<commit_message>
Atualização automática: reparaveis (24/09/2026 12:50)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
@@ -4940,7 +4940,7 @@
         <v>1353</v>
       </c>
       <c r="I2">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="K2" t="s">
         <v>1356</v>
@@ -4978,7 +4978,7 @@
         <v>1353</v>
       </c>
       <c r="I3">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="K3" t="s">
         <v>1357</v>
@@ -5016,7 +5016,7 @@
         <v>1353</v>
       </c>
       <c r="I4">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="K4" t="s">
         <v>1357</v>
@@ -5054,7 +5054,7 @@
         <v>1353</v>
       </c>
       <c r="I5">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="J5">
         <v>279</v>
@@ -5098,7 +5098,7 @@
         <v>1353</v>
       </c>
       <c r="I6">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="J6">
         <v>153</v>
@@ -5142,7 +5142,7 @@
         <v>1353</v>
       </c>
       <c r="I7">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="J7">
         <v>112</v>
@@ -5218,7 +5218,7 @@
         <v>1353</v>
       </c>
       <c r="I9">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="J9">
         <v>362</v>
@@ -5265,7 +5265,7 @@
         <v>1353</v>
       </c>
       <c r="I10">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="J10">
         <v>378</v>
@@ -5312,7 +5312,7 @@
         <v>1353</v>
       </c>
       <c r="I11">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="J11">
         <v>112</v>
@@ -5359,7 +5359,7 @@
         <v>1353</v>
       </c>
       <c r="I12">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="J12">
         <v>124</v>
@@ -5432,7 +5432,7 @@
         <v>1353</v>
       </c>
       <c r="I14">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="J14">
         <v>64</v>
@@ -5476,7 +5476,7 @@
         <v>1353</v>
       </c>
       <c r="I15">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="K15" t="s">
         <v>1359</v>
@@ -5514,7 +5514,7 @@
         <v>1353</v>
       </c>
       <c r="I16">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="K16" t="s">
         <v>1356</v>
@@ -5552,7 +5552,7 @@
         <v>1353</v>
       </c>
       <c r="I17">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="J17">
         <v>161</v>
@@ -5596,7 +5596,7 @@
         <v>1353</v>
       </c>
       <c r="I18">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="J18">
         <v>66</v>
@@ -5669,7 +5669,7 @@
         <v>1353</v>
       </c>
       <c r="I20">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="J20">
         <v>399</v>
@@ -5742,7 +5742,7 @@
         <v>1353</v>
       </c>
       <c r="I22">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="K22" t="s">
         <v>1360</v>
@@ -5780,7 +5780,7 @@
         <v>1353</v>
       </c>
       <c r="I23">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="J23">
         <v>229</v>
@@ -5885,7 +5885,7 @@
         <v>1353</v>
       </c>
       <c r="I26">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="J26">
         <v>155</v>
@@ -5932,7 +5932,7 @@
         <v>1353</v>
       </c>
       <c r="I27">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="K27" t="s">
         <v>1360</v>
@@ -6028,7 +6028,7 @@
         <v>1353</v>
       </c>
       <c r="I30">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="J30">
         <v>209</v>
@@ -6101,7 +6101,7 @@
         <v>1353</v>
       </c>
       <c r="I32">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="K32" t="s">
         <v>1356</v>
@@ -6310,7 +6310,7 @@
         <v>1353</v>
       </c>
       <c r="I39">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="K39" t="s">
         <v>1361</v>
@@ -6345,7 +6345,7 @@
         <v>1353</v>
       </c>
       <c r="I40">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="K40" t="s">
         <v>1359</v>
@@ -6476,7 +6476,7 @@
         <v>1353</v>
       </c>
       <c r="I44">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="J44">
         <v>87</v>
@@ -6523,7 +6523,7 @@
         <v>1353</v>
       </c>
       <c r="I45">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="J45">
         <v>331</v>
@@ -6570,7 +6570,7 @@
         <v>1353</v>
       </c>
       <c r="I46">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="K46" t="s">
         <v>1360</v>
@@ -6608,7 +6608,7 @@
         <v>1353</v>
       </c>
       <c r="I47">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="J47">
         <v>344</v>
@@ -6655,7 +6655,7 @@
         <v>1353</v>
       </c>
       <c r="I48">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="K48" t="s">
         <v>1360</v>
@@ -6722,7 +6722,7 @@
         <v>1353</v>
       </c>
       <c r="I50">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="K50" t="s">
         <v>1360</v>
@@ -6789,7 +6789,7 @@
         <v>1353</v>
       </c>
       <c r="I52">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="K52" t="s">
         <v>1356</v>
@@ -6827,7 +6827,7 @@
         <v>1353</v>
       </c>
       <c r="I53">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="K53" t="s">
         <v>1357</v>
@@ -6865,7 +6865,7 @@
         <v>1353</v>
       </c>
       <c r="I54">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="K54" t="s">
         <v>1357</v>
@@ -6961,7 +6961,7 @@
         <v>1353</v>
       </c>
       <c r="I57">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="K57" t="s">
         <v>1360</v>
@@ -7144,7 +7144,7 @@
         <v>1353</v>
       </c>
       <c r="I63">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="J63">
         <v>293</v>
@@ -7191,7 +7191,7 @@
         <v>1353</v>
       </c>
       <c r="I64">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="J64">
         <v>320</v>
@@ -7380,7 +7380,7 @@
         <v>1353</v>
       </c>
       <c r="I70">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="J70">
         <v>429</v>
@@ -7424,7 +7424,7 @@
         <v>1353</v>
       </c>
       <c r="I71">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="J71">
         <v>429</v>
@@ -7497,7 +7497,7 @@
         <v>1353</v>
       </c>
       <c r="I73">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="K73" t="s">
         <v>1356</v>
@@ -7564,7 +7564,7 @@
         <v>1353</v>
       </c>
       <c r="I75">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="J75">
         <v>429</v>
@@ -7608,7 +7608,7 @@
         <v>1353</v>
       </c>
       <c r="I76">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="K76" t="s">
         <v>1363</v>
@@ -7701,7 +7701,7 @@
         <v>1353</v>
       </c>
       <c r="I79">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="K79" t="s">
         <v>1363</v>
@@ -7736,7 +7736,7 @@
         <v>1353</v>
       </c>
       <c r="I80">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="J80">
         <v>429</v>
@@ -7809,7 +7809,7 @@
         <v>1353</v>
       </c>
       <c r="I82">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="K82" t="s">
         <v>1360</v>
@@ -7876,7 +7876,7 @@
         <v>1353</v>
       </c>
       <c r="I84">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="J84">
         <v>40</v>
@@ -7923,7 +7923,7 @@
         <v>1353</v>
       </c>
       <c r="I85">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="K85" t="s">
         <v>1357</v>
@@ -7961,7 +7961,7 @@
         <v>1353</v>
       </c>
       <c r="I86">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="K86" t="s">
         <v>1357</v>
@@ -7999,7 +7999,7 @@
         <v>1353</v>
       </c>
       <c r="I87">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="J87">
         <v>-16</v>
@@ -8122,7 +8122,7 @@
         <v>1353</v>
       </c>
       <c r="I90">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="K90" t="s">
         <v>1330</v>
@@ -8163,7 +8163,7 @@
         <v>1353</v>
       </c>
       <c r="I91">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="J91">
         <v>308</v>
@@ -8233,7 +8233,7 @@
         <v>1353</v>
       </c>
       <c r="I93">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="J93">
         <v>308</v>
@@ -8277,7 +8277,7 @@
         <v>1353</v>
       </c>
       <c r="I94">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="K94" t="s">
         <v>1360</v>
@@ -8315,7 +8315,7 @@
         <v>1353</v>
       </c>
       <c r="I95">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="J95">
         <v>308</v>
@@ -8359,7 +8359,7 @@
         <v>1353</v>
       </c>
       <c r="I96">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="J96">
         <v>17</v>
@@ -8406,7 +8406,7 @@
         <v>1353</v>
       </c>
       <c r="I97">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="J97">
         <v>20</v>
@@ -8453,7 +8453,7 @@
         <v>1353</v>
       </c>
       <c r="I98">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="K98" t="s">
         <v>1360</v>
@@ -8520,7 +8520,7 @@
         <v>1353</v>
       </c>
       <c r="I100">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="J100">
         <v>348</v>
@@ -8651,7 +8651,7 @@
         <v>1353</v>
       </c>
       <c r="I104">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="J104">
         <v>348</v>
@@ -8695,7 +8695,7 @@
         <v>1353</v>
       </c>
       <c r="I105">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="J105">
         <v>348</v>
@@ -8739,7 +8739,7 @@
         <v>1353</v>
       </c>
       <c r="I106">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="J106">
         <v>49</v>
@@ -8783,7 +8783,7 @@
         <v>1353</v>
       </c>
       <c r="I107">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="J107">
         <v>36</v>
@@ -8827,7 +8827,7 @@
         <v>1353</v>
       </c>
       <c r="I108">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="K108" t="s">
         <v>1357</v>
@@ -8865,7 +8865,7 @@
         <v>1353</v>
       </c>
       <c r="I109">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="K109" t="s">
         <v>1357</v>
@@ -9048,7 +9048,7 @@
         <v>1353</v>
       </c>
       <c r="I115">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="K115" t="s">
         <v>1357</v>
@@ -9086,7 +9086,7 @@
         <v>1353</v>
       </c>
       <c r="I116">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="K116" t="s">
         <v>1357</v>
@@ -9124,7 +9124,7 @@
         <v>1353</v>
       </c>
       <c r="I117">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="K117" t="s">
         <v>1357</v>
@@ -9162,7 +9162,7 @@
         <v>1353</v>
       </c>
       <c r="I118">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="K118" t="s">
         <v>1357</v>
@@ -9200,7 +9200,7 @@
         <v>1353</v>
       </c>
       <c r="I119">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="K119" t="s">
         <v>1357</v>
@@ -9238,7 +9238,7 @@
         <v>1353</v>
       </c>
       <c r="I120">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="K120" t="s">
         <v>1357</v>
@@ -9276,7 +9276,7 @@
         <v>1353</v>
       </c>
       <c r="I121">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="J121">
         <v>251</v>
@@ -9323,7 +9323,7 @@
         <v>1353</v>
       </c>
       <c r="I122">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="K122" t="s">
         <v>1357</v>
@@ -9390,7 +9390,7 @@
         <v>1353</v>
       </c>
       <c r="I124">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="K124" t="s">
         <v>1357</v>
@@ -9428,7 +9428,7 @@
         <v>1353</v>
       </c>
       <c r="I125">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="K125" t="s">
         <v>1363</v>
@@ -9524,7 +9524,7 @@
         <v>1353</v>
       </c>
       <c r="I128">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="K128" t="s">
         <v>1357</v>
@@ -9562,7 +9562,7 @@
         <v>1353</v>
       </c>
       <c r="I129">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="K129" t="s">
         <v>1356</v>
@@ -9600,7 +9600,7 @@
         <v>1353</v>
       </c>
       <c r="I130">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="J130">
         <v>47</v>
@@ -9676,7 +9676,7 @@
         <v>1353</v>
       </c>
       <c r="I132">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="J132">
         <v>145</v>
@@ -9752,7 +9752,7 @@
         <v>1353</v>
       </c>
       <c r="I134">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="K134" t="s">
         <v>1356</v>
@@ -9877,7 +9877,7 @@
         <v>1353</v>
       </c>
       <c r="I138">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="K138" t="s">
         <v>1357</v>
@@ -10176,7 +10176,7 @@
         <v>1353</v>
       </c>
       <c r="I148">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="J148">
         <v>341</v>
@@ -10220,7 +10220,7 @@
         <v>1353</v>
       </c>
       <c r="I149">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="J149">
         <v>374</v>
@@ -10267,7 +10267,7 @@
         <v>1353</v>
       </c>
       <c r="I150">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="J150">
         <v>201</v>
@@ -10343,7 +10343,7 @@
         <v>1353</v>
       </c>
       <c r="I152">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="J152">
         <v>228</v>
@@ -10457,7 +10457,7 @@
         <v>1353</v>
       </c>
       <c r="I155">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="K155" t="s">
         <v>1363</v>
@@ -10492,7 +10492,7 @@
         <v>1353</v>
       </c>
       <c r="I156">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="K156" t="s">
         <v>1357</v>
@@ -10530,7 +10530,7 @@
         <v>1353</v>
       </c>
       <c r="I157">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="J157">
         <v>371</v>
@@ -10574,7 +10574,7 @@
         <v>1353</v>
       </c>
       <c r="I158">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="J158">
         <v>52</v>
@@ -10618,7 +10618,7 @@
         <v>1353</v>
       </c>
       <c r="I159">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="K159" t="s">
         <v>1357</v>
@@ -10656,7 +10656,7 @@
         <v>1353</v>
       </c>
       <c r="I160">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="K160" t="s">
         <v>1357</v>
@@ -10694,7 +10694,7 @@
         <v>1353</v>
       </c>
       <c r="I161">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="J161">
         <v>55</v>
@@ -10741,7 +10741,7 @@
         <v>1353</v>
       </c>
       <c r="I162">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="J162">
         <v>42</v>
@@ -10788,7 +10788,7 @@
         <v>1353</v>
       </c>
       <c r="I163">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="J163">
         <v>42</v>
@@ -10835,7 +10835,7 @@
         <v>1355</v>
       </c>
       <c r="I164">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="O164" t="s">
         <v>1469</v>
@@ -10972,7 +10972,7 @@
         <v>1353</v>
       </c>
       <c r="I168">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="K168" t="s">
         <v>1360</v>
@@ -11013,7 +11013,7 @@
         <v>1353</v>
       </c>
       <c r="I169">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="K169" t="s">
         <v>1330</v>
@@ -11089,7 +11089,7 @@
         <v>1353</v>
       </c>
       <c r="I171">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="K171" t="s">
         <v>1357</v>
@@ -11226,7 +11226,7 @@
         <v>1353</v>
       </c>
       <c r="I175">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="J175">
         <v>205</v>
@@ -11273,7 +11273,7 @@
         <v>1353</v>
       </c>
       <c r="I176">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="K176" t="s">
         <v>1357</v>
@@ -11311,7 +11311,7 @@
         <v>1353</v>
       </c>
       <c r="I177">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="J177">
         <v>44</v>
@@ -11358,7 +11358,7 @@
         <v>1353</v>
       </c>
       <c r="I178">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="K178" t="s">
         <v>1356</v>
@@ -11425,7 +11425,7 @@
         <v>1353</v>
       </c>
       <c r="I180">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="K180" t="s">
         <v>1356</v>
@@ -11521,7 +11521,7 @@
         <v>1353</v>
       </c>
       <c r="I183">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="K183" t="s">
         <v>1357</v>
@@ -11559,7 +11559,7 @@
         <v>1353</v>
       </c>
       <c r="I184">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="K184" t="s">
         <v>1363</v>
@@ -11594,7 +11594,7 @@
         <v>1353</v>
       </c>
       <c r="I185">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="K185" t="s">
         <v>1357</v>
@@ -11632,7 +11632,7 @@
         <v>1353</v>
       </c>
       <c r="I186">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="K186" t="s">
         <v>1357</v>
@@ -11670,7 +11670,7 @@
         <v>1353</v>
       </c>
       <c r="I187">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="J187">
         <v>75</v>
@@ -11717,7 +11717,7 @@
         <v>1353</v>
       </c>
       <c r="I188">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="J188">
         <v>40</v>
@@ -11764,7 +11764,7 @@
         <v>1353</v>
       </c>
       <c r="I189">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="J189">
         <v>155</v>
@@ -11808,7 +11808,7 @@
         <v>1353</v>
       </c>
       <c r="I190">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="J190">
         <v>107</v>
@@ -11852,7 +11852,7 @@
         <v>1353</v>
       </c>
       <c r="I191">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="J191">
         <v>5</v>
@@ -11896,7 +11896,7 @@
         <v>1353</v>
       </c>
       <c r="I192">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="K192" t="s">
         <v>1357</v>
@@ -11934,7 +11934,7 @@
         <v>1353</v>
       </c>
       <c r="I193">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="K193" t="s">
         <v>1362</v>
@@ -12001,7 +12001,7 @@
         <v>1353</v>
       </c>
       <c r="I195">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="J195">
         <v>186</v>
@@ -12132,7 +12132,7 @@
         <v>1353</v>
       </c>
       <c r="I199">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="J199">
         <v>70</v>
@@ -12176,7 +12176,7 @@
         <v>1353</v>
       </c>
       <c r="I200">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="J200">
         <v>170</v>
@@ -12220,7 +12220,7 @@
         <v>1353</v>
       </c>
       <c r="I201">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="K201" t="s">
         <v>1357</v>
@@ -12258,7 +12258,7 @@
         <v>1353</v>
       </c>
       <c r="I202">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="K202" t="s">
         <v>1357</v>
@@ -12337,7 +12337,7 @@
         <v>1353</v>
       </c>
       <c r="I204">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="K204" t="s">
         <v>1356</v>
@@ -12375,7 +12375,7 @@
         <v>1353</v>
       </c>
       <c r="I205">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="K205" t="s">
         <v>1356</v>
@@ -12442,7 +12442,7 @@
         <v>1353</v>
       </c>
       <c r="I207">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="J207">
         <v>167</v>
@@ -12486,7 +12486,7 @@
         <v>1353</v>
       </c>
       <c r="I208">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="J208">
         <v>45</v>
@@ -12530,7 +12530,7 @@
         <v>1353</v>
       </c>
       <c r="I209">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="J209">
         <v>191</v>
@@ -12574,7 +12574,7 @@
         <v>1353</v>
       </c>
       <c r="I210">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="K210" t="s">
         <v>1360</v>
@@ -12670,7 +12670,7 @@
         <v>1353</v>
       </c>
       <c r="I213">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="K213" t="s">
         <v>1357</v>
@@ -12708,7 +12708,7 @@
         <v>1353</v>
       </c>
       <c r="I214">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="J214">
         <v>14</v>
@@ -12755,7 +12755,7 @@
         <v>1353</v>
       </c>
       <c r="I215">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="K215" t="s">
         <v>1357</v>
@@ -12822,7 +12822,7 @@
         <v>1353</v>
       </c>
       <c r="I217">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="J217">
         <v>42</v>
@@ -12866,7 +12866,7 @@
         <v>1353</v>
       </c>
       <c r="I218">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="J218">
         <v>166</v>
@@ -12954,7 +12954,7 @@
         <v>1353</v>
       </c>
       <c r="I220">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="J220">
         <v>154</v>
@@ -13112,7 +13112,7 @@
         <v>1353</v>
       </c>
       <c r="I224">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="J224">
         <v>204</v>
@@ -13267,7 +13267,7 @@
         <v>1353</v>
       </c>
       <c r="I228">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="J228">
         <v>204</v>
@@ -13346,7 +13346,7 @@
         <v>1353</v>
       </c>
       <c r="I230">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="J230">
         <v>197</v>
@@ -13390,7 +13390,7 @@
         <v>1353</v>
       </c>
       <c r="I231">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="J231">
         <v>35</v>
@@ -13492,7 +13492,7 @@
         <v>1353</v>
       </c>
       <c r="I234">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="J234">
         <v>35</v>
@@ -13539,7 +13539,7 @@
         <v>1353</v>
       </c>
       <c r="I235">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="J235">
         <v>35</v>
@@ -13586,7 +13586,7 @@
         <v>1353</v>
       </c>
       <c r="I236">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="J236">
         <v>86</v>
@@ -13703,7 +13703,7 @@
         <v>1353</v>
       </c>
       <c r="I239">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="K239" t="s">
         <v>1330</v>
@@ -13802,7 +13802,7 @@
         <v>1353</v>
       </c>
       <c r="I242">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="K242" t="s">
         <v>1356</v>
@@ -13869,7 +13869,7 @@
         <v>1353</v>
       </c>
       <c r="I244">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="J244">
         <v>15</v>
@@ -13910,7 +13910,7 @@
         <v>1353</v>
       </c>
       <c r="I245">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="J245">
         <v>15</v>
@@ -14053,7 +14053,7 @@
         <v>1353</v>
       </c>
       <c r="I249">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="K249" t="s">
         <v>1357</v>
@@ -14187,7 +14187,7 @@
         <v>1353</v>
       </c>
       <c r="I253">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="J253">
         <v>162</v>
@@ -14231,7 +14231,7 @@
         <v>1353</v>
       </c>
       <c r="I254">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="K254" t="s">
         <v>1360</v>
@@ -14269,7 +14269,7 @@
         <v>1353</v>
       </c>
       <c r="I255">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="J255">
         <v>72</v>
@@ -14313,7 +14313,7 @@
         <v>1353</v>
       </c>
       <c r="I256">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="J256">
         <v>23</v>
@@ -14415,7 +14415,7 @@
         <v>1353</v>
       </c>
       <c r="I259">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="J259">
         <v>72</v>
@@ -14459,7 +14459,7 @@
         <v>1353</v>
       </c>
       <c r="I260">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="J260">
         <v>84</v>
@@ -14503,7 +14503,7 @@
         <v>1353</v>
       </c>
       <c r="I261">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="J261">
         <v>162</v>
@@ -14620,7 +14620,7 @@
         <v>1353</v>
       </c>
       <c r="I264">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="J264">
         <v>162</v>
@@ -14664,7 +14664,7 @@
         <v>1353</v>
       </c>
       <c r="I265">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="J265">
         <v>162</v>
@@ -14708,7 +14708,7 @@
         <v>1353</v>
       </c>
       <c r="I266">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="J266">
         <v>84</v>
@@ -14752,7 +14752,7 @@
         <v>1353</v>
       </c>
       <c r="I267">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="K267" t="s">
         <v>1360</v>
@@ -14790,7 +14790,7 @@
         <v>1353</v>
       </c>
       <c r="I268">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="K268" t="s">
         <v>1357</v>
@@ -14825,7 +14825,7 @@
         <v>1353</v>
       </c>
       <c r="I269">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="K269" t="s">
         <v>1357</v>
@@ -14863,7 +14863,7 @@
         <v>1353</v>
       </c>
       <c r="I270">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="K270" t="s">
         <v>1360</v>
@@ -14901,7 +14901,7 @@
         <v>1353</v>
       </c>
       <c r="I271">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="K271" t="s">
         <v>1360</v>
@@ -15079,7 +15079,7 @@
         <v>1353</v>
       </c>
       <c r="I276">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="K276" t="s">
         <v>1361</v>
@@ -15117,7 +15117,7 @@
         <v>1353</v>
       </c>
       <c r="I277">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="K277" t="s">
         <v>1357</v>
@@ -15155,7 +15155,7 @@
         <v>1353</v>
       </c>
       <c r="I278">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="J278">
         <v>148</v>
@@ -15199,7 +15199,7 @@
         <v>1353</v>
       </c>
       <c r="I279">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="K279" t="s">
         <v>1359</v>
@@ -15240,7 +15240,7 @@
         <v>1353</v>
       </c>
       <c r="I280">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="K280" t="s">
         <v>1357</v>
@@ -15278,7 +15278,7 @@
         <v>1353</v>
       </c>
       <c r="I281">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="K281" t="s">
         <v>1357</v>
@@ -15319,7 +15319,7 @@
         <v>1353</v>
       </c>
       <c r="I282">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="K282" t="s">
         <v>1357</v>
@@ -15502,7 +15502,7 @@
         <v>1353</v>
       </c>
       <c r="I288">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="J288">
         <v>28</v>
@@ -15575,7 +15575,7 @@
         <v>1353</v>
       </c>
       <c r="I290">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="J290">
         <v>20</v>
@@ -15619,7 +15619,7 @@
         <v>1353</v>
       </c>
       <c r="I291">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="J291">
         <v>20</v>
@@ -15663,7 +15663,7 @@
         <v>1353</v>
       </c>
       <c r="I292">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="K292" t="s">
         <v>1360</v>
@@ -15701,7 +15701,7 @@
         <v>1353</v>
       </c>
       <c r="I293">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="K293" t="s">
         <v>1361</v>
@@ -15739,7 +15739,7 @@
         <v>1353</v>
       </c>
       <c r="I294">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="K294" t="s">
         <v>1366</v>
@@ -15774,7 +15774,7 @@
         <v>1353</v>
       </c>
       <c r="I295">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="K295" t="s">
         <v>1366</v>
@@ -15809,7 +15809,7 @@
         <v>1353</v>
       </c>
       <c r="I296">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="K296" t="s">
         <v>1366</v>
@@ -15882,7 +15882,7 @@
         <v>1353</v>
       </c>
       <c r="I298">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J298">
         <v>58</v>
@@ -15923,7 +15923,7 @@
         <v>1353</v>
       </c>
       <c r="I299">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J299">
         <v>100</v>
@@ -15967,7 +15967,7 @@
         <v>1353</v>
       </c>
       <c r="I300">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J300">
         <v>86</v>
@@ -16011,7 +16011,7 @@
         <v>1353</v>
       </c>
       <c r="I301">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J301">
         <v>102</v>
@@ -16055,7 +16055,7 @@
         <v>1353</v>
       </c>
       <c r="I302">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="K302" t="s">
         <v>1360</v>
@@ -16093,7 +16093,7 @@
         <v>1353</v>
       </c>
       <c r="I303">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="K303" t="s">
         <v>1357</v>
@@ -16131,7 +16131,7 @@
         <v>1353</v>
       </c>
       <c r="I304">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="K304" t="s">
         <v>1360</v>
@@ -16169,7 +16169,7 @@
         <v>1353</v>
       </c>
       <c r="I305">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J305">
         <v>35</v>
@@ -16213,7 +16213,7 @@
         <v>1353</v>
       </c>
       <c r="I306">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J306">
         <v>31</v>
@@ -16301,7 +16301,7 @@
         <v>1353</v>
       </c>
       <c r="I308">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="K308" t="s">
         <v>1356</v>
@@ -16377,7 +16377,7 @@
         <v>1353</v>
       </c>
       <c r="I310">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J310">
         <v>107</v>
@@ -16421,7 +16421,7 @@
         <v>1353</v>
       </c>
       <c r="I311">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="K311" t="s">
         <v>1356</v>
@@ -16611,7 +16611,7 @@
         <v>1353</v>
       </c>
       <c r="I316">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="K316" t="s">
         <v>1357</v>
@@ -16754,7 +16754,7 @@
         <v>1353</v>
       </c>
       <c r="I320">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="K320" t="s">
         <v>1361</v>
@@ -16792,7 +16792,7 @@
         <v>1353</v>
       </c>
       <c r="I321">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="K321" t="s">
         <v>1357</v>
@@ -16830,7 +16830,7 @@
         <v>1353</v>
       </c>
       <c r="I322">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J322">
         <v>57</v>
@@ -16944,7 +16944,7 @@
         <v>1353</v>
       </c>
       <c r="I325">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J325">
         <v>57</v>
@@ -17026,7 +17026,7 @@
         <v>1353</v>
       </c>
       <c r="I327">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J327">
         <v>57</v>
@@ -17070,7 +17070,7 @@
         <v>1353</v>
       </c>
       <c r="I328">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J328">
         <v>57</v>
@@ -17114,7 +17114,7 @@
         <v>1353</v>
       </c>
       <c r="I329">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J329">
         <v>57</v>
@@ -17158,7 +17158,7 @@
         <v>1353</v>
       </c>
       <c r="I330">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J330">
         <v>57</v>
@@ -17202,7 +17202,7 @@
         <v>1353</v>
       </c>
       <c r="I331">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="K331" t="s">
         <v>1356</v>
@@ -17240,7 +17240,7 @@
         <v>1353</v>
       </c>
       <c r="I332">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="K332" t="s">
         <v>1357</v>
@@ -17278,7 +17278,7 @@
         <v>1353</v>
       </c>
       <c r="I333">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J333">
         <v>100</v>
@@ -17322,7 +17322,7 @@
         <v>1353</v>
       </c>
       <c r="I334">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="K334" t="s">
         <v>1357</v>
@@ -17398,7 +17398,7 @@
         <v>1353</v>
       </c>
       <c r="I336">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="J336">
         <v>28</v>
@@ -17480,7 +17480,7 @@
         <v>1353</v>
       </c>
       <c r="I338">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="J338">
         <v>12</v>
@@ -17553,7 +17553,7 @@
         <v>1353</v>
       </c>
       <c r="I340">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="J340">
         <v>98</v>
@@ -17594,7 +17594,7 @@
         <v>1353</v>
       </c>
       <c r="I341">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="J341">
         <v>90</v>
@@ -17635,7 +17635,7 @@
         <v>1353</v>
       </c>
       <c r="I342">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="K342" t="s">
         <v>1356</v>
@@ -17749,7 +17749,7 @@
         <v>1353</v>
       </c>
       <c r="I345">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="K345" t="s">
         <v>1356</v>
@@ -17825,7 +17825,7 @@
         <v>1353</v>
       </c>
       <c r="I347">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="J347">
         <v>18</v>
@@ -17872,7 +17872,7 @@
         <v>1353</v>
       </c>
       <c r="I348">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="J348">
         <v>14</v>
@@ -17916,7 +17916,7 @@
         <v>1353</v>
       </c>
       <c r="I349">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="K349" t="s">
         <v>1361</v>
@@ -17954,7 +17954,7 @@
         <v>1353</v>
       </c>
       <c r="I350">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="J350">
         <v>46</v>
@@ -17992,7 +17992,7 @@
         <v>1353</v>
       </c>
       <c r="I351">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="J351">
         <v>82</v>
@@ -18036,7 +18036,7 @@
         <v>1353</v>
       </c>
       <c r="I352">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="J352">
         <v>78</v>
@@ -18080,7 +18080,7 @@
         <v>1353</v>
       </c>
       <c r="I353">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="J353">
         <v>83</v>
@@ -18124,7 +18124,7 @@
         <v>1353</v>
       </c>
       <c r="I354">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="K354" t="s">
         <v>1360</v>
@@ -18162,7 +18162,7 @@
         <v>1353</v>
       </c>
       <c r="I355">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="J355">
         <v>8</v>
@@ -18244,7 +18244,7 @@
         <v>1353</v>
       </c>
       <c r="I357">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="J357">
         <v>85</v>
@@ -18367,7 +18367,7 @@
         <v>1353</v>
       </c>
       <c r="I360">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="J360">
         <v>83</v>
@@ -18414,7 +18414,7 @@
         <v>1353</v>
       </c>
       <c r="I361">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="J361">
         <v>83</v>
@@ -18458,7 +18458,7 @@
         <v>1353</v>
       </c>
       <c r="I362">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="K362" t="s">
         <v>1360</v>
@@ -18496,7 +18496,7 @@
         <v>1353</v>
       </c>
       <c r="I363">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="K363" t="s">
         <v>1360</v>
@@ -18534,7 +18534,7 @@
         <v>1353</v>
       </c>
       <c r="I364">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="J364">
         <v>83</v>
@@ -18578,7 +18578,7 @@
         <v>1353</v>
       </c>
       <c r="I365">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="J365">
         <v>15</v>
@@ -18619,7 +18619,7 @@
         <v>1353</v>
       </c>
       <c r="I366">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="J366">
         <v>77</v>
@@ -18663,7 +18663,7 @@
         <v>1353</v>
       </c>
       <c r="I367">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="J367">
         <v>77</v>
@@ -18707,7 +18707,7 @@
         <v>1353</v>
       </c>
       <c r="I368">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="J368">
         <v>77</v>
@@ -18751,7 +18751,7 @@
         <v>1353</v>
       </c>
       <c r="I369">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="K369" t="s">
         <v>1360</v>
@@ -18789,7 +18789,7 @@
         <v>1353</v>
       </c>
       <c r="I370">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="K370" t="s">
         <v>1360</v>
@@ -18827,7 +18827,7 @@
         <v>1353</v>
       </c>
       <c r="I371">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="J371">
         <v>16</v>
@@ -18915,7 +18915,7 @@
         <v>1353</v>
       </c>
       <c r="I373">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="K373" t="s">
         <v>1356</v>
@@ -18953,7 +18953,7 @@
         <v>1353</v>
       </c>
       <c r="I374">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="K374" t="s">
         <v>1356</v>
@@ -18991,7 +18991,7 @@
         <v>1353</v>
       </c>
       <c r="I375">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="J375">
         <v>94</v>
@@ -19032,7 +19032,7 @@
         <v>1353</v>
       </c>
       <c r="I376">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="K376" t="s">
         <v>1360</v>
@@ -19111,7 +19111,7 @@
         <v>1353</v>
       </c>
       <c r="I378">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="K378" t="s">
         <v>1360</v>
@@ -19149,7 +19149,7 @@
         <v>1353</v>
       </c>
       <c r="I379">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="J379">
         <v>20</v>
@@ -19193,7 +19193,7 @@
         <v>1353</v>
       </c>
       <c r="I380">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="J380">
         <v>94</v>
@@ -19237,7 +19237,7 @@
         <v>1353</v>
       </c>
       <c r="I381">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="K381" t="s">
         <v>1360</v>
@@ -19275,7 +19275,7 @@
         <v>1353</v>
       </c>
       <c r="I382">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="K382" t="s">
         <v>1360</v>
@@ -19313,7 +19313,7 @@
         <v>1353</v>
       </c>
       <c r="I383">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="J383">
         <v>71</v>
@@ -19357,7 +19357,7 @@
         <v>1353</v>
       </c>
       <c r="I384">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="K384" t="s">
         <v>1357</v>
@@ -19395,7 +19395,7 @@
         <v>1353</v>
       </c>
       <c r="I385">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="J385">
         <v>102</v>
@@ -19442,7 +19442,7 @@
         <v>1353</v>
       </c>
       <c r="I386">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="K386" t="s">
         <v>1360</v>
@@ -19480,7 +19480,7 @@
         <v>1353</v>
       </c>
       <c r="I387">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="K387" t="s">
         <v>1360</v>
@@ -19518,7 +19518,7 @@
         <v>1353</v>
       </c>
       <c r="I388">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="J388">
         <v>-85</v>
@@ -19562,7 +19562,7 @@
         <v>1353</v>
       </c>
       <c r="I389">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="K389" t="s">
         <v>1361</v>
@@ -19720,7 +19720,7 @@
         <v>1353</v>
       </c>
       <c r="I393">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="J393">
         <v>20</v>
@@ -20016,7 +20016,7 @@
         <v>1353</v>
       </c>
       <c r="I400">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="K400" t="s">
         <v>1360</v>
@@ -20092,7 +20092,7 @@
         <v>1353</v>
       </c>
       <c r="I402">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="K402" t="s">
         <v>1360</v>
@@ -20130,7 +20130,7 @@
         <v>1353</v>
       </c>
       <c r="I403">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="J403">
         <v>83</v>
@@ -20174,7 +20174,7 @@
         <v>1353</v>
       </c>
       <c r="I404">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="K404" t="s">
         <v>1360</v>
@@ -20244,7 +20244,7 @@
         <v>1353</v>
       </c>
       <c r="I406">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="Q406" t="b">
         <v>1</v>
@@ -20276,7 +20276,7 @@
         <v>1353</v>
       </c>
       <c r="I407">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="Q407" t="b">
         <v>1</v>
@@ -20308,7 +20308,7 @@
         <v>1353</v>
       </c>
       <c r="I408">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="Q408" t="b">
         <v>1</v>
@@ -20340,7 +20340,7 @@
         <v>1353</v>
       </c>
       <c r="I409">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="Q409" t="b">
         <v>1</v>
@@ -20372,7 +20372,7 @@
         <v>1353</v>
       </c>
       <c r="I410">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="Q410" t="b">
         <v>1</v>
@@ -20404,7 +20404,7 @@
         <v>1353</v>
       </c>
       <c r="I411">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="Q411" t="b">
         <v>1</v>
@@ -20436,7 +20436,7 @@
         <v>1353</v>
       </c>
       <c r="I412">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="Q412" t="b">
         <v>1</v>
@@ -20468,7 +20468,7 @@
         <v>1353</v>
       </c>
       <c r="I413">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="Q413" t="b">
         <v>1</v>
@@ -20558,7 +20558,7 @@
         <v>1353</v>
       </c>
       <c r="I416">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="Q416" t="b">
         <v>1</v>
@@ -20648,7 +20648,7 @@
         <v>1353</v>
       </c>
       <c r="I419">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="Q419" t="b">
         <v>1</v>
@@ -20680,7 +20680,7 @@
         <v>1353</v>
       </c>
       <c r="I420">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="Q420" t="b">
         <v>1</v>
@@ -20712,7 +20712,7 @@
         <v>1353</v>
       </c>
       <c r="I421">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="Q421" t="b">
         <v>1</v>
@@ -20744,7 +20744,7 @@
         <v>1353</v>
       </c>
       <c r="I422">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="Q422" t="b">
         <v>1</v>
@@ -20776,7 +20776,7 @@
         <v>1353</v>
       </c>
       <c r="I423">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="Q423" t="b">
         <v>1</v>
@@ -20808,7 +20808,7 @@
         <v>1353</v>
       </c>
       <c r="I424">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="Q424" t="b">
         <v>1</v>
@@ -20840,7 +20840,7 @@
         <v>1353</v>
       </c>
       <c r="I425">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="Q425" t="b">
         <v>1</v>
@@ -20872,7 +20872,7 @@
         <v>1353</v>
       </c>
       <c r="I426">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="Q426" t="b">
         <v>1</v>
@@ -20904,7 +20904,7 @@
         <v>1353</v>
       </c>
       <c r="I427">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="Q427" t="b">
         <v>1</v>
@@ -20994,7 +20994,7 @@
         <v>1353</v>
       </c>
       <c r="I430">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="Q430" t="b">
         <v>1</v>
@@ -21026,7 +21026,7 @@
         <v>1353</v>
       </c>
       <c r="I431">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="Q431" t="b">
         <v>1</v>
@@ -21058,7 +21058,7 @@
         <v>1353</v>
       </c>
       <c r="I432">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="Q432" t="b">
         <v>1</v>
@@ -21090,7 +21090,7 @@
         <v>1353</v>
       </c>
       <c r="I433">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="Q433" t="b">
         <v>1</v>
@@ -21122,7 +21122,7 @@
         <v>1353</v>
       </c>
       <c r="I434">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="Q434" t="b">
         <v>1</v>
@@ -21154,7 +21154,7 @@
         <v>1353</v>
       </c>
       <c r="I435">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="Q435" t="b">
         <v>1</v>
@@ -21186,7 +21186,7 @@
         <v>1353</v>
       </c>
       <c r="I436">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="Q436" t="b">
         <v>1</v>
@@ -21218,7 +21218,7 @@
         <v>1355</v>
       </c>
       <c r="I437">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="Q437" t="b">
         <v>1</v>
@@ -21250,7 +21250,7 @@
         <v>1355</v>
       </c>
       <c r="I438">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="Q438" t="b">
         <v>1</v>
@@ -21282,7 +21282,7 @@
         <v>1353</v>
       </c>
       <c r="I439">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q439" t="b">
         <v>1</v>
@@ -21314,7 +21314,7 @@
         <v>1353</v>
       </c>
       <c r="I440">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q440" t="b">
         <v>1</v>
@@ -21346,7 +21346,7 @@
         <v>1353</v>
       </c>
       <c r="I441">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="Q441" t="b">
         <v>1</v>
@@ -21407,7 +21407,7 @@
         <v>1353</v>
       </c>
       <c r="I443">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q443" t="b">
         <v>1</v>
@@ -21497,7 +21497,7 @@
         <v>1353</v>
       </c>
       <c r="I446">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Q446" t="b">
         <v>1</v>
@@ -21529,7 +21529,7 @@
         <v>1353</v>
       </c>
       <c r="I447">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Q447" t="b">
         <v>1</v>
@@ -21561,7 +21561,7 @@
         <v>1353</v>
       </c>
       <c r="I448">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Q448" t="b">
         <v>1</v>
@@ -21593,7 +21593,7 @@
         <v>1353</v>
       </c>
       <c r="I449">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Q449" t="b">
         <v>1</v>
@@ -21625,7 +21625,7 @@
         <v>1353</v>
       </c>
       <c r="I450">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Q450" t="b">
         <v>1</v>
@@ -21657,7 +21657,7 @@
         <v>1353</v>
       </c>
       <c r="I451">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q451" t="b">
         <v>1</v>
@@ -21689,7 +21689,7 @@
         <v>1353</v>
       </c>
       <c r="I452">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q452" t="b">
         <v>1</v>
@@ -21721,7 +21721,7 @@
         <v>1353</v>
       </c>
       <c r="I453">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q453" t="b">
         <v>1</v>
@@ -21753,7 +21753,7 @@
         <v>1353</v>
       </c>
       <c r="I454">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q454" t="b">
         <v>1</v>
@@ -21785,7 +21785,7 @@
         <v>1353</v>
       </c>
       <c r="I455">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q455" t="b">
         <v>1</v>
@@ -21817,7 +21817,7 @@
         <v>1353</v>
       </c>
       <c r="I456">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q456" t="b">
         <v>1</v>
@@ -21849,7 +21849,7 @@
         <v>1353</v>
       </c>
       <c r="I457">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q457" t="b">
         <v>1</v>
@@ -21881,7 +21881,7 @@
         <v>1353</v>
       </c>
       <c r="I458">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q458" t="b">
         <v>1</v>
@@ -21913,7 +21913,7 @@
         <v>1353</v>
       </c>
       <c r="I459">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="Q459" t="b">
         <v>1</v>
@@ -21945,7 +21945,7 @@
         <v>1353</v>
       </c>
       <c r="I460">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="Q460" t="b">
         <v>1</v>
@@ -21977,7 +21977,7 @@
         <v>1353</v>
       </c>
       <c r="I461">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="Q461" t="b">
         <v>1</v>
@@ -22009,7 +22009,7 @@
         <v>1353</v>
       </c>
       <c r="I462">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="Q462" t="b">
         <v>1</v>
@@ -22041,7 +22041,7 @@
         <v>1353</v>
       </c>
       <c r="I463">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="Q463" t="b">
         <v>1</v>
@@ -22073,7 +22073,7 @@
         <v>1353</v>
       </c>
       <c r="I464">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q464" t="b">
         <v>1</v>
@@ -22105,7 +22105,7 @@
         <v>1353</v>
       </c>
       <c r="I465">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q465" t="b">
         <v>1</v>
@@ -22137,7 +22137,7 @@
         <v>1353</v>
       </c>
       <c r="I466">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q466" t="b">
         <v>1</v>
@@ -22169,7 +22169,7 @@
         <v>1353</v>
       </c>
       <c r="I467">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q467" t="b">
         <v>1</v>
@@ -22201,7 +22201,7 @@
         <v>1353</v>
       </c>
       <c r="I468">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q468" t="b">
         <v>1</v>
@@ -22233,7 +22233,7 @@
         <v>1353</v>
       </c>
       <c r="I469">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q469" t="b">
         <v>1</v>
@@ -22294,7 +22294,7 @@
         <v>1353</v>
       </c>
       <c r="I471">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q471" t="b">
         <v>1</v>
@@ -22326,7 +22326,7 @@
         <v>1353</v>
       </c>
       <c r="I472">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q472" t="b">
         <v>1</v>
@@ -22358,7 +22358,7 @@
         <v>1353</v>
       </c>
       <c r="I473">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q473" t="b">
         <v>1</v>
@@ -22390,7 +22390,7 @@
         <v>1353</v>
       </c>
       <c r="I474">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q474" t="b">
         <v>1</v>
@@ -22422,7 +22422,7 @@
         <v>1353</v>
       </c>
       <c r="I475">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q475" t="b">
         <v>1</v>
@@ -22454,7 +22454,7 @@
         <v>1353</v>
       </c>
       <c r="I476">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q476" t="b">
         <v>1</v>
@@ -22486,7 +22486,7 @@
         <v>1353</v>
       </c>
       <c r="I477">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q477" t="b">
         <v>1</v>
@@ -22518,7 +22518,7 @@
         <v>1353</v>
       </c>
       <c r="I478">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q478" t="b">
         <v>1</v>
@@ -22550,7 +22550,7 @@
         <v>1353</v>
       </c>
       <c r="I479">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q479" t="b">
         <v>1</v>
@@ -22582,7 +22582,7 @@
         <v>1353</v>
       </c>
       <c r="I480">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q480" t="b">
         <v>1</v>
@@ -22614,7 +22614,7 @@
         <v>1353</v>
       </c>
       <c r="I481">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q481" t="b">
         <v>1</v>
@@ -22646,7 +22646,7 @@
         <v>1353</v>
       </c>
       <c r="I482">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q482" t="b">
         <v>1</v>
@@ -22678,7 +22678,7 @@
         <v>1353</v>
       </c>
       <c r="I483">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q483" t="b">
         <v>1</v>
@@ -22710,7 +22710,7 @@
         <v>1353</v>
       </c>
       <c r="I484">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q484" t="b">
         <v>1</v>
@@ -22742,7 +22742,7 @@
         <v>1353</v>
       </c>
       <c r="I485">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q485" t="b">
         <v>1</v>
@@ -22774,7 +22774,7 @@
         <v>1353</v>
       </c>
       <c r="I486">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q486" t="b">
         <v>1</v>
@@ -22806,7 +22806,7 @@
         <v>1353</v>
       </c>
       <c r="I487">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q487" t="b">
         <v>1</v>
@@ -22838,7 +22838,7 @@
         <v>1353</v>
       </c>
       <c r="I488">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q488" t="b">
         <v>1</v>
@@ -22870,7 +22870,7 @@
         <v>1353</v>
       </c>
       <c r="I489">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q489" t="b">
         <v>1</v>
@@ -22902,7 +22902,7 @@
         <v>1353</v>
       </c>
       <c r="I490">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q490" t="b">
         <v>1</v>
@@ -22934,7 +22934,7 @@
         <v>1353</v>
       </c>
       <c r="I491">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q491" t="b">
         <v>1</v>
@@ -22966,7 +22966,7 @@
         <v>1355</v>
       </c>
       <c r="I492">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q492" t="b">
         <v>1</v>
@@ -22998,7 +22998,7 @@
         <v>1355</v>
       </c>
       <c r="I493">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q493" t="b">
         <v>1</v>
@@ -23030,7 +23030,7 @@
         <v>1355</v>
       </c>
       <c r="I494">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q494" t="b">
         <v>1</v>
@@ -23062,7 +23062,7 @@
         <v>1355</v>
       </c>
       <c r="I495">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q495" t="b">
         <v>1</v>
@@ -23094,7 +23094,7 @@
         <v>1355</v>
       </c>
       <c r="I496">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q496" t="b">
         <v>1</v>
@@ -23126,7 +23126,7 @@
         <v>1353</v>
       </c>
       <c r="I497">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q497" t="b">
         <v>1</v>
@@ -23158,7 +23158,7 @@
         <v>1353</v>
       </c>
       <c r="I498">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q498" t="b">
         <v>1</v>
@@ -23190,7 +23190,7 @@
         <v>1355</v>
       </c>
       <c r="I499">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q499" t="b">
         <v>1</v>
@@ -23222,7 +23222,7 @@
         <v>1353</v>
       </c>
       <c r="I500">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q500" t="b">
         <v>1</v>
@@ -23254,7 +23254,7 @@
         <v>1353</v>
       </c>
       <c r="I501">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q501" t="b">
         <v>1</v>
@@ -23286,7 +23286,7 @@
         <v>1353</v>
       </c>
       <c r="I502">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q502" t="b">
         <v>1</v>
@@ -23318,7 +23318,7 @@
         <v>1353</v>
       </c>
       <c r="I503">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q503" t="b">
         <v>1</v>
@@ -23350,7 +23350,7 @@
         <v>1353</v>
       </c>
       <c r="I504">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q504" t="b">
         <v>1</v>
@@ -23382,7 +23382,7 @@
         <v>1353</v>
       </c>
       <c r="I505">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q505" t="b">
         <v>1</v>
@@ -23414,7 +23414,7 @@
         <v>1353</v>
       </c>
       <c r="I506">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q506" t="b">
         <v>1</v>
@@ -23446,7 +23446,7 @@
         <v>1353</v>
       </c>
       <c r="I507">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Q507" t="b">
         <v>1</v>
@@ -23507,7 +23507,7 @@
         <v>1353</v>
       </c>
       <c r="I509">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Q509" t="b">
         <v>1</v>
@@ -23539,7 +23539,7 @@
         <v>1353</v>
       </c>
       <c r="I510">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Q510" t="b">
         <v>1</v>
@@ -23571,7 +23571,7 @@
         <v>1353</v>
       </c>
       <c r="I511">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="Q511" t="b">
         <v>1</v>
@@ -23603,7 +23603,7 @@
         <v>1353</v>
       </c>
       <c r="I512">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="Q512" t="b">
         <v>1</v>
@@ -23635,7 +23635,7 @@
         <v>1353</v>
       </c>
       <c r="I513">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Q513" t="b">
         <v>1</v>
@@ -23667,7 +23667,7 @@
         <v>1353</v>
       </c>
       <c r="I514">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Q514" t="b">
         <v>1</v>
@@ -23699,7 +23699,7 @@
         <v>1353</v>
       </c>
       <c r="I515">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Q515" t="b">
         <v>1</v>
@@ -23731,7 +23731,7 @@
         <v>1353</v>
       </c>
       <c r="I516">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Q516" t="b">
         <v>1</v>
@@ -23763,7 +23763,7 @@
         <v>1353</v>
       </c>
       <c r="I517">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Q517" t="b">
         <v>1</v>
@@ -23795,7 +23795,7 @@
         <v>1353</v>
       </c>
       <c r="I518">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Q518" t="b">
         <v>1</v>
@@ -23827,7 +23827,7 @@
         <v>1353</v>
       </c>
       <c r="I519">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q519" t="b">
         <v>1</v>
@@ -23859,7 +23859,7 @@
         <v>1353</v>
       </c>
       <c r="I520">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q520" t="b">
         <v>1</v>
@@ -23891,7 +23891,7 @@
         <v>1353</v>
       </c>
       <c r="I521">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q521" t="b">
         <v>1</v>
@@ -23923,7 +23923,7 @@
         <v>1353</v>
       </c>
       <c r="I522">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q522" t="b">
         <v>1</v>
@@ -23955,7 +23955,7 @@
         <v>1353</v>
       </c>
       <c r="I523">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q523" t="b">
         <v>1</v>
@@ -23987,7 +23987,7 @@
         <v>1353</v>
       </c>
       <c r="I524">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="Q524" t="b">
         <v>1</v>
@@ -24019,7 +24019,7 @@
         <v>1353</v>
       </c>
       <c r="I525">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="Q525" t="b">
         <v>1</v>
@@ -24051,7 +24051,7 @@
         <v>1353</v>
       </c>
       <c r="I526">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="Q526" t="b">
         <v>1</v>
@@ -24083,7 +24083,7 @@
         <v>1353</v>
       </c>
       <c r="I527">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="Q527" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: reparaveis (25/09/2026 12:50)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
@@ -4940,7 +4940,7 @@
         <v>1353</v>
       </c>
       <c r="I2">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="K2" t="s">
         <v>1356</v>
@@ -4978,7 +4978,7 @@
         <v>1353</v>
       </c>
       <c r="I3">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="K3" t="s">
         <v>1357</v>
@@ -5016,7 +5016,7 @@
         <v>1353</v>
       </c>
       <c r="I4">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="K4" t="s">
         <v>1357</v>
@@ -5054,7 +5054,7 @@
         <v>1353</v>
       </c>
       <c r="I5">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="J5">
         <v>279</v>
@@ -5098,7 +5098,7 @@
         <v>1353</v>
       </c>
       <c r="I6">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="J6">
         <v>153</v>
@@ -5142,7 +5142,7 @@
         <v>1353</v>
       </c>
       <c r="I7">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="J7">
         <v>112</v>
@@ -5218,7 +5218,7 @@
         <v>1353</v>
       </c>
       <c r="I9">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="J9">
         <v>362</v>
@@ -5265,7 +5265,7 @@
         <v>1353</v>
       </c>
       <c r="I10">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="J10">
         <v>378</v>
@@ -5312,7 +5312,7 @@
         <v>1353</v>
       </c>
       <c r="I11">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="J11">
         <v>112</v>
@@ -5359,7 +5359,7 @@
         <v>1353</v>
       </c>
       <c r="I12">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="J12">
         <v>124</v>
@@ -5432,7 +5432,7 @@
         <v>1353</v>
       </c>
       <c r="I14">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="J14">
         <v>64</v>
@@ -5476,7 +5476,7 @@
         <v>1353</v>
       </c>
       <c r="I15">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="K15" t="s">
         <v>1359</v>
@@ -5514,7 +5514,7 @@
         <v>1353</v>
       </c>
       <c r="I16">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="K16" t="s">
         <v>1356</v>
@@ -5552,7 +5552,7 @@
         <v>1353</v>
       </c>
       <c r="I17">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="J17">
         <v>161</v>
@@ -5596,7 +5596,7 @@
         <v>1353</v>
       </c>
       <c r="I18">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="J18">
         <v>66</v>
@@ -5669,7 +5669,7 @@
         <v>1353</v>
       </c>
       <c r="I20">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="J20">
         <v>399</v>
@@ -5742,7 +5742,7 @@
         <v>1353</v>
       </c>
       <c r="I22">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="K22" t="s">
         <v>1360</v>
@@ -5780,7 +5780,7 @@
         <v>1353</v>
       </c>
       <c r="I23">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="J23">
         <v>229</v>
@@ -5885,7 +5885,7 @@
         <v>1353</v>
       </c>
       <c r="I26">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="J26">
         <v>155</v>
@@ -5932,7 +5932,7 @@
         <v>1353</v>
       </c>
       <c r="I27">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="K27" t="s">
         <v>1360</v>
@@ -6028,7 +6028,7 @@
         <v>1353</v>
       </c>
       <c r="I30">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="J30">
         <v>209</v>
@@ -6101,7 +6101,7 @@
         <v>1353</v>
       </c>
       <c r="I32">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="K32" t="s">
         <v>1356</v>
@@ -6310,7 +6310,7 @@
         <v>1353</v>
       </c>
       <c r="I39">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="K39" t="s">
         <v>1361</v>
@@ -6345,7 +6345,7 @@
         <v>1353</v>
       </c>
       <c r="I40">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="K40" t="s">
         <v>1359</v>
@@ -6476,7 +6476,7 @@
         <v>1353</v>
       </c>
       <c r="I44">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="J44">
         <v>87</v>
@@ -6523,7 +6523,7 @@
         <v>1353</v>
       </c>
       <c r="I45">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="J45">
         <v>331</v>
@@ -6570,7 +6570,7 @@
         <v>1353</v>
       </c>
       <c r="I46">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="K46" t="s">
         <v>1360</v>
@@ -6608,7 +6608,7 @@
         <v>1353</v>
       </c>
       <c r="I47">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="J47">
         <v>344</v>
@@ -6655,7 +6655,7 @@
         <v>1353</v>
       </c>
       <c r="I48">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="K48" t="s">
         <v>1360</v>
@@ -6722,7 +6722,7 @@
         <v>1353</v>
       </c>
       <c r="I50">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="K50" t="s">
         <v>1360</v>
@@ -6789,7 +6789,7 @@
         <v>1353</v>
       </c>
       <c r="I52">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="K52" t="s">
         <v>1356</v>
@@ -6827,7 +6827,7 @@
         <v>1353</v>
       </c>
       <c r="I53">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="K53" t="s">
         <v>1357</v>
@@ -6865,7 +6865,7 @@
         <v>1353</v>
       </c>
       <c r="I54">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="K54" t="s">
         <v>1357</v>
@@ -6961,7 +6961,7 @@
         <v>1353</v>
       </c>
       <c r="I57">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="K57" t="s">
         <v>1360</v>
@@ -7144,7 +7144,7 @@
         <v>1353</v>
       </c>
       <c r="I63">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="J63">
         <v>293</v>
@@ -7191,7 +7191,7 @@
         <v>1353</v>
       </c>
       <c r="I64">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="J64">
         <v>320</v>
@@ -7380,7 +7380,7 @@
         <v>1353</v>
       </c>
       <c r="I70">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="J70">
         <v>429</v>
@@ -7424,7 +7424,7 @@
         <v>1353</v>
       </c>
       <c r="I71">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="J71">
         <v>429</v>
@@ -7497,7 +7497,7 @@
         <v>1353</v>
       </c>
       <c r="I73">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="K73" t="s">
         <v>1356</v>
@@ -7564,7 +7564,7 @@
         <v>1353</v>
       </c>
       <c r="I75">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="J75">
         <v>429</v>
@@ -7608,7 +7608,7 @@
         <v>1353</v>
       </c>
       <c r="I76">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="K76" t="s">
         <v>1363</v>
@@ -7701,7 +7701,7 @@
         <v>1353</v>
       </c>
       <c r="I79">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="K79" t="s">
         <v>1363</v>
@@ -7736,7 +7736,7 @@
         <v>1353</v>
       </c>
       <c r="I80">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="J80">
         <v>429</v>
@@ -7809,7 +7809,7 @@
         <v>1353</v>
       </c>
       <c r="I82">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="K82" t="s">
         <v>1360</v>
@@ -7876,7 +7876,7 @@
         <v>1353</v>
       </c>
       <c r="I84">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="J84">
         <v>40</v>
@@ -7923,7 +7923,7 @@
         <v>1353</v>
       </c>
       <c r="I85">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="K85" t="s">
         <v>1357</v>
@@ -7961,7 +7961,7 @@
         <v>1353</v>
       </c>
       <c r="I86">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="K86" t="s">
         <v>1357</v>
@@ -7999,7 +7999,7 @@
         <v>1353</v>
       </c>
       <c r="I87">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="J87">
         <v>-16</v>
@@ -8122,7 +8122,7 @@
         <v>1353</v>
       </c>
       <c r="I90">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="K90" t="s">
         <v>1330</v>
@@ -8163,7 +8163,7 @@
         <v>1353</v>
       </c>
       <c r="I91">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="J91">
         <v>308</v>
@@ -8233,7 +8233,7 @@
         <v>1353</v>
       </c>
       <c r="I93">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="J93">
         <v>308</v>
@@ -8277,7 +8277,7 @@
         <v>1353</v>
       </c>
       <c r="I94">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="K94" t="s">
         <v>1360</v>
@@ -8315,7 +8315,7 @@
         <v>1353</v>
       </c>
       <c r="I95">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="J95">
         <v>308</v>
@@ -8359,7 +8359,7 @@
         <v>1353</v>
       </c>
       <c r="I96">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="J96">
         <v>17</v>
@@ -8406,7 +8406,7 @@
         <v>1353</v>
       </c>
       <c r="I97">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="J97">
         <v>20</v>
@@ -8453,7 +8453,7 @@
         <v>1353</v>
       </c>
       <c r="I98">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="K98" t="s">
         <v>1360</v>
@@ -8520,7 +8520,7 @@
         <v>1353</v>
       </c>
       <c r="I100">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="J100">
         <v>348</v>
@@ -8651,7 +8651,7 @@
         <v>1353</v>
       </c>
       <c r="I104">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="J104">
         <v>348</v>
@@ -8695,7 +8695,7 @@
         <v>1353</v>
       </c>
       <c r="I105">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="J105">
         <v>348</v>
@@ -8739,7 +8739,7 @@
         <v>1353</v>
       </c>
       <c r="I106">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="J106">
         <v>49</v>
@@ -8783,7 +8783,7 @@
         <v>1353</v>
       </c>
       <c r="I107">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="J107">
         <v>36</v>
@@ -8827,7 +8827,7 @@
         <v>1353</v>
       </c>
       <c r="I108">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="K108" t="s">
         <v>1357</v>
@@ -8865,7 +8865,7 @@
         <v>1353</v>
       </c>
       <c r="I109">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="K109" t="s">
         <v>1357</v>
@@ -9048,7 +9048,7 @@
         <v>1353</v>
       </c>
       <c r="I115">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="K115" t="s">
         <v>1357</v>
@@ -9086,7 +9086,7 @@
         <v>1353</v>
       </c>
       <c r="I116">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="K116" t="s">
         <v>1357</v>
@@ -9124,7 +9124,7 @@
         <v>1353</v>
       </c>
       <c r="I117">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="K117" t="s">
         <v>1357</v>
@@ -9162,7 +9162,7 @@
         <v>1353</v>
       </c>
       <c r="I118">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="K118" t="s">
         <v>1357</v>
@@ -9200,7 +9200,7 @@
         <v>1353</v>
       </c>
       <c r="I119">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="K119" t="s">
         <v>1357</v>
@@ -9238,7 +9238,7 @@
         <v>1353</v>
       </c>
       <c r="I120">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="K120" t="s">
         <v>1357</v>
@@ -9276,7 +9276,7 @@
         <v>1353</v>
       </c>
       <c r="I121">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="J121">
         <v>251</v>
@@ -9323,7 +9323,7 @@
         <v>1353</v>
       </c>
       <c r="I122">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="K122" t="s">
         <v>1357</v>
@@ -9390,7 +9390,7 @@
         <v>1353</v>
       </c>
       <c r="I124">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="K124" t="s">
         <v>1357</v>
@@ -9428,7 +9428,7 @@
         <v>1353</v>
       </c>
       <c r="I125">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="K125" t="s">
         <v>1363</v>
@@ -9524,7 +9524,7 @@
         <v>1353</v>
       </c>
       <c r="I128">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="K128" t="s">
         <v>1357</v>
@@ -9562,7 +9562,7 @@
         <v>1353</v>
       </c>
       <c r="I129">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="K129" t="s">
         <v>1356</v>
@@ -9600,7 +9600,7 @@
         <v>1353</v>
       </c>
       <c r="I130">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="J130">
         <v>47</v>
@@ -9676,7 +9676,7 @@
         <v>1353</v>
       </c>
       <c r="I132">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="J132">
         <v>145</v>
@@ -9752,7 +9752,7 @@
         <v>1353</v>
       </c>
       <c r="I134">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="K134" t="s">
         <v>1356</v>
@@ -9877,7 +9877,7 @@
         <v>1353</v>
       </c>
       <c r="I138">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="K138" t="s">
         <v>1357</v>
@@ -10176,7 +10176,7 @@
         <v>1353</v>
       </c>
       <c r="I148">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="J148">
         <v>341</v>
@@ -10220,7 +10220,7 @@
         <v>1353</v>
       </c>
       <c r="I149">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="J149">
         <v>374</v>
@@ -10267,7 +10267,7 @@
         <v>1353</v>
       </c>
       <c r="I150">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="J150">
         <v>201</v>
@@ -10343,7 +10343,7 @@
         <v>1353</v>
       </c>
       <c r="I152">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="J152">
         <v>228</v>
@@ -10457,7 +10457,7 @@
         <v>1353</v>
       </c>
       <c r="I155">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="K155" t="s">
         <v>1363</v>
@@ -10492,7 +10492,7 @@
         <v>1353</v>
       </c>
       <c r="I156">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="K156" t="s">
         <v>1357</v>
@@ -10530,7 +10530,7 @@
         <v>1353</v>
       </c>
       <c r="I157">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="J157">
         <v>371</v>
@@ -10574,7 +10574,7 @@
         <v>1353</v>
       </c>
       <c r="I158">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="J158">
         <v>52</v>
@@ -10618,7 +10618,7 @@
         <v>1353</v>
       </c>
       <c r="I159">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="K159" t="s">
         <v>1357</v>
@@ -10656,7 +10656,7 @@
         <v>1353</v>
       </c>
       <c r="I160">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="K160" t="s">
         <v>1357</v>
@@ -10694,7 +10694,7 @@
         <v>1353</v>
       </c>
       <c r="I161">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="J161">
         <v>55</v>
@@ -10741,7 +10741,7 @@
         <v>1353</v>
       </c>
       <c r="I162">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="J162">
         <v>42</v>
@@ -10788,7 +10788,7 @@
         <v>1353</v>
       </c>
       <c r="I163">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="J163">
         <v>42</v>
@@ -10835,7 +10835,7 @@
         <v>1355</v>
       </c>
       <c r="I164">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="O164" t="s">
         <v>1469</v>
@@ -10972,7 +10972,7 @@
         <v>1353</v>
       </c>
       <c r="I168">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="K168" t="s">
         <v>1360</v>
@@ -11013,7 +11013,7 @@
         <v>1353</v>
       </c>
       <c r="I169">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="K169" t="s">
         <v>1330</v>
@@ -11089,7 +11089,7 @@
         <v>1353</v>
       </c>
       <c r="I171">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="K171" t="s">
         <v>1357</v>
@@ -11226,7 +11226,7 @@
         <v>1353</v>
       </c>
       <c r="I175">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="J175">
         <v>205</v>
@@ -11273,7 +11273,7 @@
         <v>1353</v>
       </c>
       <c r="I176">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="K176" t="s">
         <v>1357</v>
@@ -11311,7 +11311,7 @@
         <v>1353</v>
       </c>
       <c r="I177">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="J177">
         <v>44</v>
@@ -11358,7 +11358,7 @@
         <v>1353</v>
       </c>
       <c r="I178">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="K178" t="s">
         <v>1356</v>
@@ -11425,7 +11425,7 @@
         <v>1353</v>
       </c>
       <c r="I180">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="K180" t="s">
         <v>1356</v>
@@ -11521,7 +11521,7 @@
         <v>1353</v>
       </c>
       <c r="I183">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="K183" t="s">
         <v>1357</v>
@@ -11559,7 +11559,7 @@
         <v>1353</v>
       </c>
       <c r="I184">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="K184" t="s">
         <v>1363</v>
@@ -11594,7 +11594,7 @@
         <v>1353</v>
       </c>
       <c r="I185">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="K185" t="s">
         <v>1357</v>
@@ -11632,7 +11632,7 @@
         <v>1353</v>
       </c>
       <c r="I186">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="K186" t="s">
         <v>1357</v>
@@ -11670,7 +11670,7 @@
         <v>1353</v>
       </c>
       <c r="I187">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="J187">
         <v>75</v>
@@ -11717,7 +11717,7 @@
         <v>1353</v>
       </c>
       <c r="I188">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="J188">
         <v>40</v>
@@ -11764,7 +11764,7 @@
         <v>1353</v>
       </c>
       <c r="I189">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="J189">
         <v>155</v>
@@ -11808,7 +11808,7 @@
         <v>1353</v>
       </c>
       <c r="I190">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="J190">
         <v>107</v>
@@ -11852,7 +11852,7 @@
         <v>1353</v>
       </c>
       <c r="I191">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="J191">
         <v>5</v>
@@ -11896,7 +11896,7 @@
         <v>1353</v>
       </c>
       <c r="I192">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="K192" t="s">
         <v>1357</v>
@@ -11934,7 +11934,7 @@
         <v>1353</v>
       </c>
       <c r="I193">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="K193" t="s">
         <v>1362</v>
@@ -12001,7 +12001,7 @@
         <v>1353</v>
       </c>
       <c r="I195">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J195">
         <v>186</v>
@@ -12132,7 +12132,7 @@
         <v>1353</v>
       </c>
       <c r="I199">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="J199">
         <v>70</v>
@@ -12176,7 +12176,7 @@
         <v>1353</v>
       </c>
       <c r="I200">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="J200">
         <v>170</v>
@@ -12220,7 +12220,7 @@
         <v>1353</v>
       </c>
       <c r="I201">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="K201" t="s">
         <v>1357</v>
@@ -12258,7 +12258,7 @@
         <v>1353</v>
       </c>
       <c r="I202">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="K202" t="s">
         <v>1357</v>
@@ -12337,7 +12337,7 @@
         <v>1353</v>
       </c>
       <c r="I204">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="K204" t="s">
         <v>1356</v>
@@ -12375,7 +12375,7 @@
         <v>1353</v>
       </c>
       <c r="I205">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="K205" t="s">
         <v>1356</v>
@@ -12442,7 +12442,7 @@
         <v>1353</v>
       </c>
       <c r="I207">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="J207">
         <v>167</v>
@@ -12486,7 +12486,7 @@
         <v>1353</v>
       </c>
       <c r="I208">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="J208">
         <v>45</v>
@@ -12530,7 +12530,7 @@
         <v>1353</v>
       </c>
       <c r="I209">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="J209">
         <v>191</v>
@@ -12574,7 +12574,7 @@
         <v>1353</v>
       </c>
       <c r="I210">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="K210" t="s">
         <v>1360</v>
@@ -12670,7 +12670,7 @@
         <v>1353</v>
       </c>
       <c r="I213">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="K213" t="s">
         <v>1357</v>
@@ -12708,7 +12708,7 @@
         <v>1353</v>
       </c>
       <c r="I214">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="J214">
         <v>14</v>
@@ -12755,7 +12755,7 @@
         <v>1353</v>
       </c>
       <c r="I215">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="K215" t="s">
         <v>1357</v>
@@ -12822,7 +12822,7 @@
         <v>1353</v>
       </c>
       <c r="I217">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="J217">
         <v>42</v>
@@ -12866,7 +12866,7 @@
         <v>1353</v>
       </c>
       <c r="I218">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="J218">
         <v>166</v>
@@ -12954,7 +12954,7 @@
         <v>1353</v>
       </c>
       <c r="I220">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="J220">
         <v>154</v>
@@ -13112,7 +13112,7 @@
         <v>1353</v>
       </c>
       <c r="I224">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="J224">
         <v>204</v>
@@ -13267,7 +13267,7 @@
         <v>1353</v>
       </c>
       <c r="I228">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="J228">
         <v>204</v>
@@ -13346,7 +13346,7 @@
         <v>1353</v>
       </c>
       <c r="I230">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="J230">
         <v>197</v>
@@ -13390,7 +13390,7 @@
         <v>1353</v>
       </c>
       <c r="I231">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="J231">
         <v>35</v>
@@ -13492,7 +13492,7 @@
         <v>1353</v>
       </c>
       <c r="I234">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="J234">
         <v>35</v>
@@ -13539,7 +13539,7 @@
         <v>1353</v>
       </c>
       <c r="I235">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="J235">
         <v>35</v>
@@ -13586,7 +13586,7 @@
         <v>1353</v>
       </c>
       <c r="I236">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="J236">
         <v>86</v>
@@ -13703,7 +13703,7 @@
         <v>1353</v>
       </c>
       <c r="I239">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="K239" t="s">
         <v>1330</v>
@@ -13802,7 +13802,7 @@
         <v>1353</v>
       </c>
       <c r="I242">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="K242" t="s">
         <v>1356</v>
@@ -13869,7 +13869,7 @@
         <v>1353</v>
       </c>
       <c r="I244">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="J244">
         <v>15</v>
@@ -13910,7 +13910,7 @@
         <v>1353</v>
       </c>
       <c r="I245">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="J245">
         <v>15</v>
@@ -14053,7 +14053,7 @@
         <v>1353</v>
       </c>
       <c r="I249">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="K249" t="s">
         <v>1357</v>
@@ -14187,7 +14187,7 @@
         <v>1353</v>
       </c>
       <c r="I253">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="J253">
         <v>162</v>
@@ -14231,7 +14231,7 @@
         <v>1353</v>
       </c>
       <c r="I254">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="K254" t="s">
         <v>1360</v>
@@ -14269,7 +14269,7 @@
         <v>1353</v>
       </c>
       <c r="I255">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="J255">
         <v>72</v>
@@ -14313,7 +14313,7 @@
         <v>1353</v>
       </c>
       <c r="I256">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="J256">
         <v>23</v>
@@ -14415,7 +14415,7 @@
         <v>1353</v>
       </c>
       <c r="I259">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="J259">
         <v>72</v>
@@ -14459,7 +14459,7 @@
         <v>1353</v>
       </c>
       <c r="I260">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="J260">
         <v>84</v>
@@ -14503,7 +14503,7 @@
         <v>1353</v>
       </c>
       <c r="I261">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="J261">
         <v>162</v>
@@ -14620,7 +14620,7 @@
         <v>1353</v>
       </c>
       <c r="I264">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="J264">
         <v>162</v>
@@ -14664,7 +14664,7 @@
         <v>1353</v>
       </c>
       <c r="I265">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="J265">
         <v>162</v>
@@ -14708,7 +14708,7 @@
         <v>1353</v>
       </c>
       <c r="I266">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="J266">
         <v>84</v>
@@ -14752,7 +14752,7 @@
         <v>1353</v>
       </c>
       <c r="I267">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="K267" t="s">
         <v>1360</v>
@@ -14790,7 +14790,7 @@
         <v>1353</v>
       </c>
       <c r="I268">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="K268" t="s">
         <v>1357</v>
@@ -14825,7 +14825,7 @@
         <v>1353</v>
       </c>
       <c r="I269">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="K269" t="s">
         <v>1357</v>
@@ -14863,7 +14863,7 @@
         <v>1353</v>
       </c>
       <c r="I270">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="K270" t="s">
         <v>1360</v>
@@ -14901,7 +14901,7 @@
         <v>1353</v>
       </c>
       <c r="I271">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="K271" t="s">
         <v>1360</v>
@@ -15079,7 +15079,7 @@
         <v>1353</v>
       </c>
       <c r="I276">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="K276" t="s">
         <v>1361</v>
@@ -15117,7 +15117,7 @@
         <v>1353</v>
       </c>
       <c r="I277">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="K277" t="s">
         <v>1357</v>
@@ -15155,7 +15155,7 @@
         <v>1353</v>
       </c>
       <c r="I278">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J278">
         <v>148</v>
@@ -15199,7 +15199,7 @@
         <v>1353</v>
       </c>
       <c r="I279">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="K279" t="s">
         <v>1359</v>
@@ -15240,7 +15240,7 @@
         <v>1353</v>
       </c>
       <c r="I280">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="K280" t="s">
         <v>1357</v>
@@ -15278,7 +15278,7 @@
         <v>1353</v>
       </c>
       <c r="I281">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="K281" t="s">
         <v>1357</v>
@@ -15319,7 +15319,7 @@
         <v>1353</v>
       </c>
       <c r="I282">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="K282" t="s">
         <v>1357</v>
@@ -15502,7 +15502,7 @@
         <v>1353</v>
       </c>
       <c r="I288">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="J288">
         <v>28</v>
@@ -15575,7 +15575,7 @@
         <v>1353</v>
       </c>
       <c r="I290">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="J290">
         <v>20</v>
@@ -15619,7 +15619,7 @@
         <v>1353</v>
       </c>
       <c r="I291">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="J291">
         <v>20</v>
@@ -15663,7 +15663,7 @@
         <v>1353</v>
       </c>
       <c r="I292">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="K292" t="s">
         <v>1360</v>
@@ -15701,7 +15701,7 @@
         <v>1353</v>
       </c>
       <c r="I293">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="K293" t="s">
         <v>1361</v>
@@ -15739,7 +15739,7 @@
         <v>1353</v>
       </c>
       <c r="I294">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="K294" t="s">
         <v>1366</v>
@@ -15774,7 +15774,7 @@
         <v>1353</v>
       </c>
       <c r="I295">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="K295" t="s">
         <v>1366</v>
@@ -15809,7 +15809,7 @@
         <v>1353</v>
       </c>
       <c r="I296">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="K296" t="s">
         <v>1366</v>
@@ -15882,7 +15882,7 @@
         <v>1353</v>
       </c>
       <c r="I298">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J298">
         <v>58</v>
@@ -15923,7 +15923,7 @@
         <v>1353</v>
       </c>
       <c r="I299">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J299">
         <v>100</v>
@@ -15967,7 +15967,7 @@
         <v>1353</v>
       </c>
       <c r="I300">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J300">
         <v>86</v>
@@ -16011,7 +16011,7 @@
         <v>1353</v>
       </c>
       <c r="I301">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J301">
         <v>102</v>
@@ -16055,7 +16055,7 @@
         <v>1353</v>
       </c>
       <c r="I302">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="K302" t="s">
         <v>1360</v>
@@ -16093,7 +16093,7 @@
         <v>1353</v>
       </c>
       <c r="I303">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="K303" t="s">
         <v>1357</v>
@@ -16131,7 +16131,7 @@
         <v>1353</v>
       </c>
       <c r="I304">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="K304" t="s">
         <v>1360</v>
@@ -16169,7 +16169,7 @@
         <v>1353</v>
       </c>
       <c r="I305">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J305">
         <v>35</v>
@@ -16213,7 +16213,7 @@
         <v>1353</v>
       </c>
       <c r="I306">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J306">
         <v>31</v>
@@ -16301,7 +16301,7 @@
         <v>1353</v>
       </c>
       <c r="I308">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="K308" t="s">
         <v>1356</v>
@@ -16377,7 +16377,7 @@
         <v>1353</v>
       </c>
       <c r="I310">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J310">
         <v>107</v>
@@ -16421,7 +16421,7 @@
         <v>1353</v>
       </c>
       <c r="I311">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="K311" t="s">
         <v>1356</v>
@@ -16611,7 +16611,7 @@
         <v>1353</v>
       </c>
       <c r="I316">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="K316" t="s">
         <v>1357</v>
@@ -16754,7 +16754,7 @@
         <v>1353</v>
       </c>
       <c r="I320">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="K320" t="s">
         <v>1361</v>
@@ -16792,7 +16792,7 @@
         <v>1353</v>
       </c>
       <c r="I321">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="K321" t="s">
         <v>1357</v>
@@ -16830,7 +16830,7 @@
         <v>1353</v>
       </c>
       <c r="I322">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J322">
         <v>57</v>
@@ -16944,7 +16944,7 @@
         <v>1353</v>
       </c>
       <c r="I325">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J325">
         <v>57</v>
@@ -17026,7 +17026,7 @@
         <v>1353</v>
       </c>
       <c r="I327">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J327">
         <v>57</v>
@@ -17070,7 +17070,7 @@
         <v>1353</v>
       </c>
       <c r="I328">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J328">
         <v>57</v>
@@ -17114,7 +17114,7 @@
         <v>1353</v>
       </c>
       <c r="I329">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J329">
         <v>57</v>
@@ -17158,7 +17158,7 @@
         <v>1353</v>
       </c>
       <c r="I330">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J330">
         <v>57</v>
@@ -17202,7 +17202,7 @@
         <v>1353</v>
       </c>
       <c r="I331">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="K331" t="s">
         <v>1356</v>
@@ -17240,7 +17240,7 @@
         <v>1353</v>
       </c>
       <c r="I332">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="K332" t="s">
         <v>1357</v>
@@ -17278,7 +17278,7 @@
         <v>1353</v>
       </c>
       <c r="I333">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J333">
         <v>100</v>
@@ -17322,7 +17322,7 @@
         <v>1353</v>
       </c>
       <c r="I334">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="K334" t="s">
         <v>1357</v>
@@ -17398,7 +17398,7 @@
         <v>1353</v>
       </c>
       <c r="I336">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="J336">
         <v>28</v>
@@ -17480,7 +17480,7 @@
         <v>1353</v>
       </c>
       <c r="I338">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="J338">
         <v>12</v>
@@ -17553,7 +17553,7 @@
         <v>1353</v>
       </c>
       <c r="I340">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="J340">
         <v>98</v>
@@ -17594,7 +17594,7 @@
         <v>1353</v>
       </c>
       <c r="I341">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="J341">
         <v>90</v>
@@ -17635,7 +17635,7 @@
         <v>1353</v>
       </c>
       <c r="I342">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="K342" t="s">
         <v>1356</v>
@@ -17749,7 +17749,7 @@
         <v>1353</v>
       </c>
       <c r="I345">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="K345" t="s">
         <v>1356</v>
@@ -17825,7 +17825,7 @@
         <v>1353</v>
       </c>
       <c r="I347">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="J347">
         <v>18</v>
@@ -17872,7 +17872,7 @@
         <v>1353</v>
       </c>
       <c r="I348">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="J348">
         <v>14</v>
@@ -17916,7 +17916,7 @@
         <v>1353</v>
       </c>
       <c r="I349">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="K349" t="s">
         <v>1361</v>
@@ -17954,7 +17954,7 @@
         <v>1353</v>
       </c>
       <c r="I350">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="J350">
         <v>46</v>
@@ -17992,7 +17992,7 @@
         <v>1353</v>
       </c>
       <c r="I351">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="J351">
         <v>82</v>
@@ -18036,7 +18036,7 @@
         <v>1353</v>
       </c>
       <c r="I352">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="J352">
         <v>78</v>
@@ -18080,7 +18080,7 @@
         <v>1353</v>
       </c>
       <c r="I353">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="J353">
         <v>83</v>
@@ -18124,7 +18124,7 @@
         <v>1353</v>
       </c>
       <c r="I354">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="K354" t="s">
         <v>1360</v>
@@ -18162,7 +18162,7 @@
         <v>1353</v>
       </c>
       <c r="I355">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="J355">
         <v>8</v>
@@ -18244,7 +18244,7 @@
         <v>1353</v>
       </c>
       <c r="I357">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="J357">
         <v>85</v>
@@ -18367,7 +18367,7 @@
         <v>1353</v>
       </c>
       <c r="I360">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="J360">
         <v>83</v>
@@ -18414,7 +18414,7 @@
         <v>1353</v>
       </c>
       <c r="I361">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="J361">
         <v>83</v>
@@ -18458,7 +18458,7 @@
         <v>1353</v>
       </c>
       <c r="I362">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="K362" t="s">
         <v>1360</v>
@@ -18496,7 +18496,7 @@
         <v>1353</v>
       </c>
       <c r="I363">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="K363" t="s">
         <v>1360</v>
@@ -18534,7 +18534,7 @@
         <v>1353</v>
       </c>
       <c r="I364">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="J364">
         <v>83</v>
@@ -18578,7 +18578,7 @@
         <v>1353</v>
       </c>
       <c r="I365">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="J365">
         <v>15</v>
@@ -18619,7 +18619,7 @@
         <v>1353</v>
       </c>
       <c r="I366">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="J366">
         <v>77</v>
@@ -18663,7 +18663,7 @@
         <v>1353</v>
       </c>
       <c r="I367">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="J367">
         <v>77</v>
@@ -18707,7 +18707,7 @@
         <v>1353</v>
       </c>
       <c r="I368">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="J368">
         <v>77</v>
@@ -18751,7 +18751,7 @@
         <v>1353</v>
       </c>
       <c r="I369">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="K369" t="s">
         <v>1360</v>
@@ -18789,7 +18789,7 @@
         <v>1353</v>
       </c>
       <c r="I370">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="K370" t="s">
         <v>1360</v>
@@ -18827,7 +18827,7 @@
         <v>1353</v>
       </c>
       <c r="I371">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="J371">
         <v>16</v>
@@ -18915,7 +18915,7 @@
         <v>1353</v>
       </c>
       <c r="I373">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="K373" t="s">
         <v>1356</v>
@@ -18953,7 +18953,7 @@
         <v>1353</v>
       </c>
       <c r="I374">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="K374" t="s">
         <v>1356</v>
@@ -18991,7 +18991,7 @@
         <v>1353</v>
       </c>
       <c r="I375">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J375">
         <v>94</v>
@@ -19032,7 +19032,7 @@
         <v>1353</v>
       </c>
       <c r="I376">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="K376" t="s">
         <v>1360</v>
@@ -19111,7 +19111,7 @@
         <v>1353</v>
       </c>
       <c r="I378">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="K378" t="s">
         <v>1360</v>
@@ -19149,7 +19149,7 @@
         <v>1353</v>
       </c>
       <c r="I379">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J379">
         <v>20</v>
@@ -19193,7 +19193,7 @@
         <v>1353</v>
       </c>
       <c r="I380">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J380">
         <v>94</v>
@@ -19237,7 +19237,7 @@
         <v>1353</v>
       </c>
       <c r="I381">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="K381" t="s">
         <v>1360</v>
@@ -19275,7 +19275,7 @@
         <v>1353</v>
       </c>
       <c r="I382">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="K382" t="s">
         <v>1360</v>
@@ -19313,7 +19313,7 @@
         <v>1353</v>
       </c>
       <c r="I383">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J383">
         <v>71</v>
@@ -19357,7 +19357,7 @@
         <v>1353</v>
       </c>
       <c r="I384">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="K384" t="s">
         <v>1357</v>
@@ -19395,7 +19395,7 @@
         <v>1353</v>
       </c>
       <c r="I385">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="J385">
         <v>102</v>
@@ -19442,7 +19442,7 @@
         <v>1353</v>
       </c>
       <c r="I386">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="K386" t="s">
         <v>1360</v>
@@ -19480,7 +19480,7 @@
         <v>1353</v>
       </c>
       <c r="I387">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="K387" t="s">
         <v>1360</v>
@@ -19518,7 +19518,7 @@
         <v>1353</v>
       </c>
       <c r="I388">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="J388">
         <v>-85</v>
@@ -19562,7 +19562,7 @@
         <v>1353</v>
       </c>
       <c r="I389">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="K389" t="s">
         <v>1361</v>
@@ -19720,7 +19720,7 @@
         <v>1353</v>
       </c>
       <c r="I393">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="J393">
         <v>20</v>
@@ -20016,7 +20016,7 @@
         <v>1353</v>
       </c>
       <c r="I400">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="K400" t="s">
         <v>1360</v>
@@ -20092,7 +20092,7 @@
         <v>1353</v>
       </c>
       <c r="I402">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="K402" t="s">
         <v>1360</v>
@@ -20130,7 +20130,7 @@
         <v>1353</v>
       </c>
       <c r="I403">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="J403">
         <v>83</v>
@@ -20174,7 +20174,7 @@
         <v>1353</v>
       </c>
       <c r="I404">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="K404" t="s">
         <v>1360</v>
@@ -20244,7 +20244,7 @@
         <v>1353</v>
       </c>
       <c r="I406">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="Q406" t="b">
         <v>1</v>
@@ -20276,7 +20276,7 @@
         <v>1353</v>
       </c>
       <c r="I407">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="Q407" t="b">
         <v>1</v>
@@ -20308,7 +20308,7 @@
         <v>1353</v>
       </c>
       <c r="I408">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="Q408" t="b">
         <v>1</v>
@@ -20340,7 +20340,7 @@
         <v>1353</v>
       </c>
       <c r="I409">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="Q409" t="b">
         <v>1</v>
@@ -20372,7 +20372,7 @@
         <v>1353</v>
       </c>
       <c r="I410">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="Q410" t="b">
         <v>1</v>
@@ -20404,7 +20404,7 @@
         <v>1353</v>
       </c>
       <c r="I411">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="Q411" t="b">
         <v>1</v>
@@ -20436,7 +20436,7 @@
         <v>1353</v>
       </c>
       <c r="I412">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="Q412" t="b">
         <v>1</v>
@@ -20468,7 +20468,7 @@
         <v>1353</v>
       </c>
       <c r="I413">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="Q413" t="b">
         <v>1</v>
@@ -20558,7 +20558,7 @@
         <v>1353</v>
       </c>
       <c r="I416">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="Q416" t="b">
         <v>1</v>
@@ -20648,7 +20648,7 @@
         <v>1353</v>
       </c>
       <c r="I419">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="Q419" t="b">
         <v>1</v>
@@ -20680,7 +20680,7 @@
         <v>1353</v>
       </c>
       <c r="I420">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="Q420" t="b">
         <v>1</v>
@@ -20712,7 +20712,7 @@
         <v>1353</v>
       </c>
       <c r="I421">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="Q421" t="b">
         <v>1</v>
@@ -20744,7 +20744,7 @@
         <v>1353</v>
       </c>
       <c r="I422">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="Q422" t="b">
         <v>1</v>
@@ -20776,7 +20776,7 @@
         <v>1353</v>
       </c>
       <c r="I423">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="Q423" t="b">
         <v>1</v>
@@ -20808,7 +20808,7 @@
         <v>1353</v>
       </c>
       <c r="I424">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="Q424" t="b">
         <v>1</v>
@@ -20840,7 +20840,7 @@
         <v>1353</v>
       </c>
       <c r="I425">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="Q425" t="b">
         <v>1</v>
@@ -20872,7 +20872,7 @@
         <v>1353</v>
       </c>
       <c r="I426">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="Q426" t="b">
         <v>1</v>
@@ -20904,7 +20904,7 @@
         <v>1353</v>
       </c>
       <c r="I427">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="Q427" t="b">
         <v>1</v>
@@ -20994,7 +20994,7 @@
         <v>1353</v>
       </c>
       <c r="I430">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="Q430" t="b">
         <v>1</v>
@@ -21026,7 +21026,7 @@
         <v>1353</v>
       </c>
       <c r="I431">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="Q431" t="b">
         <v>1</v>
@@ -21058,7 +21058,7 @@
         <v>1353</v>
       </c>
       <c r="I432">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="Q432" t="b">
         <v>1</v>
@@ -21090,7 +21090,7 @@
         <v>1353</v>
       </c>
       <c r="I433">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="Q433" t="b">
         <v>1</v>
@@ -21122,7 +21122,7 @@
         <v>1353</v>
       </c>
       <c r="I434">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="Q434" t="b">
         <v>1</v>
@@ -21154,7 +21154,7 @@
         <v>1353</v>
       </c>
       <c r="I435">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="Q435" t="b">
         <v>1</v>
@@ -21186,7 +21186,7 @@
         <v>1353</v>
       </c>
       <c r="I436">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="Q436" t="b">
         <v>1</v>
@@ -21218,7 +21218,7 @@
         <v>1355</v>
       </c>
       <c r="I437">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="Q437" t="b">
         <v>1</v>
@@ -21250,7 +21250,7 @@
         <v>1355</v>
       </c>
       <c r="I438">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="Q438" t="b">
         <v>1</v>
@@ -21282,7 +21282,7 @@
         <v>1353</v>
       </c>
       <c r="I439">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="Q439" t="b">
         <v>1</v>
@@ -21314,7 +21314,7 @@
         <v>1353</v>
       </c>
       <c r="I440">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="Q440" t="b">
         <v>1</v>
@@ -21346,7 +21346,7 @@
         <v>1353</v>
       </c>
       <c r="I441">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="Q441" t="b">
         <v>1</v>
@@ -21407,7 +21407,7 @@
         <v>1353</v>
       </c>
       <c r="I443">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q443" t="b">
         <v>1</v>
@@ -21497,7 +21497,7 @@
         <v>1353</v>
       </c>
       <c r="I446">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="Q446" t="b">
         <v>1</v>
@@ -21529,7 +21529,7 @@
         <v>1353</v>
       </c>
       <c r="I447">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="Q447" t="b">
         <v>1</v>
@@ -21561,7 +21561,7 @@
         <v>1353</v>
       </c>
       <c r="I448">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="Q448" t="b">
         <v>1</v>
@@ -21593,7 +21593,7 @@
         <v>1353</v>
       </c>
       <c r="I449">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="Q449" t="b">
         <v>1</v>
@@ -21625,7 +21625,7 @@
         <v>1353</v>
       </c>
       <c r="I450">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="Q450" t="b">
         <v>1</v>
@@ -21657,7 +21657,7 @@
         <v>1353</v>
       </c>
       <c r="I451">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="Q451" t="b">
         <v>1</v>
@@ -21689,7 +21689,7 @@
         <v>1353</v>
       </c>
       <c r="I452">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="Q452" t="b">
         <v>1</v>
@@ -21721,7 +21721,7 @@
         <v>1353</v>
       </c>
       <c r="I453">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="Q453" t="b">
         <v>1</v>
@@ -21753,7 +21753,7 @@
         <v>1353</v>
       </c>
       <c r="I454">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="Q454" t="b">
         <v>1</v>
@@ -21785,7 +21785,7 @@
         <v>1353</v>
       </c>
       <c r="I455">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="Q455" t="b">
         <v>1</v>
@@ -21817,7 +21817,7 @@
         <v>1353</v>
       </c>
       <c r="I456">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="Q456" t="b">
         <v>1</v>
@@ -21849,7 +21849,7 @@
         <v>1353</v>
       </c>
       <c r="I457">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="Q457" t="b">
         <v>1</v>
@@ -21881,7 +21881,7 @@
         <v>1353</v>
       </c>
       <c r="I458">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q458" t="b">
         <v>1</v>
@@ -21913,7 +21913,7 @@
         <v>1353</v>
       </c>
       <c r="I459">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q459" t="b">
         <v>1</v>
@@ -21945,7 +21945,7 @@
         <v>1353</v>
       </c>
       <c r="I460">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q460" t="b">
         <v>1</v>
@@ -21977,7 +21977,7 @@
         <v>1353</v>
       </c>
       <c r="I461">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q461" t="b">
         <v>1</v>
@@ -22009,7 +22009,7 @@
         <v>1353</v>
       </c>
       <c r="I462">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q462" t="b">
         <v>1</v>
@@ -22041,7 +22041,7 @@
         <v>1353</v>
       </c>
       <c r="I463">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="Q463" t="b">
         <v>1</v>
@@ -22073,7 +22073,7 @@
         <v>1353</v>
       </c>
       <c r="I464">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="Q464" t="b">
         <v>1</v>
@@ -22105,7 +22105,7 @@
         <v>1353</v>
       </c>
       <c r="I465">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="Q465" t="b">
         <v>1</v>
@@ -22137,7 +22137,7 @@
         <v>1353</v>
       </c>
       <c r="I466">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="Q466" t="b">
         <v>1</v>
@@ -22169,7 +22169,7 @@
         <v>1353</v>
       </c>
       <c r="I467">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="Q467" t="b">
         <v>1</v>
@@ -22201,7 +22201,7 @@
         <v>1353</v>
       </c>
       <c r="I468">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="Q468" t="b">
         <v>1</v>
@@ -22233,7 +22233,7 @@
         <v>1353</v>
       </c>
       <c r="I469">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="Q469" t="b">
         <v>1</v>
@@ -22294,7 +22294,7 @@
         <v>1353</v>
       </c>
       <c r="I471">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="Q471" t="b">
         <v>1</v>
@@ -22326,7 +22326,7 @@
         <v>1353</v>
       </c>
       <c r="I472">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="Q472" t="b">
         <v>1</v>
@@ -22358,7 +22358,7 @@
         <v>1353</v>
       </c>
       <c r="I473">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="Q473" t="b">
         <v>1</v>
@@ -22390,7 +22390,7 @@
         <v>1353</v>
       </c>
       <c r="I474">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q474" t="b">
         <v>1</v>
@@ -22422,7 +22422,7 @@
         <v>1353</v>
       </c>
       <c r="I475">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q475" t="b">
         <v>1</v>
@@ -22454,7 +22454,7 @@
         <v>1353</v>
       </c>
       <c r="I476">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q476" t="b">
         <v>1</v>
@@ -22486,7 +22486,7 @@
         <v>1353</v>
       </c>
       <c r="I477">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q477" t="b">
         <v>1</v>
@@ -22518,7 +22518,7 @@
         <v>1353</v>
       </c>
       <c r="I478">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q478" t="b">
         <v>1</v>
@@ -22550,7 +22550,7 @@
         <v>1353</v>
       </c>
       <c r="I479">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q479" t="b">
         <v>1</v>
@@ -22582,7 +22582,7 @@
         <v>1353</v>
       </c>
       <c r="I480">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q480" t="b">
         <v>1</v>
@@ -22614,7 +22614,7 @@
         <v>1353</v>
       </c>
       <c r="I481">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q481" t="b">
         <v>1</v>
@@ -22646,7 +22646,7 @@
         <v>1353</v>
       </c>
       <c r="I482">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q482" t="b">
         <v>1</v>
@@ -22678,7 +22678,7 @@
         <v>1353</v>
       </c>
       <c r="I483">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q483" t="b">
         <v>1</v>
@@ -22710,7 +22710,7 @@
         <v>1353</v>
       </c>
       <c r="I484">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q484" t="b">
         <v>1</v>
@@ -22742,7 +22742,7 @@
         <v>1353</v>
       </c>
       <c r="I485">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q485" t="b">
         <v>1</v>
@@ -22774,7 +22774,7 @@
         <v>1353</v>
       </c>
       <c r="I486">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q486" t="b">
         <v>1</v>
@@ -22806,7 +22806,7 @@
         <v>1353</v>
       </c>
       <c r="I487">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q487" t="b">
         <v>1</v>
@@ -22838,7 +22838,7 @@
         <v>1353</v>
       </c>
       <c r="I488">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q488" t="b">
         <v>1</v>
@@ -22870,7 +22870,7 @@
         <v>1353</v>
       </c>
       <c r="I489">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q489" t="b">
         <v>1</v>
@@ -22902,7 +22902,7 @@
         <v>1353</v>
       </c>
       <c r="I490">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q490" t="b">
         <v>1</v>
@@ -22934,7 +22934,7 @@
         <v>1353</v>
       </c>
       <c r="I491">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q491" t="b">
         <v>1</v>
@@ -22966,7 +22966,7 @@
         <v>1355</v>
       </c>
       <c r="I492">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q492" t="b">
         <v>1</v>
@@ -22998,7 +22998,7 @@
         <v>1355</v>
       </c>
       <c r="I493">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q493" t="b">
         <v>1</v>
@@ -23030,7 +23030,7 @@
         <v>1355</v>
       </c>
       <c r="I494">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q494" t="b">
         <v>1</v>
@@ -23062,7 +23062,7 @@
         <v>1355</v>
       </c>
       <c r="I495">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q495" t="b">
         <v>1</v>
@@ -23094,7 +23094,7 @@
         <v>1355</v>
       </c>
       <c r="I496">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q496" t="b">
         <v>1</v>
@@ -23126,7 +23126,7 @@
         <v>1353</v>
       </c>
       <c r="I497">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q497" t="b">
         <v>1</v>
@@ -23158,7 +23158,7 @@
         <v>1353</v>
       </c>
       <c r="I498">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q498" t="b">
         <v>1</v>
@@ -23190,7 +23190,7 @@
         <v>1355</v>
       </c>
       <c r="I499">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q499" t="b">
         <v>1</v>
@@ -23222,7 +23222,7 @@
         <v>1353</v>
       </c>
       <c r="I500">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q500" t="b">
         <v>1</v>
@@ -23254,7 +23254,7 @@
         <v>1353</v>
       </c>
       <c r="I501">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q501" t="b">
         <v>1</v>
@@ -23286,7 +23286,7 @@
         <v>1353</v>
       </c>
       <c r="I502">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q502" t="b">
         <v>1</v>
@@ -23318,7 +23318,7 @@
         <v>1353</v>
       </c>
       <c r="I503">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q503" t="b">
         <v>1</v>
@@ -23350,7 +23350,7 @@
         <v>1353</v>
       </c>
       <c r="I504">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q504" t="b">
         <v>1</v>
@@ -23382,7 +23382,7 @@
         <v>1353</v>
       </c>
       <c r="I505">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q505" t="b">
         <v>1</v>
@@ -23414,7 +23414,7 @@
         <v>1353</v>
       </c>
       <c r="I506">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q506" t="b">
         <v>1</v>
@@ -23446,7 +23446,7 @@
         <v>1353</v>
       </c>
       <c r="I507">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Q507" t="b">
         <v>1</v>
@@ -23507,7 +23507,7 @@
         <v>1353</v>
       </c>
       <c r="I509">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Q509" t="b">
         <v>1</v>
@@ -23539,7 +23539,7 @@
         <v>1353</v>
       </c>
       <c r="I510">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Q510" t="b">
         <v>1</v>
@@ -23571,7 +23571,7 @@
         <v>1353</v>
       </c>
       <c r="I511">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q511" t="b">
         <v>1</v>
@@ -23603,7 +23603,7 @@
         <v>1353</v>
       </c>
       <c r="I512">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q512" t="b">
         <v>1</v>
@@ -23635,7 +23635,7 @@
         <v>1353</v>
       </c>
       <c r="I513">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="Q513" t="b">
         <v>1</v>
@@ -23667,7 +23667,7 @@
         <v>1353</v>
       </c>
       <c r="I514">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="Q514" t="b">
         <v>1</v>
@@ -23699,7 +23699,7 @@
         <v>1353</v>
       </c>
       <c r="I515">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="Q515" t="b">
         <v>1</v>
@@ -23731,7 +23731,7 @@
         <v>1353</v>
       </c>
       <c r="I516">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="Q516" t="b">
         <v>1</v>
@@ -23763,7 +23763,7 @@
         <v>1353</v>
       </c>
       <c r="I517">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="Q517" t="b">
         <v>1</v>
@@ -23795,7 +23795,7 @@
         <v>1353</v>
       </c>
       <c r="I518">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="Q518" t="b">
         <v>1</v>
@@ -23827,7 +23827,7 @@
         <v>1353</v>
       </c>
       <c r="I519">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q519" t="b">
         <v>1</v>
@@ -23859,7 +23859,7 @@
         <v>1353</v>
       </c>
       <c r="I520">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q520" t="b">
         <v>1</v>
@@ -23891,7 +23891,7 @@
         <v>1353</v>
       </c>
       <c r="I521">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q521" t="b">
         <v>1</v>
@@ -23923,7 +23923,7 @@
         <v>1353</v>
       </c>
       <c r="I522">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q522" t="b">
         <v>1</v>
@@ -23955,7 +23955,7 @@
         <v>1353</v>
       </c>
       <c r="I523">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q523" t="b">
         <v>1</v>
@@ -23987,7 +23987,7 @@
         <v>1353</v>
       </c>
       <c r="I524">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="Q524" t="b">
         <v>1</v>
@@ -24019,7 +24019,7 @@
         <v>1353</v>
       </c>
       <c r="I525">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="Q525" t="b">
         <v>1</v>
@@ -24051,7 +24051,7 @@
         <v>1353</v>
       </c>
       <c r="I526">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="Q526" t="b">
         <v>1</v>
@@ -24083,7 +24083,7 @@
         <v>1353</v>
       </c>
       <c r="I527">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="Q527" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: reparaveis (29/09/2026 13:54)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
@@ -4940,7 +4940,7 @@
         <v>1353</v>
       </c>
       <c r="I2">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="K2" t="s">
         <v>1356</v>
@@ -4978,7 +4978,7 @@
         <v>1353</v>
       </c>
       <c r="I3">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="K3" t="s">
         <v>1357</v>
@@ -5016,7 +5016,7 @@
         <v>1353</v>
       </c>
       <c r="I4">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="K4" t="s">
         <v>1357</v>
@@ -5054,7 +5054,7 @@
         <v>1353</v>
       </c>
       <c r="I5">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="J5">
         <v>279</v>
@@ -5098,7 +5098,7 @@
         <v>1353</v>
       </c>
       <c r="I6">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="J6">
         <v>153</v>
@@ -5142,7 +5142,7 @@
         <v>1353</v>
       </c>
       <c r="I7">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="J7">
         <v>112</v>
@@ -5218,7 +5218,7 @@
         <v>1353</v>
       </c>
       <c r="I9">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="J9">
         <v>362</v>
@@ -5265,7 +5265,7 @@
         <v>1353</v>
       </c>
       <c r="I10">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="J10">
         <v>378</v>
@@ -5312,7 +5312,7 @@
         <v>1353</v>
       </c>
       <c r="I11">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="J11">
         <v>112</v>
@@ -5359,7 +5359,7 @@
         <v>1353</v>
       </c>
       <c r="I12">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="J12">
         <v>124</v>
@@ -5432,7 +5432,7 @@
         <v>1353</v>
       </c>
       <c r="I14">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="J14">
         <v>64</v>
@@ -5476,7 +5476,7 @@
         <v>1353</v>
       </c>
       <c r="I15">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="K15" t="s">
         <v>1359</v>
@@ -5514,7 +5514,7 @@
         <v>1353</v>
       </c>
       <c r="I16">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="K16" t="s">
         <v>1356</v>
@@ -5552,7 +5552,7 @@
         <v>1353</v>
       </c>
       <c r="I17">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="J17">
         <v>161</v>
@@ -5596,7 +5596,7 @@
         <v>1353</v>
       </c>
       <c r="I18">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="J18">
         <v>66</v>
@@ -5669,7 +5669,7 @@
         <v>1353</v>
       </c>
       <c r="I20">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="J20">
         <v>399</v>
@@ -5742,7 +5742,7 @@
         <v>1353</v>
       </c>
       <c r="I22">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="K22" t="s">
         <v>1360</v>
@@ -5780,7 +5780,7 @@
         <v>1353</v>
       </c>
       <c r="I23">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="J23">
         <v>229</v>
@@ -5885,7 +5885,7 @@
         <v>1353</v>
       </c>
       <c r="I26">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="J26">
         <v>155</v>
@@ -5932,7 +5932,7 @@
         <v>1353</v>
       </c>
       <c r="I27">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="K27" t="s">
         <v>1360</v>
@@ -6028,7 +6028,7 @@
         <v>1353</v>
       </c>
       <c r="I30">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="J30">
         <v>209</v>
@@ -6101,7 +6101,7 @@
         <v>1353</v>
       </c>
       <c r="I32">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="K32" t="s">
         <v>1356</v>
@@ -6310,7 +6310,7 @@
         <v>1353</v>
       </c>
       <c r="I39">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="K39" t="s">
         <v>1361</v>
@@ -6345,7 +6345,7 @@
         <v>1353</v>
       </c>
       <c r="I40">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="K40" t="s">
         <v>1359</v>
@@ -6476,7 +6476,7 @@
         <v>1353</v>
       </c>
       <c r="I44">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="J44">
         <v>87</v>
@@ -6523,7 +6523,7 @@
         <v>1353</v>
       </c>
       <c r="I45">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="J45">
         <v>331</v>
@@ -6570,7 +6570,7 @@
         <v>1353</v>
       </c>
       <c r="I46">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="K46" t="s">
         <v>1360</v>
@@ -6608,7 +6608,7 @@
         <v>1353</v>
       </c>
       <c r="I47">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="J47">
         <v>344</v>
@@ -6655,7 +6655,7 @@
         <v>1353</v>
       </c>
       <c r="I48">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="K48" t="s">
         <v>1360</v>
@@ -6722,7 +6722,7 @@
         <v>1353</v>
       </c>
       <c r="I50">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="K50" t="s">
         <v>1360</v>
@@ -6789,7 +6789,7 @@
         <v>1353</v>
       </c>
       <c r="I52">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="K52" t="s">
         <v>1356</v>
@@ -6827,7 +6827,7 @@
         <v>1353</v>
       </c>
       <c r="I53">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="K53" t="s">
         <v>1357</v>
@@ -6865,7 +6865,7 @@
         <v>1353</v>
       </c>
       <c r="I54">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="K54" t="s">
         <v>1357</v>
@@ -6961,7 +6961,7 @@
         <v>1353</v>
       </c>
       <c r="I57">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="K57" t="s">
         <v>1360</v>
@@ -7144,7 +7144,7 @@
         <v>1353</v>
       </c>
       <c r="I63">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="J63">
         <v>293</v>
@@ -7191,7 +7191,7 @@
         <v>1353</v>
       </c>
       <c r="I64">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="J64">
         <v>320</v>
@@ -7380,7 +7380,7 @@
         <v>1353</v>
       </c>
       <c r="I70">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="J70">
         <v>429</v>
@@ -7424,7 +7424,7 @@
         <v>1353</v>
       </c>
       <c r="I71">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="J71">
         <v>429</v>
@@ -7497,7 +7497,7 @@
         <v>1353</v>
       </c>
       <c r="I73">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="K73" t="s">
         <v>1356</v>
@@ -7564,7 +7564,7 @@
         <v>1353</v>
       </c>
       <c r="I75">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="J75">
         <v>429</v>
@@ -7608,7 +7608,7 @@
         <v>1353</v>
       </c>
       <c r="I76">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="K76" t="s">
         <v>1363</v>
@@ -7701,7 +7701,7 @@
         <v>1353</v>
       </c>
       <c r="I79">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="K79" t="s">
         <v>1363</v>
@@ -7736,7 +7736,7 @@
         <v>1353</v>
       </c>
       <c r="I80">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="J80">
         <v>429</v>
@@ -7809,7 +7809,7 @@
         <v>1353</v>
       </c>
       <c r="I82">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="K82" t="s">
         <v>1360</v>
@@ -7876,7 +7876,7 @@
         <v>1353</v>
       </c>
       <c r="I84">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="J84">
         <v>40</v>
@@ -7923,7 +7923,7 @@
         <v>1353</v>
       </c>
       <c r="I85">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="K85" t="s">
         <v>1357</v>
@@ -7961,7 +7961,7 @@
         <v>1353</v>
       </c>
       <c r="I86">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="K86" t="s">
         <v>1357</v>
@@ -7999,7 +7999,7 @@
         <v>1353</v>
       </c>
       <c r="I87">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="J87">
         <v>-16</v>
@@ -8122,7 +8122,7 @@
         <v>1353</v>
       </c>
       <c r="I90">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="K90" t="s">
         <v>1330</v>
@@ -8163,7 +8163,7 @@
         <v>1353</v>
       </c>
       <c r="I91">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="J91">
         <v>308</v>
@@ -8233,7 +8233,7 @@
         <v>1353</v>
       </c>
       <c r="I93">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="J93">
         <v>308</v>
@@ -8277,7 +8277,7 @@
         <v>1353</v>
       </c>
       <c r="I94">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="K94" t="s">
         <v>1360</v>
@@ -8315,7 +8315,7 @@
         <v>1353</v>
       </c>
       <c r="I95">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="J95">
         <v>308</v>
@@ -8359,7 +8359,7 @@
         <v>1353</v>
       </c>
       <c r="I96">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="J96">
         <v>17</v>
@@ -8406,7 +8406,7 @@
         <v>1353</v>
       </c>
       <c r="I97">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="J97">
         <v>20</v>
@@ -8453,7 +8453,7 @@
         <v>1353</v>
       </c>
       <c r="I98">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="K98" t="s">
         <v>1360</v>
@@ -8520,7 +8520,7 @@
         <v>1353</v>
       </c>
       <c r="I100">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="J100">
         <v>348</v>
@@ -8651,7 +8651,7 @@
         <v>1353</v>
       </c>
       <c r="I104">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="J104">
         <v>348</v>
@@ -8695,7 +8695,7 @@
         <v>1353</v>
       </c>
       <c r="I105">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="J105">
         <v>348</v>
@@ -8739,7 +8739,7 @@
         <v>1353</v>
       </c>
       <c r="I106">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="J106">
         <v>49</v>
@@ -8783,7 +8783,7 @@
         <v>1353</v>
       </c>
       <c r="I107">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="J107">
         <v>36</v>
@@ -8827,7 +8827,7 @@
         <v>1353</v>
       </c>
       <c r="I108">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="K108" t="s">
         <v>1357</v>
@@ -8865,7 +8865,7 @@
         <v>1353</v>
       </c>
       <c r="I109">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="K109" t="s">
         <v>1357</v>
@@ -9048,7 +9048,7 @@
         <v>1353</v>
       </c>
       <c r="I115">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="K115" t="s">
         <v>1357</v>
@@ -9086,7 +9086,7 @@
         <v>1353</v>
       </c>
       <c r="I116">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="K116" t="s">
         <v>1357</v>
@@ -9124,7 +9124,7 @@
         <v>1353</v>
       </c>
       <c r="I117">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="K117" t="s">
         <v>1357</v>
@@ -9162,7 +9162,7 @@
         <v>1353</v>
       </c>
       <c r="I118">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="K118" t="s">
         <v>1357</v>
@@ -9200,7 +9200,7 @@
         <v>1353</v>
       </c>
       <c r="I119">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="K119" t="s">
         <v>1357</v>
@@ -9238,7 +9238,7 @@
         <v>1353</v>
       </c>
       <c r="I120">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="K120" t="s">
         <v>1357</v>
@@ -9276,7 +9276,7 @@
         <v>1353</v>
       </c>
       <c r="I121">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="J121">
         <v>251</v>
@@ -9323,7 +9323,7 @@
         <v>1353</v>
       </c>
       <c r="I122">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="K122" t="s">
         <v>1357</v>
@@ -9390,7 +9390,7 @@
         <v>1353</v>
       </c>
       <c r="I124">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="K124" t="s">
         <v>1357</v>
@@ -9428,7 +9428,7 @@
         <v>1353</v>
       </c>
       <c r="I125">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="K125" t="s">
         <v>1363</v>
@@ -9524,7 +9524,7 @@
         <v>1353</v>
       </c>
       <c r="I128">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="K128" t="s">
         <v>1357</v>
@@ -9562,7 +9562,7 @@
         <v>1353</v>
       </c>
       <c r="I129">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="K129" t="s">
         <v>1356</v>
@@ -9600,7 +9600,7 @@
         <v>1353</v>
       </c>
       <c r="I130">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="J130">
         <v>47</v>
@@ -9676,7 +9676,7 @@
         <v>1353</v>
       </c>
       <c r="I132">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="J132">
         <v>145</v>
@@ -9752,7 +9752,7 @@
         <v>1353</v>
       </c>
       <c r="I134">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="K134" t="s">
         <v>1356</v>
@@ -9877,7 +9877,7 @@
         <v>1353</v>
       </c>
       <c r="I138">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="K138" t="s">
         <v>1357</v>
@@ -10176,7 +10176,7 @@
         <v>1353</v>
       </c>
       <c r="I148">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="J148">
         <v>341</v>
@@ -10220,7 +10220,7 @@
         <v>1353</v>
       </c>
       <c r="I149">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="J149">
         <v>374</v>
@@ -10267,7 +10267,7 @@
         <v>1353</v>
       </c>
       <c r="I150">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="J150">
         <v>201</v>
@@ -10343,7 +10343,7 @@
         <v>1353</v>
       </c>
       <c r="I152">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="J152">
         <v>228</v>
@@ -10457,7 +10457,7 @@
         <v>1353</v>
       </c>
       <c r="I155">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="K155" t="s">
         <v>1363</v>
@@ -10492,7 +10492,7 @@
         <v>1353</v>
       </c>
       <c r="I156">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="K156" t="s">
         <v>1357</v>
@@ -10530,7 +10530,7 @@
         <v>1353</v>
       </c>
       <c r="I157">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="J157">
         <v>371</v>
@@ -10574,7 +10574,7 @@
         <v>1353</v>
       </c>
       <c r="I158">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="J158">
         <v>52</v>
@@ -10618,7 +10618,7 @@
         <v>1353</v>
       </c>
       <c r="I159">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="K159" t="s">
         <v>1357</v>
@@ -10656,7 +10656,7 @@
         <v>1353</v>
       </c>
       <c r="I160">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="K160" t="s">
         <v>1357</v>
@@ -10694,7 +10694,7 @@
         <v>1353</v>
       </c>
       <c r="I161">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="J161">
         <v>55</v>
@@ -10741,7 +10741,7 @@
         <v>1353</v>
       </c>
       <c r="I162">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="J162">
         <v>42</v>
@@ -10788,7 +10788,7 @@
         <v>1353</v>
       </c>
       <c r="I163">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="J163">
         <v>42</v>
@@ -10835,7 +10835,7 @@
         <v>1355</v>
       </c>
       <c r="I164">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="O164" t="s">
         <v>1469</v>
@@ -10972,7 +10972,7 @@
         <v>1353</v>
       </c>
       <c r="I168">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="K168" t="s">
         <v>1360</v>
@@ -11013,7 +11013,7 @@
         <v>1353</v>
       </c>
       <c r="I169">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="K169" t="s">
         <v>1330</v>
@@ -11089,7 +11089,7 @@
         <v>1353</v>
       </c>
       <c r="I171">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="K171" t="s">
         <v>1357</v>
@@ -11226,7 +11226,7 @@
         <v>1353</v>
       </c>
       <c r="I175">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="J175">
         <v>205</v>
@@ -11273,7 +11273,7 @@
         <v>1353</v>
       </c>
       <c r="I176">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="K176" t="s">
         <v>1357</v>
@@ -11311,7 +11311,7 @@
         <v>1353</v>
       </c>
       <c r="I177">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="J177">
         <v>44</v>
@@ -11358,7 +11358,7 @@
         <v>1353</v>
       </c>
       <c r="I178">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="K178" t="s">
         <v>1356</v>
@@ -11425,7 +11425,7 @@
         <v>1353</v>
       </c>
       <c r="I180">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="K180" t="s">
         <v>1356</v>
@@ -11521,7 +11521,7 @@
         <v>1353</v>
       </c>
       <c r="I183">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="K183" t="s">
         <v>1357</v>
@@ -11559,7 +11559,7 @@
         <v>1353</v>
       </c>
       <c r="I184">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="K184" t="s">
         <v>1363</v>
@@ -11594,7 +11594,7 @@
         <v>1353</v>
       </c>
       <c r="I185">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="K185" t="s">
         <v>1357</v>
@@ -11632,7 +11632,7 @@
         <v>1353</v>
       </c>
       <c r="I186">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="K186" t="s">
         <v>1357</v>
@@ -11670,7 +11670,7 @@
         <v>1353</v>
       </c>
       <c r="I187">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="J187">
         <v>75</v>
@@ -11717,7 +11717,7 @@
         <v>1353</v>
       </c>
       <c r="I188">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="J188">
         <v>40</v>
@@ -11764,7 +11764,7 @@
         <v>1353</v>
       </c>
       <c r="I189">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="J189">
         <v>155</v>
@@ -11808,7 +11808,7 @@
         <v>1353</v>
       </c>
       <c r="I190">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="J190">
         <v>107</v>
@@ -11852,7 +11852,7 @@
         <v>1353</v>
       </c>
       <c r="I191">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="J191">
         <v>5</v>
@@ -11896,7 +11896,7 @@
         <v>1353</v>
       </c>
       <c r="I192">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="K192" t="s">
         <v>1357</v>
@@ -11934,7 +11934,7 @@
         <v>1353</v>
       </c>
       <c r="I193">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="K193" t="s">
         <v>1362</v>
@@ -12001,7 +12001,7 @@
         <v>1353</v>
       </c>
       <c r="I195">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="J195">
         <v>186</v>
@@ -12132,7 +12132,7 @@
         <v>1353</v>
       </c>
       <c r="I199">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J199">
         <v>70</v>
@@ -12176,7 +12176,7 @@
         <v>1353</v>
       </c>
       <c r="I200">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="J200">
         <v>170</v>
@@ -12220,7 +12220,7 @@
         <v>1353</v>
       </c>
       <c r="I201">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="K201" t="s">
         <v>1357</v>
@@ -12258,7 +12258,7 @@
         <v>1353</v>
       </c>
       <c r="I202">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="K202" t="s">
         <v>1357</v>
@@ -12337,7 +12337,7 @@
         <v>1353</v>
       </c>
       <c r="I204">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="K204" t="s">
         <v>1356</v>
@@ -12375,7 +12375,7 @@
         <v>1353</v>
       </c>
       <c r="I205">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="K205" t="s">
         <v>1356</v>
@@ -12442,7 +12442,7 @@
         <v>1353</v>
       </c>
       <c r="I207">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="J207">
         <v>167</v>
@@ -12486,7 +12486,7 @@
         <v>1353</v>
       </c>
       <c r="I208">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="J208">
         <v>45</v>
@@ -12530,7 +12530,7 @@
         <v>1353</v>
       </c>
       <c r="I209">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="J209">
         <v>191</v>
@@ -12574,7 +12574,7 @@
         <v>1353</v>
       </c>
       <c r="I210">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="K210" t="s">
         <v>1360</v>
@@ -12670,7 +12670,7 @@
         <v>1353</v>
       </c>
       <c r="I213">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="K213" t="s">
         <v>1357</v>
@@ -12708,7 +12708,7 @@
         <v>1353</v>
       </c>
       <c r="I214">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="J214">
         <v>14</v>
@@ -12755,7 +12755,7 @@
         <v>1353</v>
       </c>
       <c r="I215">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="K215" t="s">
         <v>1357</v>
@@ -12822,7 +12822,7 @@
         <v>1353</v>
       </c>
       <c r="I217">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="J217">
         <v>42</v>
@@ -12866,7 +12866,7 @@
         <v>1353</v>
       </c>
       <c r="I218">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="J218">
         <v>166</v>
@@ -12954,7 +12954,7 @@
         <v>1353</v>
       </c>
       <c r="I220">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="J220">
         <v>154</v>
@@ -13112,7 +13112,7 @@
         <v>1353</v>
       </c>
       <c r="I224">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="J224">
         <v>204</v>
@@ -13267,7 +13267,7 @@
         <v>1353</v>
       </c>
       <c r="I228">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="J228">
         <v>204</v>
@@ -13346,7 +13346,7 @@
         <v>1353</v>
       </c>
       <c r="I230">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="J230">
         <v>197</v>
@@ -13390,7 +13390,7 @@
         <v>1353</v>
       </c>
       <c r="I231">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="J231">
         <v>35</v>
@@ -13492,7 +13492,7 @@
         <v>1353</v>
       </c>
       <c r="I234">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="J234">
         <v>35</v>
@@ -13539,7 +13539,7 @@
         <v>1353</v>
       </c>
       <c r="I235">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="J235">
         <v>35</v>
@@ -13586,7 +13586,7 @@
         <v>1353</v>
       </c>
       <c r="I236">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="J236">
         <v>86</v>
@@ -13703,7 +13703,7 @@
         <v>1353</v>
       </c>
       <c r="I239">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="K239" t="s">
         <v>1330</v>
@@ -13802,7 +13802,7 @@
         <v>1353</v>
       </c>
       <c r="I242">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="K242" t="s">
         <v>1356</v>
@@ -13869,7 +13869,7 @@
         <v>1353</v>
       </c>
       <c r="I244">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="J244">
         <v>15</v>
@@ -13910,7 +13910,7 @@
         <v>1353</v>
       </c>
       <c r="I245">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="J245">
         <v>15</v>
@@ -14053,7 +14053,7 @@
         <v>1353</v>
       </c>
       <c r="I249">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="K249" t="s">
         <v>1357</v>
@@ -14187,7 +14187,7 @@
         <v>1353</v>
       </c>
       <c r="I253">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="J253">
         <v>162</v>
@@ -14231,7 +14231,7 @@
         <v>1353</v>
       </c>
       <c r="I254">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="K254" t="s">
         <v>1360</v>
@@ -14269,7 +14269,7 @@
         <v>1353</v>
       </c>
       <c r="I255">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="J255">
         <v>72</v>
@@ -14313,7 +14313,7 @@
         <v>1353</v>
       </c>
       <c r="I256">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="J256">
         <v>23</v>
@@ -14415,7 +14415,7 @@
         <v>1353</v>
       </c>
       <c r="I259">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="J259">
         <v>72</v>
@@ -14459,7 +14459,7 @@
         <v>1353</v>
       </c>
       <c r="I260">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="J260">
         <v>84</v>
@@ -14503,7 +14503,7 @@
         <v>1353</v>
       </c>
       <c r="I261">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="J261">
         <v>162</v>
@@ -14620,7 +14620,7 @@
         <v>1353</v>
       </c>
       <c r="I264">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="J264">
         <v>162</v>
@@ -14664,7 +14664,7 @@
         <v>1353</v>
       </c>
       <c r="I265">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="J265">
         <v>162</v>
@@ -14708,7 +14708,7 @@
         <v>1353</v>
       </c>
       <c r="I266">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="J266">
         <v>84</v>
@@ -14752,7 +14752,7 @@
         <v>1353</v>
       </c>
       <c r="I267">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="K267" t="s">
         <v>1360</v>
@@ -14790,7 +14790,7 @@
         <v>1353</v>
       </c>
       <c r="I268">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="K268" t="s">
         <v>1357</v>
@@ -14825,7 +14825,7 @@
         <v>1353</v>
       </c>
       <c r="I269">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="K269" t="s">
         <v>1357</v>
@@ -14863,7 +14863,7 @@
         <v>1353</v>
       </c>
       <c r="I270">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="K270" t="s">
         <v>1360</v>
@@ -14901,7 +14901,7 @@
         <v>1353</v>
       </c>
       <c r="I271">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="K271" t="s">
         <v>1360</v>
@@ -15079,7 +15079,7 @@
         <v>1353</v>
       </c>
       <c r="I276">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="K276" t="s">
         <v>1361</v>
@@ -15117,7 +15117,7 @@
         <v>1353</v>
       </c>
       <c r="I277">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="K277" t="s">
         <v>1357</v>
@@ -15155,7 +15155,7 @@
         <v>1353</v>
       </c>
       <c r="I278">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="J278">
         <v>148</v>
@@ -15199,7 +15199,7 @@
         <v>1353</v>
       </c>
       <c r="I279">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="K279" t="s">
         <v>1359</v>
@@ -15240,7 +15240,7 @@
         <v>1353</v>
       </c>
       <c r="I280">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K280" t="s">
         <v>1357</v>
@@ -15278,7 +15278,7 @@
         <v>1353</v>
       </c>
       <c r="I281">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K281" t="s">
         <v>1357</v>
@@ -15319,7 +15319,7 @@
         <v>1353</v>
       </c>
       <c r="I282">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="K282" t="s">
         <v>1357</v>
@@ -15502,7 +15502,7 @@
         <v>1353</v>
       </c>
       <c r="I288">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="J288">
         <v>28</v>
@@ -15575,7 +15575,7 @@
         <v>1353</v>
       </c>
       <c r="I290">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="J290">
         <v>20</v>
@@ -15619,7 +15619,7 @@
         <v>1353</v>
       </c>
       <c r="I291">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="J291">
         <v>20</v>
@@ -15663,7 +15663,7 @@
         <v>1353</v>
       </c>
       <c r="I292">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="K292" t="s">
         <v>1360</v>
@@ -15701,7 +15701,7 @@
         <v>1353</v>
       </c>
       <c r="I293">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="K293" t="s">
         <v>1361</v>
@@ -15739,7 +15739,7 @@
         <v>1353</v>
       </c>
       <c r="I294">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="K294" t="s">
         <v>1366</v>
@@ -15774,7 +15774,7 @@
         <v>1353</v>
       </c>
       <c r="I295">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="K295" t="s">
         <v>1366</v>
@@ -15809,7 +15809,7 @@
         <v>1353</v>
       </c>
       <c r="I296">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="K296" t="s">
         <v>1366</v>
@@ -15882,7 +15882,7 @@
         <v>1353</v>
       </c>
       <c r="I298">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="J298">
         <v>58</v>
@@ -15923,7 +15923,7 @@
         <v>1353</v>
       </c>
       <c r="I299">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="J299">
         <v>100</v>
@@ -15967,7 +15967,7 @@
         <v>1353</v>
       </c>
       <c r="I300">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="J300">
         <v>86</v>
@@ -16011,7 +16011,7 @@
         <v>1353</v>
       </c>
       <c r="I301">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="J301">
         <v>102</v>
@@ -16055,7 +16055,7 @@
         <v>1353</v>
       </c>
       <c r="I302">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="K302" t="s">
         <v>1360</v>
@@ -16093,7 +16093,7 @@
         <v>1353</v>
       </c>
       <c r="I303">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="K303" t="s">
         <v>1357</v>
@@ -16131,7 +16131,7 @@
         <v>1353</v>
       </c>
       <c r="I304">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="K304" t="s">
         <v>1360</v>
@@ -16169,7 +16169,7 @@
         <v>1353</v>
       </c>
       <c r="I305">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="J305">
         <v>35</v>
@@ -16213,7 +16213,7 @@
         <v>1353</v>
       </c>
       <c r="I306">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="J306">
         <v>31</v>
@@ -16301,7 +16301,7 @@
         <v>1353</v>
       </c>
       <c r="I308">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="K308" t="s">
         <v>1356</v>
@@ -16377,7 +16377,7 @@
         <v>1353</v>
       </c>
       <c r="I310">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="J310">
         <v>107</v>
@@ -16421,7 +16421,7 @@
         <v>1353</v>
       </c>
       <c r="I311">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="K311" t="s">
         <v>1356</v>
@@ -16611,7 +16611,7 @@
         <v>1353</v>
       </c>
       <c r="I316">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="K316" t="s">
         <v>1357</v>
@@ -16754,7 +16754,7 @@
         <v>1353</v>
       </c>
       <c r="I320">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="K320" t="s">
         <v>1361</v>
@@ -16792,7 +16792,7 @@
         <v>1353</v>
       </c>
       <c r="I321">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="K321" t="s">
         <v>1357</v>
@@ -16830,7 +16830,7 @@
         <v>1353</v>
       </c>
       <c r="I322">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="J322">
         <v>57</v>
@@ -16944,7 +16944,7 @@
         <v>1353</v>
       </c>
       <c r="I325">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="J325">
         <v>57</v>
@@ -17026,7 +17026,7 @@
         <v>1353</v>
       </c>
       <c r="I327">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="J327">
         <v>57</v>
@@ -17070,7 +17070,7 @@
         <v>1353</v>
       </c>
       <c r="I328">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="J328">
         <v>57</v>
@@ -17114,7 +17114,7 @@
         <v>1353</v>
       </c>
       <c r="I329">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="J329">
         <v>57</v>
@@ -17158,7 +17158,7 @@
         <v>1353</v>
       </c>
       <c r="I330">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="J330">
         <v>57</v>
@@ -17202,7 +17202,7 @@
         <v>1353</v>
       </c>
       <c r="I331">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="K331" t="s">
         <v>1356</v>
@@ -17240,7 +17240,7 @@
         <v>1353</v>
       </c>
       <c r="I332">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="K332" t="s">
         <v>1357</v>
@@ -17278,7 +17278,7 @@
         <v>1353</v>
       </c>
       <c r="I333">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="J333">
         <v>100</v>
@@ -17322,7 +17322,7 @@
         <v>1353</v>
       </c>
       <c r="I334">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="K334" t="s">
         <v>1357</v>
@@ -17398,7 +17398,7 @@
         <v>1353</v>
       </c>
       <c r="I336">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="J336">
         <v>28</v>
@@ -17480,7 +17480,7 @@
         <v>1353</v>
       </c>
       <c r="I338">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="J338">
         <v>12</v>
@@ -17553,7 +17553,7 @@
         <v>1353</v>
       </c>
       <c r="I340">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="J340">
         <v>98</v>
@@ -17594,7 +17594,7 @@
         <v>1353</v>
       </c>
       <c r="I341">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="J341">
         <v>90</v>
@@ -17635,7 +17635,7 @@
         <v>1353</v>
       </c>
       <c r="I342">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="K342" t="s">
         <v>1356</v>
@@ -17749,7 +17749,7 @@
         <v>1353</v>
       </c>
       <c r="I345">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="K345" t="s">
         <v>1356</v>
@@ -17825,7 +17825,7 @@
         <v>1353</v>
       </c>
       <c r="I347">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="J347">
         <v>18</v>
@@ -17872,7 +17872,7 @@
         <v>1353</v>
       </c>
       <c r="I348">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="J348">
         <v>14</v>
@@ -17916,7 +17916,7 @@
         <v>1353</v>
       </c>
       <c r="I349">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="K349" t="s">
         <v>1361</v>
@@ -17954,7 +17954,7 @@
         <v>1353</v>
       </c>
       <c r="I350">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="J350">
         <v>46</v>
@@ -17992,7 +17992,7 @@
         <v>1353</v>
       </c>
       <c r="I351">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="J351">
         <v>82</v>
@@ -18036,7 +18036,7 @@
         <v>1353</v>
       </c>
       <c r="I352">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="J352">
         <v>78</v>
@@ -18080,7 +18080,7 @@
         <v>1353</v>
       </c>
       <c r="I353">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="J353">
         <v>83</v>
@@ -18124,7 +18124,7 @@
         <v>1353</v>
       </c>
       <c r="I354">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="K354" t="s">
         <v>1360</v>
@@ -18162,7 +18162,7 @@
         <v>1353</v>
       </c>
       <c r="I355">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="J355">
         <v>8</v>
@@ -18244,7 +18244,7 @@
         <v>1353</v>
       </c>
       <c r="I357">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="J357">
         <v>85</v>
@@ -18367,7 +18367,7 @@
         <v>1353</v>
       </c>
       <c r="I360">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="J360">
         <v>83</v>
@@ -18414,7 +18414,7 @@
         <v>1353</v>
       </c>
       <c r="I361">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="J361">
         <v>83</v>
@@ -18458,7 +18458,7 @@
         <v>1353</v>
       </c>
       <c r="I362">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="K362" t="s">
         <v>1360</v>
@@ -18496,7 +18496,7 @@
         <v>1353</v>
       </c>
       <c r="I363">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="K363" t="s">
         <v>1360</v>
@@ -18534,7 +18534,7 @@
         <v>1353</v>
       </c>
       <c r="I364">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="J364">
         <v>83</v>
@@ -18578,7 +18578,7 @@
         <v>1353</v>
       </c>
       <c r="I365">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="J365">
         <v>15</v>
@@ -18619,7 +18619,7 @@
         <v>1353</v>
       </c>
       <c r="I366">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="J366">
         <v>77</v>
@@ -18663,7 +18663,7 @@
         <v>1353</v>
       </c>
       <c r="I367">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="J367">
         <v>77</v>
@@ -18707,7 +18707,7 @@
         <v>1353</v>
       </c>
       <c r="I368">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="J368">
         <v>77</v>
@@ -18751,7 +18751,7 @@
         <v>1353</v>
       </c>
       <c r="I369">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="K369" t="s">
         <v>1360</v>
@@ -18789,7 +18789,7 @@
         <v>1353</v>
       </c>
       <c r="I370">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="K370" t="s">
         <v>1360</v>
@@ -18827,7 +18827,7 @@
         <v>1353</v>
       </c>
       <c r="I371">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="J371">
         <v>16</v>
@@ -18915,7 +18915,7 @@
         <v>1353</v>
       </c>
       <c r="I373">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="K373" t="s">
         <v>1356</v>
@@ -18953,7 +18953,7 @@
         <v>1353</v>
       </c>
       <c r="I374">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="K374" t="s">
         <v>1356</v>
@@ -18991,7 +18991,7 @@
         <v>1353</v>
       </c>
       <c r="I375">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="J375">
         <v>94</v>
@@ -19032,7 +19032,7 @@
         <v>1353</v>
       </c>
       <c r="I376">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="K376" t="s">
         <v>1360</v>
@@ -19111,7 +19111,7 @@
         <v>1353</v>
       </c>
       <c r="I378">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="K378" t="s">
         <v>1360</v>
@@ -19149,7 +19149,7 @@
         <v>1353</v>
       </c>
       <c r="I379">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="J379">
         <v>20</v>
@@ -19193,7 +19193,7 @@
         <v>1353</v>
       </c>
       <c r="I380">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="J380">
         <v>94</v>
@@ -19237,7 +19237,7 @@
         <v>1353</v>
       </c>
       <c r="I381">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="K381" t="s">
         <v>1360</v>
@@ -19275,7 +19275,7 @@
         <v>1353</v>
       </c>
       <c r="I382">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="K382" t="s">
         <v>1360</v>
@@ -19313,7 +19313,7 @@
         <v>1353</v>
       </c>
       <c r="I383">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="J383">
         <v>71</v>
@@ -19357,7 +19357,7 @@
         <v>1353</v>
       </c>
       <c r="I384">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="K384" t="s">
         <v>1357</v>
@@ -19395,7 +19395,7 @@
         <v>1353</v>
       </c>
       <c r="I385">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="J385">
         <v>102</v>
@@ -19442,7 +19442,7 @@
         <v>1353</v>
       </c>
       <c r="I386">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="K386" t="s">
         <v>1360</v>
@@ -19480,7 +19480,7 @@
         <v>1353</v>
       </c>
       <c r="I387">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="K387" t="s">
         <v>1360</v>
@@ -19518,7 +19518,7 @@
         <v>1353</v>
       </c>
       <c r="I388">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="J388">
         <v>-85</v>
@@ -19562,7 +19562,7 @@
         <v>1353</v>
       </c>
       <c r="I389">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="K389" t="s">
         <v>1361</v>
@@ -19720,7 +19720,7 @@
         <v>1353</v>
       </c>
       <c r="I393">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="J393">
         <v>20</v>
@@ -20016,7 +20016,7 @@
         <v>1353</v>
       </c>
       <c r="I400">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="K400" t="s">
         <v>1360</v>
@@ -20092,7 +20092,7 @@
         <v>1353</v>
       </c>
       <c r="I402">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="K402" t="s">
         <v>1360</v>
@@ -20130,7 +20130,7 @@
         <v>1353</v>
       </c>
       <c r="I403">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="J403">
         <v>83</v>
@@ -20174,7 +20174,7 @@
         <v>1353</v>
       </c>
       <c r="I404">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="K404" t="s">
         <v>1360</v>
@@ -20244,7 +20244,7 @@
         <v>1353</v>
       </c>
       <c r="I406">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="Q406" t="b">
         <v>1</v>
@@ -20276,7 +20276,7 @@
         <v>1353</v>
       </c>
       <c r="I407">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="Q407" t="b">
         <v>1</v>
@@ -20308,7 +20308,7 @@
         <v>1353</v>
       </c>
       <c r="I408">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="Q408" t="b">
         <v>1</v>
@@ -20340,7 +20340,7 @@
         <v>1353</v>
       </c>
       <c r="I409">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="Q409" t="b">
         <v>1</v>
@@ -20372,7 +20372,7 @@
         <v>1353</v>
       </c>
       <c r="I410">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="Q410" t="b">
         <v>1</v>
@@ -20404,7 +20404,7 @@
         <v>1353</v>
       </c>
       <c r="I411">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="Q411" t="b">
         <v>1</v>
@@ -20436,7 +20436,7 @@
         <v>1353</v>
       </c>
       <c r="I412">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="Q412" t="b">
         <v>1</v>
@@ -20468,7 +20468,7 @@
         <v>1353</v>
       </c>
       <c r="I413">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="Q413" t="b">
         <v>1</v>
@@ -20558,7 +20558,7 @@
         <v>1353</v>
       </c>
       <c r="I416">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="Q416" t="b">
         <v>1</v>
@@ -20648,7 +20648,7 @@
         <v>1353</v>
       </c>
       <c r="I419">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="Q419" t="b">
         <v>1</v>
@@ -20680,7 +20680,7 @@
         <v>1353</v>
       </c>
       <c r="I420">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="Q420" t="b">
         <v>1</v>
@@ -20712,7 +20712,7 @@
         <v>1353</v>
       </c>
       <c r="I421">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="Q421" t="b">
         <v>1</v>
@@ -20744,7 +20744,7 @@
         <v>1353</v>
       </c>
       <c r="I422">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="Q422" t="b">
         <v>1</v>
@@ -20776,7 +20776,7 @@
         <v>1353</v>
       </c>
       <c r="I423">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="Q423" t="b">
         <v>1</v>
@@ -20808,7 +20808,7 @@
         <v>1353</v>
       </c>
       <c r="I424">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="Q424" t="b">
         <v>1</v>
@@ -20840,7 +20840,7 @@
         <v>1353</v>
       </c>
       <c r="I425">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="Q425" t="b">
         <v>1</v>
@@ -20872,7 +20872,7 @@
         <v>1353</v>
       </c>
       <c r="I426">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="Q426" t="b">
         <v>1</v>
@@ -20904,7 +20904,7 @@
         <v>1353</v>
       </c>
       <c r="I427">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="Q427" t="b">
         <v>1</v>
@@ -20994,7 +20994,7 @@
         <v>1353</v>
       </c>
       <c r="I430">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="Q430" t="b">
         <v>1</v>
@@ -21026,7 +21026,7 @@
         <v>1353</v>
       </c>
       <c r="I431">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="Q431" t="b">
         <v>1</v>
@@ -21058,7 +21058,7 @@
         <v>1353</v>
       </c>
       <c r="I432">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="Q432" t="b">
         <v>1</v>
@@ -21090,7 +21090,7 @@
         <v>1353</v>
       </c>
       <c r="I433">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="Q433" t="b">
         <v>1</v>
@@ -21122,7 +21122,7 @@
         <v>1353</v>
       </c>
       <c r="I434">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="Q434" t="b">
         <v>1</v>
@@ -21154,7 +21154,7 @@
         <v>1353</v>
       </c>
       <c r="I435">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="Q435" t="b">
         <v>1</v>
@@ -21186,7 +21186,7 @@
         <v>1353</v>
       </c>
       <c r="I436">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="Q436" t="b">
         <v>1</v>
@@ -21218,7 +21218,7 @@
         <v>1355</v>
       </c>
       <c r="I437">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="Q437" t="b">
         <v>1</v>
@@ -21250,7 +21250,7 @@
         <v>1355</v>
       </c>
       <c r="I438">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="Q438" t="b">
         <v>1</v>
@@ -21282,7 +21282,7 @@
         <v>1353</v>
       </c>
       <c r="I439">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="Q439" t="b">
         <v>1</v>
@@ -21314,7 +21314,7 @@
         <v>1353</v>
       </c>
       <c r="I440">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="Q440" t="b">
         <v>1</v>
@@ -21346,7 +21346,7 @@
         <v>1353</v>
       </c>
       <c r="I441">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="Q441" t="b">
         <v>1</v>
@@ -21407,7 +21407,7 @@
         <v>1353</v>
       </c>
       <c r="I443">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="Q443" t="b">
         <v>1</v>
@@ -21497,7 +21497,7 @@
         <v>1353</v>
       </c>
       <c r="I446">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="Q446" t="b">
         <v>1</v>
@@ -21529,7 +21529,7 @@
         <v>1353</v>
       </c>
       <c r="I447">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="Q447" t="b">
         <v>1</v>
@@ -21561,7 +21561,7 @@
         <v>1353</v>
       </c>
       <c r="I448">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="Q448" t="b">
         <v>1</v>
@@ -21593,7 +21593,7 @@
         <v>1353</v>
       </c>
       <c r="I449">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="Q449" t="b">
         <v>1</v>
@@ -21625,7 +21625,7 @@
         <v>1353</v>
       </c>
       <c r="I450">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="Q450" t="b">
         <v>1</v>
@@ -21657,7 +21657,7 @@
         <v>1353</v>
       </c>
       <c r="I451">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="Q451" t="b">
         <v>1</v>
@@ -21689,7 +21689,7 @@
         <v>1353</v>
       </c>
       <c r="I452">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="Q452" t="b">
         <v>1</v>
@@ -21721,7 +21721,7 @@
         <v>1353</v>
       </c>
       <c r="I453">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="Q453" t="b">
         <v>1</v>
@@ -21753,7 +21753,7 @@
         <v>1353</v>
       </c>
       <c r="I454">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="Q454" t="b">
         <v>1</v>
@@ -21785,7 +21785,7 @@
         <v>1353</v>
       </c>
       <c r="I455">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="Q455" t="b">
         <v>1</v>
@@ -21817,7 +21817,7 @@
         <v>1353</v>
       </c>
       <c r="I456">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="Q456" t="b">
         <v>1</v>
@@ -21849,7 +21849,7 @@
         <v>1353</v>
       </c>
       <c r="I457">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="Q457" t="b">
         <v>1</v>
@@ -21881,7 +21881,7 @@
         <v>1353</v>
       </c>
       <c r="I458">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Q458" t="b">
         <v>1</v>
@@ -21913,7 +21913,7 @@
         <v>1353</v>
       </c>
       <c r="I459">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="Q459" t="b">
         <v>1</v>
@@ -21945,7 +21945,7 @@
         <v>1353</v>
       </c>
       <c r="I460">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="Q460" t="b">
         <v>1</v>
@@ -21977,7 +21977,7 @@
         <v>1353</v>
       </c>
       <c r="I461">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="Q461" t="b">
         <v>1</v>
@@ -22009,7 +22009,7 @@
         <v>1353</v>
       </c>
       <c r="I462">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="Q462" t="b">
         <v>1</v>
@@ -22041,7 +22041,7 @@
         <v>1353</v>
       </c>
       <c r="I463">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="Q463" t="b">
         <v>1</v>
@@ -22073,7 +22073,7 @@
         <v>1353</v>
       </c>
       <c r="I464">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="Q464" t="b">
         <v>1</v>
@@ -22105,7 +22105,7 @@
         <v>1353</v>
       </c>
       <c r="I465">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="Q465" t="b">
         <v>1</v>
@@ -22137,7 +22137,7 @@
         <v>1353</v>
       </c>
       <c r="I466">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="Q466" t="b">
         <v>1</v>
@@ -22169,7 +22169,7 @@
         <v>1353</v>
       </c>
       <c r="I467">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="Q467" t="b">
         <v>1</v>
@@ -22201,7 +22201,7 @@
         <v>1353</v>
       </c>
       <c r="I468">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="Q468" t="b">
         <v>1</v>
@@ -22233,7 +22233,7 @@
         <v>1353</v>
       </c>
       <c r="I469">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="Q469" t="b">
         <v>1</v>
@@ -22294,7 +22294,7 @@
         <v>1353</v>
       </c>
       <c r="I471">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="Q471" t="b">
         <v>1</v>
@@ -22326,7 +22326,7 @@
         <v>1353</v>
       </c>
       <c r="I472">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="Q472" t="b">
         <v>1</v>
@@ -22358,7 +22358,7 @@
         <v>1353</v>
       </c>
       <c r="I473">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="Q473" t="b">
         <v>1</v>
@@ -22390,7 +22390,7 @@
         <v>1353</v>
       </c>
       <c r="I474">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Q474" t="b">
         <v>1</v>
@@ -22422,7 +22422,7 @@
         <v>1353</v>
       </c>
       <c r="I475">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Q475" t="b">
         <v>1</v>
@@ -22454,7 +22454,7 @@
         <v>1353</v>
       </c>
       <c r="I476">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Q476" t="b">
         <v>1</v>
@@ -22486,7 +22486,7 @@
         <v>1353</v>
       </c>
       <c r="I477">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Q477" t="b">
         <v>1</v>
@@ -22518,7 +22518,7 @@
         <v>1353</v>
       </c>
       <c r="I478">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Q478" t="b">
         <v>1</v>
@@ -22550,7 +22550,7 @@
         <v>1353</v>
       </c>
       <c r="I479">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Q479" t="b">
         <v>1</v>
@@ -22582,7 +22582,7 @@
         <v>1353</v>
       </c>
       <c r="I480">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Q480" t="b">
         <v>1</v>
@@ -22614,7 +22614,7 @@
         <v>1353</v>
       </c>
       <c r="I481">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Q481" t="b">
         <v>1</v>
@@ -22646,7 +22646,7 @@
         <v>1353</v>
       </c>
       <c r="I482">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Q482" t="b">
         <v>1</v>
@@ -22678,7 +22678,7 @@
         <v>1353</v>
       </c>
       <c r="I483">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Q483" t="b">
         <v>1</v>
@@ -22710,7 +22710,7 @@
         <v>1353</v>
       </c>
       <c r="I484">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Q484" t="b">
         <v>1</v>
@@ -22742,7 +22742,7 @@
         <v>1353</v>
       </c>
       <c r="I485">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Q485" t="b">
         <v>1</v>
@@ -22774,7 +22774,7 @@
         <v>1353</v>
       </c>
       <c r="I486">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Q486" t="b">
         <v>1</v>
@@ -22806,7 +22806,7 @@
         <v>1353</v>
       </c>
       <c r="I487">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Q487" t="b">
         <v>1</v>
@@ -22838,7 +22838,7 @@
         <v>1353</v>
       </c>
       <c r="I488">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Q488" t="b">
         <v>1</v>
@@ -22870,7 +22870,7 @@
         <v>1353</v>
       </c>
       <c r="I489">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Q489" t="b">
         <v>1</v>
@@ -22902,7 +22902,7 @@
         <v>1353</v>
       </c>
       <c r="I490">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Q490" t="b">
         <v>1</v>
@@ -22934,7 +22934,7 @@
         <v>1353</v>
       </c>
       <c r="I491">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Q491" t="b">
         <v>1</v>
@@ -22966,7 +22966,7 @@
         <v>1355</v>
       </c>
       <c r="I492">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Q492" t="b">
         <v>1</v>
@@ -22998,7 +22998,7 @@
         <v>1355</v>
       </c>
       <c r="I493">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Q493" t="b">
         <v>1</v>
@@ -23030,7 +23030,7 @@
         <v>1355</v>
       </c>
       <c r="I494">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Q494" t="b">
         <v>1</v>
@@ -23062,7 +23062,7 @@
         <v>1355</v>
       </c>
       <c r="I495">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Q495" t="b">
         <v>1</v>
@@ -23094,7 +23094,7 @@
         <v>1355</v>
       </c>
       <c r="I496">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Q496" t="b">
         <v>1</v>
@@ -23126,7 +23126,7 @@
         <v>1353</v>
       </c>
       <c r="I497">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Q497" t="b">
         <v>1</v>
@@ -23158,7 +23158,7 @@
         <v>1353</v>
       </c>
       <c r="I498">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Q498" t="b">
         <v>1</v>
@@ -23190,7 +23190,7 @@
         <v>1355</v>
       </c>
       <c r="I499">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Q499" t="b">
         <v>1</v>
@@ -23222,7 +23222,7 @@
         <v>1353</v>
       </c>
       <c r="I500">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Q500" t="b">
         <v>1</v>
@@ -23254,7 +23254,7 @@
         <v>1353</v>
       </c>
       <c r="I501">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Q501" t="b">
         <v>1</v>
@@ -23286,7 +23286,7 @@
         <v>1353</v>
       </c>
       <c r="I502">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Q502" t="b">
         <v>1</v>
@@ -23318,7 +23318,7 @@
         <v>1353</v>
       </c>
       <c r="I503">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Q503" t="b">
         <v>1</v>
@@ -23350,7 +23350,7 @@
         <v>1353</v>
       </c>
       <c r="I504">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="Q504" t="b">
         <v>1</v>
@@ -23382,7 +23382,7 @@
         <v>1353</v>
       </c>
       <c r="I505">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="Q505" t="b">
         <v>1</v>
@@ -23414,7 +23414,7 @@
         <v>1353</v>
       </c>
       <c r="I506">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="Q506" t="b">
         <v>1</v>
@@ -23446,7 +23446,7 @@
         <v>1353</v>
       </c>
       <c r="I507">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q507" t="b">
         <v>1</v>
@@ -23507,7 +23507,7 @@
         <v>1353</v>
       </c>
       <c r="I509">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q509" t="b">
         <v>1</v>
@@ -23539,7 +23539,7 @@
         <v>1353</v>
       </c>
       <c r="I510">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q510" t="b">
         <v>1</v>
@@ -23571,7 +23571,7 @@
         <v>1353</v>
       </c>
       <c r="I511">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="Q511" t="b">
         <v>1</v>
@@ -23603,7 +23603,7 @@
         <v>1353</v>
       </c>
       <c r="I512">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="Q512" t="b">
         <v>1</v>
@@ -23635,7 +23635,7 @@
         <v>1353</v>
       </c>
       <c r="I513">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q513" t="b">
         <v>1</v>
@@ -23667,7 +23667,7 @@
         <v>1353</v>
       </c>
       <c r="I514">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q514" t="b">
         <v>1</v>
@@ -23699,7 +23699,7 @@
         <v>1353</v>
       </c>
       <c r="I515">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q515" t="b">
         <v>1</v>
@@ -23731,7 +23731,7 @@
         <v>1353</v>
       </c>
       <c r="I516">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Q516" t="b">
         <v>1</v>
@@ -23763,7 +23763,7 @@
         <v>1353</v>
       </c>
       <c r="I517">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Q517" t="b">
         <v>1</v>
@@ -23795,7 +23795,7 @@
         <v>1353</v>
       </c>
       <c r="I518">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Q518" t="b">
         <v>1</v>
@@ -23827,7 +23827,7 @@
         <v>1353</v>
       </c>
       <c r="I519">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="Q519" t="b">
         <v>1</v>
@@ -23859,7 +23859,7 @@
         <v>1353</v>
       </c>
       <c r="I520">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="Q520" t="b">
         <v>1</v>
@@ -23891,7 +23891,7 @@
         <v>1353</v>
       </c>
       <c r="I521">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="Q521" t="b">
         <v>1</v>
@@ -23923,7 +23923,7 @@
         <v>1353</v>
       </c>
       <c r="I522">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="Q522" t="b">
         <v>1</v>
@@ -23955,7 +23955,7 @@
         <v>1353</v>
       </c>
       <c r="I523">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="Q523" t="b">
         <v>1</v>
@@ -23987,7 +23987,7 @@
         <v>1353</v>
       </c>
       <c r="I524">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="Q524" t="b">
         <v>1</v>
@@ -24019,7 +24019,7 @@
         <v>1353</v>
       </c>
       <c r="I525">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="Q525" t="b">
         <v>1</v>
@@ -24051,7 +24051,7 @@
         <v>1353</v>
       </c>
       <c r="I526">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="Q526" t="b">
         <v>1</v>
@@ -24083,7 +24083,7 @@
         <v>1353</v>
       </c>
       <c r="I527">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="Q527" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: reparaveis (06/10/2026 13:47)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
@@ -5158,7 +5158,7 @@
         <v>1417</v>
       </c>
       <c r="I2">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="K2" t="s">
         <v>1420</v>
@@ -5196,7 +5196,7 @@
         <v>1417</v>
       </c>
       <c r="I3">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="K3" t="s">
         <v>1421</v>
@@ -5234,7 +5234,7 @@
         <v>1417</v>
       </c>
       <c r="I4">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="K4" t="s">
         <v>1421</v>
@@ -5272,7 +5272,7 @@
         <v>1417</v>
       </c>
       <c r="I5">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="J5">
         <v>279</v>
@@ -5316,7 +5316,7 @@
         <v>1417</v>
       </c>
       <c r="I6">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="J6">
         <v>153</v>
@@ -5360,7 +5360,7 @@
         <v>1417</v>
       </c>
       <c r="I7">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="J7">
         <v>112</v>
@@ -5436,7 +5436,7 @@
         <v>1417</v>
       </c>
       <c r="I9">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="J9">
         <v>362</v>
@@ -5483,7 +5483,7 @@
         <v>1417</v>
       </c>
       <c r="I10">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="J10">
         <v>378</v>
@@ -5530,7 +5530,7 @@
         <v>1417</v>
       </c>
       <c r="I11">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="J11">
         <v>112</v>
@@ -5577,7 +5577,7 @@
         <v>1417</v>
       </c>
       <c r="I12">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="J12">
         <v>124</v>
@@ -5650,7 +5650,7 @@
         <v>1417</v>
       </c>
       <c r="I14">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="J14">
         <v>64</v>
@@ -5729,7 +5729,7 @@
         <v>1417</v>
       </c>
       <c r="I16">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="K16" t="s">
         <v>1420</v>
@@ -5767,7 +5767,7 @@
         <v>1417</v>
       </c>
       <c r="I17">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="J17">
         <v>161</v>
@@ -5811,7 +5811,7 @@
         <v>1417</v>
       </c>
       <c r="I18">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="J18">
         <v>66</v>
@@ -5884,7 +5884,7 @@
         <v>1417</v>
       </c>
       <c r="I20">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="J20">
         <v>399</v>
@@ -5957,7 +5957,7 @@
         <v>1417</v>
       </c>
       <c r="I22">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="K22" t="s">
         <v>1424</v>
@@ -5995,7 +5995,7 @@
         <v>1417</v>
       </c>
       <c r="I23">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="J23">
         <v>229</v>
@@ -6100,7 +6100,7 @@
         <v>1417</v>
       </c>
       <c r="I26">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="J26">
         <v>155</v>
@@ -6147,7 +6147,7 @@
         <v>1417</v>
       </c>
       <c r="I27">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="K27" t="s">
         <v>1424</v>
@@ -6243,7 +6243,7 @@
         <v>1417</v>
       </c>
       <c r="I30">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="J30">
         <v>209</v>
@@ -6316,7 +6316,7 @@
         <v>1417</v>
       </c>
       <c r="I32">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="K32" t="s">
         <v>1420</v>
@@ -6525,7 +6525,7 @@
         <v>1417</v>
       </c>
       <c r="I39">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="K39" t="s">
         <v>1425</v>
@@ -6688,7 +6688,7 @@
         <v>1417</v>
       </c>
       <c r="I44">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="J44">
         <v>87</v>
@@ -6735,7 +6735,7 @@
         <v>1417</v>
       </c>
       <c r="I45">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="J45">
         <v>331</v>
@@ -6782,7 +6782,7 @@
         <v>1417</v>
       </c>
       <c r="I46">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="K46" t="s">
         <v>1424</v>
@@ -6820,7 +6820,7 @@
         <v>1417</v>
       </c>
       <c r="I47">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="J47">
         <v>344</v>
@@ -6867,7 +6867,7 @@
         <v>1417</v>
       </c>
       <c r="I48">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="K48" t="s">
         <v>1424</v>
@@ -6934,7 +6934,7 @@
         <v>1417</v>
       </c>
       <c r="I50">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="K50" t="s">
         <v>1424</v>
@@ -7001,7 +7001,7 @@
         <v>1417</v>
       </c>
       <c r="I52">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="K52" t="s">
         <v>1420</v>
@@ -7039,7 +7039,7 @@
         <v>1417</v>
       </c>
       <c r="I53">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="K53" t="s">
         <v>1421</v>
@@ -7077,7 +7077,7 @@
         <v>1417</v>
       </c>
       <c r="I54">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="K54" t="s">
         <v>1421</v>
@@ -7353,7 +7353,7 @@
         <v>1417</v>
       </c>
       <c r="I63">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="J63">
         <v>293</v>
@@ -7400,7 +7400,7 @@
         <v>1417</v>
       </c>
       <c r="I64">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="J64">
         <v>320</v>
@@ -7630,7 +7630,7 @@
         <v>1417</v>
       </c>
       <c r="I71">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="J71">
         <v>429</v>
@@ -7703,7 +7703,7 @@
         <v>1417</v>
       </c>
       <c r="I73">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="K73" t="s">
         <v>1420</v>
@@ -7811,7 +7811,7 @@
         <v>1417</v>
       </c>
       <c r="I76">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="K76" t="s">
         <v>1427</v>
@@ -7904,7 +7904,7 @@
         <v>1417</v>
       </c>
       <c r="I79">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="K79" t="s">
         <v>1427</v>
@@ -8009,7 +8009,7 @@
         <v>1417</v>
       </c>
       <c r="I82">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="K82" t="s">
         <v>1424</v>
@@ -8076,7 +8076,7 @@
         <v>1417</v>
       </c>
       <c r="I84">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="J84">
         <v>40</v>
@@ -8123,7 +8123,7 @@
         <v>1417</v>
       </c>
       <c r="I85">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="K85" t="s">
         <v>1421</v>
@@ -8161,7 +8161,7 @@
         <v>1417</v>
       </c>
       <c r="I86">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="K86" t="s">
         <v>1421</v>
@@ -8199,7 +8199,7 @@
         <v>1417</v>
       </c>
       <c r="I87">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="J87">
         <v>-16</v>
@@ -8322,7 +8322,7 @@
         <v>1417</v>
       </c>
       <c r="I90">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="K90" t="s">
         <v>1394</v>
@@ -8471,7 +8471,7 @@
         <v>1417</v>
       </c>
       <c r="I94">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="K94" t="s">
         <v>1424</v>
@@ -8550,7 +8550,7 @@
         <v>1417</v>
       </c>
       <c r="I96">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="J96">
         <v>17</v>
@@ -8597,7 +8597,7 @@
         <v>1417</v>
       </c>
       <c r="I97">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="J97">
         <v>20</v>
@@ -8644,7 +8644,7 @@
         <v>1417</v>
       </c>
       <c r="I98">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="K98" t="s">
         <v>1424</v>
@@ -8921,7 +8921,7 @@
         <v>1417</v>
       </c>
       <c r="I106">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="J106">
         <v>49</v>
@@ -8965,7 +8965,7 @@
         <v>1417</v>
       </c>
       <c r="I107">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="J107">
         <v>36</v>
@@ -9009,7 +9009,7 @@
         <v>1417</v>
       </c>
       <c r="I108">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="K108" t="s">
         <v>1421</v>
@@ -9047,7 +9047,7 @@
         <v>1417</v>
       </c>
       <c r="I109">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="K109" t="s">
         <v>1421</v>
@@ -9230,7 +9230,7 @@
         <v>1417</v>
       </c>
       <c r="I115">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="K115" t="s">
         <v>1421</v>
@@ -9268,7 +9268,7 @@
         <v>1417</v>
       </c>
       <c r="I116">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="K116" t="s">
         <v>1421</v>
@@ -9306,7 +9306,7 @@
         <v>1417</v>
       </c>
       <c r="I117">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="K117" t="s">
         <v>1421</v>
@@ -9344,7 +9344,7 @@
         <v>1417</v>
       </c>
       <c r="I118">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="K118" t="s">
         <v>1421</v>
@@ -9382,7 +9382,7 @@
         <v>1417</v>
       </c>
       <c r="I119">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="K119" t="s">
         <v>1421</v>
@@ -9420,7 +9420,7 @@
         <v>1417</v>
       </c>
       <c r="I120">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="K120" t="s">
         <v>1421</v>
@@ -9458,7 +9458,7 @@
         <v>1417</v>
       </c>
       <c r="I121">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="J121">
         <v>251</v>
@@ -9505,7 +9505,7 @@
         <v>1417</v>
       </c>
       <c r="I122">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="K122" t="s">
         <v>1421</v>
@@ -9572,7 +9572,7 @@
         <v>1417</v>
       </c>
       <c r="I124">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="K124" t="s">
         <v>1421</v>
@@ -9610,7 +9610,7 @@
         <v>1417</v>
       </c>
       <c r="I125">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="K125" t="s">
         <v>1427</v>
@@ -9706,7 +9706,7 @@
         <v>1417</v>
       </c>
       <c r="I128">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="K128" t="s">
         <v>1421</v>
@@ -9744,7 +9744,7 @@
         <v>1417</v>
       </c>
       <c r="I129">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="K129" t="s">
         <v>1420</v>
@@ -9782,7 +9782,7 @@
         <v>1417</v>
       </c>
       <c r="I130">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="J130">
         <v>47</v>
@@ -9858,7 +9858,7 @@
         <v>1417</v>
       </c>
       <c r="I132">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="J132">
         <v>145</v>
@@ -9934,7 +9934,7 @@
         <v>1417</v>
       </c>
       <c r="I134">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="K134" t="s">
         <v>1420</v>
@@ -10059,7 +10059,7 @@
         <v>1417</v>
       </c>
       <c r="I138">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="K138" t="s">
         <v>1421</v>
@@ -10443,7 +10443,7 @@
         <v>1417</v>
       </c>
       <c r="I150">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="J150">
         <v>201</v>
@@ -10630,7 +10630,7 @@
         <v>1417</v>
       </c>
       <c r="I155">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="K155" t="s">
         <v>1427</v>
@@ -10665,7 +10665,7 @@
         <v>1417</v>
       </c>
       <c r="I156">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="K156" t="s">
         <v>1421</v>
@@ -10703,7 +10703,7 @@
         <v>1417</v>
       </c>
       <c r="I157">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="J157">
         <v>371</v>
@@ -10747,7 +10747,7 @@
         <v>1417</v>
       </c>
       <c r="I158">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="J158">
         <v>52</v>
@@ -10791,7 +10791,7 @@
         <v>1417</v>
       </c>
       <c r="I159">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="K159" t="s">
         <v>1421</v>
@@ -10829,7 +10829,7 @@
         <v>1417</v>
       </c>
       <c r="I160">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="K160" t="s">
         <v>1421</v>
@@ -10867,7 +10867,7 @@
         <v>1417</v>
       </c>
       <c r="I161">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="J161">
         <v>55</v>
@@ -11002,7 +11002,7 @@
         <v>1417</v>
       </c>
       <c r="I164">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="O164" t="s">
         <v>1533</v>
@@ -11177,7 +11177,7 @@
         <v>1417</v>
       </c>
       <c r="I169">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="K169" t="s">
         <v>1394</v>
@@ -11387,7 +11387,7 @@
         <v>1417</v>
       </c>
       <c r="I175">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="J175">
         <v>205</v>
@@ -11434,7 +11434,7 @@
         <v>1417</v>
       </c>
       <c r="I176">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="K176" t="s">
         <v>1421</v>
@@ -11472,7 +11472,7 @@
         <v>1417</v>
       </c>
       <c r="I177">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="J177">
         <v>44</v>
@@ -11519,7 +11519,7 @@
         <v>1417</v>
       </c>
       <c r="I178">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="K178" t="s">
         <v>1420</v>
@@ -11586,7 +11586,7 @@
         <v>1417</v>
       </c>
       <c r="I180">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="K180" t="s">
         <v>1420</v>
@@ -11682,7 +11682,7 @@
         <v>1417</v>
       </c>
       <c r="I183">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="K183" t="s">
         <v>1421</v>
@@ -11720,7 +11720,7 @@
         <v>1417</v>
       </c>
       <c r="I184">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="K184" t="s">
         <v>1427</v>
@@ -11755,7 +11755,7 @@
         <v>1417</v>
       </c>
       <c r="I185">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="K185" t="s">
         <v>1421</v>
@@ -11793,7 +11793,7 @@
         <v>1417</v>
       </c>
       <c r="I186">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="K186" t="s">
         <v>1421</v>
@@ -11831,7 +11831,7 @@
         <v>1417</v>
       </c>
       <c r="I187">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="J187">
         <v>75</v>
@@ -11878,7 +11878,7 @@
         <v>1417</v>
       </c>
       <c r="I188">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="J188">
         <v>40</v>
@@ -11925,7 +11925,7 @@
         <v>1417</v>
       </c>
       <c r="I189">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="J189">
         <v>155</v>
@@ -11969,7 +11969,7 @@
         <v>1417</v>
       </c>
       <c r="I190">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="J190">
         <v>107</v>
@@ -12013,7 +12013,7 @@
         <v>1417</v>
       </c>
       <c r="I191">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="J191">
         <v>5</v>
@@ -12057,7 +12057,7 @@
         <v>1417</v>
       </c>
       <c r="I192">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="K192" t="s">
         <v>1421</v>
@@ -12095,7 +12095,7 @@
         <v>1417</v>
       </c>
       <c r="I193">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="K193" t="s">
         <v>1426</v>
@@ -12290,7 +12290,7 @@
         <v>1417</v>
       </c>
       <c r="I199">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="J199">
         <v>70</v>
@@ -12375,7 +12375,7 @@
         <v>1417</v>
       </c>
       <c r="I201">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="K201" t="s">
         <v>1421</v>
@@ -12413,7 +12413,7 @@
         <v>1417</v>
       </c>
       <c r="I202">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="K202" t="s">
         <v>1421</v>
@@ -12492,7 +12492,7 @@
         <v>1417</v>
       </c>
       <c r="I204">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="K204" t="s">
         <v>1420</v>
@@ -12530,7 +12530,7 @@
         <v>1417</v>
       </c>
       <c r="I205">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="K205" t="s">
         <v>1420</v>
@@ -12597,7 +12597,7 @@
         <v>1417</v>
       </c>
       <c r="I207">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J207">
         <v>167</v>
@@ -12641,7 +12641,7 @@
         <v>1417</v>
       </c>
       <c r="I208">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J208">
         <v>45</v>
@@ -12685,7 +12685,7 @@
         <v>1417</v>
       </c>
       <c r="I209">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="J209">
         <v>191</v>
@@ -12729,7 +12729,7 @@
         <v>1417</v>
       </c>
       <c r="I210">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="K210" t="s">
         <v>1424</v>
@@ -12825,7 +12825,7 @@
         <v>1417</v>
       </c>
       <c r="I213">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="K213" t="s">
         <v>1421</v>
@@ -12863,7 +12863,7 @@
         <v>1417</v>
       </c>
       <c r="I214">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="J214">
         <v>14</v>
@@ -12910,7 +12910,7 @@
         <v>1417</v>
       </c>
       <c r="I215">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="K215" t="s">
         <v>1421</v>
@@ -12977,7 +12977,7 @@
         <v>1417</v>
       </c>
       <c r="I217">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="J217">
         <v>42</v>
@@ -13021,7 +13021,7 @@
         <v>1417</v>
       </c>
       <c r="I218">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="J218">
         <v>166</v>
@@ -13109,7 +13109,7 @@
         <v>1417</v>
       </c>
       <c r="I220">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="J220">
         <v>154</v>
@@ -13495,7 +13495,7 @@
         <v>1417</v>
       </c>
       <c r="I230">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="J230">
         <v>197</v>
@@ -13539,7 +13539,7 @@
         <v>1417</v>
       </c>
       <c r="I231">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="J231">
         <v>35</v>
@@ -13641,7 +13641,7 @@
         <v>1417</v>
       </c>
       <c r="I234">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="J234">
         <v>35</v>
@@ -13688,7 +13688,7 @@
         <v>1417</v>
       </c>
       <c r="I235">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="J235">
         <v>35</v>
@@ -13735,7 +13735,7 @@
         <v>1417</v>
       </c>
       <c r="I236">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="J236">
         <v>86</v>
@@ -13852,7 +13852,7 @@
         <v>1417</v>
       </c>
       <c r="I239">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="K239" t="s">
         <v>1394</v>
@@ -13951,7 +13951,7 @@
         <v>1417</v>
       </c>
       <c r="I242">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="K242" t="s">
         <v>1420</v>
@@ -14018,7 +14018,7 @@
         <v>1417</v>
       </c>
       <c r="I244">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="J244">
         <v>15</v>
@@ -14059,7 +14059,7 @@
         <v>1417</v>
       </c>
       <c r="I245">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="J245">
         <v>15</v>
@@ -14202,7 +14202,7 @@
         <v>1417</v>
       </c>
       <c r="I249">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="K249" t="s">
         <v>1421</v>
@@ -14336,7 +14336,7 @@
         <v>1417</v>
       </c>
       <c r="I253">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="J253">
         <v>162</v>
@@ -14380,7 +14380,7 @@
         <v>1417</v>
       </c>
       <c r="I254">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="K254" t="s">
         <v>1424</v>
@@ -14459,7 +14459,7 @@
         <v>1417</v>
       </c>
       <c r="I256">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="J256">
         <v>23</v>
@@ -14643,7 +14643,7 @@
         <v>1417</v>
       </c>
       <c r="I261">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="J261">
         <v>162</v>
@@ -14801,7 +14801,7 @@
         <v>1417</v>
       </c>
       <c r="I265">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="J265">
         <v>162</v>
@@ -14886,7 +14886,7 @@
         <v>1417</v>
       </c>
       <c r="I267">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="K267" t="s">
         <v>1424</v>
@@ -14924,7 +14924,7 @@
         <v>1417</v>
       </c>
       <c r="I268">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="K268" t="s">
         <v>1421</v>
@@ -14959,7 +14959,7 @@
         <v>1417</v>
       </c>
       <c r="I269">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="K269" t="s">
         <v>1421</v>
@@ -14997,7 +14997,7 @@
         <v>1417</v>
       </c>
       <c r="I270">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="K270" t="s">
         <v>1424</v>
@@ -15035,7 +15035,7 @@
         <v>1417</v>
       </c>
       <c r="I271">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="K271" t="s">
         <v>1424</v>
@@ -15213,7 +15213,7 @@
         <v>1417</v>
       </c>
       <c r="I276">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="K276" t="s">
         <v>1425</v>
@@ -15251,7 +15251,7 @@
         <v>1417</v>
       </c>
       <c r="I277">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="K277" t="s">
         <v>1421</v>
@@ -15289,7 +15289,7 @@
         <v>1417</v>
       </c>
       <c r="I278">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="J278">
         <v>148</v>
@@ -15333,7 +15333,7 @@
         <v>1417</v>
       </c>
       <c r="I279">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="K279" t="s">
         <v>1423</v>
@@ -15374,7 +15374,7 @@
         <v>1417</v>
       </c>
       <c r="I280">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="K280" t="s">
         <v>1421</v>
@@ -15412,7 +15412,7 @@
         <v>1417</v>
       </c>
       <c r="I281">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="K281" t="s">
         <v>1421</v>
@@ -15453,7 +15453,7 @@
         <v>1417</v>
       </c>
       <c r="I282">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="K282" t="s">
         <v>1421</v>
@@ -15747,7 +15747,7 @@
         <v>1417</v>
       </c>
       <c r="I291">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="J291">
         <v>20</v>
@@ -15791,7 +15791,7 @@
         <v>1417</v>
       </c>
       <c r="I292">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="K292" t="s">
         <v>1424</v>
@@ -15829,7 +15829,7 @@
         <v>1417</v>
       </c>
       <c r="I293">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K293" t="s">
         <v>1425</v>
@@ -15867,7 +15867,7 @@
         <v>1417</v>
       </c>
       <c r="I294">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K294" t="s">
         <v>1430</v>
@@ -16004,7 +16004,7 @@
         <v>1417</v>
       </c>
       <c r="I298">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J298">
         <v>58</v>
@@ -16168,7 +16168,7 @@
         <v>1417</v>
       </c>
       <c r="I302">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K302" t="s">
         <v>1424</v>
@@ -16206,7 +16206,7 @@
         <v>1417</v>
       </c>
       <c r="I303">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K303" t="s">
         <v>1421</v>
@@ -16244,7 +16244,7 @@
         <v>1417</v>
       </c>
       <c r="I304">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K304" t="s">
         <v>1424</v>
@@ -16282,7 +16282,7 @@
         <v>1417</v>
       </c>
       <c r="I305">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J305">
         <v>35</v>
@@ -16326,7 +16326,7 @@
         <v>1417</v>
       </c>
       <c r="I306">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J306">
         <v>31</v>
@@ -16414,7 +16414,7 @@
         <v>1417</v>
       </c>
       <c r="I308">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K308" t="s">
         <v>1420</v>
@@ -16531,7 +16531,7 @@
         <v>1417</v>
       </c>
       <c r="I311">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K311" t="s">
         <v>1420</v>
@@ -16861,7 +16861,7 @@
         <v>1417</v>
       </c>
       <c r="I320">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K320" t="s">
         <v>1425</v>
@@ -16899,7 +16899,7 @@
         <v>1417</v>
       </c>
       <c r="I321">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K321" t="s">
         <v>1421</v>
@@ -16937,7 +16937,7 @@
         <v>1417</v>
       </c>
       <c r="I322">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J322">
         <v>57</v>
@@ -17051,7 +17051,7 @@
         <v>1417</v>
       </c>
       <c r="I325">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J325">
         <v>57</v>
@@ -17133,7 +17133,7 @@
         <v>1417</v>
       </c>
       <c r="I327">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J327">
         <v>57</v>
@@ -17177,7 +17177,7 @@
         <v>1417</v>
       </c>
       <c r="I328">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J328">
         <v>57</v>
@@ -17221,7 +17221,7 @@
         <v>1417</v>
       </c>
       <c r="I329">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J329">
         <v>57</v>
@@ -17265,7 +17265,7 @@
         <v>1417</v>
       </c>
       <c r="I330">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J330">
         <v>57</v>
@@ -17309,7 +17309,7 @@
         <v>1417</v>
       </c>
       <c r="I331">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K331" t="s">
         <v>1420</v>
@@ -17347,7 +17347,7 @@
         <v>1417</v>
       </c>
       <c r="I332">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K332" t="s">
         <v>1421</v>
@@ -17385,7 +17385,7 @@
         <v>1417</v>
       </c>
       <c r="I333">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J333">
         <v>100</v>
@@ -17429,7 +17429,7 @@
         <v>1417</v>
       </c>
       <c r="I334">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K334" t="s">
         <v>1421</v>
@@ -17654,7 +17654,7 @@
         <v>1417</v>
       </c>
       <c r="I340">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J340">
         <v>98</v>
@@ -17695,7 +17695,7 @@
         <v>1417</v>
       </c>
       <c r="I341">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J341">
         <v>90</v>
@@ -17736,7 +17736,7 @@
         <v>1417</v>
       </c>
       <c r="I342">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="K342" t="s">
         <v>1420</v>
@@ -17850,7 +17850,7 @@
         <v>1417</v>
       </c>
       <c r="I345">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="K345" t="s">
         <v>1420</v>
@@ -17970,7 +17970,7 @@
         <v>1417</v>
       </c>
       <c r="I348">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J348">
         <v>14</v>
@@ -18014,7 +18014,7 @@
         <v>1417</v>
       </c>
       <c r="I349">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="K349" t="s">
         <v>1425</v>
@@ -18052,7 +18052,7 @@
         <v>1417</v>
       </c>
       <c r="I350">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J350">
         <v>46</v>
@@ -18090,7 +18090,7 @@
         <v>1417</v>
       </c>
       <c r="I351">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J351">
         <v>82</v>
@@ -18134,7 +18134,7 @@
         <v>1417</v>
       </c>
       <c r="I352">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J352">
         <v>78</v>
@@ -18178,7 +18178,7 @@
         <v>1417</v>
       </c>
       <c r="I353">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J353">
         <v>83</v>
@@ -18222,7 +18222,7 @@
         <v>1417</v>
       </c>
       <c r="I354">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="K354" t="s">
         <v>1424</v>
@@ -18260,7 +18260,7 @@
         <v>1417</v>
       </c>
       <c r="I355">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J355">
         <v>8</v>
@@ -18342,7 +18342,7 @@
         <v>1417</v>
       </c>
       <c r="I357">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J357">
         <v>85</v>
@@ -18465,7 +18465,7 @@
         <v>1417</v>
       </c>
       <c r="I360">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J360">
         <v>83</v>
@@ -18512,7 +18512,7 @@
         <v>1417</v>
       </c>
       <c r="I361">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J361">
         <v>83</v>
@@ -18556,7 +18556,7 @@
         <v>1417</v>
       </c>
       <c r="I362">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="K362" t="s">
         <v>1424</v>
@@ -18594,7 +18594,7 @@
         <v>1417</v>
       </c>
       <c r="I363">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="K363" t="s">
         <v>1424</v>
@@ -18632,7 +18632,7 @@
         <v>1417</v>
       </c>
       <c r="I364">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J364">
         <v>83</v>
@@ -18676,7 +18676,7 @@
         <v>1417</v>
       </c>
       <c r="I365">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J365">
         <v>15</v>
@@ -18799,7 +18799,7 @@
         <v>1417</v>
       </c>
       <c r="I368">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J368">
         <v>77</v>
@@ -18843,7 +18843,7 @@
         <v>1417</v>
       </c>
       <c r="I369">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="K369" t="s">
         <v>1424</v>
@@ -18881,7 +18881,7 @@
         <v>1417</v>
       </c>
       <c r="I370">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="K370" t="s">
         <v>1424</v>
@@ -18919,7 +18919,7 @@
         <v>1417</v>
       </c>
       <c r="I371">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J371">
         <v>16</v>
@@ -19007,7 +19007,7 @@
         <v>1417</v>
       </c>
       <c r="I373">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="K373" t="s">
         <v>1420</v>
@@ -19045,7 +19045,7 @@
         <v>1417</v>
       </c>
       <c r="I374">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="K374" t="s">
         <v>1420</v>
@@ -19083,7 +19083,7 @@
         <v>1417</v>
       </c>
       <c r="I375">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="J375">
         <v>94</v>
@@ -19124,7 +19124,7 @@
         <v>1417</v>
       </c>
       <c r="I376">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="K376" t="s">
         <v>1424</v>
@@ -19203,7 +19203,7 @@
         <v>1417</v>
       </c>
       <c r="I378">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="K378" t="s">
         <v>1424</v>
@@ -19241,7 +19241,7 @@
         <v>1417</v>
       </c>
       <c r="I379">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="J379">
         <v>20</v>
@@ -19285,7 +19285,7 @@
         <v>1417</v>
       </c>
       <c r="I380">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="J380">
         <v>94</v>
@@ -19329,7 +19329,7 @@
         <v>1417</v>
       </c>
       <c r="I381">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="K381" t="s">
         <v>1424</v>
@@ -19367,7 +19367,7 @@
         <v>1417</v>
       </c>
       <c r="I382">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="K382" t="s">
         <v>1424</v>
@@ -19405,7 +19405,7 @@
         <v>1417</v>
       </c>
       <c r="I383">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="J383">
         <v>71</v>
@@ -19449,7 +19449,7 @@
         <v>1417</v>
       </c>
       <c r="I384">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="K384" t="s">
         <v>1421</v>
@@ -19531,7 +19531,7 @@
         <v>1417</v>
       </c>
       <c r="I386">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="K386" t="s">
         <v>1424</v>
@@ -19569,7 +19569,7 @@
         <v>1417</v>
       </c>
       <c r="I387">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="K387" t="s">
         <v>1424</v>
@@ -19607,7 +19607,7 @@
         <v>1417</v>
       </c>
       <c r="I388">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="J388">
         <v>-85</v>
@@ -19651,7 +19651,7 @@
         <v>1417</v>
       </c>
       <c r="I389">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="K389" t="s">
         <v>1425</v>
@@ -20102,7 +20102,7 @@
         <v>1417</v>
       </c>
       <c r="I400">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="K400" t="s">
         <v>1424</v>
@@ -20178,7 +20178,7 @@
         <v>1417</v>
       </c>
       <c r="I402">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="K402" t="s">
         <v>1424</v>
@@ -20216,7 +20216,7 @@
         <v>1417</v>
       </c>
       <c r="I403">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="J403">
         <v>83</v>
@@ -20260,7 +20260,7 @@
         <v>1417</v>
       </c>
       <c r="I404">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="K404" t="s">
         <v>1424</v>
@@ -20330,7 +20330,7 @@
         <v>1417</v>
       </c>
       <c r="I406">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="Q406" t="b">
         <v>1</v>
@@ -20362,7 +20362,7 @@
         <v>1417</v>
       </c>
       <c r="I407">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="Q407" t="b">
         <v>1</v>
@@ -20394,7 +20394,7 @@
         <v>1417</v>
       </c>
       <c r="I408">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="Q408" t="b">
         <v>1</v>
@@ -20426,7 +20426,7 @@
         <v>1417</v>
       </c>
       <c r="I409">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="Q409" t="b">
         <v>1</v>
@@ -20458,7 +20458,7 @@
         <v>1417</v>
       </c>
       <c r="I410">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="Q410" t="b">
         <v>1</v>
@@ -20490,7 +20490,7 @@
         <v>1417</v>
       </c>
       <c r="I411">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="Q411" t="b">
         <v>1</v>
@@ -20522,7 +20522,7 @@
         <v>1417</v>
       </c>
       <c r="I412">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="Q412" t="b">
         <v>1</v>
@@ -20554,7 +20554,7 @@
         <v>1417</v>
       </c>
       <c r="I413">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="Q413" t="b">
         <v>1</v>
@@ -20644,7 +20644,7 @@
         <v>1417</v>
       </c>
       <c r="I416">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="Q416" t="b">
         <v>1</v>
@@ -20734,7 +20734,7 @@
         <v>1417</v>
       </c>
       <c r="I419">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="Q419" t="b">
         <v>1</v>
@@ -20766,7 +20766,7 @@
         <v>1417</v>
       </c>
       <c r="I420">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="Q420" t="b">
         <v>1</v>
@@ -20798,7 +20798,7 @@
         <v>1417</v>
       </c>
       <c r="I421">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="Q421" t="b">
         <v>1</v>
@@ -20830,7 +20830,7 @@
         <v>1417</v>
       </c>
       <c r="I422">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="Q422" t="b">
         <v>1</v>
@@ -20862,7 +20862,7 @@
         <v>1417</v>
       </c>
       <c r="I423">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="Q423" t="b">
         <v>1</v>
@@ -20894,7 +20894,7 @@
         <v>1417</v>
       </c>
       <c r="I424">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="Q424" t="b">
         <v>1</v>
@@ -20926,7 +20926,7 @@
         <v>1417</v>
       </c>
       <c r="I425">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="Q425" t="b">
         <v>1</v>
@@ -20958,7 +20958,7 @@
         <v>1417</v>
       </c>
       <c r="I426">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="Q426" t="b">
         <v>1</v>
@@ -20990,7 +20990,7 @@
         <v>1417</v>
       </c>
       <c r="I427">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="Q427" t="b">
         <v>1</v>
@@ -21080,7 +21080,7 @@
         <v>1417</v>
       </c>
       <c r="I430">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="Q430" t="b">
         <v>1</v>
@@ -21112,7 +21112,7 @@
         <v>1417</v>
       </c>
       <c r="I431">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="Q431" t="b">
         <v>1</v>
@@ -21144,7 +21144,7 @@
         <v>1417</v>
       </c>
       <c r="I432">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="Q432" t="b">
         <v>1</v>
@@ -21176,7 +21176,7 @@
         <v>1417</v>
       </c>
       <c r="I433">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="Q433" t="b">
         <v>1</v>
@@ -21208,7 +21208,7 @@
         <v>1417</v>
       </c>
       <c r="I434">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="Q434" t="b">
         <v>1</v>
@@ -21240,7 +21240,7 @@
         <v>1417</v>
       </c>
       <c r="I435">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="Q435" t="b">
         <v>1</v>
@@ -21272,7 +21272,7 @@
         <v>1417</v>
       </c>
       <c r="I436">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="Q436" t="b">
         <v>1</v>
@@ -21304,7 +21304,7 @@
         <v>1419</v>
       </c>
       <c r="I437">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="Q437" t="b">
         <v>1</v>
@@ -21336,7 +21336,7 @@
         <v>1419</v>
       </c>
       <c r="I438">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="Q438" t="b">
         <v>1</v>
@@ -21368,7 +21368,7 @@
         <v>1417</v>
       </c>
       <c r="I439">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="Q439" t="b">
         <v>1</v>
@@ -21400,7 +21400,7 @@
         <v>1417</v>
       </c>
       <c r="I440">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="Q440" t="b">
         <v>1</v>
@@ -21432,7 +21432,7 @@
         <v>1417</v>
       </c>
       <c r="I441">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="Q441" t="b">
         <v>1</v>
@@ -21493,7 +21493,7 @@
         <v>1417</v>
       </c>
       <c r="I443">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="Q443" t="b">
         <v>1</v>
@@ -21583,7 +21583,7 @@
         <v>1417</v>
       </c>
       <c r="I446">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="Q446" t="b">
         <v>1</v>
@@ -21615,7 +21615,7 @@
         <v>1417</v>
       </c>
       <c r="I447">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="Q447" t="b">
         <v>1</v>
@@ -21647,7 +21647,7 @@
         <v>1417</v>
       </c>
       <c r="I448">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="Q448" t="b">
         <v>1</v>
@@ -21679,7 +21679,7 @@
         <v>1417</v>
       </c>
       <c r="I449">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="Q449" t="b">
         <v>1</v>
@@ -21711,7 +21711,7 @@
         <v>1417</v>
       </c>
       <c r="I450">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="Q450" t="b">
         <v>1</v>
@@ -21743,7 +21743,7 @@
         <v>1417</v>
       </c>
       <c r="I451">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="Q451" t="b">
         <v>1</v>
@@ -21804,7 +21804,7 @@
         <v>1417</v>
       </c>
       <c r="I453">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="Q453" t="b">
         <v>1</v>
@@ -21836,7 +21836,7 @@
         <v>1417</v>
       </c>
       <c r="I454">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="Q454" t="b">
         <v>1</v>
@@ -21868,7 +21868,7 @@
         <v>1417</v>
       </c>
       <c r="I455">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="Q455" t="b">
         <v>1</v>
@@ -21929,7 +21929,7 @@
         <v>1417</v>
       </c>
       <c r="I457">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="Q457" t="b">
         <v>1</v>
@@ -21961,7 +21961,7 @@
         <v>1417</v>
       </c>
       <c r="I458">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Q458" t="b">
         <v>1</v>
@@ -21993,7 +21993,7 @@
         <v>1417</v>
       </c>
       <c r="I459">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="Q459" t="b">
         <v>1</v>
@@ -22025,7 +22025,7 @@
         <v>1417</v>
       </c>
       <c r="I460">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="Q460" t="b">
         <v>1</v>
@@ -22057,7 +22057,7 @@
         <v>1417</v>
       </c>
       <c r="I461">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="Q461" t="b">
         <v>1</v>
@@ -22089,7 +22089,7 @@
         <v>1417</v>
       </c>
       <c r="I462">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="Q462" t="b">
         <v>1</v>
@@ -22121,7 +22121,7 @@
         <v>1417</v>
       </c>
       <c r="I463">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="Q463" t="b">
         <v>1</v>
@@ -22153,7 +22153,7 @@
         <v>1417</v>
       </c>
       <c r="I464">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="Q464" t="b">
         <v>1</v>
@@ -22185,7 +22185,7 @@
         <v>1417</v>
       </c>
       <c r="I465">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="Q465" t="b">
         <v>1</v>
@@ -22217,7 +22217,7 @@
         <v>1417</v>
       </c>
       <c r="I466">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="Q466" t="b">
         <v>1</v>
@@ -22249,7 +22249,7 @@
         <v>1417</v>
       </c>
       <c r="I467">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="Q467" t="b">
         <v>1</v>
@@ -22281,7 +22281,7 @@
         <v>1417</v>
       </c>
       <c r="I468">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="Q468" t="b">
         <v>1</v>
@@ -22313,7 +22313,7 @@
         <v>1417</v>
       </c>
       <c r="I469">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="Q469" t="b">
         <v>1</v>
@@ -22374,7 +22374,7 @@
         <v>1417</v>
       </c>
       <c r="I471">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="Q471" t="b">
         <v>1</v>
@@ -22406,7 +22406,7 @@
         <v>1417</v>
       </c>
       <c r="I472">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="Q472" t="b">
         <v>1</v>
@@ -22438,7 +22438,7 @@
         <v>1417</v>
       </c>
       <c r="I473">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="Q473" t="b">
         <v>1</v>
@@ -22470,7 +22470,7 @@
         <v>1417</v>
       </c>
       <c r="I474">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Q474" t="b">
         <v>1</v>
@@ -22502,7 +22502,7 @@
         <v>1417</v>
       </c>
       <c r="I475">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Q475" t="b">
         <v>1</v>
@@ -22534,7 +22534,7 @@
         <v>1417</v>
       </c>
       <c r="I476">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Q476" t="b">
         <v>1</v>
@@ -22566,7 +22566,7 @@
         <v>1417</v>
       </c>
       <c r="I477">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Q477" t="b">
         <v>1</v>
@@ -22598,7 +22598,7 @@
         <v>1417</v>
       </c>
       <c r="I478">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Q478" t="b">
         <v>1</v>
@@ -22630,7 +22630,7 @@
         <v>1417</v>
       </c>
       <c r="I479">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Q479" t="b">
         <v>1</v>
@@ -22662,7 +22662,7 @@
         <v>1417</v>
       </c>
       <c r="I480">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Q480" t="b">
         <v>1</v>
@@ -22694,7 +22694,7 @@
         <v>1417</v>
       </c>
       <c r="I481">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Q481" t="b">
         <v>1</v>
@@ -22726,7 +22726,7 @@
         <v>1417</v>
       </c>
       <c r="I482">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Q482" t="b">
         <v>1</v>
@@ -22758,7 +22758,7 @@
         <v>1417</v>
       </c>
       <c r="I483">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Q483" t="b">
         <v>1</v>
@@ -22790,7 +22790,7 @@
         <v>1417</v>
       </c>
       <c r="I484">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Q484" t="b">
         <v>1</v>
@@ -22822,7 +22822,7 @@
         <v>1417</v>
       </c>
       <c r="I485">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Q485" t="b">
         <v>1</v>
@@ -22854,7 +22854,7 @@
         <v>1417</v>
       </c>
       <c r="I486">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Q486" t="b">
         <v>1</v>
@@ -22886,7 +22886,7 @@
         <v>1417</v>
       </c>
       <c r="I487">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Q487" t="b">
         <v>1</v>
@@ -22918,7 +22918,7 @@
         <v>1417</v>
       </c>
       <c r="I488">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Q488" t="b">
         <v>1</v>
@@ -22950,7 +22950,7 @@
         <v>1417</v>
       </c>
       <c r="I489">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Q489" t="b">
         <v>1</v>
@@ -22982,7 +22982,7 @@
         <v>1417</v>
       </c>
       <c r="I490">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Q490" t="b">
         <v>1</v>
@@ -23014,7 +23014,7 @@
         <v>1417</v>
       </c>
       <c r="I491">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Q491" t="b">
         <v>1</v>
@@ -23046,7 +23046,7 @@
         <v>1419</v>
       </c>
       <c r="I492">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Q492" t="b">
         <v>1</v>
@@ -23078,7 +23078,7 @@
         <v>1419</v>
       </c>
       <c r="I493">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Q493" t="b">
         <v>1</v>
@@ -23110,7 +23110,7 @@
         <v>1419</v>
       </c>
       <c r="I494">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Q494" t="b">
         <v>1</v>
@@ -23142,7 +23142,7 @@
         <v>1419</v>
       </c>
       <c r="I495">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Q495" t="b">
         <v>1</v>
@@ -23174,7 +23174,7 @@
         <v>1419</v>
       </c>
       <c r="I496">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Q496" t="b">
         <v>1</v>
@@ -23206,7 +23206,7 @@
         <v>1417</v>
       </c>
       <c r="I497">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Q497" t="b">
         <v>1</v>
@@ -23238,7 +23238,7 @@
         <v>1417</v>
       </c>
       <c r="I498">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Q498" t="b">
         <v>1</v>
@@ -23270,7 +23270,7 @@
         <v>1419</v>
       </c>
       <c r="I499">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Q499" t="b">
         <v>1</v>
@@ -23302,7 +23302,7 @@
         <v>1417</v>
       </c>
       <c r="I500">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Q500" t="b">
         <v>1</v>
@@ -23334,7 +23334,7 @@
         <v>1417</v>
       </c>
       <c r="I501">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Q501" t="b">
         <v>1</v>
@@ -23366,7 +23366,7 @@
         <v>1417</v>
       </c>
       <c r="I502">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Q502" t="b">
         <v>1</v>
@@ -23398,7 +23398,7 @@
         <v>1417</v>
       </c>
       <c r="I503">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Q503" t="b">
         <v>1</v>
@@ -23430,7 +23430,7 @@
         <v>1417</v>
       </c>
       <c r="I504">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="Q504" t="b">
         <v>1</v>
@@ -23462,7 +23462,7 @@
         <v>1417</v>
       </c>
       <c r="I505">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="Q505" t="b">
         <v>1</v>
@@ -23494,7 +23494,7 @@
         <v>1417</v>
       </c>
       <c r="I506">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="Q506" t="b">
         <v>1</v>
@@ -23526,7 +23526,7 @@
         <v>1417</v>
       </c>
       <c r="I507">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="Q507" t="b">
         <v>1</v>
@@ -23587,7 +23587,7 @@
         <v>1417</v>
       </c>
       <c r="I509">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="Q509" t="b">
         <v>1</v>
@@ -23619,7 +23619,7 @@
         <v>1417</v>
       </c>
       <c r="I510">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="Q510" t="b">
         <v>1</v>
@@ -23651,7 +23651,7 @@
         <v>1417</v>
       </c>
       <c r="I511">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="Q511" t="b">
         <v>1</v>
@@ -23683,7 +23683,7 @@
         <v>1417</v>
       </c>
       <c r="I512">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="Q512" t="b">
         <v>1</v>
@@ -23715,7 +23715,7 @@
         <v>1417</v>
       </c>
       <c r="I513">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q513" t="b">
         <v>1</v>
@@ -23776,7 +23776,7 @@
         <v>1417</v>
       </c>
       <c r="I515">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q515" t="b">
         <v>1</v>
@@ -23808,7 +23808,7 @@
         <v>1417</v>
       </c>
       <c r="I516">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="Q516" t="b">
         <v>1</v>
@@ -23840,7 +23840,7 @@
         <v>1417</v>
       </c>
       <c r="I517">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="Q517" t="b">
         <v>1</v>
@@ -23872,7 +23872,7 @@
         <v>1417</v>
       </c>
       <c r="I518">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="Q518" t="b">
         <v>1</v>
@@ -23904,7 +23904,7 @@
         <v>1417</v>
       </c>
       <c r="I519">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="Q519" t="b">
         <v>1</v>
@@ -23936,7 +23936,7 @@
         <v>1417</v>
       </c>
       <c r="I520">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="Q520" t="b">
         <v>1</v>
@@ -23968,7 +23968,7 @@
         <v>1417</v>
       </c>
       <c r="I521">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="Q521" t="b">
         <v>1</v>
@@ -24000,7 +24000,7 @@
         <v>1417</v>
       </c>
       <c r="I522">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="Q522" t="b">
         <v>1</v>
@@ -24032,7 +24032,7 @@
         <v>1417</v>
       </c>
       <c r="I523">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="Q523" t="b">
         <v>1</v>
@@ -24064,7 +24064,7 @@
         <v>1417</v>
       </c>
       <c r="I524">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q524" t="b">
         <v>1</v>
@@ -24096,7 +24096,7 @@
         <v>1417</v>
       </c>
       <c r="I525">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q525" t="b">
         <v>1</v>
@@ -24128,7 +24128,7 @@
         <v>1417</v>
       </c>
       <c r="I526">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q526" t="b">
         <v>1</v>
@@ -24160,7 +24160,7 @@
         <v>1417</v>
       </c>
       <c r="I527">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q527" t="b">
         <v>1</v>
@@ -24192,7 +24192,7 @@
         <v>1417</v>
       </c>
       <c r="I528">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="Q528" t="b">
         <v>1</v>
@@ -24224,7 +24224,7 @@
         <v>1417</v>
       </c>
       <c r="I529">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Q529" t="b">
         <v>1</v>
@@ -24256,7 +24256,7 @@
         <v>1417</v>
       </c>
       <c r="I530">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Q530" t="b">
         <v>1</v>
@@ -24288,7 +24288,7 @@
         <v>1417</v>
       </c>
       <c r="I531">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Q531" t="b">
         <v>1</v>
@@ -24320,7 +24320,7 @@
         <v>1417</v>
       </c>
       <c r="I532">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Q532" t="b">
         <v>1</v>
@@ -24352,7 +24352,7 @@
         <v>1417</v>
       </c>
       <c r="I533">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Q533" t="b">
         <v>1</v>
@@ -24384,7 +24384,7 @@
         <v>1417</v>
       </c>
       <c r="I534">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Q534" t="b">
         <v>1</v>
@@ -24416,7 +24416,7 @@
         <v>1417</v>
       </c>
       <c r="I535">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Q535" t="b">
         <v>1</v>
@@ -24448,7 +24448,7 @@
         <v>1417</v>
       </c>
       <c r="I536">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Q536" t="b">
         <v>1</v>
@@ -24480,7 +24480,7 @@
         <v>1417</v>
       </c>
       <c r="I537">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Q537" t="b">
         <v>1</v>
@@ -24512,7 +24512,7 @@
         <v>1417</v>
       </c>
       <c r="I538">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Q538" t="b">
         <v>1</v>
@@ -24544,7 +24544,7 @@
         <v>1417</v>
       </c>
       <c r="I539">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Q539" t="b">
         <v>1</v>
@@ -24576,7 +24576,7 @@
         <v>1417</v>
       </c>
       <c r="I540">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Q540" t="b">
         <v>1</v>
@@ -24608,7 +24608,7 @@
         <v>1417</v>
       </c>
       <c r="I541">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Q541" t="b">
         <v>1</v>
@@ -24640,7 +24640,7 @@
         <v>1417</v>
       </c>
       <c r="I542">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Q542" t="b">
         <v>1</v>
@@ -24672,7 +24672,7 @@
         <v>1417</v>
       </c>
       <c r="I543">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Q543" t="b">
         <v>1</v>
@@ -24704,7 +24704,7 @@
         <v>1417</v>
       </c>
       <c r="I544">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Q544" t="b">
         <v>1</v>
@@ -24736,7 +24736,7 @@
         <v>1417</v>
       </c>
       <c r="I545">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Q545" t="b">
         <v>1</v>
@@ -24768,7 +24768,7 @@
         <v>1417</v>
       </c>
       <c r="I546">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="Q546" t="b">
         <v>1</v>
@@ -24800,7 +24800,7 @@
         <v>1417</v>
       </c>
       <c r="I547">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="Q547" t="b">
         <v>1</v>
@@ -24832,7 +24832,7 @@
         <v>1417</v>
       </c>
       <c r="I548">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="Q548" t="b">
         <v>1</v>
@@ -24864,7 +24864,7 @@
         <v>1417</v>
       </c>
       <c r="I549">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="Q549" t="b">
         <v>1</v>
@@ -24896,7 +24896,7 @@
         <v>1417</v>
       </c>
       <c r="I550">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="Q550" t="b">
         <v>1</v>
@@ -24928,7 +24928,7 @@
         <v>1417</v>
       </c>
       <c r="I551">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="Q551" t="b">
         <v>1</v>
@@ -24960,7 +24960,7 @@
         <v>1417</v>
       </c>
       <c r="I552">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="Q552" t="b">
         <v>1</v>
@@ -24992,7 +24992,7 @@
         <v>1417</v>
       </c>
       <c r="I553">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="Q553" t="b">
         <v>1</v>
@@ -25024,7 +25024,7 @@
         <v>1417</v>
       </c>
       <c r="I554">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="Q554" t="b">
         <v>1</v>
@@ -25056,7 +25056,7 @@
         <v>1417</v>
       </c>
       <c r="I555">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="Q555" t="b">
         <v>1</v>
@@ -25088,7 +25088,7 @@
         <v>1417</v>
       </c>
       <c r="I556">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="Q556" t="b">
         <v>1</v>
@@ -25120,7 +25120,7 @@
         <v>1417</v>
       </c>
       <c r="I557">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="Q557" t="b">
         <v>1</v>
@@ -25152,7 +25152,7 @@
         <v>1417</v>
       </c>
       <c r="I558">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="Q558" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: reparaveis (08/10/2026 14:52)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
@@ -5132,7 +5132,7 @@
         <v>1417</v>
       </c>
       <c r="I2">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="K2" t="s">
         <v>1420</v>
@@ -5170,7 +5170,7 @@
         <v>1417</v>
       </c>
       <c r="I3">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="K3" t="s">
         <v>1421</v>
@@ -5208,7 +5208,7 @@
         <v>1417</v>
       </c>
       <c r="I4">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="K4" t="s">
         <v>1421</v>
@@ -5246,7 +5246,7 @@
         <v>1417</v>
       </c>
       <c r="I5">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="J5">
         <v>279</v>
@@ -5290,7 +5290,7 @@
         <v>1417</v>
       </c>
       <c r="I6">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="J6">
         <v>153</v>
@@ -5334,7 +5334,7 @@
         <v>1417</v>
       </c>
       <c r="I7">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="J7">
         <v>112</v>
@@ -5410,7 +5410,7 @@
         <v>1417</v>
       </c>
       <c r="I9">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="J9">
         <v>362</v>
@@ -5457,7 +5457,7 @@
         <v>1417</v>
       </c>
       <c r="I10">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="J10">
         <v>378</v>
@@ -5504,7 +5504,7 @@
         <v>1417</v>
       </c>
       <c r="I11">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="J11">
         <v>112</v>
@@ -5551,7 +5551,7 @@
         <v>1417</v>
       </c>
       <c r="I12">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="J12">
         <v>124</v>
@@ -5624,7 +5624,7 @@
         <v>1417</v>
       </c>
       <c r="I14">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="J14">
         <v>64</v>
@@ -5703,7 +5703,7 @@
         <v>1417</v>
       </c>
       <c r="I16">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="K16" t="s">
         <v>1420</v>
@@ -5741,7 +5741,7 @@
         <v>1417</v>
       </c>
       <c r="I17">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="J17">
         <v>161</v>
@@ -5785,7 +5785,7 @@
         <v>1417</v>
       </c>
       <c r="I18">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="J18">
         <v>66</v>
@@ -5858,7 +5858,7 @@
         <v>1417</v>
       </c>
       <c r="I20">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="J20">
         <v>399</v>
@@ -5931,7 +5931,7 @@
         <v>1417</v>
       </c>
       <c r="I22">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="K22" t="s">
         <v>1424</v>
@@ -5969,7 +5969,7 @@
         <v>1417</v>
       </c>
       <c r="I23">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="J23">
         <v>229</v>
@@ -6074,7 +6074,7 @@
         <v>1417</v>
       </c>
       <c r="I26">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="J26">
         <v>155</v>
@@ -6121,7 +6121,7 @@
         <v>1417</v>
       </c>
       <c r="I27">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="K27" t="s">
         <v>1424</v>
@@ -6217,7 +6217,7 @@
         <v>1417</v>
       </c>
       <c r="I30">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="J30">
         <v>209</v>
@@ -6290,7 +6290,7 @@
         <v>1417</v>
       </c>
       <c r="I32">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="K32" t="s">
         <v>1420</v>
@@ -6499,7 +6499,7 @@
         <v>1417</v>
       </c>
       <c r="I39">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="K39" t="s">
         <v>1425</v>
@@ -6662,7 +6662,7 @@
         <v>1417</v>
       </c>
       <c r="I44">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="J44">
         <v>87</v>
@@ -6709,7 +6709,7 @@
         <v>1417</v>
       </c>
       <c r="I45">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="J45">
         <v>331</v>
@@ -6756,7 +6756,7 @@
         <v>1417</v>
       </c>
       <c r="I46">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="K46" t="s">
         <v>1424</v>
@@ -6797,7 +6797,7 @@
         <v>1417</v>
       </c>
       <c r="I47">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="J47">
         <v>344</v>
@@ -6844,7 +6844,7 @@
         <v>1417</v>
       </c>
       <c r="I48">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="K48" t="s">
         <v>1424</v>
@@ -6911,7 +6911,7 @@
         <v>1417</v>
       </c>
       <c r="I50">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="K50" t="s">
         <v>1424</v>
@@ -6978,7 +6978,7 @@
         <v>1417</v>
       </c>
       <c r="I52">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="K52" t="s">
         <v>1420</v>
@@ -7016,7 +7016,7 @@
         <v>1417</v>
       </c>
       <c r="I53">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="K53" t="s">
         <v>1421</v>
@@ -7054,7 +7054,7 @@
         <v>1417</v>
       </c>
       <c r="I54">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="K54" t="s">
         <v>1421</v>
@@ -7330,7 +7330,7 @@
         <v>1417</v>
       </c>
       <c r="I63">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="J63">
         <v>293</v>
@@ -7377,7 +7377,7 @@
         <v>1417</v>
       </c>
       <c r="I64">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="J64">
         <v>320</v>
@@ -7607,7 +7607,7 @@
         <v>1417</v>
       </c>
       <c r="I71">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="J71">
         <v>429</v>
@@ -7680,7 +7680,7 @@
         <v>1417</v>
       </c>
       <c r="I73">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="K73" t="s">
         <v>1420</v>
@@ -7788,7 +7788,7 @@
         <v>1417</v>
       </c>
       <c r="I76">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="K76" t="s">
         <v>1427</v>
@@ -7881,7 +7881,7 @@
         <v>1417</v>
       </c>
       <c r="I79">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="K79" t="s">
         <v>1427</v>
@@ -7986,7 +7986,7 @@
         <v>1417</v>
       </c>
       <c r="I82">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="K82" t="s">
         <v>1424</v>
@@ -8053,7 +8053,7 @@
         <v>1417</v>
       </c>
       <c r="I84">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="J84">
         <v>40</v>
@@ -8100,7 +8100,7 @@
         <v>1417</v>
       </c>
       <c r="I85">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="K85" t="s">
         <v>1421</v>
@@ -8138,7 +8138,7 @@
         <v>1417</v>
       </c>
       <c r="I86">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="K86" t="s">
         <v>1421</v>
@@ -8176,7 +8176,7 @@
         <v>1417</v>
       </c>
       <c r="I87">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="J87">
         <v>-16</v>
@@ -8299,7 +8299,7 @@
         <v>1417</v>
       </c>
       <c r="I90">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="K90" t="s">
         <v>1394</v>
@@ -8448,7 +8448,7 @@
         <v>1417</v>
       </c>
       <c r="I94">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="K94" t="s">
         <v>1424</v>
@@ -8527,7 +8527,7 @@
         <v>1417</v>
       </c>
       <c r="I96">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="J96">
         <v>17</v>
@@ -8574,7 +8574,7 @@
         <v>1417</v>
       </c>
       <c r="I97">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="J97">
         <v>20</v>
@@ -8621,7 +8621,7 @@
         <v>1417</v>
       </c>
       <c r="I98">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="K98" t="s">
         <v>1424</v>
@@ -8898,7 +8898,7 @@
         <v>1417</v>
       </c>
       <c r="I106">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="J106">
         <v>49</v>
@@ -8942,7 +8942,7 @@
         <v>1417</v>
       </c>
       <c r="I107">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="J107">
         <v>36</v>
@@ -8986,7 +8986,7 @@
         <v>1417</v>
       </c>
       <c r="I108">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="K108" t="s">
         <v>1421</v>
@@ -9024,7 +9024,7 @@
         <v>1417</v>
       </c>
       <c r="I109">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="K109" t="s">
         <v>1421</v>
@@ -9207,7 +9207,7 @@
         <v>1417</v>
       </c>
       <c r="I115">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="K115" t="s">
         <v>1421</v>
@@ -9245,7 +9245,7 @@
         <v>1417</v>
       </c>
       <c r="I116">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="K116" t="s">
         <v>1421</v>
@@ -9283,7 +9283,7 @@
         <v>1417</v>
       </c>
       <c r="I117">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="K117" t="s">
         <v>1421</v>
@@ -9321,7 +9321,7 @@
         <v>1417</v>
       </c>
       <c r="I118">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="K118" t="s">
         <v>1421</v>
@@ -9359,7 +9359,7 @@
         <v>1417</v>
       </c>
       <c r="I119">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="K119" t="s">
         <v>1421</v>
@@ -9397,7 +9397,7 @@
         <v>1417</v>
       </c>
       <c r="I120">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="K120" t="s">
         <v>1421</v>
@@ -9435,7 +9435,7 @@
         <v>1417</v>
       </c>
       <c r="I121">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="J121">
         <v>251</v>
@@ -9482,7 +9482,7 @@
         <v>1417</v>
       </c>
       <c r="I122">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="K122" t="s">
         <v>1421</v>
@@ -9549,7 +9549,7 @@
         <v>1417</v>
       </c>
       <c r="I124">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="K124" t="s">
         <v>1421</v>
@@ -9587,7 +9587,7 @@
         <v>1417</v>
       </c>
       <c r="I125">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="K125" t="s">
         <v>1427</v>
@@ -9683,7 +9683,7 @@
         <v>1417</v>
       </c>
       <c r="I128">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="K128" t="s">
         <v>1421</v>
@@ -9721,7 +9721,7 @@
         <v>1417</v>
       </c>
       <c r="I129">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="K129" t="s">
         <v>1420</v>
@@ -9759,7 +9759,7 @@
         <v>1417</v>
       </c>
       <c r="I130">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="J130">
         <v>47</v>
@@ -9835,7 +9835,7 @@
         <v>1417</v>
       </c>
       <c r="I132">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="J132">
         <v>145</v>
@@ -9911,7 +9911,7 @@
         <v>1417</v>
       </c>
       <c r="I134">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="K134" t="s">
         <v>1420</v>
@@ -10036,7 +10036,7 @@
         <v>1417</v>
       </c>
       <c r="I138">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="K138" t="s">
         <v>1421</v>
@@ -10420,7 +10420,7 @@
         <v>1417</v>
       </c>
       <c r="I150">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="J150">
         <v>201</v>
@@ -10607,7 +10607,7 @@
         <v>1417</v>
       </c>
       <c r="I155">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="K155" t="s">
         <v>1427</v>
@@ -10642,7 +10642,7 @@
         <v>1417</v>
       </c>
       <c r="I156">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="K156" t="s">
         <v>1421</v>
@@ -10680,7 +10680,7 @@
         <v>1417</v>
       </c>
       <c r="I157">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="J157">
         <v>371</v>
@@ -10724,7 +10724,7 @@
         <v>1417</v>
       </c>
       <c r="I158">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="J158">
         <v>52</v>
@@ -10768,7 +10768,7 @@
         <v>1417</v>
       </c>
       <c r="I159">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="K159" t="s">
         <v>1421</v>
@@ -10806,7 +10806,7 @@
         <v>1417</v>
       </c>
       <c r="I160">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="K160" t="s">
         <v>1421</v>
@@ -10844,7 +10844,7 @@
         <v>1417</v>
       </c>
       <c r="I161">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="J161">
         <v>55</v>
@@ -10979,7 +10979,7 @@
         <v>1417</v>
       </c>
       <c r="I164">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="O164" t="s">
         <v>1533</v>
@@ -11154,7 +11154,7 @@
         <v>1417</v>
       </c>
       <c r="I169">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="K169" t="s">
         <v>1394</v>
@@ -11364,7 +11364,7 @@
         <v>1417</v>
       </c>
       <c r="I175">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J175">
         <v>205</v>
@@ -11411,7 +11411,7 @@
         <v>1417</v>
       </c>
       <c r="I176">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="K176" t="s">
         <v>1421</v>
@@ -11449,7 +11449,7 @@
         <v>1417</v>
       </c>
       <c r="I177">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J177">
         <v>44</v>
@@ -11496,7 +11496,7 @@
         <v>1417</v>
       </c>
       <c r="I178">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="K178" t="s">
         <v>1420</v>
@@ -11563,7 +11563,7 @@
         <v>1417</v>
       </c>
       <c r="I180">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="K180" t="s">
         <v>1420</v>
@@ -11659,7 +11659,7 @@
         <v>1417</v>
       </c>
       <c r="I183">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="K183" t="s">
         <v>1421</v>
@@ -11697,7 +11697,7 @@
         <v>1417</v>
       </c>
       <c r="I184">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="K184" t="s">
         <v>1427</v>
@@ -11732,7 +11732,7 @@
         <v>1417</v>
       </c>
       <c r="I185">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="K185" t="s">
         <v>1421</v>
@@ -11770,7 +11770,7 @@
         <v>1417</v>
       </c>
       <c r="I186">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="K186" t="s">
         <v>1421</v>
@@ -11808,7 +11808,7 @@
         <v>1417</v>
       </c>
       <c r="I187">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="J187">
         <v>75</v>
@@ -11855,7 +11855,7 @@
         <v>1417</v>
       </c>
       <c r="I188">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="J188">
         <v>40</v>
@@ -11902,7 +11902,7 @@
         <v>1417</v>
       </c>
       <c r="I189">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="J189">
         <v>155</v>
@@ -11946,7 +11946,7 @@
         <v>1417</v>
       </c>
       <c r="I190">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="J190">
         <v>107</v>
@@ -11990,7 +11990,7 @@
         <v>1417</v>
       </c>
       <c r="I191">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="J191">
         <v>5</v>
@@ -12034,7 +12034,7 @@
         <v>1417</v>
       </c>
       <c r="I192">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="K192" t="s">
         <v>1421</v>
@@ -12072,7 +12072,7 @@
         <v>1417</v>
       </c>
       <c r="I193">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="K193" t="s">
         <v>1426</v>
@@ -12267,7 +12267,7 @@
         <v>1417</v>
       </c>
       <c r="I199">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="J199">
         <v>70</v>
@@ -12352,7 +12352,7 @@
         <v>1417</v>
       </c>
       <c r="I201">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="K201" t="s">
         <v>1421</v>
@@ -12390,7 +12390,7 @@
         <v>1417</v>
       </c>
       <c r="I202">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="K202" t="s">
         <v>1421</v>
@@ -12469,7 +12469,7 @@
         <v>1417</v>
       </c>
       <c r="I204">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="K204" t="s">
         <v>1420</v>
@@ -12507,7 +12507,7 @@
         <v>1417</v>
       </c>
       <c r="I205">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="K205" t="s">
         <v>1420</v>
@@ -12574,7 +12574,7 @@
         <v>1417</v>
       </c>
       <c r="I207">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="J207">
         <v>167</v>
@@ -12618,7 +12618,7 @@
         <v>1417</v>
       </c>
       <c r="I208">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="J208">
         <v>45</v>
@@ -12662,7 +12662,7 @@
         <v>1417</v>
       </c>
       <c r="I209">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="J209">
         <v>191</v>
@@ -12706,7 +12706,7 @@
         <v>1417</v>
       </c>
       <c r="I210">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="K210" t="s">
         <v>1424</v>
@@ -12802,7 +12802,7 @@
         <v>1417</v>
       </c>
       <c r="I213">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="K213" t="s">
         <v>1421</v>
@@ -12840,7 +12840,7 @@
         <v>1417</v>
       </c>
       <c r="I214">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="J214">
         <v>14</v>
@@ -12887,7 +12887,7 @@
         <v>1417</v>
       </c>
       <c r="I215">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="K215" t="s">
         <v>1421</v>
@@ -12954,7 +12954,7 @@
         <v>1417</v>
       </c>
       <c r="I217">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="J217">
         <v>42</v>
@@ -12998,7 +12998,7 @@
         <v>1417</v>
       </c>
       <c r="I218">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="J218">
         <v>166</v>
@@ -13086,7 +13086,7 @@
         <v>1417</v>
       </c>
       <c r="I220">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="J220">
         <v>154</v>
@@ -13472,7 +13472,7 @@
         <v>1417</v>
       </c>
       <c r="I230">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="J230">
         <v>197</v>
@@ -13516,7 +13516,7 @@
         <v>1417</v>
       </c>
       <c r="I231">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="J231">
         <v>35</v>
@@ -13618,7 +13618,7 @@
         <v>1417</v>
       </c>
       <c r="I234">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="J234">
         <v>35</v>
@@ -13665,7 +13665,7 @@
         <v>1417</v>
       </c>
       <c r="I235">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="J235">
         <v>35</v>
@@ -13712,7 +13712,7 @@
         <v>1417</v>
       </c>
       <c r="I236">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="J236">
         <v>86</v>
@@ -13829,7 +13829,7 @@
         <v>1417</v>
       </c>
       <c r="I239">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="K239" t="s">
         <v>1394</v>
@@ -13928,7 +13928,7 @@
         <v>1417</v>
       </c>
       <c r="I242">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="K242" t="s">
         <v>1420</v>
@@ -13995,7 +13995,7 @@
         <v>1417</v>
       </c>
       <c r="I244">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="J244">
         <v>15</v>
@@ -14036,7 +14036,7 @@
         <v>1417</v>
       </c>
       <c r="I245">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="J245">
         <v>15</v>
@@ -14179,7 +14179,7 @@
         <v>1417</v>
       </c>
       <c r="I249">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="K249" t="s">
         <v>1421</v>
@@ -14313,7 +14313,7 @@
         <v>1417</v>
       </c>
       <c r="I253">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="J253">
         <v>162</v>
@@ -14357,7 +14357,7 @@
         <v>1417</v>
       </c>
       <c r="I254">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="K254" t="s">
         <v>1424</v>
@@ -14436,7 +14436,7 @@
         <v>1417</v>
       </c>
       <c r="I256">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="J256">
         <v>23</v>
@@ -14620,7 +14620,7 @@
         <v>1417</v>
       </c>
       <c r="I261">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="J261">
         <v>162</v>
@@ -14778,7 +14778,7 @@
         <v>1417</v>
       </c>
       <c r="I265">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="J265">
         <v>162</v>
@@ -14863,7 +14863,7 @@
         <v>1417</v>
       </c>
       <c r="I267">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="K267" t="s">
         <v>1424</v>
@@ -14901,7 +14901,7 @@
         <v>1417</v>
       </c>
       <c r="I268">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="K268" t="s">
         <v>1421</v>
@@ -14936,7 +14936,7 @@
         <v>1417</v>
       </c>
       <c r="I269">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="K269" t="s">
         <v>1421</v>
@@ -14974,7 +14974,7 @@
         <v>1417</v>
       </c>
       <c r="I270">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="K270" t="s">
         <v>1424</v>
@@ -15012,7 +15012,7 @@
         <v>1417</v>
       </c>
       <c r="I271">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="K271" t="s">
         <v>1424</v>
@@ -15190,7 +15190,7 @@
         <v>1417</v>
       </c>
       <c r="I276">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="K276" t="s">
         <v>1425</v>
@@ -15228,7 +15228,7 @@
         <v>1417</v>
       </c>
       <c r="I277">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="K277" t="s">
         <v>1421</v>
@@ -15266,7 +15266,7 @@
         <v>1417</v>
       </c>
       <c r="I278">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="J278">
         <v>148</v>
@@ -15310,7 +15310,7 @@
         <v>1417</v>
       </c>
       <c r="I279">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="K279" t="s">
         <v>1423</v>
@@ -15351,7 +15351,7 @@
         <v>1417</v>
       </c>
       <c r="I280">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="K280" t="s">
         <v>1421</v>
@@ -15389,7 +15389,7 @@
         <v>1417</v>
       </c>
       <c r="I281">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="K281" t="s">
         <v>1421</v>
@@ -15430,7 +15430,7 @@
         <v>1417</v>
       </c>
       <c r="I282">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="K282" t="s">
         <v>1421</v>
@@ -15724,7 +15724,7 @@
         <v>1417</v>
       </c>
       <c r="I291">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="J291">
         <v>20</v>
@@ -15768,7 +15768,7 @@
         <v>1417</v>
       </c>
       <c r="I292">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="K292" t="s">
         <v>1424</v>
@@ -15806,7 +15806,7 @@
         <v>1417</v>
       </c>
       <c r="I293">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="K293" t="s">
         <v>1425</v>
@@ -15844,7 +15844,7 @@
         <v>1417</v>
       </c>
       <c r="I294">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="K294" t="s">
         <v>1430</v>
@@ -15981,7 +15981,7 @@
         <v>1417</v>
       </c>
       <c r="I298">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="J298">
         <v>58</v>
@@ -16145,7 +16145,7 @@
         <v>1417</v>
       </c>
       <c r="I302">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="K302" t="s">
         <v>1424</v>
@@ -16183,7 +16183,7 @@
         <v>1417</v>
       </c>
       <c r="I303">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="K303" t="s">
         <v>1421</v>
@@ -16221,7 +16221,7 @@
         <v>1417</v>
       </c>
       <c r="I304">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="K304" t="s">
         <v>1424</v>
@@ -16259,7 +16259,7 @@
         <v>1417</v>
       </c>
       <c r="I305">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="J305">
         <v>35</v>
@@ -16303,7 +16303,7 @@
         <v>1417</v>
       </c>
       <c r="I306">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="J306">
         <v>31</v>
@@ -16391,7 +16391,7 @@
         <v>1417</v>
       </c>
       <c r="I308">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="K308" t="s">
         <v>1420</v>
@@ -16508,7 +16508,7 @@
         <v>1417</v>
       </c>
       <c r="I311">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="K311" t="s">
         <v>1420</v>
@@ -16838,7 +16838,7 @@
         <v>1417</v>
       </c>
       <c r="I320">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="K320" t="s">
         <v>1425</v>
@@ -16876,7 +16876,7 @@
         <v>1417</v>
       </c>
       <c r="I321">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="K321" t="s">
         <v>1421</v>
@@ -16914,7 +16914,7 @@
         <v>1417</v>
       </c>
       <c r="I322">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="J322">
         <v>57</v>
@@ -17028,7 +17028,7 @@
         <v>1417</v>
       </c>
       <c r="I325">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="J325">
         <v>57</v>
@@ -17110,7 +17110,7 @@
         <v>1417</v>
       </c>
       <c r="I327">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="J327">
         <v>57</v>
@@ -17154,7 +17154,7 @@
         <v>1417</v>
       </c>
       <c r="I328">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="J328">
         <v>57</v>
@@ -17198,7 +17198,7 @@
         <v>1417</v>
       </c>
       <c r="I329">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="J329">
         <v>57</v>
@@ -17242,7 +17242,7 @@
         <v>1417</v>
       </c>
       <c r="I330">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="J330">
         <v>57</v>
@@ -17286,7 +17286,7 @@
         <v>1417</v>
       </c>
       <c r="I331">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="K331" t="s">
         <v>1420</v>
@@ -17324,7 +17324,7 @@
         <v>1417</v>
       </c>
       <c r="I332">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="K332" t="s">
         <v>1421</v>
@@ -17362,7 +17362,7 @@
         <v>1417</v>
       </c>
       <c r="I333">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="J333">
         <v>100</v>
@@ -17406,7 +17406,7 @@
         <v>1417</v>
       </c>
       <c r="I334">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="K334" t="s">
         <v>1421</v>
@@ -17631,7 +17631,7 @@
         <v>1417</v>
       </c>
       <c r="I340">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="J340">
         <v>98</v>
@@ -17672,7 +17672,7 @@
         <v>1417</v>
       </c>
       <c r="I341">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="J341">
         <v>90</v>
@@ -17713,7 +17713,7 @@
         <v>1417</v>
       </c>
       <c r="I342">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="K342" t="s">
         <v>1420</v>
@@ -17827,7 +17827,7 @@
         <v>1417</v>
       </c>
       <c r="I345">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="K345" t="s">
         <v>1420</v>
@@ -17947,7 +17947,7 @@
         <v>1417</v>
       </c>
       <c r="I348">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="J348">
         <v>14</v>
@@ -17991,7 +17991,7 @@
         <v>1417</v>
       </c>
       <c r="I349">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="K349" t="s">
         <v>1425</v>
@@ -18029,7 +18029,7 @@
         <v>1417</v>
       </c>
       <c r="I350">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="J350">
         <v>46</v>
@@ -18067,7 +18067,7 @@
         <v>1417</v>
       </c>
       <c r="I351">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="J351">
         <v>82</v>
@@ -18111,7 +18111,7 @@
         <v>1417</v>
       </c>
       <c r="I352">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="J352">
         <v>78</v>
@@ -18155,7 +18155,7 @@
         <v>1417</v>
       </c>
       <c r="I353">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="J353">
         <v>83</v>
@@ -18199,7 +18199,7 @@
         <v>1417</v>
       </c>
       <c r="I354">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="K354" t="s">
         <v>1424</v>
@@ -18237,7 +18237,7 @@
         <v>1417</v>
       </c>
       <c r="I355">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="J355">
         <v>8</v>
@@ -18319,7 +18319,7 @@
         <v>1417</v>
       </c>
       <c r="I357">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="J357">
         <v>85</v>
@@ -18442,7 +18442,7 @@
         <v>1417</v>
       </c>
       <c r="I360">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="J360">
         <v>83</v>
@@ -18489,7 +18489,7 @@
         <v>1417</v>
       </c>
       <c r="I361">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="J361">
         <v>83</v>
@@ -18533,7 +18533,7 @@
         <v>1417</v>
       </c>
       <c r="I362">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="K362" t="s">
         <v>1424</v>
@@ -18571,7 +18571,7 @@
         <v>1417</v>
       </c>
       <c r="I363">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="K363" t="s">
         <v>1424</v>
@@ -18609,7 +18609,7 @@
         <v>1417</v>
       </c>
       <c r="I364">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="J364">
         <v>83</v>
@@ -18653,7 +18653,7 @@
         <v>1417</v>
       </c>
       <c r="I365">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="J365">
         <v>15</v>
@@ -18776,7 +18776,7 @@
         <v>1417</v>
       </c>
       <c r="I368">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="J368">
         <v>77</v>
@@ -18820,7 +18820,7 @@
         <v>1417</v>
       </c>
       <c r="I369">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="K369" t="s">
         <v>1424</v>
@@ -18858,7 +18858,7 @@
         <v>1417</v>
       </c>
       <c r="I370">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="K370" t="s">
         <v>1424</v>
@@ -18896,7 +18896,7 @@
         <v>1417</v>
       </c>
       <c r="I371">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="J371">
         <v>16</v>
@@ -18984,7 +18984,7 @@
         <v>1417</v>
       </c>
       <c r="I373">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="K373" t="s">
         <v>1420</v>
@@ -19022,7 +19022,7 @@
         <v>1417</v>
       </c>
       <c r="I374">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="K374" t="s">
         <v>1420</v>
@@ -19060,7 +19060,7 @@
         <v>1417</v>
       </c>
       <c r="I375">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="J375">
         <v>94</v>
@@ -19101,7 +19101,7 @@
         <v>1417</v>
       </c>
       <c r="I376">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="K376" t="s">
         <v>1424</v>
@@ -19180,7 +19180,7 @@
         <v>1417</v>
       </c>
       <c r="I378">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="K378" t="s">
         <v>1424</v>
@@ -19218,7 +19218,7 @@
         <v>1417</v>
       </c>
       <c r="I379">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="J379">
         <v>20</v>
@@ -19262,7 +19262,7 @@
         <v>1417</v>
       </c>
       <c r="I380">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="J380">
         <v>94</v>
@@ -19306,7 +19306,7 @@
         <v>1417</v>
       </c>
       <c r="I381">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="K381" t="s">
         <v>1424</v>
@@ -19344,7 +19344,7 @@
         <v>1417</v>
       </c>
       <c r="I382">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="K382" t="s">
         <v>1424</v>
@@ -19382,7 +19382,7 @@
         <v>1417</v>
       </c>
       <c r="I383">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="J383">
         <v>71</v>
@@ -19426,7 +19426,7 @@
         <v>1417</v>
       </c>
       <c r="I384">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="K384" t="s">
         <v>1421</v>
@@ -19508,7 +19508,7 @@
         <v>1417</v>
       </c>
       <c r="I386">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="K386" t="s">
         <v>1424</v>
@@ -19546,7 +19546,7 @@
         <v>1417</v>
       </c>
       <c r="I387">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="K387" t="s">
         <v>1424</v>
@@ -19584,7 +19584,7 @@
         <v>1417</v>
       </c>
       <c r="I388">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="J388">
         <v>-85</v>
@@ -19628,7 +19628,7 @@
         <v>1417</v>
       </c>
       <c r="I389">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="K389" t="s">
         <v>1425</v>
@@ -20079,7 +20079,7 @@
         <v>1417</v>
       </c>
       <c r="I400">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="K400" t="s">
         <v>1424</v>
@@ -20155,7 +20155,7 @@
         <v>1417</v>
       </c>
       <c r="I402">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="K402" t="s">
         <v>1424</v>
@@ -20193,7 +20193,7 @@
         <v>1417</v>
       </c>
       <c r="I403">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="J403">
         <v>83</v>
@@ -20237,7 +20237,7 @@
         <v>1417</v>
       </c>
       <c r="I404">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="K404" t="s">
         <v>1424</v>
@@ -20307,7 +20307,7 @@
         <v>1417</v>
       </c>
       <c r="I406">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="Q406" t="b">
         <v>1</v>
@@ -20339,7 +20339,7 @@
         <v>1417</v>
       </c>
       <c r="I407">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="Q407" t="b">
         <v>1</v>
@@ -20371,7 +20371,7 @@
         <v>1417</v>
       </c>
       <c r="I408">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="Q408" t="b">
         <v>1</v>
@@ -20403,7 +20403,7 @@
         <v>1417</v>
       </c>
       <c r="I409">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="Q409" t="b">
         <v>1</v>
@@ -20435,7 +20435,7 @@
         <v>1417</v>
       </c>
       <c r="I410">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="Q410" t="b">
         <v>1</v>
@@ -20467,7 +20467,7 @@
         <v>1417</v>
       </c>
       <c r="I411">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="Q411" t="b">
         <v>1</v>
@@ -20499,7 +20499,7 @@
         <v>1417</v>
       </c>
       <c r="I412">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="Q412" t="b">
         <v>1</v>
@@ -20531,7 +20531,7 @@
         <v>1417</v>
       </c>
       <c r="I413">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="Q413" t="b">
         <v>1</v>
@@ -20621,7 +20621,7 @@
         <v>1417</v>
       </c>
       <c r="I416">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="Q416" t="b">
         <v>1</v>
@@ -20711,7 +20711,7 @@
         <v>1417</v>
       </c>
       <c r="I419">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="Q419" t="b">
         <v>1</v>
@@ -20743,7 +20743,7 @@
         <v>1417</v>
       </c>
       <c r="I420">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="Q420" t="b">
         <v>1</v>
@@ -20775,7 +20775,7 @@
         <v>1417</v>
       </c>
       <c r="I421">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="Q421" t="b">
         <v>1</v>
@@ -20807,7 +20807,7 @@
         <v>1417</v>
       </c>
       <c r="I422">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="Q422" t="b">
         <v>1</v>
@@ -20839,7 +20839,7 @@
         <v>1417</v>
       </c>
       <c r="I423">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="Q423" t="b">
         <v>1</v>
@@ -20871,7 +20871,7 @@
         <v>1417</v>
       </c>
       <c r="I424">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="Q424" t="b">
         <v>1</v>
@@ -20903,7 +20903,7 @@
         <v>1417</v>
       </c>
       <c r="I425">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="Q425" t="b">
         <v>1</v>
@@ -20935,7 +20935,7 @@
         <v>1417</v>
       </c>
       <c r="I426">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="Q426" t="b">
         <v>1</v>
@@ -20967,7 +20967,7 @@
         <v>1417</v>
       </c>
       <c r="I427">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="Q427" t="b">
         <v>1</v>
@@ -21057,7 +21057,7 @@
         <v>1417</v>
       </c>
       <c r="I430">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="Q430" t="b">
         <v>1</v>
@@ -21089,7 +21089,7 @@
         <v>1417</v>
       </c>
       <c r="I431">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="Q431" t="b">
         <v>1</v>
@@ -21121,7 +21121,7 @@
         <v>1417</v>
       </c>
       <c r="I432">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="Q432" t="b">
         <v>1</v>
@@ -21153,7 +21153,7 @@
         <v>1417</v>
       </c>
       <c r="I433">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="Q433" t="b">
         <v>1</v>
@@ -21185,7 +21185,7 @@
         <v>1417</v>
       </c>
       <c r="I434">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="Q434" t="b">
         <v>1</v>
@@ -21217,7 +21217,7 @@
         <v>1417</v>
       </c>
       <c r="I435">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="Q435" t="b">
         <v>1</v>
@@ -21249,7 +21249,7 @@
         <v>1417</v>
       </c>
       <c r="I436">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="Q436" t="b">
         <v>1</v>
@@ -21281,7 +21281,7 @@
         <v>1419</v>
       </c>
       <c r="I437">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="Q437" t="b">
         <v>1</v>
@@ -21313,7 +21313,7 @@
         <v>1419</v>
       </c>
       <c r="I438">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="Q438" t="b">
         <v>1</v>
@@ -21345,7 +21345,7 @@
         <v>1417</v>
       </c>
       <c r="I439">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="Q439" t="b">
         <v>1</v>
@@ -21377,7 +21377,7 @@
         <v>1417</v>
       </c>
       <c r="I440">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="Q440" t="b">
         <v>1</v>
@@ -21409,7 +21409,7 @@
         <v>1417</v>
       </c>
       <c r="I441">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="Q441" t="b">
         <v>1</v>
@@ -21470,7 +21470,7 @@
         <v>1417</v>
       </c>
       <c r="I443">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="Q443" t="b">
         <v>1</v>
@@ -21560,7 +21560,7 @@
         <v>1417</v>
       </c>
       <c r="I446">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q446" t="b">
         <v>1</v>
@@ -21592,7 +21592,7 @@
         <v>1417</v>
       </c>
       <c r="I447">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q447" t="b">
         <v>1</v>
@@ -21624,7 +21624,7 @@
         <v>1417</v>
       </c>
       <c r="I448">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="Q448" t="b">
         <v>1</v>
@@ -21656,7 +21656,7 @@
         <v>1417</v>
       </c>
       <c r="I449">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="Q449" t="b">
         <v>1</v>
@@ -21688,7 +21688,7 @@
         <v>1417</v>
       </c>
       <c r="I450">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="Q450" t="b">
         <v>1</v>
@@ -21720,7 +21720,7 @@
         <v>1417</v>
       </c>
       <c r="I451">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q451" t="b">
         <v>1</v>
@@ -21781,7 +21781,7 @@
         <v>1417</v>
       </c>
       <c r="I453">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q453" t="b">
         <v>1</v>
@@ -21813,7 +21813,7 @@
         <v>1417</v>
       </c>
       <c r="I454">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q454" t="b">
         <v>1</v>
@@ -21845,7 +21845,7 @@
         <v>1417</v>
       </c>
       <c r="I455">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q455" t="b">
         <v>1</v>
@@ -21906,7 +21906,7 @@
         <v>1417</v>
       </c>
       <c r="I457">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q457" t="b">
         <v>1</v>
@@ -21938,7 +21938,7 @@
         <v>1417</v>
       </c>
       <c r="I458">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="Q458" t="b">
         <v>1</v>
@@ -21970,7 +21970,7 @@
         <v>1417</v>
       </c>
       <c r="I459">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Q459" t="b">
         <v>1</v>
@@ -22002,7 +22002,7 @@
         <v>1417</v>
       </c>
       <c r="I460">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Q460" t="b">
         <v>1</v>
@@ -22034,7 +22034,7 @@
         <v>1417</v>
       </c>
       <c r="I461">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Q461" t="b">
         <v>1</v>
@@ -22066,7 +22066,7 @@
         <v>1417</v>
       </c>
       <c r="I462">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Q462" t="b">
         <v>1</v>
@@ -22098,7 +22098,7 @@
         <v>1417</v>
       </c>
       <c r="I463">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="Q463" t="b">
         <v>1</v>
@@ -22130,7 +22130,7 @@
         <v>1417</v>
       </c>
       <c r="I464">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q464" t="b">
         <v>1</v>
@@ -22162,7 +22162,7 @@
         <v>1417</v>
       </c>
       <c r="I465">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q465" t="b">
         <v>1</v>
@@ -22194,7 +22194,7 @@
         <v>1417</v>
       </c>
       <c r="I466">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q466" t="b">
         <v>1</v>
@@ -22226,7 +22226,7 @@
         <v>1417</v>
       </c>
       <c r="I467">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q467" t="b">
         <v>1</v>
@@ -22258,7 +22258,7 @@
         <v>1417</v>
       </c>
       <c r="I468">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q468" t="b">
         <v>1</v>
@@ -22290,7 +22290,7 @@
         <v>1417</v>
       </c>
       <c r="I469">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q469" t="b">
         <v>1</v>
@@ -22351,7 +22351,7 @@
         <v>1417</v>
       </c>
       <c r="I471">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q471" t="b">
         <v>1</v>
@@ -22383,7 +22383,7 @@
         <v>1417</v>
       </c>
       <c r="I472">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q472" t="b">
         <v>1</v>
@@ -22415,7 +22415,7 @@
         <v>1417</v>
       </c>
       <c r="I473">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q473" t="b">
         <v>1</v>
@@ -22447,7 +22447,7 @@
         <v>1417</v>
       </c>
       <c r="I474">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="Q474" t="b">
         <v>1</v>
@@ -22479,7 +22479,7 @@
         <v>1417</v>
       </c>
       <c r="I475">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="Q475" t="b">
         <v>1</v>
@@ -22511,7 +22511,7 @@
         <v>1417</v>
       </c>
       <c r="I476">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="Q476" t="b">
         <v>1</v>
@@ -22543,7 +22543,7 @@
         <v>1417</v>
       </c>
       <c r="I477">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="Q477" t="b">
         <v>1</v>
@@ -22575,7 +22575,7 @@
         <v>1417</v>
       </c>
       <c r="I478">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="Q478" t="b">
         <v>1</v>
@@ -22607,7 +22607,7 @@
         <v>1417</v>
       </c>
       <c r="I479">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="Q479" t="b">
         <v>1</v>
@@ -22639,7 +22639,7 @@
         <v>1417</v>
       </c>
       <c r="I480">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="Q480" t="b">
         <v>1</v>
@@ -22671,7 +22671,7 @@
         <v>1417</v>
       </c>
       <c r="I481">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="Q481" t="b">
         <v>1</v>
@@ -22703,7 +22703,7 @@
         <v>1417</v>
       </c>
       <c r="I482">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="Q482" t="b">
         <v>1</v>
@@ -22735,7 +22735,7 @@
         <v>1417</v>
       </c>
       <c r="I483">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="Q483" t="b">
         <v>1</v>
@@ -22767,7 +22767,7 @@
         <v>1417</v>
       </c>
       <c r="I484">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="Q484" t="b">
         <v>1</v>
@@ -22799,7 +22799,7 @@
         <v>1417</v>
       </c>
       <c r="I485">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="Q485" t="b">
         <v>1</v>
@@ -22831,7 +22831,7 @@
         <v>1417</v>
       </c>
       <c r="I486">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="Q486" t="b">
         <v>1</v>
@@ -22863,7 +22863,7 @@
         <v>1417</v>
       </c>
       <c r="I487">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="Q487" t="b">
         <v>1</v>
@@ -22895,7 +22895,7 @@
         <v>1417</v>
       </c>
       <c r="I488">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="Q488" t="b">
         <v>1</v>
@@ -22927,7 +22927,7 @@
         <v>1417</v>
       </c>
       <c r="I489">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="Q489" t="b">
         <v>1</v>
@@ -22959,7 +22959,7 @@
         <v>1417</v>
       </c>
       <c r="I490">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="Q490" t="b">
         <v>1</v>
@@ -22991,7 +22991,7 @@
         <v>1417</v>
       </c>
       <c r="I491">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="Q491" t="b">
         <v>1</v>
@@ -23023,7 +23023,7 @@
         <v>1419</v>
       </c>
       <c r="I492">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="Q492" t="b">
         <v>1</v>
@@ -23055,7 +23055,7 @@
         <v>1419</v>
       </c>
       <c r="I493">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="Q493" t="b">
         <v>1</v>
@@ -23087,7 +23087,7 @@
         <v>1419</v>
       </c>
       <c r="I494">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="Q494" t="b">
         <v>1</v>
@@ -23119,7 +23119,7 @@
         <v>1419</v>
       </c>
       <c r="I495">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="Q495" t="b">
         <v>1</v>
@@ -23151,7 +23151,7 @@
         <v>1419</v>
       </c>
       <c r="I496">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="Q496" t="b">
         <v>1</v>
@@ -23183,7 +23183,7 @@
         <v>1417</v>
       </c>
       <c r="I497">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="Q497" t="b">
         <v>1</v>
@@ -23215,7 +23215,7 @@
         <v>1417</v>
       </c>
       <c r="I498">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="Q498" t="b">
         <v>1</v>
@@ -23247,7 +23247,7 @@
         <v>1419</v>
       </c>
       <c r="I499">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="Q499" t="b">
         <v>1</v>
@@ -23279,7 +23279,7 @@
         <v>1417</v>
       </c>
       <c r="I500">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="Q500" t="b">
         <v>1</v>
@@ -23311,7 +23311,7 @@
         <v>1417</v>
       </c>
       <c r="I501">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="Q501" t="b">
         <v>1</v>
@@ -23343,7 +23343,7 @@
         <v>1417</v>
       </c>
       <c r="I502">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="Q502" t="b">
         <v>1</v>
@@ -23375,7 +23375,7 @@
         <v>1417</v>
       </c>
       <c r="I503">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="Q503" t="b">
         <v>1</v>
@@ -23407,7 +23407,7 @@
         <v>1417</v>
       </c>
       <c r="I504">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="Q504" t="b">
         <v>1</v>
@@ -23439,7 +23439,7 @@
         <v>1417</v>
       </c>
       <c r="I505">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="Q505" t="b">
         <v>1</v>
@@ -23471,7 +23471,7 @@
         <v>1417</v>
       </c>
       <c r="I506">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="Q506" t="b">
         <v>1</v>
@@ -23503,7 +23503,7 @@
         <v>1417</v>
       </c>
       <c r="I507">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="Q507" t="b">
         <v>1</v>
@@ -23564,7 +23564,7 @@
         <v>1417</v>
       </c>
       <c r="I509">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="Q509" t="b">
         <v>1</v>
@@ -23596,7 +23596,7 @@
         <v>1417</v>
       </c>
       <c r="I510">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="Q510" t="b">
         <v>1</v>
@@ -23628,7 +23628,7 @@
         <v>1417</v>
       </c>
       <c r="I511">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Q511" t="b">
         <v>1</v>
@@ -23660,7 +23660,7 @@
         <v>1417</v>
       </c>
       <c r="I512">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Q512" t="b">
         <v>1</v>
@@ -23692,7 +23692,7 @@
         <v>1417</v>
       </c>
       <c r="I513">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q513" t="b">
         <v>1</v>
@@ -23753,7 +23753,7 @@
         <v>1417</v>
       </c>
       <c r="I515">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q515" t="b">
         <v>1</v>
@@ -23785,7 +23785,7 @@
         <v>1417</v>
       </c>
       <c r="I516">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q516" t="b">
         <v>1</v>
@@ -23817,7 +23817,7 @@
         <v>1417</v>
       </c>
       <c r="I517">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q517" t="b">
         <v>1</v>
@@ -23849,7 +23849,7 @@
         <v>1417</v>
       </c>
       <c r="I518">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q518" t="b">
         <v>1</v>
@@ -23881,7 +23881,7 @@
         <v>1417</v>
       </c>
       <c r="I519">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="Q519" t="b">
         <v>1</v>
@@ -23913,7 +23913,7 @@
         <v>1417</v>
       </c>
       <c r="I520">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="Q520" t="b">
         <v>1</v>
@@ -23945,7 +23945,7 @@
         <v>1417</v>
       </c>
       <c r="I521">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="Q521" t="b">
         <v>1</v>
@@ -23977,7 +23977,7 @@
         <v>1417</v>
       </c>
       <c r="I522">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="Q522" t="b">
         <v>1</v>
@@ -24009,7 +24009,7 @@
         <v>1417</v>
       </c>
       <c r="I523">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="Q523" t="b">
         <v>1</v>
@@ -24041,7 +24041,7 @@
         <v>1417</v>
       </c>
       <c r="I524">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="Q524" t="b">
         <v>1</v>
@@ -24073,7 +24073,7 @@
         <v>1417</v>
       </c>
       <c r="I525">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="Q525" t="b">
         <v>1</v>
@@ -24105,7 +24105,7 @@
         <v>1417</v>
       </c>
       <c r="I526">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="Q526" t="b">
         <v>1</v>
@@ -24137,7 +24137,7 @@
         <v>1417</v>
       </c>
       <c r="I527">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="Q527" t="b">
         <v>1</v>
@@ -24169,7 +24169,7 @@
         <v>1417</v>
       </c>
       <c r="I528">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q528" t="b">
         <v>1</v>
@@ -24201,7 +24201,7 @@
         <v>1417</v>
       </c>
       <c r="I529">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="Q529" t="b">
         <v>1</v>
@@ -24233,7 +24233,7 @@
         <v>1417</v>
       </c>
       <c r="I530">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="Q530" t="b">
         <v>1</v>
@@ -24265,7 +24265,7 @@
         <v>1417</v>
       </c>
       <c r="I531">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="Q531" t="b">
         <v>1</v>
@@ -24297,7 +24297,7 @@
         <v>1417</v>
       </c>
       <c r="I532">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="Q532" t="b">
         <v>1</v>
@@ -24329,7 +24329,7 @@
         <v>1417</v>
       </c>
       <c r="I533">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="Q533" t="b">
         <v>1</v>
@@ -24361,7 +24361,7 @@
         <v>1417</v>
       </c>
       <c r="I534">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="Q534" t="b">
         <v>1</v>
@@ -24393,7 +24393,7 @@
         <v>1417</v>
       </c>
       <c r="I535">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="Q535" t="b">
         <v>1</v>
@@ -24425,7 +24425,7 @@
         <v>1417</v>
       </c>
       <c r="I536">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="Q536" t="b">
         <v>1</v>
@@ -24457,7 +24457,7 @@
         <v>1417</v>
       </c>
       <c r="I537">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="Q537" t="b">
         <v>1</v>
@@ -24489,7 +24489,7 @@
         <v>1417</v>
       </c>
       <c r="I538">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="Q538" t="b">
         <v>1</v>
@@ -24521,7 +24521,7 @@
         <v>1417</v>
       </c>
       <c r="I539">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="Q539" t="b">
         <v>1</v>
@@ -24553,7 +24553,7 @@
         <v>1417</v>
       </c>
       <c r="I540">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="Q540" t="b">
         <v>1</v>
@@ -24585,7 +24585,7 @@
         <v>1417</v>
       </c>
       <c r="I541">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="Q541" t="b">
         <v>1</v>
@@ -24617,7 +24617,7 @@
         <v>1417</v>
       </c>
       <c r="I542">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="Q542" t="b">
         <v>1</v>
@@ -24649,7 +24649,7 @@
         <v>1417</v>
       </c>
       <c r="I543">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="Q543" t="b">
         <v>1</v>
@@ -24681,7 +24681,7 @@
         <v>1417</v>
       </c>
       <c r="I544">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="Q544" t="b">
         <v>1</v>
@@ -24713,7 +24713,7 @@
         <v>1417</v>
       </c>
       <c r="I545">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="Q545" t="b">
         <v>1</v>
@@ -24745,7 +24745,7 @@
         <v>1417</v>
       </c>
       <c r="I546">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="Q546" t="b">
         <v>1</v>
@@ -24777,7 +24777,7 @@
         <v>1417</v>
       </c>
       <c r="I547">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="Q547" t="b">
         <v>1</v>
@@ -24809,7 +24809,7 @@
         <v>1417</v>
       </c>
       <c r="I548">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="Q548" t="b">
         <v>1</v>
@@ -24841,7 +24841,7 @@
         <v>1417</v>
       </c>
       <c r="I549">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="Q549" t="b">
         <v>1</v>
@@ -24873,7 +24873,7 @@
         <v>1417</v>
       </c>
       <c r="I550">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="Q550" t="b">
         <v>1</v>
@@ -24905,7 +24905,7 @@
         <v>1417</v>
       </c>
       <c r="I551">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="Q551" t="b">
         <v>1</v>
@@ -24937,7 +24937,7 @@
         <v>1417</v>
       </c>
       <c r="I552">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="Q552" t="b">
         <v>1</v>
@@ -24969,7 +24969,7 @@
         <v>1417</v>
       </c>
       <c r="I553">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="Q553" t="b">
         <v>1</v>
@@ -25001,7 +25001,7 @@
         <v>1417</v>
       </c>
       <c r="I554">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="Q554" t="b">
         <v>1</v>
@@ -25033,7 +25033,7 @@
         <v>1417</v>
       </c>
       <c r="I555">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="Q555" t="b">
         <v>1</v>
@@ -25065,7 +25065,7 @@
         <v>1417</v>
       </c>
       <c r="I556">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="Q556" t="b">
         <v>1</v>
@@ -25097,7 +25097,7 @@
         <v>1417</v>
       </c>
       <c r="I557">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q557" t="b">
         <v>1</v>
@@ -25129,7 +25129,7 @@
         <v>1417</v>
       </c>
       <c r="I558">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q558" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: reparaveis (09/10/2026 14:27)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
@@ -5132,7 +5132,7 @@
         <v>1417</v>
       </c>
       <c r="I2">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="K2" t="s">
         <v>1420</v>
@@ -5170,7 +5170,7 @@
         <v>1417</v>
       </c>
       <c r="I3">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="K3" t="s">
         <v>1421</v>
@@ -5208,7 +5208,7 @@
         <v>1417</v>
       </c>
       <c r="I4">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="K4" t="s">
         <v>1421</v>
@@ -5246,7 +5246,7 @@
         <v>1417</v>
       </c>
       <c r="I5">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="J5">
         <v>279</v>
@@ -5290,7 +5290,7 @@
         <v>1417</v>
       </c>
       <c r="I6">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="J6">
         <v>153</v>
@@ -5334,7 +5334,7 @@
         <v>1417</v>
       </c>
       <c r="I7">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="J7">
         <v>112</v>
@@ -5410,7 +5410,7 @@
         <v>1417</v>
       </c>
       <c r="I9">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="J9">
         <v>362</v>
@@ -5457,7 +5457,7 @@
         <v>1417</v>
       </c>
       <c r="I10">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="J10">
         <v>378</v>
@@ -5504,7 +5504,7 @@
         <v>1417</v>
       </c>
       <c r="I11">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="J11">
         <v>112</v>
@@ -5551,7 +5551,7 @@
         <v>1417</v>
       </c>
       <c r="I12">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="J12">
         <v>124</v>
@@ -5624,7 +5624,7 @@
         <v>1417</v>
       </c>
       <c r="I14">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="J14">
         <v>64</v>
@@ -5703,7 +5703,7 @@
         <v>1417</v>
       </c>
       <c r="I16">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="K16" t="s">
         <v>1420</v>
@@ -5741,7 +5741,7 @@
         <v>1417</v>
       </c>
       <c r="I17">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="J17">
         <v>161</v>
@@ -5785,7 +5785,7 @@
         <v>1417</v>
       </c>
       <c r="I18">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="J18">
         <v>66</v>
@@ -5858,7 +5858,7 @@
         <v>1417</v>
       </c>
       <c r="I20">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="J20">
         <v>399</v>
@@ -5931,7 +5931,7 @@
         <v>1417</v>
       </c>
       <c r="I22">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="K22" t="s">
         <v>1424</v>
@@ -5969,7 +5969,7 @@
         <v>1417</v>
       </c>
       <c r="I23">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="J23">
         <v>229</v>
@@ -6074,7 +6074,7 @@
         <v>1417</v>
       </c>
       <c r="I26">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="J26">
         <v>155</v>
@@ -6121,7 +6121,7 @@
         <v>1417</v>
       </c>
       <c r="I27">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="K27" t="s">
         <v>1424</v>
@@ -6217,7 +6217,7 @@
         <v>1417</v>
       </c>
       <c r="I30">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="J30">
         <v>209</v>
@@ -6290,7 +6290,7 @@
         <v>1417</v>
       </c>
       <c r="I32">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="K32" t="s">
         <v>1420</v>
@@ -6499,7 +6499,7 @@
         <v>1417</v>
       </c>
       <c r="I39">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="K39" t="s">
         <v>1425</v>
@@ -6662,7 +6662,7 @@
         <v>1417</v>
       </c>
       <c r="I44">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="J44">
         <v>87</v>
@@ -6709,7 +6709,7 @@
         <v>1417</v>
       </c>
       <c r="I45">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="J45">
         <v>331</v>
@@ -6756,7 +6756,7 @@
         <v>1417</v>
       </c>
       <c r="I46">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="K46" t="s">
         <v>1424</v>
@@ -6797,7 +6797,7 @@
         <v>1417</v>
       </c>
       <c r="I47">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="J47">
         <v>344</v>
@@ -6844,7 +6844,7 @@
         <v>1417</v>
       </c>
       <c r="I48">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="K48" t="s">
         <v>1424</v>
@@ -6911,7 +6911,7 @@
         <v>1417</v>
       </c>
       <c r="I50">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="K50" t="s">
         <v>1424</v>
@@ -6978,7 +6978,7 @@
         <v>1417</v>
       </c>
       <c r="I52">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="K52" t="s">
         <v>1420</v>
@@ -7016,7 +7016,7 @@
         <v>1417</v>
       </c>
       <c r="I53">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="K53" t="s">
         <v>1421</v>
@@ -7054,7 +7054,7 @@
         <v>1417</v>
       </c>
       <c r="I54">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="K54" t="s">
         <v>1421</v>
@@ -7330,7 +7330,7 @@
         <v>1417</v>
       </c>
       <c r="I63">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="J63">
         <v>293</v>
@@ -7377,7 +7377,7 @@
         <v>1417</v>
       </c>
       <c r="I64">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="J64">
         <v>320</v>
@@ -7607,7 +7607,7 @@
         <v>1417</v>
       </c>
       <c r="I71">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="J71">
         <v>429</v>
@@ -7680,7 +7680,7 @@
         <v>1417</v>
       </c>
       <c r="I73">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="K73" t="s">
         <v>1420</v>
@@ -7788,7 +7788,7 @@
         <v>1417</v>
       </c>
       <c r="I76">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="K76" t="s">
         <v>1427</v>
@@ -7881,7 +7881,7 @@
         <v>1417</v>
       </c>
       <c r="I79">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="K79" t="s">
         <v>1427</v>
@@ -7986,7 +7986,7 @@
         <v>1417</v>
       </c>
       <c r="I82">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="K82" t="s">
         <v>1424</v>
@@ -8053,7 +8053,7 @@
         <v>1417</v>
       </c>
       <c r="I84">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="J84">
         <v>40</v>
@@ -8100,7 +8100,7 @@
         <v>1417</v>
       </c>
       <c r="I85">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="K85" t="s">
         <v>1421</v>
@@ -8138,7 +8138,7 @@
         <v>1417</v>
       </c>
       <c r="I86">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="K86" t="s">
         <v>1421</v>
@@ -8176,7 +8176,7 @@
         <v>1417</v>
       </c>
       <c r="I87">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="J87">
         <v>-16</v>
@@ -8299,7 +8299,7 @@
         <v>1417</v>
       </c>
       <c r="I90">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="K90" t="s">
         <v>1394</v>
@@ -8448,7 +8448,7 @@
         <v>1417</v>
       </c>
       <c r="I94">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="K94" t="s">
         <v>1424</v>
@@ -8527,7 +8527,7 @@
         <v>1417</v>
       </c>
       <c r="I96">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="J96">
         <v>17</v>
@@ -8574,7 +8574,7 @@
         <v>1417</v>
       </c>
       <c r="I97">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="J97">
         <v>20</v>
@@ -8621,7 +8621,7 @@
         <v>1417</v>
       </c>
       <c r="I98">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="K98" t="s">
         <v>1424</v>
@@ -8898,7 +8898,7 @@
         <v>1417</v>
       </c>
       <c r="I106">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="J106">
         <v>49</v>
@@ -8942,7 +8942,7 @@
         <v>1417</v>
       </c>
       <c r="I107">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="J107">
         <v>36</v>
@@ -8986,7 +8986,7 @@
         <v>1417</v>
       </c>
       <c r="I108">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="K108" t="s">
         <v>1421</v>
@@ -9024,7 +9024,7 @@
         <v>1417</v>
       </c>
       <c r="I109">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="K109" t="s">
         <v>1421</v>
@@ -9207,7 +9207,7 @@
         <v>1417</v>
       </c>
       <c r="I115">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="K115" t="s">
         <v>1421</v>
@@ -9245,7 +9245,7 @@
         <v>1417</v>
       </c>
       <c r="I116">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="K116" t="s">
         <v>1421</v>
@@ -9283,7 +9283,7 @@
         <v>1417</v>
       </c>
       <c r="I117">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="K117" t="s">
         <v>1421</v>
@@ -9321,7 +9321,7 @@
         <v>1417</v>
       </c>
       <c r="I118">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="K118" t="s">
         <v>1421</v>
@@ -9359,7 +9359,7 @@
         <v>1417</v>
       </c>
       <c r="I119">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="K119" t="s">
         <v>1421</v>
@@ -9397,7 +9397,7 @@
         <v>1417</v>
       </c>
       <c r="I120">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="K120" t="s">
         <v>1421</v>
@@ -9435,7 +9435,7 @@
         <v>1417</v>
       </c>
       <c r="I121">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="J121">
         <v>251</v>
@@ -9482,7 +9482,7 @@
         <v>1417</v>
       </c>
       <c r="I122">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="K122" t="s">
         <v>1421</v>
@@ -9549,7 +9549,7 @@
         <v>1417</v>
       </c>
       <c r="I124">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="K124" t="s">
         <v>1421</v>
@@ -9587,7 +9587,7 @@
         <v>1417</v>
       </c>
       <c r="I125">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="K125" t="s">
         <v>1427</v>
@@ -9683,7 +9683,7 @@
         <v>1417</v>
       </c>
       <c r="I128">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="K128" t="s">
         <v>1421</v>
@@ -9721,7 +9721,7 @@
         <v>1417</v>
       </c>
       <c r="I129">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="K129" t="s">
         <v>1420</v>
@@ -9759,7 +9759,7 @@
         <v>1417</v>
       </c>
       <c r="I130">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="J130">
         <v>47</v>
@@ -9835,7 +9835,7 @@
         <v>1417</v>
       </c>
       <c r="I132">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="J132">
         <v>145</v>
@@ -9911,7 +9911,7 @@
         <v>1417</v>
       </c>
       <c r="I134">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="K134" t="s">
         <v>1420</v>
@@ -10036,7 +10036,7 @@
         <v>1417</v>
       </c>
       <c r="I138">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="K138" t="s">
         <v>1421</v>
@@ -10420,7 +10420,7 @@
         <v>1417</v>
       </c>
       <c r="I150">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="J150">
         <v>201</v>
@@ -10607,7 +10607,7 @@
         <v>1417</v>
       </c>
       <c r="I155">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="K155" t="s">
         <v>1427</v>
@@ -10642,7 +10642,7 @@
         <v>1417</v>
       </c>
       <c r="I156">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="K156" t="s">
         <v>1421</v>
@@ -10680,7 +10680,7 @@
         <v>1417</v>
       </c>
       <c r="I157">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="J157">
         <v>371</v>
@@ -10724,7 +10724,7 @@
         <v>1417</v>
       </c>
       <c r="I158">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="J158">
         <v>52</v>
@@ -10768,7 +10768,7 @@
         <v>1417</v>
       </c>
       <c r="I159">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="K159" t="s">
         <v>1421</v>
@@ -10806,7 +10806,7 @@
         <v>1417</v>
       </c>
       <c r="I160">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="K160" t="s">
         <v>1421</v>
@@ -10844,7 +10844,7 @@
         <v>1417</v>
       </c>
       <c r="I161">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="J161">
         <v>55</v>
@@ -10979,7 +10979,7 @@
         <v>1417</v>
       </c>
       <c r="I164">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="O164" t="s">
         <v>1533</v>
@@ -11154,7 +11154,7 @@
         <v>1417</v>
       </c>
       <c r="I169">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="K169" t="s">
         <v>1394</v>
@@ -11364,7 +11364,7 @@
         <v>1417</v>
       </c>
       <c r="I175">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="J175">
         <v>205</v>
@@ -11411,7 +11411,7 @@
         <v>1417</v>
       </c>
       <c r="I176">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="K176" t="s">
         <v>1421</v>
@@ -11449,7 +11449,7 @@
         <v>1417</v>
       </c>
       <c r="I177">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="J177">
         <v>44</v>
@@ -11496,7 +11496,7 @@
         <v>1417</v>
       </c>
       <c r="I178">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="K178" t="s">
         <v>1420</v>
@@ -11563,7 +11563,7 @@
         <v>1417</v>
       </c>
       <c r="I180">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="K180" t="s">
         <v>1420</v>
@@ -11659,7 +11659,7 @@
         <v>1417</v>
       </c>
       <c r="I183">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="K183" t="s">
         <v>1421</v>
@@ -11697,7 +11697,7 @@
         <v>1417</v>
       </c>
       <c r="I184">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="K184" t="s">
         <v>1427</v>
@@ -11732,7 +11732,7 @@
         <v>1417</v>
       </c>
       <c r="I185">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="K185" t="s">
         <v>1421</v>
@@ -11770,7 +11770,7 @@
         <v>1417</v>
       </c>
       <c r="I186">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="K186" t="s">
         <v>1421</v>
@@ -11808,7 +11808,7 @@
         <v>1417</v>
       </c>
       <c r="I187">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="J187">
         <v>75</v>
@@ -11855,7 +11855,7 @@
         <v>1417</v>
       </c>
       <c r="I188">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="J188">
         <v>40</v>
@@ -11902,7 +11902,7 @@
         <v>1417</v>
       </c>
       <c r="I189">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="J189">
         <v>155</v>
@@ -11946,7 +11946,7 @@
         <v>1417</v>
       </c>
       <c r="I190">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="J190">
         <v>107</v>
@@ -11990,7 +11990,7 @@
         <v>1417</v>
       </c>
       <c r="I191">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="J191">
         <v>5</v>
@@ -12034,7 +12034,7 @@
         <v>1417</v>
       </c>
       <c r="I192">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="K192" t="s">
         <v>1421</v>
@@ -12072,7 +12072,7 @@
         <v>1417</v>
       </c>
       <c r="I193">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="K193" t="s">
         <v>1426</v>
@@ -12267,7 +12267,7 @@
         <v>1417</v>
       </c>
       <c r="I199">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="J199">
         <v>70</v>
@@ -12352,7 +12352,7 @@
         <v>1417</v>
       </c>
       <c r="I201">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="K201" t="s">
         <v>1421</v>
@@ -12390,7 +12390,7 @@
         <v>1417</v>
       </c>
       <c r="I202">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="K202" t="s">
         <v>1421</v>
@@ -12469,7 +12469,7 @@
         <v>1417</v>
       </c>
       <c r="I204">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="K204" t="s">
         <v>1420</v>
@@ -12507,7 +12507,7 @@
         <v>1417</v>
       </c>
       <c r="I205">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="K205" t="s">
         <v>1420</v>
@@ -12574,7 +12574,7 @@
         <v>1417</v>
       </c>
       <c r="I207">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="J207">
         <v>167</v>
@@ -12618,7 +12618,7 @@
         <v>1417</v>
       </c>
       <c r="I208">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="J208">
         <v>45</v>
@@ -12662,7 +12662,7 @@
         <v>1417</v>
       </c>
       <c r="I209">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="J209">
         <v>191</v>
@@ -12706,7 +12706,7 @@
         <v>1417</v>
       </c>
       <c r="I210">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="K210" t="s">
         <v>1424</v>
@@ -12802,7 +12802,7 @@
         <v>1417</v>
       </c>
       <c r="I213">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="K213" t="s">
         <v>1421</v>
@@ -12840,7 +12840,7 @@
         <v>1417</v>
       </c>
       <c r="I214">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="J214">
         <v>14</v>
@@ -12887,7 +12887,7 @@
         <v>1417</v>
       </c>
       <c r="I215">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="K215" t="s">
         <v>1421</v>
@@ -12954,7 +12954,7 @@
         <v>1417</v>
       </c>
       <c r="I217">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="J217">
         <v>42</v>
@@ -12998,7 +12998,7 @@
         <v>1417</v>
       </c>
       <c r="I218">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="J218">
         <v>166</v>
@@ -13086,7 +13086,7 @@
         <v>1417</v>
       </c>
       <c r="I220">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="J220">
         <v>154</v>
@@ -13472,7 +13472,7 @@
         <v>1417</v>
       </c>
       <c r="I230">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="J230">
         <v>197</v>
@@ -13516,7 +13516,7 @@
         <v>1417</v>
       </c>
       <c r="I231">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="J231">
         <v>35</v>
@@ -13618,7 +13618,7 @@
         <v>1417</v>
       </c>
       <c r="I234">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="J234">
         <v>35</v>
@@ -13665,7 +13665,7 @@
         <v>1417</v>
       </c>
       <c r="I235">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="J235">
         <v>35</v>
@@ -13712,7 +13712,7 @@
         <v>1417</v>
       </c>
       <c r="I236">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="J236">
         <v>86</v>
@@ -13829,7 +13829,7 @@
         <v>1417</v>
       </c>
       <c r="I239">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="K239" t="s">
         <v>1394</v>
@@ -13928,7 +13928,7 @@
         <v>1417</v>
       </c>
       <c r="I242">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="K242" t="s">
         <v>1420</v>
@@ -13995,7 +13995,7 @@
         <v>1417</v>
       </c>
       <c r="I244">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="J244">
         <v>15</v>
@@ -14036,7 +14036,7 @@
         <v>1417</v>
       </c>
       <c r="I245">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="J245">
         <v>15</v>
@@ -14179,7 +14179,7 @@
         <v>1417</v>
       </c>
       <c r="I249">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="K249" t="s">
         <v>1421</v>
@@ -14313,7 +14313,7 @@
         <v>1417</v>
       </c>
       <c r="I253">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="J253">
         <v>162</v>
@@ -14357,7 +14357,7 @@
         <v>1417</v>
       </c>
       <c r="I254">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="K254" t="s">
         <v>1424</v>
@@ -14436,7 +14436,7 @@
         <v>1417</v>
       </c>
       <c r="I256">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="J256">
         <v>23</v>
@@ -14620,7 +14620,7 @@
         <v>1417</v>
       </c>
       <c r="I261">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="J261">
         <v>162</v>
@@ -14778,7 +14778,7 @@
         <v>1417</v>
       </c>
       <c r="I265">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="J265">
         <v>162</v>
@@ -14863,7 +14863,7 @@
         <v>1417</v>
       </c>
       <c r="I267">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="K267" t="s">
         <v>1424</v>
@@ -14901,7 +14901,7 @@
         <v>1417</v>
       </c>
       <c r="I268">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="K268" t="s">
         <v>1421</v>
@@ -14936,7 +14936,7 @@
         <v>1417</v>
       </c>
       <c r="I269">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="K269" t="s">
         <v>1421</v>
@@ -14974,7 +14974,7 @@
         <v>1417</v>
       </c>
       <c r="I270">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="K270" t="s">
         <v>1424</v>
@@ -15012,7 +15012,7 @@
         <v>1417</v>
       </c>
       <c r="I271">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="K271" t="s">
         <v>1424</v>
@@ -15190,7 +15190,7 @@
         <v>1417</v>
       </c>
       <c r="I276">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="K276" t="s">
         <v>1425</v>
@@ -15228,7 +15228,7 @@
         <v>1417</v>
       </c>
       <c r="I277">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="K277" t="s">
         <v>1421</v>
@@ -15266,7 +15266,7 @@
         <v>1417</v>
       </c>
       <c r="I278">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="J278">
         <v>148</v>
@@ -15310,7 +15310,7 @@
         <v>1417</v>
       </c>
       <c r="I279">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="K279" t="s">
         <v>1423</v>
@@ -15351,7 +15351,7 @@
         <v>1417</v>
       </c>
       <c r="I280">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="K280" t="s">
         <v>1421</v>
@@ -15389,7 +15389,7 @@
         <v>1417</v>
       </c>
       <c r="I281">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="K281" t="s">
         <v>1421</v>
@@ -15430,7 +15430,7 @@
         <v>1417</v>
       </c>
       <c r="I282">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="K282" t="s">
         <v>1421</v>
@@ -15724,7 +15724,7 @@
         <v>1417</v>
       </c>
       <c r="I291">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="J291">
         <v>20</v>
@@ -15768,7 +15768,7 @@
         <v>1417</v>
       </c>
       <c r="I292">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="K292" t="s">
         <v>1424</v>
@@ -15806,7 +15806,7 @@
         <v>1417</v>
       </c>
       <c r="I293">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="K293" t="s">
         <v>1425</v>
@@ -15844,7 +15844,7 @@
         <v>1417</v>
       </c>
       <c r="I294">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="K294" t="s">
         <v>1430</v>
@@ -15981,7 +15981,7 @@
         <v>1417</v>
       </c>
       <c r="I298">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="J298">
         <v>58</v>
@@ -16145,7 +16145,7 @@
         <v>1417</v>
       </c>
       <c r="I302">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="K302" t="s">
         <v>1424</v>
@@ -16183,7 +16183,7 @@
         <v>1417</v>
       </c>
       <c r="I303">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="K303" t="s">
         <v>1421</v>
@@ -16221,7 +16221,7 @@
         <v>1417</v>
       </c>
       <c r="I304">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="K304" t="s">
         <v>1424</v>
@@ -16259,7 +16259,7 @@
         <v>1417</v>
       </c>
       <c r="I305">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="J305">
         <v>35</v>
@@ -16303,7 +16303,7 @@
         <v>1417</v>
       </c>
       <c r="I306">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="J306">
         <v>31</v>
@@ -16391,7 +16391,7 @@
         <v>1417</v>
       </c>
       <c r="I308">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="K308" t="s">
         <v>1420</v>
@@ -16508,7 +16508,7 @@
         <v>1417</v>
       </c>
       <c r="I311">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="K311" t="s">
         <v>1420</v>
@@ -16838,7 +16838,7 @@
         <v>1417</v>
       </c>
       <c r="I320">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="K320" t="s">
         <v>1425</v>
@@ -16876,7 +16876,7 @@
         <v>1417</v>
       </c>
       <c r="I321">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="K321" t="s">
         <v>1421</v>
@@ -16914,7 +16914,7 @@
         <v>1417</v>
       </c>
       <c r="I322">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="J322">
         <v>57</v>
@@ -17028,7 +17028,7 @@
         <v>1417</v>
       </c>
       <c r="I325">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="J325">
         <v>57</v>
@@ -17110,7 +17110,7 @@
         <v>1417</v>
       </c>
       <c r="I327">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="J327">
         <v>57</v>
@@ -17154,7 +17154,7 @@
         <v>1417</v>
       </c>
       <c r="I328">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="J328">
         <v>57</v>
@@ -17198,7 +17198,7 @@
         <v>1417</v>
       </c>
       <c r="I329">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="J329">
         <v>57</v>
@@ -17242,7 +17242,7 @@
         <v>1417</v>
       </c>
       <c r="I330">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="J330">
         <v>57</v>
@@ -17286,7 +17286,7 @@
         <v>1417</v>
       </c>
       <c r="I331">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="K331" t="s">
         <v>1420</v>
@@ -17324,7 +17324,7 @@
         <v>1417</v>
       </c>
       <c r="I332">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="K332" t="s">
         <v>1421</v>
@@ -17362,7 +17362,7 @@
         <v>1417</v>
       </c>
       <c r="I333">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="J333">
         <v>100</v>
@@ -17406,7 +17406,7 @@
         <v>1417</v>
       </c>
       <c r="I334">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="K334" t="s">
         <v>1421</v>
@@ -17631,7 +17631,7 @@
         <v>1417</v>
       </c>
       <c r="I340">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="J340">
         <v>98</v>
@@ -17672,7 +17672,7 @@
         <v>1417</v>
       </c>
       <c r="I341">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="J341">
         <v>90</v>
@@ -17713,7 +17713,7 @@
         <v>1417</v>
       </c>
       <c r="I342">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="K342" t="s">
         <v>1420</v>
@@ -17827,7 +17827,7 @@
         <v>1417</v>
       </c>
       <c r="I345">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="K345" t="s">
         <v>1420</v>
@@ -17947,7 +17947,7 @@
         <v>1417</v>
       </c>
       <c r="I348">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="J348">
         <v>14</v>
@@ -17991,7 +17991,7 @@
         <v>1417</v>
       </c>
       <c r="I349">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="K349" t="s">
         <v>1425</v>
@@ -18029,7 +18029,7 @@
         <v>1417</v>
       </c>
       <c r="I350">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="J350">
         <v>46</v>
@@ -18067,7 +18067,7 @@
         <v>1417</v>
       </c>
       <c r="I351">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="J351">
         <v>82</v>
@@ -18111,7 +18111,7 @@
         <v>1417</v>
       </c>
       <c r="I352">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="J352">
         <v>78</v>
@@ -18155,7 +18155,7 @@
         <v>1417</v>
       </c>
       <c r="I353">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="J353">
         <v>83</v>
@@ -18199,7 +18199,7 @@
         <v>1417</v>
       </c>
       <c r="I354">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="K354" t="s">
         <v>1424</v>
@@ -18237,7 +18237,7 @@
         <v>1417</v>
       </c>
       <c r="I355">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="J355">
         <v>8</v>
@@ -18319,7 +18319,7 @@
         <v>1417</v>
       </c>
       <c r="I357">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="J357">
         <v>85</v>
@@ -18442,7 +18442,7 @@
         <v>1417</v>
       </c>
       <c r="I360">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="J360">
         <v>83</v>
@@ -18489,7 +18489,7 @@
         <v>1417</v>
       </c>
       <c r="I361">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="J361">
         <v>83</v>
@@ -18533,7 +18533,7 @@
         <v>1417</v>
       </c>
       <c r="I362">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="K362" t="s">
         <v>1424</v>
@@ -18571,7 +18571,7 @@
         <v>1417</v>
       </c>
       <c r="I363">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="K363" t="s">
         <v>1424</v>
@@ -18609,7 +18609,7 @@
         <v>1417</v>
       </c>
       <c r="I364">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="J364">
         <v>83</v>
@@ -18653,7 +18653,7 @@
         <v>1417</v>
       </c>
       <c r="I365">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="J365">
         <v>15</v>
@@ -18776,7 +18776,7 @@
         <v>1417</v>
       </c>
       <c r="I368">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="J368">
         <v>77</v>
@@ -18820,7 +18820,7 @@
         <v>1417</v>
       </c>
       <c r="I369">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="K369" t="s">
         <v>1424</v>
@@ -18858,7 +18858,7 @@
         <v>1417</v>
       </c>
       <c r="I370">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="K370" t="s">
         <v>1424</v>
@@ -18896,7 +18896,7 @@
         <v>1417</v>
       </c>
       <c r="I371">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="J371">
         <v>16</v>
@@ -18984,7 +18984,7 @@
         <v>1417</v>
       </c>
       <c r="I373">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="K373" t="s">
         <v>1420</v>
@@ -19022,7 +19022,7 @@
         <v>1417</v>
       </c>
       <c r="I374">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="K374" t="s">
         <v>1420</v>
@@ -19060,7 +19060,7 @@
         <v>1417</v>
       </c>
       <c r="I375">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="J375">
         <v>94</v>
@@ -19101,7 +19101,7 @@
         <v>1417</v>
       </c>
       <c r="I376">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="K376" t="s">
         <v>1424</v>
@@ -19180,7 +19180,7 @@
         <v>1417</v>
       </c>
       <c r="I378">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="K378" t="s">
         <v>1424</v>
@@ -19218,7 +19218,7 @@
         <v>1417</v>
       </c>
       <c r="I379">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="J379">
         <v>20</v>
@@ -19262,7 +19262,7 @@
         <v>1417</v>
       </c>
       <c r="I380">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="J380">
         <v>94</v>
@@ -19306,7 +19306,7 @@
         <v>1417</v>
       </c>
       <c r="I381">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="K381" t="s">
         <v>1424</v>
@@ -19344,7 +19344,7 @@
         <v>1417</v>
       </c>
       <c r="I382">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="K382" t="s">
         <v>1424</v>
@@ -19382,7 +19382,7 @@
         <v>1417</v>
       </c>
       <c r="I383">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="J383">
         <v>71</v>
@@ -19426,7 +19426,7 @@
         <v>1417</v>
       </c>
       <c r="I384">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="K384" t="s">
         <v>1421</v>
@@ -19508,7 +19508,7 @@
         <v>1417</v>
       </c>
       <c r="I386">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="K386" t="s">
         <v>1424</v>
@@ -19546,7 +19546,7 @@
         <v>1417</v>
       </c>
       <c r="I387">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="K387" t="s">
         <v>1424</v>
@@ -19584,7 +19584,7 @@
         <v>1417</v>
       </c>
       <c r="I388">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="J388">
         <v>-85</v>
@@ -19628,7 +19628,7 @@
         <v>1417</v>
       </c>
       <c r="I389">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="K389" t="s">
         <v>1425</v>
@@ -20079,7 +20079,7 @@
         <v>1417</v>
       </c>
       <c r="I400">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="K400" t="s">
         <v>1424</v>
@@ -20155,7 +20155,7 @@
         <v>1417</v>
       </c>
       <c r="I402">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="K402" t="s">
         <v>1424</v>
@@ -20193,7 +20193,7 @@
         <v>1417</v>
       </c>
       <c r="I403">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="J403">
         <v>83</v>
@@ -20237,7 +20237,7 @@
         <v>1417</v>
       </c>
       <c r="I404">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="K404" t="s">
         <v>1424</v>
@@ -20307,7 +20307,7 @@
         <v>1417</v>
       </c>
       <c r="I406">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="Q406" t="b">
         <v>1</v>
@@ -20339,7 +20339,7 @@
         <v>1417</v>
       </c>
       <c r="I407">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="Q407" t="b">
         <v>1</v>
@@ -20371,7 +20371,7 @@
         <v>1417</v>
       </c>
       <c r="I408">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="Q408" t="b">
         <v>1</v>
@@ -20403,7 +20403,7 @@
         <v>1417</v>
       </c>
       <c r="I409">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="Q409" t="b">
         <v>1</v>
@@ -20435,7 +20435,7 @@
         <v>1417</v>
       </c>
       <c r="I410">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="Q410" t="b">
         <v>1</v>
@@ -20467,7 +20467,7 @@
         <v>1417</v>
       </c>
       <c r="I411">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="Q411" t="b">
         <v>1</v>
@@ -20499,7 +20499,7 @@
         <v>1417</v>
       </c>
       <c r="I412">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="Q412" t="b">
         <v>1</v>
@@ -20531,7 +20531,7 @@
         <v>1417</v>
       </c>
       <c r="I413">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="Q413" t="b">
         <v>1</v>
@@ -20621,7 +20621,7 @@
         <v>1417</v>
       </c>
       <c r="I416">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="Q416" t="b">
         <v>1</v>
@@ -20711,7 +20711,7 @@
         <v>1417</v>
       </c>
       <c r="I419">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="Q419" t="b">
         <v>1</v>
@@ -20743,7 +20743,7 @@
         <v>1417</v>
       </c>
       <c r="I420">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="Q420" t="b">
         <v>1</v>
@@ -20775,7 +20775,7 @@
         <v>1417</v>
       </c>
       <c r="I421">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="Q421" t="b">
         <v>1</v>
@@ -20807,7 +20807,7 @@
         <v>1417</v>
       </c>
       <c r="I422">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="Q422" t="b">
         <v>1</v>
@@ -20839,7 +20839,7 @@
         <v>1417</v>
       </c>
       <c r="I423">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="Q423" t="b">
         <v>1</v>
@@ -20871,7 +20871,7 @@
         <v>1417</v>
       </c>
       <c r="I424">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="Q424" t="b">
         <v>1</v>
@@ -20903,7 +20903,7 @@
         <v>1417</v>
       </c>
       <c r="I425">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="Q425" t="b">
         <v>1</v>
@@ -20935,7 +20935,7 @@
         <v>1417</v>
       </c>
       <c r="I426">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="Q426" t="b">
         <v>1</v>
@@ -20967,7 +20967,7 @@
         <v>1417</v>
       </c>
       <c r="I427">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="Q427" t="b">
         <v>1</v>
@@ -21057,7 +21057,7 @@
         <v>1417</v>
       </c>
       <c r="I430">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="Q430" t="b">
         <v>1</v>
@@ -21089,7 +21089,7 @@
         <v>1417</v>
       </c>
       <c r="I431">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="Q431" t="b">
         <v>1</v>
@@ -21121,7 +21121,7 @@
         <v>1417</v>
       </c>
       <c r="I432">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="Q432" t="b">
         <v>1</v>
@@ -21153,7 +21153,7 @@
         <v>1417</v>
       </c>
       <c r="I433">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="Q433" t="b">
         <v>1</v>
@@ -21185,7 +21185,7 @@
         <v>1417</v>
       </c>
       <c r="I434">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="Q434" t="b">
         <v>1</v>
@@ -21217,7 +21217,7 @@
         <v>1417</v>
       </c>
       <c r="I435">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="Q435" t="b">
         <v>1</v>
@@ -21249,7 +21249,7 @@
         <v>1417</v>
       </c>
       <c r="I436">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="Q436" t="b">
         <v>1</v>
@@ -21281,7 +21281,7 @@
         <v>1419</v>
       </c>
       <c r="I437">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="Q437" t="b">
         <v>1</v>
@@ -21313,7 +21313,7 @@
         <v>1419</v>
       </c>
       <c r="I438">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="Q438" t="b">
         <v>1</v>
@@ -21345,7 +21345,7 @@
         <v>1417</v>
       </c>
       <c r="I439">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="Q439" t="b">
         <v>1</v>
@@ -21377,7 +21377,7 @@
         <v>1417</v>
       </c>
       <c r="I440">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="Q440" t="b">
         <v>1</v>
@@ -21409,7 +21409,7 @@
         <v>1417</v>
       </c>
       <c r="I441">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="Q441" t="b">
         <v>1</v>
@@ -21470,7 +21470,7 @@
         <v>1417</v>
       </c>
       <c r="I443">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="Q443" t="b">
         <v>1</v>
@@ -21560,7 +21560,7 @@
         <v>1417</v>
       </c>
       <c r="I446">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q446" t="b">
         <v>1</v>
@@ -21592,7 +21592,7 @@
         <v>1417</v>
       </c>
       <c r="I447">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q447" t="b">
         <v>1</v>
@@ -21624,7 +21624,7 @@
         <v>1417</v>
       </c>
       <c r="I448">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Q448" t="b">
         <v>1</v>
@@ -21656,7 +21656,7 @@
         <v>1417</v>
       </c>
       <c r="I449">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Q449" t="b">
         <v>1</v>
@@ -21688,7 +21688,7 @@
         <v>1417</v>
       </c>
       <c r="I450">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Q450" t="b">
         <v>1</v>
@@ -21720,7 +21720,7 @@
         <v>1417</v>
       </c>
       <c r="I451">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="Q451" t="b">
         <v>1</v>
@@ -21781,7 +21781,7 @@
         <v>1417</v>
       </c>
       <c r="I453">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="Q453" t="b">
         <v>1</v>
@@ -21813,7 +21813,7 @@
         <v>1417</v>
       </c>
       <c r="I454">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="Q454" t="b">
         <v>1</v>
@@ -21845,7 +21845,7 @@
         <v>1417</v>
       </c>
       <c r="I455">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="Q455" t="b">
         <v>1</v>
@@ -21906,7 +21906,7 @@
         <v>1417</v>
       </c>
       <c r="I457">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="Q457" t="b">
         <v>1</v>
@@ -21938,7 +21938,7 @@
         <v>1417</v>
       </c>
       <c r="I458">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q458" t="b">
         <v>1</v>
@@ -21970,7 +21970,7 @@
         <v>1417</v>
       </c>
       <c r="I459">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="Q459" t="b">
         <v>1</v>
@@ -22002,7 +22002,7 @@
         <v>1417</v>
       </c>
       <c r="I460">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="Q460" t="b">
         <v>1</v>
@@ -22034,7 +22034,7 @@
         <v>1417</v>
       </c>
       <c r="I461">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="Q461" t="b">
         <v>1</v>
@@ -22066,7 +22066,7 @@
         <v>1417</v>
       </c>
       <c r="I462">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="Q462" t="b">
         <v>1</v>
@@ -22098,7 +22098,7 @@
         <v>1417</v>
       </c>
       <c r="I463">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Q463" t="b">
         <v>1</v>
@@ -22130,7 +22130,7 @@
         <v>1417</v>
       </c>
       <c r="I464">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="Q464" t="b">
         <v>1</v>
@@ -22162,7 +22162,7 @@
         <v>1417</v>
       </c>
       <c r="I465">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="Q465" t="b">
         <v>1</v>
@@ -22194,7 +22194,7 @@
         <v>1417</v>
       </c>
       <c r="I466">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="Q466" t="b">
         <v>1</v>
@@ -22226,7 +22226,7 @@
         <v>1417</v>
       </c>
       <c r="I467">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="Q467" t="b">
         <v>1</v>
@@ -22258,7 +22258,7 @@
         <v>1417</v>
       </c>
       <c r="I468">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="Q468" t="b">
         <v>1</v>
@@ -22290,7 +22290,7 @@
         <v>1417</v>
       </c>
       <c r="I469">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="Q469" t="b">
         <v>1</v>
@@ -22351,7 +22351,7 @@
         <v>1417</v>
       </c>
       <c r="I471">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="Q471" t="b">
         <v>1</v>
@@ -22383,7 +22383,7 @@
         <v>1417</v>
       </c>
       <c r="I472">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="Q472" t="b">
         <v>1</v>
@@ -22415,7 +22415,7 @@
         <v>1417</v>
       </c>
       <c r="I473">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="Q473" t="b">
         <v>1</v>
@@ -22447,7 +22447,7 @@
         <v>1417</v>
       </c>
       <c r="I474">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q474" t="b">
         <v>1</v>
@@ -22479,7 +22479,7 @@
         <v>1417</v>
       </c>
       <c r="I475">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q475" t="b">
         <v>1</v>
@@ -22511,7 +22511,7 @@
         <v>1417</v>
       </c>
       <c r="I476">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q476" t="b">
         <v>1</v>
@@ -22543,7 +22543,7 @@
         <v>1417</v>
       </c>
       <c r="I477">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q477" t="b">
         <v>1</v>
@@ -22575,7 +22575,7 @@
         <v>1417</v>
       </c>
       <c r="I478">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q478" t="b">
         <v>1</v>
@@ -22607,7 +22607,7 @@
         <v>1417</v>
       </c>
       <c r="I479">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q479" t="b">
         <v>1</v>
@@ -22639,7 +22639,7 @@
         <v>1417</v>
       </c>
       <c r="I480">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q480" t="b">
         <v>1</v>
@@ -22671,7 +22671,7 @@
         <v>1417</v>
       </c>
       <c r="I481">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q481" t="b">
         <v>1</v>
@@ -22703,7 +22703,7 @@
         <v>1417</v>
       </c>
       <c r="I482">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q482" t="b">
         <v>1</v>
@@ -22735,7 +22735,7 @@
         <v>1417</v>
       </c>
       <c r="I483">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q483" t="b">
         <v>1</v>
@@ -22767,7 +22767,7 @@
         <v>1417</v>
       </c>
       <c r="I484">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q484" t="b">
         <v>1</v>
@@ -22799,7 +22799,7 @@
         <v>1417</v>
       </c>
       <c r="I485">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q485" t="b">
         <v>1</v>
@@ -22831,7 +22831,7 @@
         <v>1417</v>
       </c>
       <c r="I486">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q486" t="b">
         <v>1</v>
@@ -22863,7 +22863,7 @@
         <v>1417</v>
       </c>
       <c r="I487">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q487" t="b">
         <v>1</v>
@@ -22895,7 +22895,7 @@
         <v>1417</v>
       </c>
       <c r="I488">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q488" t="b">
         <v>1</v>
@@ -22927,7 +22927,7 @@
         <v>1417</v>
       </c>
       <c r="I489">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q489" t="b">
         <v>1</v>
@@ -22959,7 +22959,7 @@
         <v>1417</v>
       </c>
       <c r="I490">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q490" t="b">
         <v>1</v>
@@ -22991,7 +22991,7 @@
         <v>1417</v>
       </c>
       <c r="I491">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q491" t="b">
         <v>1</v>
@@ -23023,7 +23023,7 @@
         <v>1419</v>
       </c>
       <c r="I492">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q492" t="b">
         <v>1</v>
@@ -23055,7 +23055,7 @@
         <v>1419</v>
       </c>
       <c r="I493">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q493" t="b">
         <v>1</v>
@@ -23087,7 +23087,7 @@
         <v>1419</v>
       </c>
       <c r="I494">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q494" t="b">
         <v>1</v>
@@ -23119,7 +23119,7 @@
         <v>1419</v>
       </c>
       <c r="I495">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q495" t="b">
         <v>1</v>
@@ -23151,7 +23151,7 @@
         <v>1419</v>
       </c>
       <c r="I496">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q496" t="b">
         <v>1</v>
@@ -23183,7 +23183,7 @@
         <v>1417</v>
       </c>
       <c r="I497">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q497" t="b">
         <v>1</v>
@@ -23215,7 +23215,7 @@
         <v>1417</v>
       </c>
       <c r="I498">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q498" t="b">
         <v>1</v>
@@ -23247,7 +23247,7 @@
         <v>1419</v>
       </c>
       <c r="I499">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q499" t="b">
         <v>1</v>
@@ -23279,7 +23279,7 @@
         <v>1417</v>
       </c>
       <c r="I500">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q500" t="b">
         <v>1</v>
@@ -23311,7 +23311,7 @@
         <v>1417</v>
       </c>
       <c r="I501">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q501" t="b">
         <v>1</v>
@@ -23343,7 +23343,7 @@
         <v>1417</v>
       </c>
       <c r="I502">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q502" t="b">
         <v>1</v>
@@ -23375,7 +23375,7 @@
         <v>1417</v>
       </c>
       <c r="I503">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q503" t="b">
         <v>1</v>
@@ -23407,7 +23407,7 @@
         <v>1417</v>
       </c>
       <c r="I504">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="Q504" t="b">
         <v>1</v>
@@ -23439,7 +23439,7 @@
         <v>1417</v>
       </c>
       <c r="I505">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="Q505" t="b">
         <v>1</v>
@@ -23471,7 +23471,7 @@
         <v>1417</v>
       </c>
       <c r="I506">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="Q506" t="b">
         <v>1</v>
@@ -23503,7 +23503,7 @@
         <v>1417</v>
       </c>
       <c r="I507">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="Q507" t="b">
         <v>1</v>
@@ -23564,7 +23564,7 @@
         <v>1417</v>
       </c>
       <c r="I509">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="Q509" t="b">
         <v>1</v>
@@ -23596,7 +23596,7 @@
         <v>1417</v>
       </c>
       <c r="I510">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="Q510" t="b">
         <v>1</v>
@@ -23628,7 +23628,7 @@
         <v>1417</v>
       </c>
       <c r="I511">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="Q511" t="b">
         <v>1</v>
@@ -23660,7 +23660,7 @@
         <v>1417</v>
       </c>
       <c r="I512">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="Q512" t="b">
         <v>1</v>
@@ -23692,7 +23692,7 @@
         <v>1417</v>
       </c>
       <c r="I513">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="Q513" t="b">
         <v>1</v>
@@ -23753,7 +23753,7 @@
         <v>1417</v>
       </c>
       <c r="I515">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="Q515" t="b">
         <v>1</v>
@@ -23785,7 +23785,7 @@
         <v>1417</v>
       </c>
       <c r="I516">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Q516" t="b">
         <v>1</v>
@@ -23817,7 +23817,7 @@
         <v>1417</v>
       </c>
       <c r="I517">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Q517" t="b">
         <v>1</v>
@@ -23849,7 +23849,7 @@
         <v>1417</v>
       </c>
       <c r="I518">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Q518" t="b">
         <v>1</v>
@@ -23881,7 +23881,7 @@
         <v>1417</v>
       </c>
       <c r="I519">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q519" t="b">
         <v>1</v>
@@ -23913,7 +23913,7 @@
         <v>1417</v>
       </c>
       <c r="I520">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q520" t="b">
         <v>1</v>
@@ -23945,7 +23945,7 @@
         <v>1417</v>
       </c>
       <c r="I521">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q521" t="b">
         <v>1</v>
@@ -23977,7 +23977,7 @@
         <v>1417</v>
       </c>
       <c r="I522">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q522" t="b">
         <v>1</v>
@@ -24009,7 +24009,7 @@
         <v>1417</v>
       </c>
       <c r="I523">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q523" t="b">
         <v>1</v>
@@ -24041,7 +24041,7 @@
         <v>1417</v>
       </c>
       <c r="I524">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="Q524" t="b">
         <v>1</v>
@@ -24073,7 +24073,7 @@
         <v>1417</v>
       </c>
       <c r="I525">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="Q525" t="b">
         <v>1</v>
@@ -24105,7 +24105,7 @@
         <v>1417</v>
       </c>
       <c r="I526">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="Q526" t="b">
         <v>1</v>
@@ -24137,7 +24137,7 @@
         <v>1417</v>
       </c>
       <c r="I527">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="Q527" t="b">
         <v>1</v>
@@ -24169,7 +24169,7 @@
         <v>1417</v>
       </c>
       <c r="I528">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q528" t="b">
         <v>1</v>
@@ -24201,7 +24201,7 @@
         <v>1417</v>
       </c>
       <c r="I529">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="Q529" t="b">
         <v>1</v>
@@ -24233,7 +24233,7 @@
         <v>1417</v>
       </c>
       <c r="I530">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="Q530" t="b">
         <v>1</v>
@@ -24265,7 +24265,7 @@
         <v>1417</v>
       </c>
       <c r="I531">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="Q531" t="b">
         <v>1</v>
@@ -24297,7 +24297,7 @@
         <v>1417</v>
       </c>
       <c r="I532">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="Q532" t="b">
         <v>1</v>
@@ -24329,7 +24329,7 @@
         <v>1417</v>
       </c>
       <c r="I533">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="Q533" t="b">
         <v>1</v>
@@ -24361,7 +24361,7 @@
         <v>1417</v>
       </c>
       <c r="I534">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="Q534" t="b">
         <v>1</v>
@@ -24393,7 +24393,7 @@
         <v>1417</v>
       </c>
       <c r="I535">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="Q535" t="b">
         <v>1</v>
@@ -24425,7 +24425,7 @@
         <v>1417</v>
       </c>
       <c r="I536">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="Q536" t="b">
         <v>1</v>
@@ -24457,7 +24457,7 @@
         <v>1417</v>
       </c>
       <c r="I537">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="Q537" t="b">
         <v>1</v>
@@ -24489,7 +24489,7 @@
         <v>1417</v>
       </c>
       <c r="I538">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="Q538" t="b">
         <v>1</v>
@@ -24521,7 +24521,7 @@
         <v>1417</v>
       </c>
       <c r="I539">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="Q539" t="b">
         <v>1</v>
@@ -24553,7 +24553,7 @@
         <v>1417</v>
       </c>
       <c r="I540">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="Q540" t="b">
         <v>1</v>
@@ -24585,7 +24585,7 @@
         <v>1417</v>
       </c>
       <c r="I541">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="Q541" t="b">
         <v>1</v>
@@ -24617,7 +24617,7 @@
         <v>1417</v>
       </c>
       <c r="I542">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="Q542" t="b">
         <v>1</v>
@@ -24649,7 +24649,7 @@
         <v>1417</v>
       </c>
       <c r="I543">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="Q543" t="b">
         <v>1</v>
@@ -24681,7 +24681,7 @@
         <v>1417</v>
       </c>
       <c r="I544">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="Q544" t="b">
         <v>1</v>
@@ -24713,7 +24713,7 @@
         <v>1417</v>
       </c>
       <c r="I545">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="Q545" t="b">
         <v>1</v>
@@ -24745,7 +24745,7 @@
         <v>1417</v>
       </c>
       <c r="I546">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="Q546" t="b">
         <v>1</v>
@@ -24777,7 +24777,7 @@
         <v>1417</v>
       </c>
       <c r="I547">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="Q547" t="b">
         <v>1</v>
@@ -24809,7 +24809,7 @@
         <v>1417</v>
       </c>
       <c r="I548">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="Q548" t="b">
         <v>1</v>
@@ -24841,7 +24841,7 @@
         <v>1417</v>
       </c>
       <c r="I549">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="Q549" t="b">
         <v>1</v>
@@ -24873,7 +24873,7 @@
         <v>1417</v>
       </c>
       <c r="I550">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="Q550" t="b">
         <v>1</v>
@@ -24905,7 +24905,7 @@
         <v>1417</v>
       </c>
       <c r="I551">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="Q551" t="b">
         <v>1</v>
@@ -24937,7 +24937,7 @@
         <v>1417</v>
       </c>
       <c r="I552">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="Q552" t="b">
         <v>1</v>
@@ -24969,7 +24969,7 @@
         <v>1417</v>
       </c>
       <c r="I553">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="Q553" t="b">
         <v>1</v>
@@ -25001,7 +25001,7 @@
         <v>1417</v>
       </c>
       <c r="I554">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="Q554" t="b">
         <v>1</v>
@@ -25033,7 +25033,7 @@
         <v>1417</v>
       </c>
       <c r="I555">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="Q555" t="b">
         <v>1</v>
@@ -25065,7 +25065,7 @@
         <v>1417</v>
       </c>
       <c r="I556">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="Q556" t="b">
         <v>1</v>
@@ -25097,7 +25097,7 @@
         <v>1417</v>
       </c>
       <c r="I557">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="Q557" t="b">
         <v>1</v>
@@ -25129,7 +25129,7 @@
         <v>1417</v>
       </c>
       <c r="I558">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="Q558" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: reparaveis (12/10/2026 17:16)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
@@ -5132,7 +5132,7 @@
         <v>1417</v>
       </c>
       <c r="I2">
-        <v>606</v>
+        <v>609</v>
       </c>
       <c r="K2" t="s">
         <v>1420</v>
@@ -5170,7 +5170,7 @@
         <v>1417</v>
       </c>
       <c r="I3">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="K3" t="s">
         <v>1421</v>
@@ -5208,7 +5208,7 @@
         <v>1417</v>
       </c>
       <c r="I4">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="K4" t="s">
         <v>1421</v>
@@ -5246,7 +5246,7 @@
         <v>1417</v>
       </c>
       <c r="I5">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="J5">
         <v>279</v>
@@ -5290,7 +5290,7 @@
         <v>1417</v>
       </c>
       <c r="I6">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="J6">
         <v>153</v>
@@ -5334,7 +5334,7 @@
         <v>1417</v>
       </c>
       <c r="I7">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="J7">
         <v>112</v>
@@ -5410,7 +5410,7 @@
         <v>1417</v>
       </c>
       <c r="I9">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="J9">
         <v>362</v>
@@ -5457,7 +5457,7 @@
         <v>1417</v>
       </c>
       <c r="I10">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="J10">
         <v>378</v>
@@ -5504,7 +5504,7 @@
         <v>1417</v>
       </c>
       <c r="I11">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="J11">
         <v>112</v>
@@ -5551,7 +5551,7 @@
         <v>1417</v>
       </c>
       <c r="I12">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="J12">
         <v>124</v>
@@ -5624,7 +5624,7 @@
         <v>1417</v>
       </c>
       <c r="I14">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="J14">
         <v>64</v>
@@ -5703,7 +5703,7 @@
         <v>1417</v>
       </c>
       <c r="I16">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="K16" t="s">
         <v>1420</v>
@@ -5741,7 +5741,7 @@
         <v>1417</v>
       </c>
       <c r="I17">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="J17">
         <v>161</v>
@@ -5785,7 +5785,7 @@
         <v>1417</v>
       </c>
       <c r="I18">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="J18">
         <v>66</v>
@@ -5858,7 +5858,7 @@
         <v>1417</v>
       </c>
       <c r="I20">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="J20">
         <v>399</v>
@@ -5931,7 +5931,7 @@
         <v>1417</v>
       </c>
       <c r="I22">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="K22" t="s">
         <v>1424</v>
@@ -5969,7 +5969,7 @@
         <v>1417</v>
       </c>
       <c r="I23">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="J23">
         <v>229</v>
@@ -6074,7 +6074,7 @@
         <v>1417</v>
       </c>
       <c r="I26">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="J26">
         <v>155</v>
@@ -6121,7 +6121,7 @@
         <v>1417</v>
       </c>
       <c r="I27">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="K27" t="s">
         <v>1424</v>
@@ -6217,7 +6217,7 @@
         <v>1417</v>
       </c>
       <c r="I30">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="J30">
         <v>209</v>
@@ -6290,7 +6290,7 @@
         <v>1417</v>
       </c>
       <c r="I32">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="K32" t="s">
         <v>1420</v>
@@ -6499,7 +6499,7 @@
         <v>1417</v>
       </c>
       <c r="I39">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="K39" t="s">
         <v>1425</v>
@@ -6662,7 +6662,7 @@
         <v>1417</v>
       </c>
       <c r="I44">
-        <v>535</v>
+        <v>538</v>
       </c>
       <c r="J44">
         <v>87</v>
@@ -6709,7 +6709,7 @@
         <v>1417</v>
       </c>
       <c r="I45">
-        <v>535</v>
+        <v>538</v>
       </c>
       <c r="J45">
         <v>331</v>
@@ -6756,7 +6756,7 @@
         <v>1417</v>
       </c>
       <c r="I46">
-        <v>535</v>
+        <v>538</v>
       </c>
       <c r="K46" t="s">
         <v>1424</v>
@@ -6797,7 +6797,7 @@
         <v>1417</v>
       </c>
       <c r="I47">
-        <v>535</v>
+        <v>538</v>
       </c>
       <c r="J47">
         <v>344</v>
@@ -6844,7 +6844,7 @@
         <v>1417</v>
       </c>
       <c r="I48">
-        <v>535</v>
+        <v>538</v>
       </c>
       <c r="K48" t="s">
         <v>1424</v>
@@ -6911,7 +6911,7 @@
         <v>1417</v>
       </c>
       <c r="I50">
-        <v>535</v>
+        <v>538</v>
       </c>
       <c r="K50" t="s">
         <v>1424</v>
@@ -6978,7 +6978,7 @@
         <v>1417</v>
       </c>
       <c r="I52">
-        <v>535</v>
+        <v>538</v>
       </c>
       <c r="K52" t="s">
         <v>1420</v>
@@ -7016,7 +7016,7 @@
         <v>1417</v>
       </c>
       <c r="I53">
-        <v>535</v>
+        <v>538</v>
       </c>
       <c r="K53" t="s">
         <v>1421</v>
@@ -7054,7 +7054,7 @@
         <v>1417</v>
       </c>
       <c r="I54">
-        <v>535</v>
+        <v>538</v>
       </c>
       <c r="K54" t="s">
         <v>1421</v>
@@ -7330,7 +7330,7 @@
         <v>1417</v>
       </c>
       <c r="I63">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="J63">
         <v>293</v>
@@ -7377,7 +7377,7 @@
         <v>1417</v>
       </c>
       <c r="I64">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="J64">
         <v>320</v>
@@ -7607,7 +7607,7 @@
         <v>1417</v>
       </c>
       <c r="I71">
-        <v>501</v>
+        <v>504</v>
       </c>
       <c r="J71">
         <v>429</v>
@@ -7680,7 +7680,7 @@
         <v>1417</v>
       </c>
       <c r="I73">
-        <v>501</v>
+        <v>504</v>
       </c>
       <c r="K73" t="s">
         <v>1420</v>
@@ -7788,7 +7788,7 @@
         <v>1417</v>
       </c>
       <c r="I76">
-        <v>501</v>
+        <v>504</v>
       </c>
       <c r="K76" t="s">
         <v>1427</v>
@@ -7881,7 +7881,7 @@
         <v>1417</v>
       </c>
       <c r="I79">
-        <v>501</v>
+        <v>504</v>
       </c>
       <c r="K79" t="s">
         <v>1427</v>
@@ -7986,7 +7986,7 @@
         <v>1417</v>
       </c>
       <c r="I82">
-        <v>491</v>
+        <v>494</v>
       </c>
       <c r="K82" t="s">
         <v>1424</v>
@@ -8053,7 +8053,7 @@
         <v>1417</v>
       </c>
       <c r="I84">
-        <v>491</v>
+        <v>494</v>
       </c>
       <c r="J84">
         <v>40</v>
@@ -8100,7 +8100,7 @@
         <v>1417</v>
       </c>
       <c r="I85">
-        <v>491</v>
+        <v>494</v>
       </c>
       <c r="K85" t="s">
         <v>1421</v>
@@ -8138,7 +8138,7 @@
         <v>1417</v>
       </c>
       <c r="I86">
-        <v>491</v>
+        <v>494</v>
       </c>
       <c r="K86" t="s">
         <v>1421</v>
@@ -8176,7 +8176,7 @@
         <v>1417</v>
       </c>
       <c r="I87">
-        <v>491</v>
+        <v>494</v>
       </c>
       <c r="J87">
         <v>-16</v>
@@ -8299,7 +8299,7 @@
         <v>1417</v>
       </c>
       <c r="I90">
-        <v>473</v>
+        <v>476</v>
       </c>
       <c r="K90" t="s">
         <v>1394</v>
@@ -8448,7 +8448,7 @@
         <v>1417</v>
       </c>
       <c r="I94">
-        <v>473</v>
+        <v>476</v>
       </c>
       <c r="K94" t="s">
         <v>1424</v>
@@ -8527,7 +8527,7 @@
         <v>1417</v>
       </c>
       <c r="I96">
-        <v>473</v>
+        <v>476</v>
       </c>
       <c r="J96">
         <v>17</v>
@@ -8574,7 +8574,7 @@
         <v>1417</v>
       </c>
       <c r="I97">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="J97">
         <v>20</v>
@@ -8621,7 +8621,7 @@
         <v>1417</v>
       </c>
       <c r="I98">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="K98" t="s">
         <v>1424</v>
@@ -8898,7 +8898,7 @@
         <v>1417</v>
       </c>
       <c r="I106">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="J106">
         <v>49</v>
@@ -8942,7 +8942,7 @@
         <v>1417</v>
       </c>
       <c r="I107">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="J107">
         <v>36</v>
@@ -8986,7 +8986,7 @@
         <v>1417</v>
       </c>
       <c r="I108">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="K108" t="s">
         <v>1421</v>
@@ -9024,7 +9024,7 @@
         <v>1417</v>
       </c>
       <c r="I109">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="K109" t="s">
         <v>1421</v>
@@ -9207,7 +9207,7 @@
         <v>1417</v>
       </c>
       <c r="I115">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="K115" t="s">
         <v>1421</v>
@@ -9245,7 +9245,7 @@
         <v>1417</v>
       </c>
       <c r="I116">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="K116" t="s">
         <v>1421</v>
@@ -9283,7 +9283,7 @@
         <v>1417</v>
       </c>
       <c r="I117">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="K117" t="s">
         <v>1421</v>
@@ -9321,7 +9321,7 @@
         <v>1417</v>
       </c>
       <c r="I118">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="K118" t="s">
         <v>1421</v>
@@ -9359,7 +9359,7 @@
         <v>1417</v>
       </c>
       <c r="I119">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="K119" t="s">
         <v>1421</v>
@@ -9397,7 +9397,7 @@
         <v>1417</v>
       </c>
       <c r="I120">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="K120" t="s">
         <v>1421</v>
@@ -9435,7 +9435,7 @@
         <v>1417</v>
       </c>
       <c r="I121">
-        <v>455</v>
+        <v>458</v>
       </c>
       <c r="J121">
         <v>251</v>
@@ -9482,7 +9482,7 @@
         <v>1417</v>
       </c>
       <c r="I122">
-        <v>455</v>
+        <v>458</v>
       </c>
       <c r="K122" t="s">
         <v>1421</v>
@@ -9549,7 +9549,7 @@
         <v>1417</v>
       </c>
       <c r="I124">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="K124" t="s">
         <v>1421</v>
@@ -9587,7 +9587,7 @@
         <v>1417</v>
       </c>
       <c r="I125">
-        <v>449</v>
+        <v>452</v>
       </c>
       <c r="K125" t="s">
         <v>1427</v>
@@ -9683,7 +9683,7 @@
         <v>1417</v>
       </c>
       <c r="I128">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="K128" t="s">
         <v>1421</v>
@@ -9721,7 +9721,7 @@
         <v>1417</v>
       </c>
       <c r="I129">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="K129" t="s">
         <v>1420</v>
@@ -9759,7 +9759,7 @@
         <v>1417</v>
       </c>
       <c r="I130">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="J130">
         <v>47</v>
@@ -9835,7 +9835,7 @@
         <v>1417</v>
       </c>
       <c r="I132">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="J132">
         <v>145</v>
@@ -9911,7 +9911,7 @@
         <v>1417</v>
       </c>
       <c r="I134">
-        <v>422</v>
+        <v>425</v>
       </c>
       <c r="K134" t="s">
         <v>1420</v>
@@ -10036,7 +10036,7 @@
         <v>1417</v>
       </c>
       <c r="I138">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="K138" t="s">
         <v>1421</v>
@@ -10420,7 +10420,7 @@
         <v>1417</v>
       </c>
       <c r="I150">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="J150">
         <v>201</v>
@@ -10607,7 +10607,7 @@
         <v>1417</v>
       </c>
       <c r="I155">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="K155" t="s">
         <v>1427</v>
@@ -10642,7 +10642,7 @@
         <v>1417</v>
       </c>
       <c r="I156">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="K156" t="s">
         <v>1421</v>
@@ -10680,7 +10680,7 @@
         <v>1417</v>
       </c>
       <c r="I157">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="J157">
         <v>371</v>
@@ -10724,7 +10724,7 @@
         <v>1417</v>
       </c>
       <c r="I158">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="J158">
         <v>52</v>
@@ -10768,7 +10768,7 @@
         <v>1417</v>
       </c>
       <c r="I159">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="K159" t="s">
         <v>1421</v>
@@ -10806,7 +10806,7 @@
         <v>1417</v>
       </c>
       <c r="I160">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="K160" t="s">
         <v>1421</v>
@@ -10844,7 +10844,7 @@
         <v>1417</v>
       </c>
       <c r="I161">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="J161">
         <v>55</v>
@@ -10979,7 +10979,7 @@
         <v>1417</v>
       </c>
       <c r="I164">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="O164" t="s">
         <v>1533</v>
@@ -11154,7 +11154,7 @@
         <v>1417</v>
       </c>
       <c r="I169">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="K169" t="s">
         <v>1394</v>
@@ -11364,7 +11364,7 @@
         <v>1417</v>
       </c>
       <c r="I175">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="J175">
         <v>205</v>
@@ -11411,7 +11411,7 @@
         <v>1417</v>
       </c>
       <c r="I176">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="K176" t="s">
         <v>1421</v>
@@ -11449,7 +11449,7 @@
         <v>1417</v>
       </c>
       <c r="I177">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="J177">
         <v>44</v>
@@ -11496,7 +11496,7 @@
         <v>1417</v>
       </c>
       <c r="I178">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="K178" t="s">
         <v>1420</v>
@@ -11563,7 +11563,7 @@
         <v>1417</v>
       </c>
       <c r="I180">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="K180" t="s">
         <v>1420</v>
@@ -11659,7 +11659,7 @@
         <v>1417</v>
       </c>
       <c r="I183">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="K183" t="s">
         <v>1421</v>
@@ -11697,7 +11697,7 @@
         <v>1417</v>
       </c>
       <c r="I184">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="K184" t="s">
         <v>1427</v>
@@ -11732,7 +11732,7 @@
         <v>1417</v>
       </c>
       <c r="I185">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="K185" t="s">
         <v>1421</v>
@@ -11770,7 +11770,7 @@
         <v>1417</v>
       </c>
       <c r="I186">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="K186" t="s">
         <v>1421</v>
@@ -11808,7 +11808,7 @@
         <v>1417</v>
       </c>
       <c r="I187">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="J187">
         <v>75</v>
@@ -11855,7 +11855,7 @@
         <v>1417</v>
       </c>
       <c r="I188">
-        <v>358</v>
+        <v>361</v>
       </c>
       <c r="J188">
         <v>40</v>
@@ -11902,7 +11902,7 @@
         <v>1417</v>
       </c>
       <c r="I189">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="J189">
         <v>155</v>
@@ -11946,7 +11946,7 @@
         <v>1417</v>
       </c>
       <c r="I190">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="J190">
         <v>107</v>
@@ -11990,7 +11990,7 @@
         <v>1417</v>
       </c>
       <c r="I191">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="J191">
         <v>5</v>
@@ -12034,7 +12034,7 @@
         <v>1417</v>
       </c>
       <c r="I192">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="K192" t="s">
         <v>1421</v>
@@ -12072,7 +12072,7 @@
         <v>1417</v>
       </c>
       <c r="I193">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="K193" t="s">
         <v>1426</v>
@@ -12267,7 +12267,7 @@
         <v>1417</v>
       </c>
       <c r="I199">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="J199">
         <v>70</v>
@@ -12352,7 +12352,7 @@
         <v>1417</v>
       </c>
       <c r="I201">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="K201" t="s">
         <v>1421</v>
@@ -12390,7 +12390,7 @@
         <v>1417</v>
       </c>
       <c r="I202">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="K202" t="s">
         <v>1421</v>
@@ -12469,7 +12469,7 @@
         <v>1417</v>
       </c>
       <c r="I204">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="K204" t="s">
         <v>1420</v>
@@ -12507,7 +12507,7 @@
         <v>1417</v>
       </c>
       <c r="I205">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="K205" t="s">
         <v>1420</v>
@@ -12574,7 +12574,7 @@
         <v>1417</v>
       </c>
       <c r="I207">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="J207">
         <v>167</v>
@@ -12618,7 +12618,7 @@
         <v>1417</v>
       </c>
       <c r="I208">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="J208">
         <v>45</v>
@@ -12662,7 +12662,7 @@
         <v>1417</v>
       </c>
       <c r="I209">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="J209">
         <v>191</v>
@@ -12706,7 +12706,7 @@
         <v>1417</v>
       </c>
       <c r="I210">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="K210" t="s">
         <v>1424</v>
@@ -12802,7 +12802,7 @@
         <v>1417</v>
       </c>
       <c r="I213">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="K213" t="s">
         <v>1421</v>
@@ -12840,7 +12840,7 @@
         <v>1417</v>
       </c>
       <c r="I214">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="J214">
         <v>14</v>
@@ -12887,7 +12887,7 @@
         <v>1417</v>
       </c>
       <c r="I215">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="K215" t="s">
         <v>1421</v>
@@ -12954,7 +12954,7 @@
         <v>1417</v>
       </c>
       <c r="I217">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="J217">
         <v>42</v>
@@ -12998,7 +12998,7 @@
         <v>1417</v>
       </c>
       <c r="I218">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="J218">
         <v>166</v>
@@ -13086,7 +13086,7 @@
         <v>1417</v>
       </c>
       <c r="I220">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="J220">
         <v>154</v>
@@ -13472,7 +13472,7 @@
         <v>1417</v>
       </c>
       <c r="I230">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="J230">
         <v>197</v>
@@ -13516,7 +13516,7 @@
         <v>1417</v>
       </c>
       <c r="I231">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="J231">
         <v>35</v>
@@ -13618,7 +13618,7 @@
         <v>1417</v>
       </c>
       <c r="I234">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="J234">
         <v>35</v>
@@ -13665,7 +13665,7 @@
         <v>1417</v>
       </c>
       <c r="I235">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="J235">
         <v>35</v>
@@ -13712,7 +13712,7 @@
         <v>1417</v>
       </c>
       <c r="I236">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="J236">
         <v>86</v>
@@ -13829,7 +13829,7 @@
         <v>1417</v>
       </c>
       <c r="I239">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="K239" t="s">
         <v>1394</v>
@@ -13928,7 +13928,7 @@
         <v>1417</v>
       </c>
       <c r="I242">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="K242" t="s">
         <v>1420</v>
@@ -13995,7 +13995,7 @@
         <v>1417</v>
       </c>
       <c r="I244">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="J244">
         <v>15</v>
@@ -14036,7 +14036,7 @@
         <v>1417</v>
       </c>
       <c r="I245">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="J245">
         <v>15</v>
@@ -14179,7 +14179,7 @@
         <v>1417</v>
       </c>
       <c r="I249">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="K249" t="s">
         <v>1421</v>
@@ -14313,7 +14313,7 @@
         <v>1417</v>
       </c>
       <c r="I253">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="J253">
         <v>162</v>
@@ -14357,7 +14357,7 @@
         <v>1417</v>
       </c>
       <c r="I254">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="K254" t="s">
         <v>1424</v>
@@ -14436,7 +14436,7 @@
         <v>1417</v>
       </c>
       <c r="I256">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="J256">
         <v>23</v>
@@ -14620,7 +14620,7 @@
         <v>1417</v>
       </c>
       <c r="I261">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="J261">
         <v>162</v>
@@ -14778,7 +14778,7 @@
         <v>1417</v>
       </c>
       <c r="I265">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="J265">
         <v>162</v>
@@ -14863,7 +14863,7 @@
         <v>1417</v>
       </c>
       <c r="I267">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="K267" t="s">
         <v>1424</v>
@@ -14901,7 +14901,7 @@
         <v>1417</v>
       </c>
       <c r="I268">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="K268" t="s">
         <v>1421</v>
@@ -14936,7 +14936,7 @@
         <v>1417</v>
       </c>
       <c r="I269">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="K269" t="s">
         <v>1421</v>
@@ -14974,7 +14974,7 @@
         <v>1417</v>
       </c>
       <c r="I270">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="K270" t="s">
         <v>1424</v>
@@ -15012,7 +15012,7 @@
         <v>1417</v>
       </c>
       <c r="I271">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="K271" t="s">
         <v>1424</v>
@@ -15190,7 +15190,7 @@
         <v>1417</v>
       </c>
       <c r="I276">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="K276" t="s">
         <v>1425</v>
@@ -15228,7 +15228,7 @@
         <v>1417</v>
       </c>
       <c r="I277">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="K277" t="s">
         <v>1421</v>
@@ -15266,7 +15266,7 @@
         <v>1417</v>
       </c>
       <c r="I278">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="J278">
         <v>148</v>
@@ -15310,7 +15310,7 @@
         <v>1417</v>
       </c>
       <c r="I279">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="K279" t="s">
         <v>1423</v>
@@ -15351,7 +15351,7 @@
         <v>1417</v>
       </c>
       <c r="I280">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="K280" t="s">
         <v>1421</v>
@@ -15389,7 +15389,7 @@
         <v>1417</v>
       </c>
       <c r="I281">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="K281" t="s">
         <v>1421</v>
@@ -15430,7 +15430,7 @@
         <v>1417</v>
       </c>
       <c r="I282">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="K282" t="s">
         <v>1421</v>
@@ -15724,7 +15724,7 @@
         <v>1417</v>
       </c>
       <c r="I291">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="J291">
         <v>20</v>
@@ -15768,7 +15768,7 @@
         <v>1417</v>
       </c>
       <c r="I292">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="K292" t="s">
         <v>1424</v>
@@ -15806,7 +15806,7 @@
         <v>1417</v>
       </c>
       <c r="I293">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="K293" t="s">
         <v>1425</v>
@@ -15844,7 +15844,7 @@
         <v>1417</v>
       </c>
       <c r="I294">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="K294" t="s">
         <v>1430</v>
@@ -15981,7 +15981,7 @@
         <v>1417</v>
       </c>
       <c r="I298">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="J298">
         <v>58</v>
@@ -16145,7 +16145,7 @@
         <v>1417</v>
       </c>
       <c r="I302">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="K302" t="s">
         <v>1424</v>
@@ -16183,7 +16183,7 @@
         <v>1417</v>
       </c>
       <c r="I303">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="K303" t="s">
         <v>1421</v>
@@ -16221,7 +16221,7 @@
         <v>1417</v>
       </c>
       <c r="I304">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="K304" t="s">
         <v>1424</v>
@@ -16259,7 +16259,7 @@
         <v>1417</v>
       </c>
       <c r="I305">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="J305">
         <v>35</v>
@@ -16303,7 +16303,7 @@
         <v>1417</v>
       </c>
       <c r="I306">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="J306">
         <v>31</v>
@@ -16391,7 +16391,7 @@
         <v>1417</v>
       </c>
       <c r="I308">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="K308" t="s">
         <v>1420</v>
@@ -16508,7 +16508,7 @@
         <v>1417</v>
       </c>
       <c r="I311">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="K311" t="s">
         <v>1420</v>
@@ -16838,7 +16838,7 @@
         <v>1417</v>
       </c>
       <c r="I320">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="K320" t="s">
         <v>1425</v>
@@ -16876,7 +16876,7 @@
         <v>1417</v>
       </c>
       <c r="I321">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="K321" t="s">
         <v>1421</v>
@@ -16914,7 +16914,7 @@
         <v>1417</v>
       </c>
       <c r="I322">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="J322">
         <v>57</v>
@@ -17028,7 +17028,7 @@
         <v>1417</v>
       </c>
       <c r="I325">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="J325">
         <v>57</v>
@@ -17110,7 +17110,7 @@
         <v>1417</v>
       </c>
       <c r="I327">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="J327">
         <v>57</v>
@@ -17154,7 +17154,7 @@
         <v>1417</v>
       </c>
       <c r="I328">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="J328">
         <v>57</v>
@@ -17198,7 +17198,7 @@
         <v>1417</v>
       </c>
       <c r="I329">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="J329">
         <v>57</v>
@@ -17242,7 +17242,7 @@
         <v>1417</v>
       </c>
       <c r="I330">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="J330">
         <v>57</v>
@@ -17286,7 +17286,7 @@
         <v>1417</v>
       </c>
       <c r="I331">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="K331" t="s">
         <v>1420</v>
@@ -17324,7 +17324,7 @@
         <v>1417</v>
       </c>
       <c r="I332">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="K332" t="s">
         <v>1421</v>
@@ -17362,7 +17362,7 @@
         <v>1417</v>
       </c>
       <c r="I333">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="J333">
         <v>100</v>
@@ -17406,7 +17406,7 @@
         <v>1417</v>
       </c>
       <c r="I334">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="K334" t="s">
         <v>1421</v>
@@ -17631,7 +17631,7 @@
         <v>1417</v>
       </c>
       <c r="I340">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="J340">
         <v>98</v>
@@ -17672,7 +17672,7 @@
         <v>1417</v>
       </c>
       <c r="I341">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="J341">
         <v>90</v>
@@ -17713,7 +17713,7 @@
         <v>1417</v>
       </c>
       <c r="I342">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="K342" t="s">
         <v>1420</v>
@@ -17827,7 +17827,7 @@
         <v>1417</v>
       </c>
       <c r="I345">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="K345" t="s">
         <v>1420</v>
@@ -17947,7 +17947,7 @@
         <v>1417</v>
       </c>
       <c r="I348">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="J348">
         <v>14</v>
@@ -17991,7 +17991,7 @@
         <v>1417</v>
       </c>
       <c r="I349">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="K349" t="s">
         <v>1425</v>
@@ -18029,7 +18029,7 @@
         <v>1417</v>
       </c>
       <c r="I350">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="J350">
         <v>46</v>
@@ -18067,7 +18067,7 @@
         <v>1417</v>
       </c>
       <c r="I351">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="J351">
         <v>82</v>
@@ -18111,7 +18111,7 @@
         <v>1417</v>
       </c>
       <c r="I352">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="J352">
         <v>78</v>
@@ -18155,7 +18155,7 @@
         <v>1417</v>
       </c>
       <c r="I353">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="J353">
         <v>83</v>
@@ -18199,7 +18199,7 @@
         <v>1417</v>
       </c>
       <c r="I354">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="K354" t="s">
         <v>1424</v>
@@ -18237,7 +18237,7 @@
         <v>1417</v>
       </c>
       <c r="I355">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="J355">
         <v>8</v>
@@ -18319,7 +18319,7 @@
         <v>1417</v>
       </c>
       <c r="I357">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="J357">
         <v>85</v>
@@ -18442,7 +18442,7 @@
         <v>1417</v>
       </c>
       <c r="I360">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="J360">
         <v>83</v>
@@ -18489,7 +18489,7 @@
         <v>1417</v>
       </c>
       <c r="I361">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="J361">
         <v>83</v>
@@ -18533,7 +18533,7 @@
         <v>1417</v>
       </c>
       <c r="I362">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="K362" t="s">
         <v>1424</v>
@@ -18571,7 +18571,7 @@
         <v>1417</v>
       </c>
       <c r="I363">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="K363" t="s">
         <v>1424</v>
@@ -18609,7 +18609,7 @@
         <v>1417</v>
       </c>
       <c r="I364">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="J364">
         <v>83</v>
@@ -18653,7 +18653,7 @@
         <v>1417</v>
       </c>
       <c r="I365">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="J365">
         <v>15</v>
@@ -18776,7 +18776,7 @@
         <v>1417</v>
       </c>
       <c r="I368">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="J368">
         <v>77</v>
@@ -18820,7 +18820,7 @@
         <v>1417</v>
       </c>
       <c r="I369">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="K369" t="s">
         <v>1424</v>
@@ -18858,7 +18858,7 @@
         <v>1417</v>
       </c>
       <c r="I370">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="K370" t="s">
         <v>1424</v>
@@ -18896,7 +18896,7 @@
         <v>1417</v>
       </c>
       <c r="I371">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="J371">
         <v>16</v>
@@ -18984,7 +18984,7 @@
         <v>1417</v>
       </c>
       <c r="I373">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="K373" t="s">
         <v>1420</v>
@@ -19022,7 +19022,7 @@
         <v>1417</v>
       </c>
       <c r="I374">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="K374" t="s">
         <v>1420</v>
@@ -19060,7 +19060,7 @@
         <v>1417</v>
       </c>
       <c r="I375">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="J375">
         <v>94</v>
@@ -19101,7 +19101,7 @@
         <v>1417</v>
       </c>
       <c r="I376">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="K376" t="s">
         <v>1424</v>
@@ -19180,7 +19180,7 @@
         <v>1417</v>
       </c>
       <c r="I378">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="K378" t="s">
         <v>1424</v>
@@ -19218,7 +19218,7 @@
         <v>1417</v>
       </c>
       <c r="I379">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="J379">
         <v>20</v>
@@ -19262,7 +19262,7 @@
         <v>1417</v>
       </c>
       <c r="I380">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="J380">
         <v>94</v>
@@ -19306,7 +19306,7 @@
         <v>1417</v>
       </c>
       <c r="I381">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="K381" t="s">
         <v>1424</v>
@@ -19344,7 +19344,7 @@
         <v>1417</v>
       </c>
       <c r="I382">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="K382" t="s">
         <v>1424</v>
@@ -19382,7 +19382,7 @@
         <v>1417</v>
       </c>
       <c r="I383">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="J383">
         <v>71</v>
@@ -19426,7 +19426,7 @@
         <v>1417</v>
       </c>
       <c r="I384">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="K384" t="s">
         <v>1421</v>
@@ -19508,7 +19508,7 @@
         <v>1417</v>
       </c>
       <c r="I386">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="K386" t="s">
         <v>1424</v>
@@ -19546,7 +19546,7 @@
         <v>1417</v>
       </c>
       <c r="I387">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="K387" t="s">
         <v>1424</v>
@@ -19584,7 +19584,7 @@
         <v>1417</v>
       </c>
       <c r="I388">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="J388">
         <v>-85</v>
@@ -19628,7 +19628,7 @@
         <v>1417</v>
       </c>
       <c r="I389">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="K389" t="s">
         <v>1425</v>
@@ -20079,7 +20079,7 @@
         <v>1417</v>
       </c>
       <c r="I400">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="K400" t="s">
         <v>1424</v>
@@ -20155,7 +20155,7 @@
         <v>1417</v>
       </c>
       <c r="I402">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="K402" t="s">
         <v>1424</v>
@@ -20193,7 +20193,7 @@
         <v>1417</v>
       </c>
       <c r="I403">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="J403">
         <v>83</v>
@@ -20237,7 +20237,7 @@
         <v>1417</v>
       </c>
       <c r="I404">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="K404" t="s">
         <v>1424</v>
@@ -20307,7 +20307,7 @@
         <v>1417</v>
       </c>
       <c r="I406">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="Q406" t="b">
         <v>1</v>
@@ -20339,7 +20339,7 @@
         <v>1417</v>
       </c>
       <c r="I407">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="Q407" t="b">
         <v>1</v>
@@ -20371,7 +20371,7 @@
         <v>1417</v>
       </c>
       <c r="I408">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="Q408" t="b">
         <v>1</v>
@@ -20403,7 +20403,7 @@
         <v>1417</v>
       </c>
       <c r="I409">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="Q409" t="b">
         <v>1</v>
@@ -20435,7 +20435,7 @@
         <v>1417</v>
       </c>
       <c r="I410">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="Q410" t="b">
         <v>1</v>
@@ -20467,7 +20467,7 @@
         <v>1417</v>
       </c>
       <c r="I411">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="Q411" t="b">
         <v>1</v>
@@ -20499,7 +20499,7 @@
         <v>1417</v>
       </c>
       <c r="I412">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="Q412" t="b">
         <v>1</v>
@@ -20531,7 +20531,7 @@
         <v>1417</v>
       </c>
       <c r="I413">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="Q413" t="b">
         <v>1</v>
@@ -20621,7 +20621,7 @@
         <v>1417</v>
       </c>
       <c r="I416">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="Q416" t="b">
         <v>1</v>
@@ -20711,7 +20711,7 @@
         <v>1417</v>
       </c>
       <c r="I419">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="Q419" t="b">
         <v>1</v>
@@ -20743,7 +20743,7 @@
         <v>1417</v>
       </c>
       <c r="I420">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="Q420" t="b">
         <v>1</v>
@@ -20775,7 +20775,7 @@
         <v>1417</v>
       </c>
       <c r="I421">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="Q421" t="b">
         <v>1</v>
@@ -20807,7 +20807,7 @@
         <v>1417</v>
       </c>
       <c r="I422">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="Q422" t="b">
         <v>1</v>
@@ -20839,7 +20839,7 @@
         <v>1417</v>
       </c>
       <c r="I423">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="Q423" t="b">
         <v>1</v>
@@ -20871,7 +20871,7 @@
         <v>1417</v>
       </c>
       <c r="I424">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="Q424" t="b">
         <v>1</v>
@@ -20903,7 +20903,7 @@
         <v>1417</v>
       </c>
       <c r="I425">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="Q425" t="b">
         <v>1</v>
@@ -20935,7 +20935,7 @@
         <v>1417</v>
       </c>
       <c r="I426">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="Q426" t="b">
         <v>1</v>
@@ -20967,7 +20967,7 @@
         <v>1417</v>
       </c>
       <c r="I427">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="Q427" t="b">
         <v>1</v>
@@ -21057,7 +21057,7 @@
         <v>1417</v>
       </c>
       <c r="I430">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="Q430" t="b">
         <v>1</v>
@@ -21089,7 +21089,7 @@
         <v>1417</v>
       </c>
       <c r="I431">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="Q431" t="b">
         <v>1</v>
@@ -21121,7 +21121,7 @@
         <v>1417</v>
       </c>
       <c r="I432">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="Q432" t="b">
         <v>1</v>
@@ -21153,7 +21153,7 @@
         <v>1417</v>
       </c>
       <c r="I433">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="Q433" t="b">
         <v>1</v>
@@ -21185,7 +21185,7 @@
         <v>1417</v>
       </c>
       <c r="I434">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="Q434" t="b">
         <v>1</v>
@@ -21217,7 +21217,7 @@
         <v>1417</v>
       </c>
       <c r="I435">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="Q435" t="b">
         <v>1</v>
@@ -21249,7 +21249,7 @@
         <v>1417</v>
       </c>
       <c r="I436">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="Q436" t="b">
         <v>1</v>
@@ -21281,7 +21281,7 @@
         <v>1419</v>
       </c>
       <c r="I437">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="Q437" t="b">
         <v>1</v>
@@ -21313,7 +21313,7 @@
         <v>1419</v>
       </c>
       <c r="I438">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="Q438" t="b">
         <v>1</v>
@@ -21345,7 +21345,7 @@
         <v>1417</v>
       </c>
       <c r="I439">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="Q439" t="b">
         <v>1</v>
@@ -21377,7 +21377,7 @@
         <v>1417</v>
       </c>
       <c r="I440">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="Q440" t="b">
         <v>1</v>
@@ -21409,7 +21409,7 @@
         <v>1417</v>
       </c>
       <c r="I441">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="Q441" t="b">
         <v>1</v>
@@ -21470,7 +21470,7 @@
         <v>1417</v>
       </c>
       <c r="I443">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="Q443" t="b">
         <v>1</v>
@@ -21560,7 +21560,7 @@
         <v>1417</v>
       </c>
       <c r="I446">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="Q446" t="b">
         <v>1</v>
@@ -21592,7 +21592,7 @@
         <v>1417</v>
       </c>
       <c r="I447">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="Q447" t="b">
         <v>1</v>
@@ -21624,7 +21624,7 @@
         <v>1417</v>
       </c>
       <c r="I448">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="Q448" t="b">
         <v>1</v>
@@ -21656,7 +21656,7 @@
         <v>1417</v>
       </c>
       <c r="I449">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="Q449" t="b">
         <v>1</v>
@@ -21688,7 +21688,7 @@
         <v>1417</v>
       </c>
       <c r="I450">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="Q450" t="b">
         <v>1</v>
@@ -21720,7 +21720,7 @@
         <v>1417</v>
       </c>
       <c r="I451">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="Q451" t="b">
         <v>1</v>
@@ -21781,7 +21781,7 @@
         <v>1417</v>
       </c>
       <c r="I453">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="Q453" t="b">
         <v>1</v>
@@ -21813,7 +21813,7 @@
         <v>1417</v>
       </c>
       <c r="I454">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="Q454" t="b">
         <v>1</v>
@@ -21845,7 +21845,7 @@
         <v>1417</v>
       </c>
       <c r="I455">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="Q455" t="b">
         <v>1</v>
@@ -21906,7 +21906,7 @@
         <v>1417</v>
       </c>
       <c r="I457">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="Q457" t="b">
         <v>1</v>
@@ -21938,7 +21938,7 @@
         <v>1417</v>
       </c>
       <c r="I458">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="Q458" t="b">
         <v>1</v>
@@ -21970,7 +21970,7 @@
         <v>1417</v>
       </c>
       <c r="I459">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="Q459" t="b">
         <v>1</v>
@@ -22002,7 +22002,7 @@
         <v>1417</v>
       </c>
       <c r="I460">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="Q460" t="b">
         <v>1</v>
@@ -22034,7 +22034,7 @@
         <v>1417</v>
       </c>
       <c r="I461">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="Q461" t="b">
         <v>1</v>
@@ -22066,7 +22066,7 @@
         <v>1417</v>
       </c>
       <c r="I462">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="Q462" t="b">
         <v>1</v>
@@ -22098,7 +22098,7 @@
         <v>1417</v>
       </c>
       <c r="I463">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="Q463" t="b">
         <v>1</v>
@@ -22130,7 +22130,7 @@
         <v>1417</v>
       </c>
       <c r="I464">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="Q464" t="b">
         <v>1</v>
@@ -22162,7 +22162,7 @@
         <v>1417</v>
       </c>
       <c r="I465">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="Q465" t="b">
         <v>1</v>
@@ -22194,7 +22194,7 @@
         <v>1417</v>
       </c>
       <c r="I466">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="Q466" t="b">
         <v>1</v>
@@ -22226,7 +22226,7 @@
         <v>1417</v>
       </c>
       <c r="I467">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="Q467" t="b">
         <v>1</v>
@@ -22258,7 +22258,7 @@
         <v>1417</v>
       </c>
       <c r="I468">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="Q468" t="b">
         <v>1</v>
@@ -22290,7 +22290,7 @@
         <v>1417</v>
       </c>
       <c r="I469">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="Q469" t="b">
         <v>1</v>
@@ -22351,7 +22351,7 @@
         <v>1417</v>
       </c>
       <c r="I471">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="Q471" t="b">
         <v>1</v>
@@ -22383,7 +22383,7 @@
         <v>1417</v>
       </c>
       <c r="I472">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="Q472" t="b">
         <v>1</v>
@@ -22415,7 +22415,7 @@
         <v>1417</v>
       </c>
       <c r="I473">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="Q473" t="b">
         <v>1</v>
@@ -22447,7 +22447,7 @@
         <v>1417</v>
       </c>
       <c r="I474">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="Q474" t="b">
         <v>1</v>
@@ -22479,7 +22479,7 @@
         <v>1417</v>
       </c>
       <c r="I475">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="Q475" t="b">
         <v>1</v>
@@ -22511,7 +22511,7 @@
         <v>1417</v>
       </c>
       <c r="I476">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="Q476" t="b">
         <v>1</v>
@@ -22543,7 +22543,7 @@
         <v>1417</v>
       </c>
       <c r="I477">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="Q477" t="b">
         <v>1</v>
@@ -22575,7 +22575,7 @@
         <v>1417</v>
       </c>
       <c r="I478">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="Q478" t="b">
         <v>1</v>
@@ -22607,7 +22607,7 @@
         <v>1417</v>
       </c>
       <c r="I479">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="Q479" t="b">
         <v>1</v>
@@ -22639,7 +22639,7 @@
         <v>1417</v>
       </c>
       <c r="I480">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="Q480" t="b">
         <v>1</v>
@@ -22671,7 +22671,7 @@
         <v>1417</v>
       </c>
       <c r="I481">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="Q481" t="b">
         <v>1</v>
@@ -22703,7 +22703,7 @@
         <v>1417</v>
       </c>
       <c r="I482">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="Q482" t="b">
         <v>1</v>
@@ -22735,7 +22735,7 @@
         <v>1417</v>
       </c>
       <c r="I483">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="Q483" t="b">
         <v>1</v>
@@ -22767,7 +22767,7 @@
         <v>1417</v>
       </c>
       <c r="I484">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="Q484" t="b">
         <v>1</v>
@@ -22799,7 +22799,7 @@
         <v>1417</v>
       </c>
       <c r="I485">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="Q485" t="b">
         <v>1</v>
@@ -22831,7 +22831,7 @@
         <v>1417</v>
       </c>
       <c r="I486">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="Q486" t="b">
         <v>1</v>
@@ -22863,7 +22863,7 @@
         <v>1417</v>
       </c>
       <c r="I487">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="Q487" t="b">
         <v>1</v>
@@ -22895,7 +22895,7 @@
         <v>1417</v>
       </c>
       <c r="I488">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="Q488" t="b">
         <v>1</v>
@@ -22927,7 +22927,7 @@
         <v>1417</v>
       </c>
       <c r="I489">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="Q489" t="b">
         <v>1</v>
@@ -22959,7 +22959,7 @@
         <v>1417</v>
       </c>
       <c r="I490">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="Q490" t="b">
         <v>1</v>
@@ -22991,7 +22991,7 @@
         <v>1417</v>
       </c>
       <c r="I491">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="Q491" t="b">
         <v>1</v>
@@ -23023,7 +23023,7 @@
         <v>1419</v>
       </c>
       <c r="I492">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="Q492" t="b">
         <v>1</v>
@@ -23055,7 +23055,7 @@
         <v>1419</v>
       </c>
       <c r="I493">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="Q493" t="b">
         <v>1</v>
@@ -23087,7 +23087,7 @@
         <v>1419</v>
       </c>
       <c r="I494">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="Q494" t="b">
         <v>1</v>
@@ -23119,7 +23119,7 @@
         <v>1419</v>
       </c>
       <c r="I495">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="Q495" t="b">
         <v>1</v>
@@ -23151,7 +23151,7 @@
         <v>1419</v>
       </c>
       <c r="I496">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="Q496" t="b">
         <v>1</v>
@@ -23183,7 +23183,7 @@
         <v>1417</v>
       </c>
       <c r="I497">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="Q497" t="b">
         <v>1</v>
@@ -23215,7 +23215,7 @@
         <v>1417</v>
       </c>
       <c r="I498">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="Q498" t="b">
         <v>1</v>
@@ -23247,7 +23247,7 @@
         <v>1419</v>
       </c>
       <c r="I499">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="Q499" t="b">
         <v>1</v>
@@ -23279,7 +23279,7 @@
         <v>1417</v>
       </c>
       <c r="I500">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="Q500" t="b">
         <v>1</v>
@@ -23311,7 +23311,7 @@
         <v>1417</v>
       </c>
       <c r="I501">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="Q501" t="b">
         <v>1</v>
@@ -23343,7 +23343,7 @@
         <v>1417</v>
       </c>
       <c r="I502">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="Q502" t="b">
         <v>1</v>
@@ -23375,7 +23375,7 @@
         <v>1417</v>
       </c>
       <c r="I503">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="Q503" t="b">
         <v>1</v>
@@ -23407,7 +23407,7 @@
         <v>1417</v>
       </c>
       <c r="I504">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="Q504" t="b">
         <v>1</v>
@@ -23439,7 +23439,7 @@
         <v>1417</v>
       </c>
       <c r="I505">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="Q505" t="b">
         <v>1</v>
@@ -23471,7 +23471,7 @@
         <v>1417</v>
       </c>
       <c r="I506">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="Q506" t="b">
         <v>1</v>
@@ -23503,7 +23503,7 @@
         <v>1417</v>
       </c>
       <c r="I507">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="Q507" t="b">
         <v>1</v>
@@ -23564,7 +23564,7 @@
         <v>1417</v>
       </c>
       <c r="I509">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="Q509" t="b">
         <v>1</v>
@@ -23596,7 +23596,7 @@
         <v>1417</v>
       </c>
       <c r="I510">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="Q510" t="b">
         <v>1</v>
@@ -23628,7 +23628,7 @@
         <v>1417</v>
       </c>
       <c r="I511">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="Q511" t="b">
         <v>1</v>
@@ -23660,7 +23660,7 @@
         <v>1417</v>
       </c>
       <c r="I512">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="Q512" t="b">
         <v>1</v>
@@ -23692,7 +23692,7 @@
         <v>1417</v>
       </c>
       <c r="I513">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="Q513" t="b">
         <v>1</v>
@@ -23753,7 +23753,7 @@
         <v>1417</v>
       </c>
       <c r="I515">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="Q515" t="b">
         <v>1</v>
@@ -23785,7 +23785,7 @@
         <v>1417</v>
       </c>
       <c r="I516">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="Q516" t="b">
         <v>1</v>
@@ -23817,7 +23817,7 @@
         <v>1417</v>
       </c>
       <c r="I517">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="Q517" t="b">
         <v>1</v>
@@ -23849,7 +23849,7 @@
         <v>1417</v>
       </c>
       <c r="I518">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="Q518" t="b">
         <v>1</v>
@@ -23881,7 +23881,7 @@
         <v>1417</v>
       </c>
       <c r="I519">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="Q519" t="b">
         <v>1</v>
@@ -23913,7 +23913,7 @@
         <v>1417</v>
       </c>
       <c r="I520">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="Q520" t="b">
         <v>1</v>
@@ -23945,7 +23945,7 @@
         <v>1417</v>
       </c>
       <c r="I521">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="Q521" t="b">
         <v>1</v>
@@ -23977,7 +23977,7 @@
         <v>1417</v>
       </c>
       <c r="I522">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="Q522" t="b">
         <v>1</v>
@@ -24009,7 +24009,7 @@
         <v>1417</v>
       </c>
       <c r="I523">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="Q523" t="b">
         <v>1</v>
@@ -24041,7 +24041,7 @@
         <v>1417</v>
       </c>
       <c r="I524">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="Q524" t="b">
         <v>1</v>
@@ -24073,7 +24073,7 @@
         <v>1417</v>
       </c>
       <c r="I525">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="Q525" t="b">
         <v>1</v>
@@ -24105,7 +24105,7 @@
         <v>1417</v>
       </c>
       <c r="I526">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="Q526" t="b">
         <v>1</v>
@@ -24137,7 +24137,7 @@
         <v>1417</v>
       </c>
       <c r="I527">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="Q527" t="b">
         <v>1</v>
@@ -24169,7 +24169,7 @@
         <v>1417</v>
       </c>
       <c r="I528">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="Q528" t="b">
         <v>1</v>
@@ -24201,7 +24201,7 @@
         <v>1417</v>
       </c>
       <c r="I529">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="Q529" t="b">
         <v>1</v>
@@ -24233,7 +24233,7 @@
         <v>1417</v>
       </c>
       <c r="I530">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="Q530" t="b">
         <v>1</v>
@@ -24265,7 +24265,7 @@
         <v>1417</v>
       </c>
       <c r="I531">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="Q531" t="b">
         <v>1</v>
@@ -24297,7 +24297,7 @@
         <v>1417</v>
       </c>
       <c r="I532">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="Q532" t="b">
         <v>1</v>
@@ -24329,7 +24329,7 @@
         <v>1417</v>
       </c>
       <c r="I533">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="Q533" t="b">
         <v>1</v>
@@ -24361,7 +24361,7 @@
         <v>1417</v>
       </c>
       <c r="I534">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="Q534" t="b">
         <v>1</v>
@@ -24393,7 +24393,7 @@
         <v>1417</v>
       </c>
       <c r="I535">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="Q535" t="b">
         <v>1</v>
@@ -24425,7 +24425,7 @@
         <v>1417</v>
       </c>
       <c r="I536">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="Q536" t="b">
         <v>1</v>
@@ -24457,7 +24457,7 @@
         <v>1417</v>
       </c>
       <c r="I537">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="Q537" t="b">
         <v>1</v>
@@ -24489,7 +24489,7 @@
         <v>1417</v>
       </c>
       <c r="I538">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="Q538" t="b">
         <v>1</v>
@@ -24521,7 +24521,7 @@
         <v>1417</v>
       </c>
       <c r="I539">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="Q539" t="b">
         <v>1</v>
@@ -24553,7 +24553,7 @@
         <v>1417</v>
       </c>
       <c r="I540">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="Q540" t="b">
         <v>1</v>
@@ -24585,7 +24585,7 @@
         <v>1417</v>
       </c>
       <c r="I541">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="Q541" t="b">
         <v>1</v>
@@ -24617,7 +24617,7 @@
         <v>1417</v>
       </c>
       <c r="I542">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="Q542" t="b">
         <v>1</v>
@@ -24649,7 +24649,7 @@
         <v>1417</v>
       </c>
       <c r="I543">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="Q543" t="b">
         <v>1</v>
@@ -24681,7 +24681,7 @@
         <v>1417</v>
       </c>
       <c r="I544">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="Q544" t="b">
         <v>1</v>
@@ -24713,7 +24713,7 @@
         <v>1417</v>
       </c>
       <c r="I545">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="Q545" t="b">
         <v>1</v>
@@ -24745,7 +24745,7 @@
         <v>1417</v>
       </c>
       <c r="I546">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="Q546" t="b">
         <v>1</v>
@@ -24777,7 +24777,7 @@
         <v>1417</v>
       </c>
       <c r="I547">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="Q547" t="b">
         <v>1</v>
@@ -24809,7 +24809,7 @@
         <v>1417</v>
       </c>
       <c r="I548">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="Q548" t="b">
         <v>1</v>
@@ -24841,7 +24841,7 @@
         <v>1417</v>
       </c>
       <c r="I549">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="Q549" t="b">
         <v>1</v>
@@ -24873,7 +24873,7 @@
         <v>1417</v>
       </c>
       <c r="I550">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="Q550" t="b">
         <v>1</v>
@@ -24905,7 +24905,7 @@
         <v>1417</v>
       </c>
       <c r="I551">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="Q551" t="b">
         <v>1</v>
@@ -24937,7 +24937,7 @@
         <v>1417</v>
       </c>
       <c r="I552">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="Q552" t="b">
         <v>1</v>
@@ -24969,7 +24969,7 @@
         <v>1417</v>
       </c>
       <c r="I553">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="Q553" t="b">
         <v>1</v>
@@ -25001,7 +25001,7 @@
         <v>1417</v>
       </c>
       <c r="I554">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="Q554" t="b">
         <v>1</v>
@@ -25033,7 +25033,7 @@
         <v>1417</v>
       </c>
       <c r="I555">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="Q555" t="b">
         <v>1</v>
@@ -25065,7 +25065,7 @@
         <v>1417</v>
       </c>
       <c r="I556">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="Q556" t="b">
         <v>1</v>
@@ -25097,7 +25097,7 @@
         <v>1417</v>
       </c>
       <c r="I557">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="Q557" t="b">
         <v>1</v>
@@ -25129,7 +25129,7 @@
         <v>1417</v>
       </c>
       <c r="I558">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="Q558" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: reparaveis (14/10/2026 12:49)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
@@ -5132,7 +5132,7 @@
         <v>1417</v>
       </c>
       <c r="I2">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="K2" t="s">
         <v>1420</v>
@@ -5170,7 +5170,7 @@
         <v>1417</v>
       </c>
       <c r="I3">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="K3" t="s">
         <v>1421</v>
@@ -5208,7 +5208,7 @@
         <v>1417</v>
       </c>
       <c r="I4">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="K4" t="s">
         <v>1421</v>
@@ -5246,7 +5246,7 @@
         <v>1417</v>
       </c>
       <c r="I5">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="J5">
         <v>279</v>
@@ -5290,7 +5290,7 @@
         <v>1417</v>
       </c>
       <c r="I6">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="J6">
         <v>153</v>
@@ -5334,7 +5334,7 @@
         <v>1417</v>
       </c>
       <c r="I7">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="J7">
         <v>112</v>
@@ -5410,7 +5410,7 @@
         <v>1417</v>
       </c>
       <c r="I9">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="J9">
         <v>362</v>
@@ -5457,7 +5457,7 @@
         <v>1417</v>
       </c>
       <c r="I10">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="J10">
         <v>378</v>
@@ -5504,7 +5504,7 @@
         <v>1417</v>
       </c>
       <c r="I11">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="J11">
         <v>112</v>
@@ -5551,7 +5551,7 @@
         <v>1417</v>
       </c>
       <c r="I12">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="J12">
         <v>124</v>
@@ -5624,7 +5624,7 @@
         <v>1417</v>
       </c>
       <c r="I14">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="J14">
         <v>64</v>
@@ -5703,7 +5703,7 @@
         <v>1417</v>
       </c>
       <c r="I16">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="K16" t="s">
         <v>1420</v>
@@ -5741,7 +5741,7 @@
         <v>1417</v>
       </c>
       <c r="I17">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="J17">
         <v>161</v>
@@ -5785,7 +5785,7 @@
         <v>1417</v>
       </c>
       <c r="I18">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="J18">
         <v>66</v>
@@ -5858,7 +5858,7 @@
         <v>1417</v>
       </c>
       <c r="I20">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="J20">
         <v>399</v>
@@ -5931,7 +5931,7 @@
         <v>1417</v>
       </c>
       <c r="I22">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="K22" t="s">
         <v>1424</v>
@@ -5969,7 +5969,7 @@
         <v>1417</v>
       </c>
       <c r="I23">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="J23">
         <v>229</v>
@@ -6074,7 +6074,7 @@
         <v>1417</v>
       </c>
       <c r="I26">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="J26">
         <v>155</v>
@@ -6121,7 +6121,7 @@
         <v>1417</v>
       </c>
       <c r="I27">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="K27" t="s">
         <v>1424</v>
@@ -6217,7 +6217,7 @@
         <v>1417</v>
       </c>
       <c r="I30">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="J30">
         <v>209</v>
@@ -6290,7 +6290,7 @@
         <v>1417</v>
       </c>
       <c r="I32">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="K32" t="s">
         <v>1420</v>
@@ -6499,7 +6499,7 @@
         <v>1417</v>
       </c>
       <c r="I39">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="K39" t="s">
         <v>1425</v>
@@ -6662,7 +6662,7 @@
         <v>1417</v>
       </c>
       <c r="I44">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="J44">
         <v>87</v>
@@ -6709,7 +6709,7 @@
         <v>1417</v>
       </c>
       <c r="I45">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="J45">
         <v>331</v>
@@ -6756,7 +6756,7 @@
         <v>1417</v>
       </c>
       <c r="I46">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="K46" t="s">
         <v>1424</v>
@@ -6797,7 +6797,7 @@
         <v>1417</v>
       </c>
       <c r="I47">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="J47">
         <v>344</v>
@@ -6844,7 +6844,7 @@
         <v>1417</v>
       </c>
       <c r="I48">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="K48" t="s">
         <v>1424</v>
@@ -6911,7 +6911,7 @@
         <v>1417</v>
       </c>
       <c r="I50">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="K50" t="s">
         <v>1424</v>
@@ -6978,7 +6978,7 @@
         <v>1417</v>
       </c>
       <c r="I52">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="K52" t="s">
         <v>1420</v>
@@ -7016,7 +7016,7 @@
         <v>1417</v>
       </c>
       <c r="I53">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="K53" t="s">
         <v>1421</v>
@@ -7054,7 +7054,7 @@
         <v>1417</v>
       </c>
       <c r="I54">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="K54" t="s">
         <v>1421</v>
@@ -7330,7 +7330,7 @@
         <v>1417</v>
       </c>
       <c r="I63">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="J63">
         <v>293</v>
@@ -7377,7 +7377,7 @@
         <v>1417</v>
       </c>
       <c r="I64">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="J64">
         <v>320</v>
@@ -7607,7 +7607,7 @@
         <v>1417</v>
       </c>
       <c r="I71">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="J71">
         <v>429</v>
@@ -7680,7 +7680,7 @@
         <v>1417</v>
       </c>
       <c r="I73">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="K73" t="s">
         <v>1420</v>
@@ -7788,7 +7788,7 @@
         <v>1417</v>
       </c>
       <c r="I76">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="K76" t="s">
         <v>1427</v>
@@ -7881,7 +7881,7 @@
         <v>1417</v>
       </c>
       <c r="I79">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="K79" t="s">
         <v>1427</v>
@@ -7986,7 +7986,7 @@
         <v>1417</v>
       </c>
       <c r="I82">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="K82" t="s">
         <v>1424</v>
@@ -8053,7 +8053,7 @@
         <v>1417</v>
       </c>
       <c r="I84">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="J84">
         <v>40</v>
@@ -8100,7 +8100,7 @@
         <v>1417</v>
       </c>
       <c r="I85">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="K85" t="s">
         <v>1421</v>
@@ -8138,7 +8138,7 @@
         <v>1417</v>
       </c>
       <c r="I86">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="K86" t="s">
         <v>1421</v>
@@ -8176,7 +8176,7 @@
         <v>1417</v>
       </c>
       <c r="I87">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="J87">
         <v>-16</v>
@@ -8299,7 +8299,7 @@
         <v>1417</v>
       </c>
       <c r="I90">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="K90" t="s">
         <v>1394</v>
@@ -8448,7 +8448,7 @@
         <v>1417</v>
       </c>
       <c r="I94">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="K94" t="s">
         <v>1424</v>
@@ -8527,7 +8527,7 @@
         <v>1417</v>
       </c>
       <c r="I96">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="J96">
         <v>17</v>
@@ -8574,7 +8574,7 @@
         <v>1417</v>
       </c>
       <c r="I97">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="J97">
         <v>20</v>
@@ -8621,7 +8621,7 @@
         <v>1417</v>
       </c>
       <c r="I98">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="K98" t="s">
         <v>1424</v>
@@ -8898,7 +8898,7 @@
         <v>1417</v>
       </c>
       <c r="I106">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="J106">
         <v>49</v>
@@ -8942,7 +8942,7 @@
         <v>1417</v>
       </c>
       <c r="I107">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="J107">
         <v>36</v>
@@ -8986,7 +8986,7 @@
         <v>1417</v>
       </c>
       <c r="I108">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="K108" t="s">
         <v>1421</v>
@@ -9024,7 +9024,7 @@
         <v>1417</v>
       </c>
       <c r="I109">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="K109" t="s">
         <v>1421</v>
@@ -9207,7 +9207,7 @@
         <v>1417</v>
       </c>
       <c r="I115">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="K115" t="s">
         <v>1421</v>
@@ -9245,7 +9245,7 @@
         <v>1417</v>
       </c>
       <c r="I116">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="K116" t="s">
         <v>1421</v>
@@ -9283,7 +9283,7 @@
         <v>1417</v>
       </c>
       <c r="I117">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="K117" t="s">
         <v>1421</v>
@@ -9321,7 +9321,7 @@
         <v>1417</v>
       </c>
       <c r="I118">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="K118" t="s">
         <v>1421</v>
@@ -9359,7 +9359,7 @@
         <v>1417</v>
       </c>
       <c r="I119">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="K119" t="s">
         <v>1421</v>
@@ -9397,7 +9397,7 @@
         <v>1417</v>
       </c>
       <c r="I120">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="K120" t="s">
         <v>1421</v>
@@ -9435,7 +9435,7 @@
         <v>1417</v>
       </c>
       <c r="I121">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="J121">
         <v>251</v>
@@ -9482,7 +9482,7 @@
         <v>1417</v>
       </c>
       <c r="I122">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="K122" t="s">
         <v>1421</v>
@@ -9549,7 +9549,7 @@
         <v>1417</v>
       </c>
       <c r="I124">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="K124" t="s">
         <v>1421</v>
@@ -9587,7 +9587,7 @@
         <v>1417</v>
       </c>
       <c r="I125">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="K125" t="s">
         <v>1427</v>
@@ -9683,7 +9683,7 @@
         <v>1417</v>
       </c>
       <c r="I128">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="K128" t="s">
         <v>1421</v>
@@ -9721,7 +9721,7 @@
         <v>1417</v>
       </c>
       <c r="I129">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="K129" t="s">
         <v>1420</v>
@@ -9759,7 +9759,7 @@
         <v>1417</v>
       </c>
       <c r="I130">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="J130">
         <v>47</v>
@@ -9835,7 +9835,7 @@
         <v>1417</v>
       </c>
       <c r="I132">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="J132">
         <v>145</v>
@@ -9911,7 +9911,7 @@
         <v>1417</v>
       </c>
       <c r="I134">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="K134" t="s">
         <v>1420</v>
@@ -10036,7 +10036,7 @@
         <v>1417</v>
       </c>
       <c r="I138">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="K138" t="s">
         <v>1421</v>
@@ -10420,7 +10420,7 @@
         <v>1417</v>
       </c>
       <c r="I150">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="J150">
         <v>201</v>
@@ -10607,7 +10607,7 @@
         <v>1417</v>
       </c>
       <c r="I155">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="K155" t="s">
         <v>1427</v>
@@ -10642,7 +10642,7 @@
         <v>1417</v>
       </c>
       <c r="I156">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="K156" t="s">
         <v>1421</v>
@@ -10680,7 +10680,7 @@
         <v>1417</v>
       </c>
       <c r="I157">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="J157">
         <v>371</v>
@@ -10724,7 +10724,7 @@
         <v>1417</v>
       </c>
       <c r="I158">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="J158">
         <v>52</v>
@@ -10768,7 +10768,7 @@
         <v>1417</v>
       </c>
       <c r="I159">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="K159" t="s">
         <v>1421</v>
@@ -10806,7 +10806,7 @@
         <v>1417</v>
       </c>
       <c r="I160">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="K160" t="s">
         <v>1421</v>
@@ -10844,7 +10844,7 @@
         <v>1417</v>
       </c>
       <c r="I161">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="J161">
         <v>55</v>
@@ -10979,7 +10979,7 @@
         <v>1417</v>
       </c>
       <c r="I164">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="O164" t="s">
         <v>1533</v>
@@ -11154,7 +11154,7 @@
         <v>1417</v>
       </c>
       <c r="I169">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="K169" t="s">
         <v>1394</v>
@@ -11364,7 +11364,7 @@
         <v>1417</v>
       </c>
       <c r="I175">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="J175">
         <v>205</v>
@@ -11411,7 +11411,7 @@
         <v>1417</v>
       </c>
       <c r="I176">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="K176" t="s">
         <v>1421</v>
@@ -11449,7 +11449,7 @@
         <v>1417</v>
       </c>
       <c r="I177">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="J177">
         <v>44</v>
@@ -11496,7 +11496,7 @@
         <v>1417</v>
       </c>
       <c r="I178">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="K178" t="s">
         <v>1420</v>
@@ -11563,7 +11563,7 @@
         <v>1417</v>
       </c>
       <c r="I180">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="K180" t="s">
         <v>1420</v>
@@ -11659,7 +11659,7 @@
         <v>1417</v>
       </c>
       <c r="I183">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="K183" t="s">
         <v>1421</v>
@@ -11697,7 +11697,7 @@
         <v>1417</v>
       </c>
       <c r="I184">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="K184" t="s">
         <v>1427</v>
@@ -11732,7 +11732,7 @@
         <v>1417</v>
       </c>
       <c r="I185">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="K185" t="s">
         <v>1421</v>
@@ -11770,7 +11770,7 @@
         <v>1417</v>
       </c>
       <c r="I186">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="K186" t="s">
         <v>1421</v>
@@ -11808,7 +11808,7 @@
         <v>1417</v>
       </c>
       <c r="I187">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="J187">
         <v>75</v>
@@ -11855,7 +11855,7 @@
         <v>1417</v>
       </c>
       <c r="I188">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="J188">
         <v>40</v>
@@ -11902,7 +11902,7 @@
         <v>1417</v>
       </c>
       <c r="I189">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="J189">
         <v>155</v>
@@ -11946,7 +11946,7 @@
         <v>1417</v>
       </c>
       <c r="I190">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="J190">
         <v>107</v>
@@ -11990,7 +11990,7 @@
         <v>1417</v>
       </c>
       <c r="I191">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="J191">
         <v>5</v>
@@ -12034,7 +12034,7 @@
         <v>1417</v>
       </c>
       <c r="I192">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="K192" t="s">
         <v>1421</v>
@@ -12072,7 +12072,7 @@
         <v>1417</v>
       </c>
       <c r="I193">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="K193" t="s">
         <v>1426</v>
@@ -12267,7 +12267,7 @@
         <v>1417</v>
       </c>
       <c r="I199">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="J199">
         <v>70</v>
@@ -12352,7 +12352,7 @@
         <v>1417</v>
       </c>
       <c r="I201">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="K201" t="s">
         <v>1421</v>
@@ -12390,7 +12390,7 @@
         <v>1417</v>
       </c>
       <c r="I202">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="K202" t="s">
         <v>1421</v>
@@ -12469,7 +12469,7 @@
         <v>1417</v>
       </c>
       <c r="I204">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="K204" t="s">
         <v>1420</v>
@@ -12507,7 +12507,7 @@
         <v>1417</v>
       </c>
       <c r="I205">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="K205" t="s">
         <v>1420</v>
@@ -12574,7 +12574,7 @@
         <v>1417</v>
       </c>
       <c r="I207">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="J207">
         <v>167</v>
@@ -12618,7 +12618,7 @@
         <v>1417</v>
       </c>
       <c r="I208">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="J208">
         <v>45</v>
@@ -12662,7 +12662,7 @@
         <v>1417</v>
       </c>
       <c r="I209">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="J209">
         <v>191</v>
@@ -12706,7 +12706,7 @@
         <v>1417</v>
       </c>
       <c r="I210">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="K210" t="s">
         <v>1424</v>
@@ -12802,7 +12802,7 @@
         <v>1417</v>
       </c>
       <c r="I213">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="K213" t="s">
         <v>1421</v>
@@ -12840,7 +12840,7 @@
         <v>1417</v>
       </c>
       <c r="I214">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="J214">
         <v>14</v>
@@ -12887,7 +12887,7 @@
         <v>1417</v>
       </c>
       <c r="I215">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="K215" t="s">
         <v>1421</v>
@@ -12954,7 +12954,7 @@
         <v>1417</v>
       </c>
       <c r="I217">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="J217">
         <v>42</v>
@@ -12998,7 +12998,7 @@
         <v>1417</v>
       </c>
       <c r="I218">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="J218">
         <v>166</v>
@@ -13086,7 +13086,7 @@
         <v>1417</v>
       </c>
       <c r="I220">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="J220">
         <v>154</v>
@@ -13472,7 +13472,7 @@
         <v>1417</v>
       </c>
       <c r="I230">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="J230">
         <v>197</v>
@@ -13516,7 +13516,7 @@
         <v>1417</v>
       </c>
       <c r="I231">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="J231">
         <v>35</v>
@@ -13618,7 +13618,7 @@
         <v>1417</v>
       </c>
       <c r="I234">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="J234">
         <v>35</v>
@@ -13665,7 +13665,7 @@
         <v>1417</v>
       </c>
       <c r="I235">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="J235">
         <v>35</v>
@@ -13712,7 +13712,7 @@
         <v>1417</v>
       </c>
       <c r="I236">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="J236">
         <v>86</v>
@@ -13829,7 +13829,7 @@
         <v>1417</v>
       </c>
       <c r="I239">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="K239" t="s">
         <v>1394</v>
@@ -13928,7 +13928,7 @@
         <v>1417</v>
       </c>
       <c r="I242">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="K242" t="s">
         <v>1420</v>
@@ -13995,7 +13995,7 @@
         <v>1417</v>
       </c>
       <c r="I244">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="J244">
         <v>15</v>
@@ -14036,7 +14036,7 @@
         <v>1417</v>
       </c>
       <c r="I245">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="J245">
         <v>15</v>
@@ -14179,7 +14179,7 @@
         <v>1417</v>
       </c>
       <c r="I249">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="K249" t="s">
         <v>1421</v>
@@ -14313,7 +14313,7 @@
         <v>1417</v>
       </c>
       <c r="I253">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="J253">
         <v>162</v>
@@ -14357,7 +14357,7 @@
         <v>1417</v>
       </c>
       <c r="I254">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="K254" t="s">
         <v>1424</v>
@@ -14436,7 +14436,7 @@
         <v>1417</v>
       </c>
       <c r="I256">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="J256">
         <v>23</v>
@@ -14620,7 +14620,7 @@
         <v>1417</v>
       </c>
       <c r="I261">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="J261">
         <v>162</v>
@@ -14778,7 +14778,7 @@
         <v>1417</v>
       </c>
       <c r="I265">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="J265">
         <v>162</v>
@@ -14863,7 +14863,7 @@
         <v>1417</v>
       </c>
       <c r="I267">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="K267" t="s">
         <v>1424</v>
@@ -14901,7 +14901,7 @@
         <v>1417</v>
       </c>
       <c r="I268">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="K268" t="s">
         <v>1421</v>
@@ -14936,7 +14936,7 @@
         <v>1417</v>
       </c>
       <c r="I269">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="K269" t="s">
         <v>1421</v>
@@ -14974,7 +14974,7 @@
         <v>1417</v>
       </c>
       <c r="I270">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="K270" t="s">
         <v>1424</v>
@@ -15012,7 +15012,7 @@
         <v>1417</v>
       </c>
       <c r="I271">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="K271" t="s">
         <v>1424</v>
@@ -15190,7 +15190,7 @@
         <v>1417</v>
       </c>
       <c r="I276">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="K276" t="s">
         <v>1425</v>
@@ -15228,7 +15228,7 @@
         <v>1417</v>
       </c>
       <c r="I277">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="K277" t="s">
         <v>1421</v>
@@ -15266,7 +15266,7 @@
         <v>1417</v>
       </c>
       <c r="I278">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="J278">
         <v>148</v>
@@ -15310,7 +15310,7 @@
         <v>1417</v>
       </c>
       <c r="I279">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="K279" t="s">
         <v>1423</v>
@@ -15351,7 +15351,7 @@
         <v>1417</v>
       </c>
       <c r="I280">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="K280" t="s">
         <v>1421</v>
@@ -15389,7 +15389,7 @@
         <v>1417</v>
       </c>
       <c r="I281">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="K281" t="s">
         <v>1421</v>
@@ -15430,7 +15430,7 @@
         <v>1417</v>
       </c>
       <c r="I282">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="K282" t="s">
         <v>1421</v>
@@ -15724,7 +15724,7 @@
         <v>1417</v>
       </c>
       <c r="I291">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="J291">
         <v>20</v>
@@ -15768,7 +15768,7 @@
         <v>1417</v>
       </c>
       <c r="I292">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="K292" t="s">
         <v>1424</v>
@@ -15806,7 +15806,7 @@
         <v>1417</v>
       </c>
       <c r="I293">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="K293" t="s">
         <v>1425</v>
@@ -15844,7 +15844,7 @@
         <v>1417</v>
       </c>
       <c r="I294">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="K294" t="s">
         <v>1430</v>
@@ -15981,7 +15981,7 @@
         <v>1417</v>
       </c>
       <c r="I298">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="J298">
         <v>58</v>
@@ -16145,7 +16145,7 @@
         <v>1417</v>
       </c>
       <c r="I302">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="K302" t="s">
         <v>1424</v>
@@ -16183,7 +16183,7 @@
         <v>1417</v>
       </c>
       <c r="I303">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="K303" t="s">
         <v>1421</v>
@@ -16221,7 +16221,7 @@
         <v>1417</v>
       </c>
       <c r="I304">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="K304" t="s">
         <v>1424</v>
@@ -16259,7 +16259,7 @@
         <v>1417</v>
       </c>
       <c r="I305">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="J305">
         <v>35</v>
@@ -16303,7 +16303,7 @@
         <v>1417</v>
       </c>
       <c r="I306">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="J306">
         <v>31</v>
@@ -16391,7 +16391,7 @@
         <v>1417</v>
       </c>
       <c r="I308">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="K308" t="s">
         <v>1420</v>
@@ -16508,7 +16508,7 @@
         <v>1417</v>
       </c>
       <c r="I311">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="K311" t="s">
         <v>1420</v>
@@ -16838,7 +16838,7 @@
         <v>1417</v>
       </c>
       <c r="I320">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="K320" t="s">
         <v>1425</v>
@@ -16876,7 +16876,7 @@
         <v>1417</v>
       </c>
       <c r="I321">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="K321" t="s">
         <v>1421</v>
@@ -16914,7 +16914,7 @@
         <v>1417</v>
       </c>
       <c r="I322">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="J322">
         <v>57</v>
@@ -17028,7 +17028,7 @@
         <v>1417</v>
       </c>
       <c r="I325">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="J325">
         <v>57</v>
@@ -17110,7 +17110,7 @@
         <v>1417</v>
       </c>
       <c r="I327">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="J327">
         <v>57</v>
@@ -17154,7 +17154,7 @@
         <v>1417</v>
       </c>
       <c r="I328">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="J328">
         <v>57</v>
@@ -17198,7 +17198,7 @@
         <v>1417</v>
       </c>
       <c r="I329">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="J329">
         <v>57</v>
@@ -17242,7 +17242,7 @@
         <v>1417</v>
       </c>
       <c r="I330">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="J330">
         <v>57</v>
@@ -17286,7 +17286,7 @@
         <v>1417</v>
       </c>
       <c r="I331">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="K331" t="s">
         <v>1420</v>
@@ -17324,7 +17324,7 @@
         <v>1417</v>
       </c>
       <c r="I332">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="K332" t="s">
         <v>1421</v>
@@ -17362,7 +17362,7 @@
         <v>1417</v>
       </c>
       <c r="I333">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="J333">
         <v>100</v>
@@ -17406,7 +17406,7 @@
         <v>1417</v>
       </c>
       <c r="I334">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="K334" t="s">
         <v>1421</v>
@@ -17631,7 +17631,7 @@
         <v>1417</v>
       </c>
       <c r="I340">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="J340">
         <v>98</v>
@@ -17672,7 +17672,7 @@
         <v>1417</v>
       </c>
       <c r="I341">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="J341">
         <v>90</v>
@@ -17713,7 +17713,7 @@
         <v>1417</v>
       </c>
       <c r="I342">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="K342" t="s">
         <v>1420</v>
@@ -17827,7 +17827,7 @@
         <v>1417</v>
       </c>
       <c r="I345">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="K345" t="s">
         <v>1420</v>
@@ -17947,7 +17947,7 @@
         <v>1417</v>
       </c>
       <c r="I348">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="J348">
         <v>14</v>
@@ -17991,7 +17991,7 @@
         <v>1417</v>
       </c>
       <c r="I349">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="K349" t="s">
         <v>1425</v>
@@ -18029,7 +18029,7 @@
         <v>1417</v>
       </c>
       <c r="I350">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="J350">
         <v>46</v>
@@ -18067,7 +18067,7 @@
         <v>1417</v>
       </c>
       <c r="I351">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="J351">
         <v>82</v>
@@ -18111,7 +18111,7 @@
         <v>1417</v>
       </c>
       <c r="I352">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="J352">
         <v>78</v>
@@ -18155,7 +18155,7 @@
         <v>1417</v>
       </c>
       <c r="I353">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="J353">
         <v>83</v>
@@ -18199,7 +18199,7 @@
         <v>1417</v>
       </c>
       <c r="I354">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="K354" t="s">
         <v>1424</v>
@@ -18237,7 +18237,7 @@
         <v>1417</v>
       </c>
       <c r="I355">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="J355">
         <v>8</v>
@@ -18319,7 +18319,7 @@
         <v>1417</v>
       </c>
       <c r="I357">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="J357">
         <v>85</v>
@@ -18442,7 +18442,7 @@
         <v>1417</v>
       </c>
       <c r="I360">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="J360">
         <v>83</v>
@@ -18489,7 +18489,7 @@
         <v>1417</v>
       </c>
       <c r="I361">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="J361">
         <v>83</v>
@@ -18533,7 +18533,7 @@
         <v>1417</v>
       </c>
       <c r="I362">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="K362" t="s">
         <v>1424</v>
@@ -18571,7 +18571,7 @@
         <v>1417</v>
       </c>
       <c r="I363">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="K363" t="s">
         <v>1424</v>
@@ -18609,7 +18609,7 @@
         <v>1417</v>
       </c>
       <c r="I364">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="J364">
         <v>83</v>
@@ -18653,7 +18653,7 @@
         <v>1417</v>
       </c>
       <c r="I365">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="J365">
         <v>15</v>
@@ -18776,7 +18776,7 @@
         <v>1417</v>
       </c>
       <c r="I368">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="J368">
         <v>77</v>
@@ -18820,7 +18820,7 @@
         <v>1417</v>
       </c>
       <c r="I369">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="K369" t="s">
         <v>1424</v>
@@ -18858,7 +18858,7 @@
         <v>1417</v>
       </c>
       <c r="I370">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="K370" t="s">
         <v>1424</v>
@@ -18896,7 +18896,7 @@
         <v>1417</v>
       </c>
       <c r="I371">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="J371">
         <v>16</v>
@@ -18984,7 +18984,7 @@
         <v>1417</v>
       </c>
       <c r="I373">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="K373" t="s">
         <v>1420</v>
@@ -19022,7 +19022,7 @@
         <v>1417</v>
       </c>
       <c r="I374">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="K374" t="s">
         <v>1420</v>
@@ -19060,7 +19060,7 @@
         <v>1417</v>
       </c>
       <c r="I375">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="J375">
         <v>94</v>
@@ -19101,7 +19101,7 @@
         <v>1417</v>
       </c>
       <c r="I376">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="K376" t="s">
         <v>1424</v>
@@ -19180,7 +19180,7 @@
         <v>1417</v>
       </c>
       <c r="I378">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="K378" t="s">
         <v>1424</v>
@@ -19218,7 +19218,7 @@
         <v>1417</v>
       </c>
       <c r="I379">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="J379">
         <v>20</v>
@@ -19262,7 +19262,7 @@
         <v>1417</v>
       </c>
       <c r="I380">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="J380">
         <v>94</v>
@@ -19306,7 +19306,7 @@
         <v>1417</v>
       </c>
       <c r="I381">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="K381" t="s">
         <v>1424</v>
@@ -19344,7 +19344,7 @@
         <v>1417</v>
       </c>
       <c r="I382">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="K382" t="s">
         <v>1424</v>
@@ -19382,7 +19382,7 @@
         <v>1417</v>
       </c>
       <c r="I383">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="J383">
         <v>71</v>
@@ -19426,7 +19426,7 @@
         <v>1417</v>
       </c>
       <c r="I384">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="K384" t="s">
         <v>1421</v>
@@ -19508,7 +19508,7 @@
         <v>1417</v>
       </c>
       <c r="I386">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="K386" t="s">
         <v>1424</v>
@@ -19546,7 +19546,7 @@
         <v>1417</v>
       </c>
       <c r="I387">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="K387" t="s">
         <v>1424</v>
@@ -19584,7 +19584,7 @@
         <v>1417</v>
       </c>
       <c r="I388">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="J388">
         <v>-85</v>
@@ -19628,7 +19628,7 @@
         <v>1417</v>
       </c>
       <c r="I389">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="K389" t="s">
         <v>1425</v>
@@ -20079,7 +20079,7 @@
         <v>1417</v>
       </c>
       <c r="I400">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="K400" t="s">
         <v>1424</v>
@@ -20155,7 +20155,7 @@
         <v>1417</v>
       </c>
       <c r="I402">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="K402" t="s">
         <v>1424</v>
@@ -20193,7 +20193,7 @@
         <v>1417</v>
       </c>
       <c r="I403">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="J403">
         <v>83</v>
@@ -20237,7 +20237,7 @@
         <v>1417</v>
       </c>
       <c r="I404">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="K404" t="s">
         <v>1424</v>
@@ -20307,7 +20307,7 @@
         <v>1417</v>
       </c>
       <c r="I406">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="Q406" t="b">
         <v>1</v>
@@ -20339,7 +20339,7 @@
         <v>1417</v>
       </c>
       <c r="I407">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="Q407" t="b">
         <v>1</v>
@@ -20371,7 +20371,7 @@
         <v>1417</v>
       </c>
       <c r="I408">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="Q408" t="b">
         <v>1</v>
@@ -20403,7 +20403,7 @@
         <v>1417</v>
       </c>
       <c r="I409">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="Q409" t="b">
         <v>1</v>
@@ -20435,7 +20435,7 @@
         <v>1417</v>
       </c>
       <c r="I410">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="Q410" t="b">
         <v>1</v>
@@ -20467,7 +20467,7 @@
         <v>1417</v>
       </c>
       <c r="I411">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="Q411" t="b">
         <v>1</v>
@@ -20499,7 +20499,7 @@
         <v>1417</v>
       </c>
       <c r="I412">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="Q412" t="b">
         <v>1</v>
@@ -20531,7 +20531,7 @@
         <v>1417</v>
       </c>
       <c r="I413">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="Q413" t="b">
         <v>1</v>
@@ -20621,7 +20621,7 @@
         <v>1417</v>
       </c>
       <c r="I416">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="Q416" t="b">
         <v>1</v>
@@ -20711,7 +20711,7 @@
         <v>1417</v>
       </c>
       <c r="I419">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="Q419" t="b">
         <v>1</v>
@@ -20743,7 +20743,7 @@
         <v>1417</v>
       </c>
       <c r="I420">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="Q420" t="b">
         <v>1</v>
@@ -20775,7 +20775,7 @@
         <v>1417</v>
       </c>
       <c r="I421">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="Q421" t="b">
         <v>1</v>
@@ -20807,7 +20807,7 @@
         <v>1417</v>
       </c>
       <c r="I422">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="Q422" t="b">
         <v>1</v>
@@ -20839,7 +20839,7 @@
         <v>1417</v>
       </c>
       <c r="I423">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="Q423" t="b">
         <v>1</v>
@@ -20871,7 +20871,7 @@
         <v>1417</v>
       </c>
       <c r="I424">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="Q424" t="b">
         <v>1</v>
@@ -20903,7 +20903,7 @@
         <v>1417</v>
       </c>
       <c r="I425">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="Q425" t="b">
         <v>1</v>
@@ -20935,7 +20935,7 @@
         <v>1417</v>
       </c>
       <c r="I426">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="Q426" t="b">
         <v>1</v>
@@ -20967,7 +20967,7 @@
         <v>1417</v>
       </c>
       <c r="I427">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="Q427" t="b">
         <v>1</v>
@@ -21057,7 +21057,7 @@
         <v>1417</v>
       </c>
       <c r="I430">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="Q430" t="b">
         <v>1</v>
@@ -21089,7 +21089,7 @@
         <v>1417</v>
       </c>
       <c r="I431">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="Q431" t="b">
         <v>1</v>
@@ -21121,7 +21121,7 @@
         <v>1417</v>
       </c>
       <c r="I432">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="Q432" t="b">
         <v>1</v>
@@ -21153,7 +21153,7 @@
         <v>1417</v>
       </c>
       <c r="I433">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="Q433" t="b">
         <v>1</v>
@@ -21185,7 +21185,7 @@
         <v>1417</v>
       </c>
       <c r="I434">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="Q434" t="b">
         <v>1</v>
@@ -21217,7 +21217,7 @@
         <v>1417</v>
       </c>
       <c r="I435">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="Q435" t="b">
         <v>1</v>
@@ -21249,7 +21249,7 @@
         <v>1417</v>
       </c>
       <c r="I436">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="Q436" t="b">
         <v>1</v>
@@ -21281,7 +21281,7 @@
         <v>1419</v>
       </c>
       <c r="I437">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="Q437" t="b">
         <v>1</v>
@@ -21313,7 +21313,7 @@
         <v>1419</v>
       </c>
       <c r="I438">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="Q438" t="b">
         <v>1</v>
@@ -21345,7 +21345,7 @@
         <v>1417</v>
       </c>
       <c r="I439">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="Q439" t="b">
         <v>1</v>
@@ -21377,7 +21377,7 @@
         <v>1417</v>
       </c>
       <c r="I440">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="Q440" t="b">
         <v>1</v>
@@ -21409,7 +21409,7 @@
         <v>1417</v>
       </c>
       <c r="I441">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="Q441" t="b">
         <v>1</v>
@@ -21470,7 +21470,7 @@
         <v>1417</v>
       </c>
       <c r="I443">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="Q443" t="b">
         <v>1</v>
@@ -21560,7 +21560,7 @@
         <v>1417</v>
       </c>
       <c r="I446">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="Q446" t="b">
         <v>1</v>
@@ -21592,7 +21592,7 @@
         <v>1417</v>
       </c>
       <c r="I447">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="Q447" t="b">
         <v>1</v>
@@ -21624,7 +21624,7 @@
         <v>1417</v>
       </c>
       <c r="I448">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="Q448" t="b">
         <v>1</v>
@@ -21656,7 +21656,7 @@
         <v>1417</v>
       </c>
       <c r="I449">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="Q449" t="b">
         <v>1</v>
@@ -21688,7 +21688,7 @@
         <v>1417</v>
       </c>
       <c r="I450">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="Q450" t="b">
         <v>1</v>
@@ -21720,7 +21720,7 @@
         <v>1417</v>
       </c>
       <c r="I451">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="Q451" t="b">
         <v>1</v>
@@ -21781,7 +21781,7 @@
         <v>1417</v>
       </c>
       <c r="I453">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="Q453" t="b">
         <v>1</v>
@@ -21813,7 +21813,7 @@
         <v>1417</v>
       </c>
       <c r="I454">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="Q454" t="b">
         <v>1</v>
@@ -21845,7 +21845,7 @@
         <v>1417</v>
       </c>
       <c r="I455">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="Q455" t="b">
         <v>1</v>
@@ -21906,7 +21906,7 @@
         <v>1417</v>
       </c>
       <c r="I457">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="Q457" t="b">
         <v>1</v>
@@ -21938,7 +21938,7 @@
         <v>1417</v>
       </c>
       <c r="I458">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Q458" t="b">
         <v>1</v>
@@ -21970,7 +21970,7 @@
         <v>1417</v>
       </c>
       <c r="I459">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="Q459" t="b">
         <v>1</v>
@@ -22002,7 +22002,7 @@
         <v>1417</v>
       </c>
       <c r="I460">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="Q460" t="b">
         <v>1</v>
@@ -22034,7 +22034,7 @@
         <v>1417</v>
       </c>
       <c r="I461">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="Q461" t="b">
         <v>1</v>
@@ -22066,7 +22066,7 @@
         <v>1417</v>
       </c>
       <c r="I462">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="Q462" t="b">
         <v>1</v>
@@ -22098,7 +22098,7 @@
         <v>1417</v>
       </c>
       <c r="I463">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="Q463" t="b">
         <v>1</v>
@@ -22130,7 +22130,7 @@
         <v>1417</v>
       </c>
       <c r="I464">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="Q464" t="b">
         <v>1</v>
@@ -22162,7 +22162,7 @@
         <v>1417</v>
       </c>
       <c r="I465">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="Q465" t="b">
         <v>1</v>
@@ -22194,7 +22194,7 @@
         <v>1417</v>
       </c>
       <c r="I466">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="Q466" t="b">
         <v>1</v>
@@ -22226,7 +22226,7 @@
         <v>1417</v>
       </c>
       <c r="I467">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="Q467" t="b">
         <v>1</v>
@@ -22258,7 +22258,7 @@
         <v>1417</v>
       </c>
       <c r="I468">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="Q468" t="b">
         <v>1</v>
@@ -22290,7 +22290,7 @@
         <v>1417</v>
       </c>
       <c r="I469">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="Q469" t="b">
         <v>1</v>
@@ -22351,7 +22351,7 @@
         <v>1417</v>
       </c>
       <c r="I471">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="Q471" t="b">
         <v>1</v>
@@ -22383,7 +22383,7 @@
         <v>1417</v>
       </c>
       <c r="I472">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="Q472" t="b">
         <v>1</v>
@@ -22415,7 +22415,7 @@
         <v>1417</v>
       </c>
       <c r="I473">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="Q473" t="b">
         <v>1</v>
@@ -22447,7 +22447,7 @@
         <v>1417</v>
       </c>
       <c r="I474">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Q474" t="b">
         <v>1</v>
@@ -22479,7 +22479,7 @@
         <v>1417</v>
       </c>
       <c r="I475">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Q475" t="b">
         <v>1</v>
@@ -22511,7 +22511,7 @@
         <v>1417</v>
       </c>
       <c r="I476">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Q476" t="b">
         <v>1</v>
@@ -22543,7 +22543,7 @@
         <v>1417</v>
       </c>
       <c r="I477">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Q477" t="b">
         <v>1</v>
@@ -22575,7 +22575,7 @@
         <v>1417</v>
       </c>
       <c r="I478">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Q478" t="b">
         <v>1</v>
@@ -22607,7 +22607,7 @@
         <v>1417</v>
       </c>
       <c r="I479">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Q479" t="b">
         <v>1</v>
@@ -22639,7 +22639,7 @@
         <v>1417</v>
       </c>
       <c r="I480">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Q480" t="b">
         <v>1</v>
@@ -22671,7 +22671,7 @@
         <v>1417</v>
       </c>
       <c r="I481">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Q481" t="b">
         <v>1</v>
@@ -22703,7 +22703,7 @@
         <v>1417</v>
       </c>
       <c r="I482">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Q482" t="b">
         <v>1</v>
@@ -22735,7 +22735,7 @@
         <v>1417</v>
       </c>
       <c r="I483">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Q483" t="b">
         <v>1</v>
@@ -22767,7 +22767,7 @@
         <v>1417</v>
       </c>
       <c r="I484">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Q484" t="b">
         <v>1</v>
@@ -22799,7 +22799,7 @@
         <v>1417</v>
       </c>
       <c r="I485">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Q485" t="b">
         <v>1</v>
@@ -22831,7 +22831,7 @@
         <v>1417</v>
       </c>
       <c r="I486">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Q486" t="b">
         <v>1</v>
@@ -22863,7 +22863,7 @@
         <v>1417</v>
       </c>
       <c r="I487">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Q487" t="b">
         <v>1</v>
@@ -22895,7 +22895,7 @@
         <v>1417</v>
       </c>
       <c r="I488">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Q488" t="b">
         <v>1</v>
@@ -22927,7 +22927,7 @@
         <v>1417</v>
       </c>
       <c r="I489">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Q489" t="b">
         <v>1</v>
@@ -22959,7 +22959,7 @@
         <v>1417</v>
       </c>
       <c r="I490">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Q490" t="b">
         <v>1</v>
@@ -22991,7 +22991,7 @@
         <v>1417</v>
       </c>
       <c r="I491">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Q491" t="b">
         <v>1</v>
@@ -23023,7 +23023,7 @@
         <v>1419</v>
       </c>
       <c r="I492">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Q492" t="b">
         <v>1</v>
@@ -23055,7 +23055,7 @@
         <v>1419</v>
       </c>
       <c r="I493">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Q493" t="b">
         <v>1</v>
@@ -23087,7 +23087,7 @@
         <v>1419</v>
       </c>
       <c r="I494">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Q494" t="b">
         <v>1</v>
@@ -23119,7 +23119,7 @@
         <v>1419</v>
       </c>
       <c r="I495">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Q495" t="b">
         <v>1</v>
@@ -23151,7 +23151,7 @@
         <v>1419</v>
       </c>
       <c r="I496">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Q496" t="b">
         <v>1</v>
@@ -23183,7 +23183,7 @@
         <v>1417</v>
       </c>
       <c r="I497">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Q497" t="b">
         <v>1</v>
@@ -23215,7 +23215,7 @@
         <v>1417</v>
       </c>
       <c r="I498">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Q498" t="b">
         <v>1</v>
@@ -23247,7 +23247,7 @@
         <v>1419</v>
       </c>
       <c r="I499">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Q499" t="b">
         <v>1</v>
@@ -23279,7 +23279,7 @@
         <v>1417</v>
       </c>
       <c r="I500">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Q500" t="b">
         <v>1</v>
@@ -23311,7 +23311,7 @@
         <v>1417</v>
       </c>
       <c r="I501">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Q501" t="b">
         <v>1</v>
@@ -23343,7 +23343,7 @@
         <v>1417</v>
       </c>
       <c r="I502">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Q502" t="b">
         <v>1</v>
@@ -23375,7 +23375,7 @@
         <v>1417</v>
       </c>
       <c r="I503">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Q503" t="b">
         <v>1</v>
@@ -23407,7 +23407,7 @@
         <v>1417</v>
       </c>
       <c r="I504">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="Q504" t="b">
         <v>1</v>
@@ -23439,7 +23439,7 @@
         <v>1417</v>
       </c>
       <c r="I505">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="Q505" t="b">
         <v>1</v>
@@ -23471,7 +23471,7 @@
         <v>1417</v>
       </c>
       <c r="I506">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="Q506" t="b">
         <v>1</v>
@@ -23503,7 +23503,7 @@
         <v>1417</v>
       </c>
       <c r="I507">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="Q507" t="b">
         <v>1</v>
@@ -23564,7 +23564,7 @@
         <v>1417</v>
       </c>
       <c r="I509">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="Q509" t="b">
         <v>1</v>
@@ -23596,7 +23596,7 @@
         <v>1417</v>
       </c>
       <c r="I510">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="Q510" t="b">
         <v>1</v>
@@ -23628,7 +23628,7 @@
         <v>1417</v>
       </c>
       <c r="I511">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="Q511" t="b">
         <v>1</v>
@@ -23660,7 +23660,7 @@
         <v>1417</v>
       </c>
       <c r="I512">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="Q512" t="b">
         <v>1</v>
@@ -23692,7 +23692,7 @@
         <v>1417</v>
       </c>
       <c r="I513">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="Q513" t="b">
         <v>1</v>
@@ -23753,7 +23753,7 @@
         <v>1417</v>
       </c>
       <c r="I515">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="Q515" t="b">
         <v>1</v>
@@ -23785,7 +23785,7 @@
         <v>1417</v>
       </c>
       <c r="I516">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q516" t="b">
         <v>1</v>
@@ -23817,7 +23817,7 @@
         <v>1417</v>
       </c>
       <c r="I517">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q517" t="b">
         <v>1</v>
@@ -23849,7 +23849,7 @@
         <v>1417</v>
       </c>
       <c r="I518">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q518" t="b">
         <v>1</v>
@@ -23881,7 +23881,7 @@
         <v>1417</v>
       </c>
       <c r="I519">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="Q519" t="b">
         <v>1</v>
@@ -23913,7 +23913,7 @@
         <v>1417</v>
       </c>
       <c r="I520">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="Q520" t="b">
         <v>1</v>
@@ -23945,7 +23945,7 @@
         <v>1417</v>
       </c>
       <c r="I521">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="Q521" t="b">
         <v>1</v>
@@ -23977,7 +23977,7 @@
         <v>1417</v>
       </c>
       <c r="I522">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="Q522" t="b">
         <v>1</v>
@@ -24009,7 +24009,7 @@
         <v>1417</v>
       </c>
       <c r="I523">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="Q523" t="b">
         <v>1</v>
@@ -24041,7 +24041,7 @@
         <v>1417</v>
       </c>
       <c r="I524">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q524" t="b">
         <v>1</v>
@@ -24073,7 +24073,7 @@
         <v>1417</v>
       </c>
       <c r="I525">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q525" t="b">
         <v>1</v>
@@ -24105,7 +24105,7 @@
         <v>1417</v>
       </c>
       <c r="I526">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q526" t="b">
         <v>1</v>
@@ -24137,7 +24137,7 @@
         <v>1417</v>
       </c>
       <c r="I527">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q527" t="b">
         <v>1</v>
@@ -24169,7 +24169,7 @@
         <v>1417</v>
       </c>
       <c r="I528">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="Q528" t="b">
         <v>1</v>
@@ -24201,7 +24201,7 @@
         <v>1417</v>
       </c>
       <c r="I529">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q529" t="b">
         <v>1</v>
@@ -24233,7 +24233,7 @@
         <v>1417</v>
       </c>
       <c r="I530">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q530" t="b">
         <v>1</v>
@@ -24265,7 +24265,7 @@
         <v>1417</v>
       </c>
       <c r="I531">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q531" t="b">
         <v>1</v>
@@ -24297,7 +24297,7 @@
         <v>1417</v>
       </c>
       <c r="I532">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q532" t="b">
         <v>1</v>
@@ -24329,7 +24329,7 @@
         <v>1417</v>
       </c>
       <c r="I533">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q533" t="b">
         <v>1</v>
@@ -24361,7 +24361,7 @@
         <v>1417</v>
       </c>
       <c r="I534">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q534" t="b">
         <v>1</v>
@@ -24393,7 +24393,7 @@
         <v>1417</v>
       </c>
       <c r="I535">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q535" t="b">
         <v>1</v>
@@ -24425,7 +24425,7 @@
         <v>1417</v>
       </c>
       <c r="I536">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q536" t="b">
         <v>1</v>
@@ -24457,7 +24457,7 @@
         <v>1417</v>
       </c>
       <c r="I537">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q537" t="b">
         <v>1</v>
@@ -24489,7 +24489,7 @@
         <v>1417</v>
       </c>
       <c r="I538">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q538" t="b">
         <v>1</v>
@@ -24521,7 +24521,7 @@
         <v>1417</v>
       </c>
       <c r="I539">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q539" t="b">
         <v>1</v>
@@ -24553,7 +24553,7 @@
         <v>1417</v>
       </c>
       <c r="I540">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q540" t="b">
         <v>1</v>
@@ -24585,7 +24585,7 @@
         <v>1417</v>
       </c>
       <c r="I541">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q541" t="b">
         <v>1</v>
@@ -24617,7 +24617,7 @@
         <v>1417</v>
       </c>
       <c r="I542">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q542" t="b">
         <v>1</v>
@@ -24649,7 +24649,7 @@
         <v>1417</v>
       </c>
       <c r="I543">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q543" t="b">
         <v>1</v>
@@ -24681,7 +24681,7 @@
         <v>1417</v>
       </c>
       <c r="I544">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q544" t="b">
         <v>1</v>
@@ -24713,7 +24713,7 @@
         <v>1417</v>
       </c>
       <c r="I545">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q545" t="b">
         <v>1</v>
@@ -24745,7 +24745,7 @@
         <v>1417</v>
       </c>
       <c r="I546">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="Q546" t="b">
         <v>1</v>
@@ -24777,7 +24777,7 @@
         <v>1417</v>
       </c>
       <c r="I547">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="Q547" t="b">
         <v>1</v>
@@ -24809,7 +24809,7 @@
         <v>1417</v>
       </c>
       <c r="I548">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="Q548" t="b">
         <v>1</v>
@@ -24841,7 +24841,7 @@
         <v>1417</v>
       </c>
       <c r="I549">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="Q549" t="b">
         <v>1</v>
@@ -24873,7 +24873,7 @@
         <v>1417</v>
       </c>
       <c r="I550">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="Q550" t="b">
         <v>1</v>
@@ -24905,7 +24905,7 @@
         <v>1417</v>
       </c>
       <c r="I551">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="Q551" t="b">
         <v>1</v>
@@ -24937,7 +24937,7 @@
         <v>1417</v>
       </c>
       <c r="I552">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="Q552" t="b">
         <v>1</v>
@@ -24969,7 +24969,7 @@
         <v>1417</v>
       </c>
       <c r="I553">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="Q553" t="b">
         <v>1</v>
@@ -25001,7 +25001,7 @@
         <v>1417</v>
       </c>
       <c r="I554">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="Q554" t="b">
         <v>1</v>
@@ -25033,7 +25033,7 @@
         <v>1417</v>
       </c>
       <c r="I555">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="Q555" t="b">
         <v>1</v>
@@ -25065,7 +25065,7 @@
         <v>1417</v>
       </c>
       <c r="I556">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="Q556" t="b">
         <v>1</v>
@@ -25097,7 +25097,7 @@
         <v>1417</v>
       </c>
       <c r="I557">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="Q557" t="b">
         <v>1</v>
@@ -25129,7 +25129,7 @@
         <v>1417</v>
       </c>
       <c r="I558">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="Q558" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: reparaveis (20/10/2026 12:39)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
@@ -5132,7 +5132,7 @@
         <v>1417</v>
       </c>
       <c r="I2">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="K2" t="s">
         <v>1420</v>
@@ -5170,7 +5170,7 @@
         <v>1417</v>
       </c>
       <c r="I3">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="K3" t="s">
         <v>1421</v>
@@ -5208,7 +5208,7 @@
         <v>1417</v>
       </c>
       <c r="I4">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="K4" t="s">
         <v>1421</v>
@@ -5246,7 +5246,7 @@
         <v>1417</v>
       </c>
       <c r="I5">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="J5">
         <v>279</v>
@@ -5290,7 +5290,7 @@
         <v>1417</v>
       </c>
       <c r="I6">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="J6">
         <v>153</v>
@@ -5334,7 +5334,7 @@
         <v>1417</v>
       </c>
       <c r="I7">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="J7">
         <v>112</v>
@@ -5410,7 +5410,7 @@
         <v>1417</v>
       </c>
       <c r="I9">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="J9">
         <v>362</v>
@@ -5457,7 +5457,7 @@
         <v>1417</v>
       </c>
       <c r="I10">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="J10">
         <v>378</v>
@@ -5504,7 +5504,7 @@
         <v>1417</v>
       </c>
       <c r="I11">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="J11">
         <v>112</v>
@@ -5551,7 +5551,7 @@
         <v>1417</v>
       </c>
       <c r="I12">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="J12">
         <v>124</v>
@@ -5624,7 +5624,7 @@
         <v>1417</v>
       </c>
       <c r="I14">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="J14">
         <v>64</v>
@@ -5703,7 +5703,7 @@
         <v>1417</v>
       </c>
       <c r="I16">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="K16" t="s">
         <v>1420</v>
@@ -5741,7 +5741,7 @@
         <v>1417</v>
       </c>
       <c r="I17">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="J17">
         <v>161</v>
@@ -5785,7 +5785,7 @@
         <v>1417</v>
       </c>
       <c r="I18">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="J18">
         <v>66</v>
@@ -5858,7 +5858,7 @@
         <v>1417</v>
       </c>
       <c r="I20">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="J20">
         <v>399</v>
@@ -5931,7 +5931,7 @@
         <v>1417</v>
       </c>
       <c r="I22">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="K22" t="s">
         <v>1424</v>
@@ -5969,7 +5969,7 @@
         <v>1417</v>
       </c>
       <c r="I23">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="J23">
         <v>229</v>
@@ -6074,7 +6074,7 @@
         <v>1417</v>
       </c>
       <c r="I26">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="J26">
         <v>155</v>
@@ -6121,7 +6121,7 @@
         <v>1417</v>
       </c>
       <c r="I27">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="K27" t="s">
         <v>1424</v>
@@ -6217,7 +6217,7 @@
         <v>1417</v>
       </c>
       <c r="I30">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="J30">
         <v>209</v>
@@ -6290,7 +6290,7 @@
         <v>1417</v>
       </c>
       <c r="I32">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="K32" t="s">
         <v>1420</v>
@@ -6499,7 +6499,7 @@
         <v>1417</v>
       </c>
       <c r="I39">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="K39" t="s">
         <v>1425</v>
@@ -6662,7 +6662,7 @@
         <v>1417</v>
       </c>
       <c r="I44">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="J44">
         <v>87</v>
@@ -6709,7 +6709,7 @@
         <v>1417</v>
       </c>
       <c r="I45">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="J45">
         <v>331</v>
@@ -6756,7 +6756,7 @@
         <v>1417</v>
       </c>
       <c r="I46">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="K46" t="s">
         <v>1424</v>
@@ -6797,7 +6797,7 @@
         <v>1417</v>
       </c>
       <c r="I47">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="J47">
         <v>344</v>
@@ -6844,7 +6844,7 @@
         <v>1417</v>
       </c>
       <c r="I48">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="K48" t="s">
         <v>1424</v>
@@ -6911,7 +6911,7 @@
         <v>1417</v>
       </c>
       <c r="I50">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="K50" t="s">
         <v>1424</v>
@@ -6978,7 +6978,7 @@
         <v>1417</v>
       </c>
       <c r="I52">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="K52" t="s">
         <v>1420</v>
@@ -7016,7 +7016,7 @@
         <v>1417</v>
       </c>
       <c r="I53">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="K53" t="s">
         <v>1421</v>
@@ -7054,7 +7054,7 @@
         <v>1417</v>
       </c>
       <c r="I54">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="K54" t="s">
         <v>1421</v>
@@ -7330,7 +7330,7 @@
         <v>1417</v>
       </c>
       <c r="I63">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="J63">
         <v>293</v>
@@ -7377,7 +7377,7 @@
         <v>1417</v>
       </c>
       <c r="I64">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="J64">
         <v>320</v>
@@ -7607,7 +7607,7 @@
         <v>1417</v>
       </c>
       <c r="I71">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="J71">
         <v>429</v>
@@ -7680,7 +7680,7 @@
         <v>1417</v>
       </c>
       <c r="I73">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="K73" t="s">
         <v>1420</v>
@@ -7788,7 +7788,7 @@
         <v>1417</v>
       </c>
       <c r="I76">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="K76" t="s">
         <v>1427</v>
@@ -7881,7 +7881,7 @@
         <v>1417</v>
       </c>
       <c r="I79">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="K79" t="s">
         <v>1427</v>
@@ -7986,7 +7986,7 @@
         <v>1417</v>
       </c>
       <c r="I82">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="K82" t="s">
         <v>1424</v>
@@ -8053,7 +8053,7 @@
         <v>1417</v>
       </c>
       <c r="I84">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="J84">
         <v>40</v>
@@ -8100,7 +8100,7 @@
         <v>1417</v>
       </c>
       <c r="I85">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="K85" t="s">
         <v>1421</v>
@@ -8138,7 +8138,7 @@
         <v>1417</v>
       </c>
       <c r="I86">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="K86" t="s">
         <v>1421</v>
@@ -8176,7 +8176,7 @@
         <v>1417</v>
       </c>
       <c r="I87">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="J87">
         <v>-16</v>
@@ -8299,7 +8299,7 @@
         <v>1417</v>
       </c>
       <c r="I90">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="K90" t="s">
         <v>1394</v>
@@ -8448,7 +8448,7 @@
         <v>1417</v>
       </c>
       <c r="I94">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="K94" t="s">
         <v>1424</v>
@@ -8527,7 +8527,7 @@
         <v>1417</v>
       </c>
       <c r="I96">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="J96">
         <v>17</v>
@@ -8574,7 +8574,7 @@
         <v>1417</v>
       </c>
       <c r="I97">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="J97">
         <v>20</v>
@@ -8621,7 +8621,7 @@
         <v>1417</v>
       </c>
       <c r="I98">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="K98" t="s">
         <v>1424</v>
@@ -8898,7 +8898,7 @@
         <v>1417</v>
       </c>
       <c r="I106">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="J106">
         <v>49</v>
@@ -8942,7 +8942,7 @@
         <v>1417</v>
       </c>
       <c r="I107">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="J107">
         <v>36</v>
@@ -8986,7 +8986,7 @@
         <v>1417</v>
       </c>
       <c r="I108">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="K108" t="s">
         <v>1421</v>
@@ -9024,7 +9024,7 @@
         <v>1417</v>
       </c>
       <c r="I109">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="K109" t="s">
         <v>1421</v>
@@ -9207,7 +9207,7 @@
         <v>1417</v>
       </c>
       <c r="I115">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="K115" t="s">
         <v>1421</v>
@@ -9245,7 +9245,7 @@
         <v>1417</v>
       </c>
       <c r="I116">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="K116" t="s">
         <v>1421</v>
@@ -9283,7 +9283,7 @@
         <v>1417</v>
       </c>
       <c r="I117">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="K117" t="s">
         <v>1421</v>
@@ -9321,7 +9321,7 @@
         <v>1417</v>
       </c>
       <c r="I118">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="K118" t="s">
         <v>1421</v>
@@ -9359,7 +9359,7 @@
         <v>1417</v>
       </c>
       <c r="I119">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="K119" t="s">
         <v>1421</v>
@@ -9397,7 +9397,7 @@
         <v>1417</v>
       </c>
       <c r="I120">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="K120" t="s">
         <v>1421</v>
@@ -9435,7 +9435,7 @@
         <v>1417</v>
       </c>
       <c r="I121">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="J121">
         <v>251</v>
@@ -9482,7 +9482,7 @@
         <v>1417</v>
       </c>
       <c r="I122">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="K122" t="s">
         <v>1421</v>
@@ -9549,7 +9549,7 @@
         <v>1417</v>
       </c>
       <c r="I124">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="K124" t="s">
         <v>1421</v>
@@ -9587,7 +9587,7 @@
         <v>1417</v>
       </c>
       <c r="I125">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="K125" t="s">
         <v>1427</v>
@@ -9683,7 +9683,7 @@
         <v>1417</v>
       </c>
       <c r="I128">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="K128" t="s">
         <v>1421</v>
@@ -9721,7 +9721,7 @@
         <v>1417</v>
       </c>
       <c r="I129">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="K129" t="s">
         <v>1420</v>
@@ -9759,7 +9759,7 @@
         <v>1417</v>
       </c>
       <c r="I130">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="J130">
         <v>47</v>
@@ -9835,7 +9835,7 @@
         <v>1417</v>
       </c>
       <c r="I132">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="J132">
         <v>145</v>
@@ -9911,7 +9911,7 @@
         <v>1417</v>
       </c>
       <c r="I134">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="K134" t="s">
         <v>1420</v>
@@ -10036,7 +10036,7 @@
         <v>1417</v>
       </c>
       <c r="I138">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="K138" t="s">
         <v>1421</v>
@@ -10420,7 +10420,7 @@
         <v>1417</v>
       </c>
       <c r="I150">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="J150">
         <v>201</v>
@@ -10607,7 +10607,7 @@
         <v>1417</v>
       </c>
       <c r="I155">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="K155" t="s">
         <v>1427</v>
@@ -10642,7 +10642,7 @@
         <v>1417</v>
       </c>
       <c r="I156">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="K156" t="s">
         <v>1421</v>
@@ -10680,7 +10680,7 @@
         <v>1417</v>
       </c>
       <c r="I157">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="J157">
         <v>371</v>
@@ -10724,7 +10724,7 @@
         <v>1417</v>
       </c>
       <c r="I158">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="J158">
         <v>52</v>
@@ -10768,7 +10768,7 @@
         <v>1417</v>
       </c>
       <c r="I159">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="K159" t="s">
         <v>1421</v>
@@ -10806,7 +10806,7 @@
         <v>1417</v>
       </c>
       <c r="I160">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="K160" t="s">
         <v>1421</v>
@@ -10844,7 +10844,7 @@
         <v>1417</v>
       </c>
       <c r="I161">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="J161">
         <v>55</v>
@@ -10979,7 +10979,7 @@
         <v>1417</v>
       </c>
       <c r="I164">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="O164" t="s">
         <v>1533</v>
@@ -11154,7 +11154,7 @@
         <v>1417</v>
       </c>
       <c r="I169">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="K169" t="s">
         <v>1394</v>
@@ -11364,7 +11364,7 @@
         <v>1417</v>
       </c>
       <c r="I175">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="J175">
         <v>205</v>
@@ -11411,7 +11411,7 @@
         <v>1417</v>
       </c>
       <c r="I176">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="K176" t="s">
         <v>1421</v>
@@ -11449,7 +11449,7 @@
         <v>1417</v>
       </c>
       <c r="I177">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="J177">
         <v>44</v>
@@ -11496,7 +11496,7 @@
         <v>1417</v>
       </c>
       <c r="I178">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="K178" t="s">
         <v>1420</v>
@@ -11563,7 +11563,7 @@
         <v>1417</v>
       </c>
       <c r="I180">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="K180" t="s">
         <v>1420</v>
@@ -11659,7 +11659,7 @@
         <v>1417</v>
       </c>
       <c r="I183">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="K183" t="s">
         <v>1421</v>
@@ -11697,7 +11697,7 @@
         <v>1417</v>
       </c>
       <c r="I184">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="K184" t="s">
         <v>1427</v>
@@ -11732,7 +11732,7 @@
         <v>1417</v>
       </c>
       <c r="I185">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="K185" t="s">
         <v>1421</v>
@@ -11770,7 +11770,7 @@
         <v>1417</v>
       </c>
       <c r="I186">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="K186" t="s">
         <v>1421</v>
@@ -11808,7 +11808,7 @@
         <v>1417</v>
       </c>
       <c r="I187">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="J187">
         <v>75</v>
@@ -11855,7 +11855,7 @@
         <v>1417</v>
       </c>
       <c r="I188">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="J188">
         <v>40</v>
@@ -11902,7 +11902,7 @@
         <v>1417</v>
       </c>
       <c r="I189">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="J189">
         <v>155</v>
@@ -11946,7 +11946,7 @@
         <v>1417</v>
       </c>
       <c r="I190">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="J190">
         <v>107</v>
@@ -11990,7 +11990,7 @@
         <v>1417</v>
       </c>
       <c r="I191">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="J191">
         <v>5</v>
@@ -12034,7 +12034,7 @@
         <v>1417</v>
       </c>
       <c r="I192">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="K192" t="s">
         <v>1421</v>
@@ -12072,7 +12072,7 @@
         <v>1417</v>
       </c>
       <c r="I193">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="K193" t="s">
         <v>1426</v>
@@ -12267,7 +12267,7 @@
         <v>1417</v>
       </c>
       <c r="I199">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="J199">
         <v>70</v>
@@ -12352,7 +12352,7 @@
         <v>1417</v>
       </c>
       <c r="I201">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="K201" t="s">
         <v>1421</v>
@@ -12390,7 +12390,7 @@
         <v>1417</v>
       </c>
       <c r="I202">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="K202" t="s">
         <v>1421</v>
@@ -12469,7 +12469,7 @@
         <v>1417</v>
       </c>
       <c r="I204">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="K204" t="s">
         <v>1420</v>
@@ -12507,7 +12507,7 @@
         <v>1417</v>
       </c>
       <c r="I205">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="K205" t="s">
         <v>1420</v>
@@ -12574,7 +12574,7 @@
         <v>1417</v>
       </c>
       <c r="I207">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="J207">
         <v>167</v>
@@ -12618,7 +12618,7 @@
         <v>1417</v>
       </c>
       <c r="I208">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="J208">
         <v>45</v>
@@ -12662,7 +12662,7 @@
         <v>1417</v>
       </c>
       <c r="I209">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J209">
         <v>191</v>
@@ -12706,7 +12706,7 @@
         <v>1417</v>
       </c>
       <c r="I210">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="K210" t="s">
         <v>1424</v>
@@ -12802,7 +12802,7 @@
         <v>1417</v>
       </c>
       <c r="I213">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="K213" t="s">
         <v>1421</v>
@@ -12840,7 +12840,7 @@
         <v>1417</v>
       </c>
       <c r="I214">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="J214">
         <v>14</v>
@@ -12887,7 +12887,7 @@
         <v>1417</v>
       </c>
       <c r="I215">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="K215" t="s">
         <v>1421</v>
@@ -12954,7 +12954,7 @@
         <v>1417</v>
       </c>
       <c r="I217">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="J217">
         <v>42</v>
@@ -12998,7 +12998,7 @@
         <v>1417</v>
       </c>
       <c r="I218">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="J218">
         <v>166</v>
@@ -13086,7 +13086,7 @@
         <v>1417</v>
       </c>
       <c r="I220">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="J220">
         <v>154</v>
@@ -13472,7 +13472,7 @@
         <v>1417</v>
       </c>
       <c r="I230">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="J230">
         <v>197</v>
@@ -13516,7 +13516,7 @@
         <v>1417</v>
       </c>
       <c r="I231">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="J231">
         <v>35</v>
@@ -13618,7 +13618,7 @@
         <v>1417</v>
       </c>
       <c r="I234">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="J234">
         <v>35</v>
@@ -13665,7 +13665,7 @@
         <v>1417</v>
       </c>
       <c r="I235">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="J235">
         <v>35</v>
@@ -13712,7 +13712,7 @@
         <v>1417</v>
       </c>
       <c r="I236">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="J236">
         <v>86</v>
@@ -13829,7 +13829,7 @@
         <v>1417</v>
       </c>
       <c r="I239">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="K239" t="s">
         <v>1394</v>
@@ -13928,7 +13928,7 @@
         <v>1417</v>
       </c>
       <c r="I242">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="K242" t="s">
         <v>1420</v>
@@ -13995,7 +13995,7 @@
         <v>1417</v>
       </c>
       <c r="I244">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="J244">
         <v>15</v>
@@ -14036,7 +14036,7 @@
         <v>1417</v>
       </c>
       <c r="I245">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="J245">
         <v>15</v>
@@ -14179,7 +14179,7 @@
         <v>1417</v>
       </c>
       <c r="I249">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="K249" t="s">
         <v>1421</v>
@@ -14313,7 +14313,7 @@
         <v>1417</v>
       </c>
       <c r="I253">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="J253">
         <v>162</v>
@@ -14357,7 +14357,7 @@
         <v>1417</v>
       </c>
       <c r="I254">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="K254" t="s">
         <v>1424</v>
@@ -14436,7 +14436,7 @@
         <v>1417</v>
       </c>
       <c r="I256">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="J256">
         <v>23</v>
@@ -14620,7 +14620,7 @@
         <v>1417</v>
       </c>
       <c r="I261">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="J261">
         <v>162</v>
@@ -14778,7 +14778,7 @@
         <v>1417</v>
       </c>
       <c r="I265">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="J265">
         <v>162</v>
@@ -14863,7 +14863,7 @@
         <v>1417</v>
       </c>
       <c r="I267">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="K267" t="s">
         <v>1424</v>
@@ -14901,7 +14901,7 @@
         <v>1417</v>
       </c>
       <c r="I268">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="K268" t="s">
         <v>1421</v>
@@ -14936,7 +14936,7 @@
         <v>1417</v>
       </c>
       <c r="I269">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="K269" t="s">
         <v>1421</v>
@@ -14974,7 +14974,7 @@
         <v>1417</v>
       </c>
       <c r="I270">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="K270" t="s">
         <v>1424</v>
@@ -15012,7 +15012,7 @@
         <v>1417</v>
       </c>
       <c r="I271">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="K271" t="s">
         <v>1424</v>
@@ -15190,7 +15190,7 @@
         <v>1417</v>
       </c>
       <c r="I276">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="K276" t="s">
         <v>1425</v>
@@ -15228,7 +15228,7 @@
         <v>1417</v>
       </c>
       <c r="I277">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="K277" t="s">
         <v>1421</v>
@@ -15266,7 +15266,7 @@
         <v>1417</v>
       </c>
       <c r="I278">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="J278">
         <v>148</v>
@@ -15310,7 +15310,7 @@
         <v>1417</v>
       </c>
       <c r="I279">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="K279" t="s">
         <v>1423</v>
@@ -15351,7 +15351,7 @@
         <v>1417</v>
       </c>
       <c r="I280">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="K280" t="s">
         <v>1421</v>
@@ -15389,7 +15389,7 @@
         <v>1417</v>
       </c>
       <c r="I281">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="K281" t="s">
         <v>1421</v>
@@ -15430,7 +15430,7 @@
         <v>1417</v>
       </c>
       <c r="I282">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="K282" t="s">
         <v>1421</v>
@@ -15724,7 +15724,7 @@
         <v>1417</v>
       </c>
       <c r="I291">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="J291">
         <v>20</v>
@@ -15768,7 +15768,7 @@
         <v>1417</v>
       </c>
       <c r="I292">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="K292" t="s">
         <v>1424</v>
@@ -15806,7 +15806,7 @@
         <v>1417</v>
       </c>
       <c r="I293">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="K293" t="s">
         <v>1425</v>
@@ -15844,7 +15844,7 @@
         <v>1417</v>
       </c>
       <c r="I294">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="K294" t="s">
         <v>1430</v>
@@ -15981,7 +15981,7 @@
         <v>1417</v>
       </c>
       <c r="I298">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="J298">
         <v>58</v>
@@ -16145,7 +16145,7 @@
         <v>1417</v>
       </c>
       <c r="I302">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="K302" t="s">
         <v>1424</v>
@@ -16183,7 +16183,7 @@
         <v>1417</v>
       </c>
       <c r="I303">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="K303" t="s">
         <v>1421</v>
@@ -16221,7 +16221,7 @@
         <v>1417</v>
       </c>
       <c r="I304">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="K304" t="s">
         <v>1424</v>
@@ -16259,7 +16259,7 @@
         <v>1417</v>
       </c>
       <c r="I305">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="J305">
         <v>35</v>
@@ -16303,7 +16303,7 @@
         <v>1417</v>
       </c>
       <c r="I306">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="J306">
         <v>31</v>
@@ -16391,7 +16391,7 @@
         <v>1417</v>
       </c>
       <c r="I308">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="K308" t="s">
         <v>1420</v>
@@ -16508,7 +16508,7 @@
         <v>1417</v>
       </c>
       <c r="I311">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="K311" t="s">
         <v>1420</v>
@@ -16838,7 +16838,7 @@
         <v>1417</v>
       </c>
       <c r="I320">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="K320" t="s">
         <v>1425</v>
@@ -16876,7 +16876,7 @@
         <v>1417</v>
       </c>
       <c r="I321">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="K321" t="s">
         <v>1421</v>
@@ -16914,7 +16914,7 @@
         <v>1417</v>
       </c>
       <c r="I322">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="J322">
         <v>57</v>
@@ -17028,7 +17028,7 @@
         <v>1417</v>
       </c>
       <c r="I325">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="J325">
         <v>57</v>
@@ -17110,7 +17110,7 @@
         <v>1417</v>
       </c>
       <c r="I327">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="J327">
         <v>57</v>
@@ -17154,7 +17154,7 @@
         <v>1417</v>
       </c>
       <c r="I328">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="J328">
         <v>57</v>
@@ -17198,7 +17198,7 @@
         <v>1417</v>
       </c>
       <c r="I329">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="J329">
         <v>57</v>
@@ -17242,7 +17242,7 @@
         <v>1417</v>
       </c>
       <c r="I330">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="J330">
         <v>57</v>
@@ -17286,7 +17286,7 @@
         <v>1417</v>
       </c>
       <c r="I331">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="K331" t="s">
         <v>1420</v>
@@ -17324,7 +17324,7 @@
         <v>1417</v>
       </c>
       <c r="I332">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="K332" t="s">
         <v>1421</v>
@@ -17362,7 +17362,7 @@
         <v>1417</v>
       </c>
       <c r="I333">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="J333">
         <v>100</v>
@@ -17406,7 +17406,7 @@
         <v>1417</v>
       </c>
       <c r="I334">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="K334" t="s">
         <v>1421</v>
@@ -17631,7 +17631,7 @@
         <v>1417</v>
       </c>
       <c r="I340">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="J340">
         <v>98</v>
@@ -17672,7 +17672,7 @@
         <v>1417</v>
       </c>
       <c r="I341">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="J341">
         <v>90</v>
@@ -17713,7 +17713,7 @@
         <v>1417</v>
       </c>
       <c r="I342">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="K342" t="s">
         <v>1420</v>
@@ -17827,7 +17827,7 @@
         <v>1417</v>
       </c>
       <c r="I345">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="K345" t="s">
         <v>1420</v>
@@ -17947,7 +17947,7 @@
         <v>1417</v>
       </c>
       <c r="I348">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="J348">
         <v>14</v>
@@ -17991,7 +17991,7 @@
         <v>1417</v>
       </c>
       <c r="I349">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="K349" t="s">
         <v>1425</v>
@@ -18029,7 +18029,7 @@
         <v>1417</v>
       </c>
       <c r="I350">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="J350">
         <v>46</v>
@@ -18067,7 +18067,7 @@
         <v>1417</v>
       </c>
       <c r="I351">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="J351">
         <v>82</v>
@@ -18111,7 +18111,7 @@
         <v>1417</v>
       </c>
       <c r="I352">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="J352">
         <v>78</v>
@@ -18155,7 +18155,7 @@
         <v>1417</v>
       </c>
       <c r="I353">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="J353">
         <v>83</v>
@@ -18199,7 +18199,7 @@
         <v>1417</v>
       </c>
       <c r="I354">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="K354" t="s">
         <v>1424</v>
@@ -18237,7 +18237,7 @@
         <v>1417</v>
       </c>
       <c r="I355">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="J355">
         <v>8</v>
@@ -18319,7 +18319,7 @@
         <v>1417</v>
       </c>
       <c r="I357">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="J357">
         <v>85</v>
@@ -18442,7 +18442,7 @@
         <v>1417</v>
       </c>
       <c r="I360">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="J360">
         <v>83</v>
@@ -18489,7 +18489,7 @@
         <v>1417</v>
       </c>
       <c r="I361">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="J361">
         <v>83</v>
@@ -18533,7 +18533,7 @@
         <v>1417</v>
       </c>
       <c r="I362">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="K362" t="s">
         <v>1424</v>
@@ -18571,7 +18571,7 @@
         <v>1417</v>
       </c>
       <c r="I363">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="K363" t="s">
         <v>1424</v>
@@ -18609,7 +18609,7 @@
         <v>1417</v>
       </c>
       <c r="I364">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="J364">
         <v>83</v>
@@ -18653,7 +18653,7 @@
         <v>1417</v>
       </c>
       <c r="I365">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="J365">
         <v>15</v>
@@ -18776,7 +18776,7 @@
         <v>1417</v>
       </c>
       <c r="I368">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="J368">
         <v>77</v>
@@ -18820,7 +18820,7 @@
         <v>1417</v>
       </c>
       <c r="I369">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="K369" t="s">
         <v>1424</v>
@@ -18858,7 +18858,7 @@
         <v>1417</v>
       </c>
       <c r="I370">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="K370" t="s">
         <v>1424</v>
@@ -18896,7 +18896,7 @@
         <v>1417</v>
       </c>
       <c r="I371">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="J371">
         <v>16</v>
@@ -18984,7 +18984,7 @@
         <v>1417</v>
       </c>
       <c r="I373">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="K373" t="s">
         <v>1420</v>
@@ -19022,7 +19022,7 @@
         <v>1417</v>
       </c>
       <c r="I374">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="K374" t="s">
         <v>1420</v>
@@ -19060,7 +19060,7 @@
         <v>1417</v>
       </c>
       <c r="I375">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="J375">
         <v>94</v>
@@ -19101,7 +19101,7 @@
         <v>1417</v>
       </c>
       <c r="I376">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="K376" t="s">
         <v>1424</v>
@@ -19180,7 +19180,7 @@
         <v>1417</v>
       </c>
       <c r="I378">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="K378" t="s">
         <v>1424</v>
@@ -19218,7 +19218,7 @@
         <v>1417</v>
       </c>
       <c r="I379">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="J379">
         <v>20</v>
@@ -19262,7 +19262,7 @@
         <v>1417</v>
       </c>
       <c r="I380">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="J380">
         <v>94</v>
@@ -19306,7 +19306,7 @@
         <v>1417</v>
       </c>
       <c r="I381">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="K381" t="s">
         <v>1424</v>
@@ -19344,7 +19344,7 @@
         <v>1417</v>
       </c>
       <c r="I382">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="K382" t="s">
         <v>1424</v>
@@ -19382,7 +19382,7 @@
         <v>1417</v>
       </c>
       <c r="I383">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="J383">
         <v>71</v>
@@ -19426,7 +19426,7 @@
         <v>1417</v>
       </c>
       <c r="I384">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="K384" t="s">
         <v>1421</v>
@@ -19508,7 +19508,7 @@
         <v>1417</v>
       </c>
       <c r="I386">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="K386" t="s">
         <v>1424</v>
@@ -19546,7 +19546,7 @@
         <v>1417</v>
       </c>
       <c r="I387">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="K387" t="s">
         <v>1424</v>
@@ -19584,7 +19584,7 @@
         <v>1417</v>
       </c>
       <c r="I388">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="J388">
         <v>-85</v>
@@ -19628,7 +19628,7 @@
         <v>1417</v>
       </c>
       <c r="I389">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="K389" t="s">
         <v>1425</v>
@@ -20079,7 +20079,7 @@
         <v>1417</v>
       </c>
       <c r="I400">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="K400" t="s">
         <v>1424</v>
@@ -20155,7 +20155,7 @@
         <v>1417</v>
       </c>
       <c r="I402">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="K402" t="s">
         <v>1424</v>
@@ -20193,7 +20193,7 @@
         <v>1417</v>
       </c>
       <c r="I403">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="J403">
         <v>83</v>
@@ -20237,7 +20237,7 @@
         <v>1417</v>
       </c>
       <c r="I404">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="K404" t="s">
         <v>1424</v>
@@ -20307,7 +20307,7 @@
         <v>1417</v>
       </c>
       <c r="I406">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="Q406" t="b">
         <v>1</v>
@@ -20339,7 +20339,7 @@
         <v>1417</v>
       </c>
       <c r="I407">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="Q407" t="b">
         <v>1</v>
@@ -20371,7 +20371,7 @@
         <v>1417</v>
       </c>
       <c r="I408">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="Q408" t="b">
         <v>1</v>
@@ -20403,7 +20403,7 @@
         <v>1417</v>
       </c>
       <c r="I409">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="Q409" t="b">
         <v>1</v>
@@ -20435,7 +20435,7 @@
         <v>1417</v>
       </c>
       <c r="I410">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="Q410" t="b">
         <v>1</v>
@@ -20467,7 +20467,7 @@
         <v>1417</v>
       </c>
       <c r="I411">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="Q411" t="b">
         <v>1</v>
@@ -20499,7 +20499,7 @@
         <v>1417</v>
       </c>
       <c r="I412">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="Q412" t="b">
         <v>1</v>
@@ -20531,7 +20531,7 @@
         <v>1417</v>
       </c>
       <c r="I413">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="Q413" t="b">
         <v>1</v>
@@ -20621,7 +20621,7 @@
         <v>1417</v>
       </c>
       <c r="I416">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="Q416" t="b">
         <v>1</v>
@@ -20711,7 +20711,7 @@
         <v>1417</v>
       </c>
       <c r="I419">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="Q419" t="b">
         <v>1</v>
@@ -20743,7 +20743,7 @@
         <v>1417</v>
       </c>
       <c r="I420">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="Q420" t="b">
         <v>1</v>
@@ -20775,7 +20775,7 @@
         <v>1417</v>
       </c>
       <c r="I421">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="Q421" t="b">
         <v>1</v>
@@ -20807,7 +20807,7 @@
         <v>1417</v>
       </c>
       <c r="I422">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="Q422" t="b">
         <v>1</v>
@@ -20839,7 +20839,7 @@
         <v>1417</v>
       </c>
       <c r="I423">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="Q423" t="b">
         <v>1</v>
@@ -20871,7 +20871,7 @@
         <v>1417</v>
       </c>
       <c r="I424">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="Q424" t="b">
         <v>1</v>
@@ -20903,7 +20903,7 @@
         <v>1417</v>
       </c>
       <c r="I425">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="Q425" t="b">
         <v>1</v>
@@ -20935,7 +20935,7 @@
         <v>1417</v>
       </c>
       <c r="I426">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="Q426" t="b">
         <v>1</v>
@@ -20967,7 +20967,7 @@
         <v>1417</v>
       </c>
       <c r="I427">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="Q427" t="b">
         <v>1</v>
@@ -21057,7 +21057,7 @@
         <v>1417</v>
       </c>
       <c r="I430">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="Q430" t="b">
         <v>1</v>
@@ -21089,7 +21089,7 @@
         <v>1417</v>
       </c>
       <c r="I431">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="Q431" t="b">
         <v>1</v>
@@ -21121,7 +21121,7 @@
         <v>1417</v>
       </c>
       <c r="I432">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="Q432" t="b">
         <v>1</v>
@@ -21153,7 +21153,7 @@
         <v>1417</v>
       </c>
       <c r="I433">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="Q433" t="b">
         <v>1</v>
@@ -21185,7 +21185,7 @@
         <v>1417</v>
       </c>
       <c r="I434">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="Q434" t="b">
         <v>1</v>
@@ -21217,7 +21217,7 @@
         <v>1417</v>
       </c>
       <c r="I435">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="Q435" t="b">
         <v>1</v>
@@ -21249,7 +21249,7 @@
         <v>1417</v>
       </c>
       <c r="I436">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="Q436" t="b">
         <v>1</v>
@@ -21281,7 +21281,7 @@
         <v>1419</v>
       </c>
       <c r="I437">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="Q437" t="b">
         <v>1</v>
@@ -21313,7 +21313,7 @@
         <v>1419</v>
       </c>
       <c r="I438">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="Q438" t="b">
         <v>1</v>
@@ -21345,7 +21345,7 @@
         <v>1417</v>
       </c>
       <c r="I439">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="Q439" t="b">
         <v>1</v>
@@ -21377,7 +21377,7 @@
         <v>1417</v>
       </c>
       <c r="I440">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="Q440" t="b">
         <v>1</v>
@@ -21409,7 +21409,7 @@
         <v>1417</v>
       </c>
       <c r="I441">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="Q441" t="b">
         <v>1</v>
@@ -21470,7 +21470,7 @@
         <v>1417</v>
       </c>
       <c r="I443">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="Q443" t="b">
         <v>1</v>
@@ -21560,7 +21560,7 @@
         <v>1417</v>
       </c>
       <c r="I446">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="Q446" t="b">
         <v>1</v>
@@ -21592,7 +21592,7 @@
         <v>1417</v>
       </c>
       <c r="I447">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="Q447" t="b">
         <v>1</v>
@@ -21624,7 +21624,7 @@
         <v>1417</v>
       </c>
       <c r="I448">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="Q448" t="b">
         <v>1</v>
@@ -21656,7 +21656,7 @@
         <v>1417</v>
       </c>
       <c r="I449">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="Q449" t="b">
         <v>1</v>
@@ -21688,7 +21688,7 @@
         <v>1417</v>
       </c>
       <c r="I450">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="Q450" t="b">
         <v>1</v>
@@ -21720,7 +21720,7 @@
         <v>1417</v>
       </c>
       <c r="I451">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q451" t="b">
         <v>1</v>
@@ -21781,7 +21781,7 @@
         <v>1417</v>
       </c>
       <c r="I453">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q453" t="b">
         <v>1</v>
@@ -21813,7 +21813,7 @@
         <v>1417</v>
       </c>
       <c r="I454">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q454" t="b">
         <v>1</v>
@@ -21845,7 +21845,7 @@
         <v>1417</v>
       </c>
       <c r="I455">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q455" t="b">
         <v>1</v>
@@ -21906,7 +21906,7 @@
         <v>1417</v>
       </c>
       <c r="I457">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q457" t="b">
         <v>1</v>
@@ -21938,7 +21938,7 @@
         <v>1417</v>
       </c>
       <c r="I458">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q458" t="b">
         <v>1</v>
@@ -21970,7 +21970,7 @@
         <v>1417</v>
       </c>
       <c r="I459">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="Q459" t="b">
         <v>1</v>
@@ -22002,7 +22002,7 @@
         <v>1417</v>
       </c>
       <c r="I460">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="Q460" t="b">
         <v>1</v>
@@ -22034,7 +22034,7 @@
         <v>1417</v>
       </c>
       <c r="I461">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="Q461" t="b">
         <v>1</v>
@@ -22066,7 +22066,7 @@
         <v>1417</v>
       </c>
       <c r="I462">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="Q462" t="b">
         <v>1</v>
@@ -22098,7 +22098,7 @@
         <v>1417</v>
       </c>
       <c r="I463">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="Q463" t="b">
         <v>1</v>
@@ -22130,7 +22130,7 @@
         <v>1417</v>
       </c>
       <c r="I464">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q464" t="b">
         <v>1</v>
@@ -22162,7 +22162,7 @@
         <v>1417</v>
       </c>
       <c r="I465">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q465" t="b">
         <v>1</v>
@@ -22194,7 +22194,7 @@
         <v>1417</v>
       </c>
       <c r="I466">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q466" t="b">
         <v>1</v>
@@ -22226,7 +22226,7 @@
         <v>1417</v>
       </c>
       <c r="I467">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q467" t="b">
         <v>1</v>
@@ -22258,7 +22258,7 @@
         <v>1417</v>
       </c>
       <c r="I468">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q468" t="b">
         <v>1</v>
@@ -22290,7 +22290,7 @@
         <v>1417</v>
       </c>
       <c r="I469">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q469" t="b">
         <v>1</v>
@@ -22351,7 +22351,7 @@
         <v>1417</v>
       </c>
       <c r="I471">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q471" t="b">
         <v>1</v>
@@ -22383,7 +22383,7 @@
         <v>1417</v>
       </c>
       <c r="I472">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q472" t="b">
         <v>1</v>
@@ -22415,7 +22415,7 @@
         <v>1417</v>
       </c>
       <c r="I473">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q473" t="b">
         <v>1</v>
@@ -22447,7 +22447,7 @@
         <v>1417</v>
       </c>
       <c r="I474">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q474" t="b">
         <v>1</v>
@@ -22479,7 +22479,7 @@
         <v>1417</v>
       </c>
       <c r="I475">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q475" t="b">
         <v>1</v>
@@ -22511,7 +22511,7 @@
         <v>1417</v>
       </c>
       <c r="I476">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q476" t="b">
         <v>1</v>
@@ -22543,7 +22543,7 @@
         <v>1417</v>
       </c>
       <c r="I477">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q477" t="b">
         <v>1</v>
@@ -22575,7 +22575,7 @@
         <v>1417</v>
       </c>
       <c r="I478">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q478" t="b">
         <v>1</v>
@@ -22607,7 +22607,7 @@
         <v>1417</v>
       </c>
       <c r="I479">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q479" t="b">
         <v>1</v>
@@ -22639,7 +22639,7 @@
         <v>1417</v>
       </c>
       <c r="I480">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q480" t="b">
         <v>1</v>
@@ -22671,7 +22671,7 @@
         <v>1417</v>
       </c>
       <c r="I481">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q481" t="b">
         <v>1</v>
@@ -22703,7 +22703,7 @@
         <v>1417</v>
       </c>
       <c r="I482">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q482" t="b">
         <v>1</v>
@@ -22735,7 +22735,7 @@
         <v>1417</v>
       </c>
       <c r="I483">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q483" t="b">
         <v>1</v>
@@ -22767,7 +22767,7 @@
         <v>1417</v>
       </c>
       <c r="I484">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q484" t="b">
         <v>1</v>
@@ -22799,7 +22799,7 @@
         <v>1417</v>
       </c>
       <c r="I485">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q485" t="b">
         <v>1</v>
@@ -22831,7 +22831,7 @@
         <v>1417</v>
       </c>
       <c r="I486">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q486" t="b">
         <v>1</v>
@@ -22863,7 +22863,7 @@
         <v>1417</v>
       </c>
       <c r="I487">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q487" t="b">
         <v>1</v>
@@ -22895,7 +22895,7 @@
         <v>1417</v>
       </c>
       <c r="I488">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q488" t="b">
         <v>1</v>
@@ -22927,7 +22927,7 @@
         <v>1417</v>
       </c>
       <c r="I489">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q489" t="b">
         <v>1</v>
@@ -22959,7 +22959,7 @@
         <v>1417</v>
       </c>
       <c r="I490">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q490" t="b">
         <v>1</v>
@@ -22991,7 +22991,7 @@
         <v>1417</v>
       </c>
       <c r="I491">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q491" t="b">
         <v>1</v>
@@ -23023,7 +23023,7 @@
         <v>1419</v>
       </c>
       <c r="I492">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q492" t="b">
         <v>1</v>
@@ -23055,7 +23055,7 @@
         <v>1419</v>
       </c>
       <c r="I493">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q493" t="b">
         <v>1</v>
@@ -23087,7 +23087,7 @@
         <v>1419</v>
       </c>
       <c r="I494">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q494" t="b">
         <v>1</v>
@@ -23119,7 +23119,7 @@
         <v>1419</v>
       </c>
       <c r="I495">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q495" t="b">
         <v>1</v>
@@ -23151,7 +23151,7 @@
         <v>1419</v>
       </c>
       <c r="I496">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q496" t="b">
         <v>1</v>
@@ -23183,7 +23183,7 @@
         <v>1417</v>
       </c>
       <c r="I497">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q497" t="b">
         <v>1</v>
@@ -23215,7 +23215,7 @@
         <v>1417</v>
       </c>
       <c r="I498">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q498" t="b">
         <v>1</v>
@@ -23247,7 +23247,7 @@
         <v>1419</v>
       </c>
       <c r="I499">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q499" t="b">
         <v>1</v>
@@ -23279,7 +23279,7 @@
         <v>1417</v>
       </c>
       <c r="I500">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q500" t="b">
         <v>1</v>
@@ -23311,7 +23311,7 @@
         <v>1417</v>
       </c>
       <c r="I501">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q501" t="b">
         <v>1</v>
@@ -23343,7 +23343,7 @@
         <v>1417</v>
       </c>
       <c r="I502">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q502" t="b">
         <v>1</v>
@@ -23375,7 +23375,7 @@
         <v>1417</v>
       </c>
       <c r="I503">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q503" t="b">
         <v>1</v>
@@ -23407,7 +23407,7 @@
         <v>1417</v>
       </c>
       <c r="I504">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="Q504" t="b">
         <v>1</v>
@@ -23439,7 +23439,7 @@
         <v>1417</v>
       </c>
       <c r="I505">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="Q505" t="b">
         <v>1</v>
@@ -23471,7 +23471,7 @@
         <v>1417</v>
       </c>
       <c r="I506">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="Q506" t="b">
         <v>1</v>
@@ -23503,7 +23503,7 @@
         <v>1417</v>
       </c>
       <c r="I507">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Q507" t="b">
         <v>1</v>
@@ -23564,7 +23564,7 @@
         <v>1417</v>
       </c>
       <c r="I509">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Q509" t="b">
         <v>1</v>
@@ -23596,7 +23596,7 @@
         <v>1417</v>
       </c>
       <c r="I510">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Q510" t="b">
         <v>1</v>
@@ -23628,7 +23628,7 @@
         <v>1417</v>
       </c>
       <c r="I511">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="Q511" t="b">
         <v>1</v>
@@ -23660,7 +23660,7 @@
         <v>1417</v>
       </c>
       <c r="I512">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="Q512" t="b">
         <v>1</v>
@@ -23692,7 +23692,7 @@
         <v>1417</v>
       </c>
       <c r="I513">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="Q513" t="b">
         <v>1</v>
@@ -23753,7 +23753,7 @@
         <v>1417</v>
       </c>
       <c r="I515">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="Q515" t="b">
         <v>1</v>
@@ -23785,7 +23785,7 @@
         <v>1417</v>
       </c>
       <c r="I516">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Q516" t="b">
         <v>1</v>
@@ -23817,7 +23817,7 @@
         <v>1417</v>
       </c>
       <c r="I517">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Q517" t="b">
         <v>1</v>
@@ -23849,7 +23849,7 @@
         <v>1417</v>
       </c>
       <c r="I518">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Q518" t="b">
         <v>1</v>
@@ -23881,7 +23881,7 @@
         <v>1417</v>
       </c>
       <c r="I519">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="Q519" t="b">
         <v>1</v>
@@ -23913,7 +23913,7 @@
         <v>1417</v>
       </c>
       <c r="I520">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="Q520" t="b">
         <v>1</v>
@@ -23945,7 +23945,7 @@
         <v>1417</v>
       </c>
       <c r="I521">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="Q521" t="b">
         <v>1</v>
@@ -23977,7 +23977,7 @@
         <v>1417</v>
       </c>
       <c r="I522">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="Q522" t="b">
         <v>1</v>
@@ -24009,7 +24009,7 @@
         <v>1417</v>
       </c>
       <c r="I523">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="Q523" t="b">
         <v>1</v>
@@ -24041,7 +24041,7 @@
         <v>1417</v>
       </c>
       <c r="I524">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q524" t="b">
         <v>1</v>
@@ -24073,7 +24073,7 @@
         <v>1417</v>
       </c>
       <c r="I525">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q525" t="b">
         <v>1</v>
@@ -24105,7 +24105,7 @@
         <v>1417</v>
       </c>
       <c r="I526">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q526" t="b">
         <v>1</v>
@@ -24137,7 +24137,7 @@
         <v>1417</v>
       </c>
       <c r="I527">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q527" t="b">
         <v>1</v>
@@ -24169,7 +24169,7 @@
         <v>1417</v>
       </c>
       <c r="I528">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="Q528" t="b">
         <v>1</v>
@@ -24201,7 +24201,7 @@
         <v>1417</v>
       </c>
       <c r="I529">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="Q529" t="b">
         <v>1</v>
@@ -24233,7 +24233,7 @@
         <v>1417</v>
       </c>
       <c r="I530">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="Q530" t="b">
         <v>1</v>
@@ -24265,7 +24265,7 @@
         <v>1417</v>
       </c>
       <c r="I531">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="Q531" t="b">
         <v>1</v>
@@ -24297,7 +24297,7 @@
         <v>1417</v>
       </c>
       <c r="I532">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="Q532" t="b">
         <v>1</v>
@@ -24329,7 +24329,7 @@
         <v>1417</v>
       </c>
       <c r="I533">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="Q533" t="b">
         <v>1</v>
@@ -24361,7 +24361,7 @@
         <v>1417</v>
       </c>
       <c r="I534">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="Q534" t="b">
         <v>1</v>
@@ -24393,7 +24393,7 @@
         <v>1417</v>
       </c>
       <c r="I535">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="Q535" t="b">
         <v>1</v>
@@ -24425,7 +24425,7 @@
         <v>1417</v>
       </c>
       <c r="I536">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="Q536" t="b">
         <v>1</v>
@@ -24457,7 +24457,7 @@
         <v>1417</v>
       </c>
       <c r="I537">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="Q537" t="b">
         <v>1</v>
@@ -24489,7 +24489,7 @@
         <v>1417</v>
       </c>
       <c r="I538">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="Q538" t="b">
         <v>1</v>
@@ -24521,7 +24521,7 @@
         <v>1417</v>
       </c>
       <c r="I539">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="Q539" t="b">
         <v>1</v>
@@ -24553,7 +24553,7 @@
         <v>1417</v>
       </c>
       <c r="I540">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="Q540" t="b">
         <v>1</v>
@@ -24585,7 +24585,7 @@
         <v>1417</v>
       </c>
       <c r="I541">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="Q541" t="b">
         <v>1</v>
@@ -24617,7 +24617,7 @@
         <v>1417</v>
       </c>
       <c r="I542">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="Q542" t="b">
         <v>1</v>
@@ -24649,7 +24649,7 @@
         <v>1417</v>
       </c>
       <c r="I543">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="Q543" t="b">
         <v>1</v>
@@ -24681,7 +24681,7 @@
         <v>1417</v>
       </c>
       <c r="I544">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="Q544" t="b">
         <v>1</v>
@@ -24713,7 +24713,7 @@
         <v>1417</v>
       </c>
       <c r="I545">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="Q545" t="b">
         <v>1</v>
@@ -24745,7 +24745,7 @@
         <v>1417</v>
       </c>
       <c r="I546">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q546" t="b">
         <v>1</v>
@@ -24777,7 +24777,7 @@
         <v>1417</v>
       </c>
       <c r="I547">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q547" t="b">
         <v>1</v>
@@ -24809,7 +24809,7 @@
         <v>1417</v>
       </c>
       <c r="I548">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q548" t="b">
         <v>1</v>
@@ -24841,7 +24841,7 @@
         <v>1417</v>
       </c>
       <c r="I549">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q549" t="b">
         <v>1</v>
@@ -24873,7 +24873,7 @@
         <v>1417</v>
       </c>
       <c r="I550">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q550" t="b">
         <v>1</v>
@@ -24905,7 +24905,7 @@
         <v>1417</v>
       </c>
       <c r="I551">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q551" t="b">
         <v>1</v>
@@ -24937,7 +24937,7 @@
         <v>1417</v>
       </c>
       <c r="I552">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q552" t="b">
         <v>1</v>
@@ -24969,7 +24969,7 @@
         <v>1417</v>
       </c>
       <c r="I553">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q553" t="b">
         <v>1</v>
@@ -25001,7 +25001,7 @@
         <v>1417</v>
       </c>
       <c r="I554">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q554" t="b">
         <v>1</v>
@@ -25033,7 +25033,7 @@
         <v>1417</v>
       </c>
       <c r="I555">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q555" t="b">
         <v>1</v>
@@ -25065,7 +25065,7 @@
         <v>1417</v>
       </c>
       <c r="I556">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q556" t="b">
         <v>1</v>
@@ -25097,7 +25097,7 @@
         <v>1417</v>
       </c>
       <c r="I557">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Q557" t="b">
         <v>1</v>
@@ -25129,7 +25129,7 @@
         <v>1417</v>
       </c>
       <c r="I558">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Q558" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: reparaveis (21/10/2026 12:57)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
@@ -5132,7 +5132,7 @@
         <v>1417</v>
       </c>
       <c r="I2">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="K2" t="s">
         <v>1420</v>
@@ -5170,7 +5170,7 @@
         <v>1417</v>
       </c>
       <c r="I3">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="K3" t="s">
         <v>1421</v>
@@ -5208,7 +5208,7 @@
         <v>1417</v>
       </c>
       <c r="I4">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="K4" t="s">
         <v>1421</v>
@@ -5246,7 +5246,7 @@
         <v>1417</v>
       </c>
       <c r="I5">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="J5">
         <v>279</v>
@@ -5290,7 +5290,7 @@
         <v>1417</v>
       </c>
       <c r="I6">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="J6">
         <v>153</v>
@@ -5334,7 +5334,7 @@
         <v>1417</v>
       </c>
       <c r="I7">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="J7">
         <v>112</v>
@@ -5410,7 +5410,7 @@
         <v>1417</v>
       </c>
       <c r="I9">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="J9">
         <v>362</v>
@@ -5457,7 +5457,7 @@
         <v>1417</v>
       </c>
       <c r="I10">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="J10">
         <v>378</v>
@@ -5504,7 +5504,7 @@
         <v>1417</v>
       </c>
       <c r="I11">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="J11">
         <v>112</v>
@@ -5551,7 +5551,7 @@
         <v>1417</v>
       </c>
       <c r="I12">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="J12">
         <v>124</v>
@@ -5624,7 +5624,7 @@
         <v>1417</v>
       </c>
       <c r="I14">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="J14">
         <v>64</v>
@@ -5703,7 +5703,7 @@
         <v>1417</v>
       </c>
       <c r="I16">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="K16" t="s">
         <v>1420</v>
@@ -5741,7 +5741,7 @@
         <v>1417</v>
       </c>
       <c r="I17">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="J17">
         <v>161</v>
@@ -5785,7 +5785,7 @@
         <v>1417</v>
       </c>
       <c r="I18">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="J18">
         <v>66</v>
@@ -5858,7 +5858,7 @@
         <v>1417</v>
       </c>
       <c r="I20">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="J20">
         <v>399</v>
@@ -5931,7 +5931,7 @@
         <v>1417</v>
       </c>
       <c r="I22">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="K22" t="s">
         <v>1424</v>
@@ -5969,7 +5969,7 @@
         <v>1417</v>
       </c>
       <c r="I23">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="J23">
         <v>229</v>
@@ -6074,7 +6074,7 @@
         <v>1417</v>
       </c>
       <c r="I26">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="J26">
         <v>155</v>
@@ -6121,7 +6121,7 @@
         <v>1417</v>
       </c>
       <c r="I27">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="K27" t="s">
         <v>1424</v>
@@ -6217,7 +6217,7 @@
         <v>1417</v>
       </c>
       <c r="I30">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="J30">
         <v>209</v>
@@ -6290,7 +6290,7 @@
         <v>1417</v>
       </c>
       <c r="I32">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="K32" t="s">
         <v>1420</v>
@@ -6499,7 +6499,7 @@
         <v>1417</v>
       </c>
       <c r="I39">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="K39" t="s">
         <v>1425</v>
@@ -6662,7 +6662,7 @@
         <v>1417</v>
       </c>
       <c r="I44">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="J44">
         <v>87</v>
@@ -6709,7 +6709,7 @@
         <v>1417</v>
       </c>
       <c r="I45">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="J45">
         <v>331</v>
@@ -6756,7 +6756,7 @@
         <v>1417</v>
       </c>
       <c r="I46">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="K46" t="s">
         <v>1424</v>
@@ -6797,7 +6797,7 @@
         <v>1417</v>
       </c>
       <c r="I47">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="J47">
         <v>344</v>
@@ -6844,7 +6844,7 @@
         <v>1417</v>
       </c>
       <c r="I48">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="K48" t="s">
         <v>1424</v>
@@ -6911,7 +6911,7 @@
         <v>1417</v>
       </c>
       <c r="I50">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="K50" t="s">
         <v>1424</v>
@@ -6978,7 +6978,7 @@
         <v>1417</v>
       </c>
       <c r="I52">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="K52" t="s">
         <v>1420</v>
@@ -7016,7 +7016,7 @@
         <v>1417</v>
       </c>
       <c r="I53">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="K53" t="s">
         <v>1421</v>
@@ -7054,7 +7054,7 @@
         <v>1417</v>
       </c>
       <c r="I54">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="K54" t="s">
         <v>1421</v>
@@ -7330,7 +7330,7 @@
         <v>1417</v>
       </c>
       <c r="I63">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="J63">
         <v>293</v>
@@ -7377,7 +7377,7 @@
         <v>1417</v>
       </c>
       <c r="I64">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="J64">
         <v>320</v>
@@ -7607,7 +7607,7 @@
         <v>1417</v>
       </c>
       <c r="I71">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="J71">
         <v>429</v>
@@ -7680,7 +7680,7 @@
         <v>1417</v>
       </c>
       <c r="I73">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="K73" t="s">
         <v>1420</v>
@@ -7788,7 +7788,7 @@
         <v>1417</v>
       </c>
       <c r="I76">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="K76" t="s">
         <v>1427</v>
@@ -7881,7 +7881,7 @@
         <v>1417</v>
       </c>
       <c r="I79">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="K79" t="s">
         <v>1427</v>
@@ -7986,7 +7986,7 @@
         <v>1417</v>
       </c>
       <c r="I82">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="K82" t="s">
         <v>1424</v>
@@ -8053,7 +8053,7 @@
         <v>1417</v>
       </c>
       <c r="I84">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="J84">
         <v>40</v>
@@ -8100,7 +8100,7 @@
         <v>1417</v>
       </c>
       <c r="I85">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="K85" t="s">
         <v>1421</v>
@@ -8138,7 +8138,7 @@
         <v>1417</v>
       </c>
       <c r="I86">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="K86" t="s">
         <v>1421</v>
@@ -8176,7 +8176,7 @@
         <v>1417</v>
       </c>
       <c r="I87">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="J87">
         <v>-16</v>
@@ -8299,7 +8299,7 @@
         <v>1417</v>
       </c>
       <c r="I90">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="K90" t="s">
         <v>1394</v>
@@ -8448,7 +8448,7 @@
         <v>1417</v>
       </c>
       <c r="I94">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="K94" t="s">
         <v>1424</v>
@@ -8527,7 +8527,7 @@
         <v>1417</v>
       </c>
       <c r="I96">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="J96">
         <v>17</v>
@@ -8574,7 +8574,7 @@
         <v>1417</v>
       </c>
       <c r="I97">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="J97">
         <v>20</v>
@@ -8621,7 +8621,7 @@
         <v>1417</v>
       </c>
       <c r="I98">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="K98" t="s">
         <v>1424</v>
@@ -8898,7 +8898,7 @@
         <v>1417</v>
       </c>
       <c r="I106">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="J106">
         <v>49</v>
@@ -8942,7 +8942,7 @@
         <v>1417</v>
       </c>
       <c r="I107">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="J107">
         <v>36</v>
@@ -8986,7 +8986,7 @@
         <v>1417</v>
       </c>
       <c r="I108">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="K108" t="s">
         <v>1421</v>
@@ -9024,7 +9024,7 @@
         <v>1417</v>
       </c>
       <c r="I109">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="K109" t="s">
         <v>1421</v>
@@ -9207,7 +9207,7 @@
         <v>1417</v>
       </c>
       <c r="I115">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="K115" t="s">
         <v>1421</v>
@@ -9245,7 +9245,7 @@
         <v>1417</v>
       </c>
       <c r="I116">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="K116" t="s">
         <v>1421</v>
@@ -9283,7 +9283,7 @@
         <v>1417</v>
       </c>
       <c r="I117">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="K117" t="s">
         <v>1421</v>
@@ -9321,7 +9321,7 @@
         <v>1417</v>
       </c>
       <c r="I118">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="K118" t="s">
         <v>1421</v>
@@ -9359,7 +9359,7 @@
         <v>1417</v>
       </c>
       <c r="I119">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="K119" t="s">
         <v>1421</v>
@@ -9397,7 +9397,7 @@
         <v>1417</v>
       </c>
       <c r="I120">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="K120" t="s">
         <v>1421</v>
@@ -9435,7 +9435,7 @@
         <v>1417</v>
       </c>
       <c r="I121">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="J121">
         <v>251</v>
@@ -9482,7 +9482,7 @@
         <v>1417</v>
       </c>
       <c r="I122">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="K122" t="s">
         <v>1421</v>
@@ -9549,7 +9549,7 @@
         <v>1417</v>
       </c>
       <c r="I124">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="K124" t="s">
         <v>1421</v>
@@ -9587,7 +9587,7 @@
         <v>1417</v>
       </c>
       <c r="I125">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="K125" t="s">
         <v>1427</v>
@@ -9683,7 +9683,7 @@
         <v>1417</v>
       </c>
       <c r="I128">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="K128" t="s">
         <v>1421</v>
@@ -9721,7 +9721,7 @@
         <v>1417</v>
       </c>
       <c r="I129">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="K129" t="s">
         <v>1420</v>
@@ -9759,7 +9759,7 @@
         <v>1417</v>
       </c>
       <c r="I130">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="J130">
         <v>47</v>
@@ -9835,7 +9835,7 @@
         <v>1417</v>
       </c>
       <c r="I132">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="J132">
         <v>145</v>
@@ -9911,7 +9911,7 @@
         <v>1417</v>
       </c>
       <c r="I134">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="K134" t="s">
         <v>1420</v>
@@ -10036,7 +10036,7 @@
         <v>1417</v>
       </c>
       <c r="I138">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="K138" t="s">
         <v>1421</v>
@@ -10420,7 +10420,7 @@
         <v>1417</v>
       </c>
       <c r="I150">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="J150">
         <v>201</v>
@@ -10607,7 +10607,7 @@
         <v>1417</v>
       </c>
       <c r="I155">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="K155" t="s">
         <v>1427</v>
@@ -10642,7 +10642,7 @@
         <v>1417</v>
       </c>
       <c r="I156">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="K156" t="s">
         <v>1421</v>
@@ -10680,7 +10680,7 @@
         <v>1417</v>
       </c>
       <c r="I157">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="J157">
         <v>371</v>
@@ -10724,7 +10724,7 @@
         <v>1417</v>
       </c>
       <c r="I158">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="J158">
         <v>52</v>
@@ -10768,7 +10768,7 @@
         <v>1417</v>
       </c>
       <c r="I159">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="K159" t="s">
         <v>1421</v>
@@ -10806,7 +10806,7 @@
         <v>1417</v>
       </c>
       <c r="I160">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="K160" t="s">
         <v>1421</v>
@@ -10844,7 +10844,7 @@
         <v>1417</v>
       </c>
       <c r="I161">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="J161">
         <v>55</v>
@@ -10979,7 +10979,7 @@
         <v>1417</v>
       </c>
       <c r="I164">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="O164" t="s">
         <v>1533</v>
@@ -11154,7 +11154,7 @@
         <v>1417</v>
       </c>
       <c r="I169">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="K169" t="s">
         <v>1394</v>
@@ -11364,7 +11364,7 @@
         <v>1417</v>
       </c>
       <c r="I175">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="J175">
         <v>205</v>
@@ -11411,7 +11411,7 @@
         <v>1417</v>
       </c>
       <c r="I176">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="K176" t="s">
         <v>1421</v>
@@ -11449,7 +11449,7 @@
         <v>1417</v>
       </c>
       <c r="I177">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="J177">
         <v>44</v>
@@ -11496,7 +11496,7 @@
         <v>1417</v>
       </c>
       <c r="I178">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="K178" t="s">
         <v>1420</v>
@@ -11563,7 +11563,7 @@
         <v>1417</v>
       </c>
       <c r="I180">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="K180" t="s">
         <v>1420</v>
@@ -11659,7 +11659,7 @@
         <v>1417</v>
       </c>
       <c r="I183">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="K183" t="s">
         <v>1421</v>
@@ -11697,7 +11697,7 @@
         <v>1417</v>
       </c>
       <c r="I184">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="K184" t="s">
         <v>1427</v>
@@ -11732,7 +11732,7 @@
         <v>1417</v>
       </c>
       <c r="I185">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="K185" t="s">
         <v>1421</v>
@@ -11770,7 +11770,7 @@
         <v>1417</v>
       </c>
       <c r="I186">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="K186" t="s">
         <v>1421</v>
@@ -11808,7 +11808,7 @@
         <v>1417</v>
       </c>
       <c r="I187">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="J187">
         <v>75</v>
@@ -11855,7 +11855,7 @@
         <v>1417</v>
       </c>
       <c r="I188">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="J188">
         <v>40</v>
@@ -11902,7 +11902,7 @@
         <v>1417</v>
       </c>
       <c r="I189">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="J189">
         <v>155</v>
@@ -11946,7 +11946,7 @@
         <v>1417</v>
       </c>
       <c r="I190">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="J190">
         <v>107</v>
@@ -11990,7 +11990,7 @@
         <v>1417</v>
       </c>
       <c r="I191">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="J191">
         <v>5</v>
@@ -12034,7 +12034,7 @@
         <v>1417</v>
       </c>
       <c r="I192">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="K192" t="s">
         <v>1421</v>
@@ -12072,7 +12072,7 @@
         <v>1417</v>
       </c>
       <c r="I193">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="K193" t="s">
         <v>1426</v>
@@ -12267,7 +12267,7 @@
         <v>1417</v>
       </c>
       <c r="I199">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="J199">
         <v>70</v>
@@ -12352,7 +12352,7 @@
         <v>1417</v>
       </c>
       <c r="I201">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="K201" t="s">
         <v>1421</v>
@@ -12390,7 +12390,7 @@
         <v>1417</v>
       </c>
       <c r="I202">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="K202" t="s">
         <v>1421</v>
@@ -12469,7 +12469,7 @@
         <v>1417</v>
       </c>
       <c r="I204">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="K204" t="s">
         <v>1420</v>
@@ -12507,7 +12507,7 @@
         <v>1417</v>
       </c>
       <c r="I205">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="K205" t="s">
         <v>1420</v>
@@ -12574,7 +12574,7 @@
         <v>1417</v>
       </c>
       <c r="I207">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="J207">
         <v>167</v>
@@ -12618,7 +12618,7 @@
         <v>1417</v>
       </c>
       <c r="I208">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="J208">
         <v>45</v>
@@ -12662,7 +12662,7 @@
         <v>1417</v>
       </c>
       <c r="I209">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="J209">
         <v>191</v>
@@ -12706,7 +12706,7 @@
         <v>1417</v>
       </c>
       <c r="I210">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="K210" t="s">
         <v>1424</v>
@@ -12802,7 +12802,7 @@
         <v>1417</v>
       </c>
       <c r="I213">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="K213" t="s">
         <v>1421</v>
@@ -12840,7 +12840,7 @@
         <v>1417</v>
       </c>
       <c r="I214">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="J214">
         <v>14</v>
@@ -12887,7 +12887,7 @@
         <v>1417</v>
       </c>
       <c r="I215">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="K215" t="s">
         <v>1421</v>
@@ -12954,7 +12954,7 @@
         <v>1417</v>
       </c>
       <c r="I217">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="J217">
         <v>42</v>
@@ -12998,7 +12998,7 @@
         <v>1417</v>
       </c>
       <c r="I218">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="J218">
         <v>166</v>
@@ -13086,7 +13086,7 @@
         <v>1417</v>
       </c>
       <c r="I220">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="J220">
         <v>154</v>
@@ -13472,7 +13472,7 @@
         <v>1417</v>
       </c>
       <c r="I230">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="J230">
         <v>197</v>
@@ -13516,7 +13516,7 @@
         <v>1417</v>
       </c>
       <c r="I231">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="J231">
         <v>35</v>
@@ -13618,7 +13618,7 @@
         <v>1417</v>
       </c>
       <c r="I234">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="J234">
         <v>35</v>
@@ -13665,7 +13665,7 @@
         <v>1417</v>
       </c>
       <c r="I235">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="J235">
         <v>35</v>
@@ -13712,7 +13712,7 @@
         <v>1417</v>
       </c>
       <c r="I236">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="J236">
         <v>86</v>
@@ -13829,7 +13829,7 @@
         <v>1417</v>
       </c>
       <c r="I239">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="K239" t="s">
         <v>1394</v>
@@ -13928,7 +13928,7 @@
         <v>1417</v>
       </c>
       <c r="I242">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="K242" t="s">
         <v>1420</v>
@@ -13995,7 +13995,7 @@
         <v>1417</v>
       </c>
       <c r="I244">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="J244">
         <v>15</v>
@@ -14036,7 +14036,7 @@
         <v>1417</v>
       </c>
       <c r="I245">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="J245">
         <v>15</v>
@@ -14179,7 +14179,7 @@
         <v>1417</v>
       </c>
       <c r="I249">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="K249" t="s">
         <v>1421</v>
@@ -14313,7 +14313,7 @@
         <v>1417</v>
       </c>
       <c r="I253">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="J253">
         <v>162</v>
@@ -14357,7 +14357,7 @@
         <v>1417</v>
       </c>
       <c r="I254">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="K254" t="s">
         <v>1424</v>
@@ -14436,7 +14436,7 @@
         <v>1417</v>
       </c>
       <c r="I256">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="J256">
         <v>23</v>
@@ -14620,7 +14620,7 @@
         <v>1417</v>
       </c>
       <c r="I261">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="J261">
         <v>162</v>
@@ -14778,7 +14778,7 @@
         <v>1417</v>
       </c>
       <c r="I265">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="J265">
         <v>162</v>
@@ -14863,7 +14863,7 @@
         <v>1417</v>
       </c>
       <c r="I267">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="K267" t="s">
         <v>1424</v>
@@ -14901,7 +14901,7 @@
         <v>1417</v>
       </c>
       <c r="I268">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="K268" t="s">
         <v>1421</v>
@@ -14936,7 +14936,7 @@
         <v>1417</v>
       </c>
       <c r="I269">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="K269" t="s">
         <v>1421</v>
@@ -14974,7 +14974,7 @@
         <v>1417</v>
       </c>
       <c r="I270">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="K270" t="s">
         <v>1424</v>
@@ -15012,7 +15012,7 @@
         <v>1417</v>
       </c>
       <c r="I271">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="K271" t="s">
         <v>1424</v>
@@ -15190,7 +15190,7 @@
         <v>1417</v>
       </c>
       <c r="I276">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="K276" t="s">
         <v>1425</v>
@@ -15228,7 +15228,7 @@
         <v>1417</v>
       </c>
       <c r="I277">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="K277" t="s">
         <v>1421</v>
@@ -15266,7 +15266,7 @@
         <v>1417</v>
       </c>
       <c r="I278">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="J278">
         <v>148</v>
@@ -15310,7 +15310,7 @@
         <v>1417</v>
       </c>
       <c r="I279">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="K279" t="s">
         <v>1423</v>
@@ -15351,7 +15351,7 @@
         <v>1417</v>
       </c>
       <c r="I280">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="K280" t="s">
         <v>1421</v>
@@ -15389,7 +15389,7 @@
         <v>1417</v>
       </c>
       <c r="I281">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="K281" t="s">
         <v>1421</v>
@@ -15430,7 +15430,7 @@
         <v>1417</v>
       </c>
       <c r="I282">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="K282" t="s">
         <v>1421</v>
@@ -15724,7 +15724,7 @@
         <v>1417</v>
       </c>
       <c r="I291">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="J291">
         <v>20</v>
@@ -15768,7 +15768,7 @@
         <v>1417</v>
       </c>
       <c r="I292">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="K292" t="s">
         <v>1424</v>
@@ -15806,7 +15806,7 @@
         <v>1417</v>
       </c>
       <c r="I293">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="K293" t="s">
         <v>1425</v>
@@ -15844,7 +15844,7 @@
         <v>1417</v>
       </c>
       <c r="I294">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="K294" t="s">
         <v>1430</v>
@@ -15981,7 +15981,7 @@
         <v>1417</v>
       </c>
       <c r="I298">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="J298">
         <v>58</v>
@@ -16145,7 +16145,7 @@
         <v>1417</v>
       </c>
       <c r="I302">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="K302" t="s">
         <v>1424</v>
@@ -16183,7 +16183,7 @@
         <v>1417</v>
       </c>
       <c r="I303">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="K303" t="s">
         <v>1421</v>
@@ -16221,7 +16221,7 @@
         <v>1417</v>
       </c>
       <c r="I304">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="K304" t="s">
         <v>1424</v>
@@ -16259,7 +16259,7 @@
         <v>1417</v>
       </c>
       <c r="I305">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="J305">
         <v>35</v>
@@ -16303,7 +16303,7 @@
         <v>1417</v>
       </c>
       <c r="I306">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="J306">
         <v>31</v>
@@ -16391,7 +16391,7 @@
         <v>1417</v>
       </c>
       <c r="I308">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="K308" t="s">
         <v>1420</v>
@@ -16508,7 +16508,7 @@
         <v>1417</v>
       </c>
       <c r="I311">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="K311" t="s">
         <v>1420</v>
@@ -16838,7 +16838,7 @@
         <v>1417</v>
       </c>
       <c r="I320">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="K320" t="s">
         <v>1425</v>
@@ -16876,7 +16876,7 @@
         <v>1417</v>
       </c>
       <c r="I321">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="K321" t="s">
         <v>1421</v>
@@ -16914,7 +16914,7 @@
         <v>1417</v>
       </c>
       <c r="I322">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="J322">
         <v>57</v>
@@ -17028,7 +17028,7 @@
         <v>1417</v>
       </c>
       <c r="I325">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="J325">
         <v>57</v>
@@ -17110,7 +17110,7 @@
         <v>1417</v>
       </c>
       <c r="I327">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="J327">
         <v>57</v>
@@ -17154,7 +17154,7 @@
         <v>1417</v>
       </c>
       <c r="I328">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="J328">
         <v>57</v>
@@ -17198,7 +17198,7 @@
         <v>1417</v>
       </c>
       <c r="I329">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="J329">
         <v>57</v>
@@ -17242,7 +17242,7 @@
         <v>1417</v>
       </c>
       <c r="I330">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="J330">
         <v>57</v>
@@ -17286,7 +17286,7 @@
         <v>1417</v>
       </c>
       <c r="I331">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="K331" t="s">
         <v>1420</v>
@@ -17324,7 +17324,7 @@
         <v>1417</v>
       </c>
       <c r="I332">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="K332" t="s">
         <v>1421</v>
@@ -17362,7 +17362,7 @@
         <v>1417</v>
       </c>
       <c r="I333">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="J333">
         <v>100</v>
@@ -17406,7 +17406,7 @@
         <v>1417</v>
       </c>
       <c r="I334">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="K334" t="s">
         <v>1421</v>
@@ -17631,7 +17631,7 @@
         <v>1417</v>
       </c>
       <c r="I340">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J340">
         <v>98</v>
@@ -17672,7 +17672,7 @@
         <v>1417</v>
       </c>
       <c r="I341">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J341">
         <v>90</v>
@@ -17713,7 +17713,7 @@
         <v>1417</v>
       </c>
       <c r="I342">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="K342" t="s">
         <v>1420</v>
@@ -17827,7 +17827,7 @@
         <v>1417</v>
       </c>
       <c r="I345">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="K345" t="s">
         <v>1420</v>
@@ -17947,7 +17947,7 @@
         <v>1417</v>
       </c>
       <c r="I348">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J348">
         <v>14</v>
@@ -17991,7 +17991,7 @@
         <v>1417</v>
       </c>
       <c r="I349">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="K349" t="s">
         <v>1425</v>
@@ -18029,7 +18029,7 @@
         <v>1417</v>
       </c>
       <c r="I350">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J350">
         <v>46</v>
@@ -18067,7 +18067,7 @@
         <v>1417</v>
       </c>
       <c r="I351">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J351">
         <v>82</v>
@@ -18111,7 +18111,7 @@
         <v>1417</v>
       </c>
       <c r="I352">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J352">
         <v>78</v>
@@ -18155,7 +18155,7 @@
         <v>1417</v>
       </c>
       <c r="I353">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J353">
         <v>83</v>
@@ -18199,7 +18199,7 @@
         <v>1417</v>
       </c>
       <c r="I354">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="K354" t="s">
         <v>1424</v>
@@ -18237,7 +18237,7 @@
         <v>1417</v>
       </c>
       <c r="I355">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J355">
         <v>8</v>
@@ -18319,7 +18319,7 @@
         <v>1417</v>
       </c>
       <c r="I357">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J357">
         <v>85</v>
@@ -18442,7 +18442,7 @@
         <v>1417</v>
       </c>
       <c r="I360">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J360">
         <v>83</v>
@@ -18489,7 +18489,7 @@
         <v>1417</v>
       </c>
       <c r="I361">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J361">
         <v>83</v>
@@ -18533,7 +18533,7 @@
         <v>1417</v>
       </c>
       <c r="I362">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="K362" t="s">
         <v>1424</v>
@@ -18571,7 +18571,7 @@
         <v>1417</v>
       </c>
       <c r="I363">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="K363" t="s">
         <v>1424</v>
@@ -18609,7 +18609,7 @@
         <v>1417</v>
       </c>
       <c r="I364">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J364">
         <v>83</v>
@@ -18653,7 +18653,7 @@
         <v>1417</v>
       </c>
       <c r="I365">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J365">
         <v>15</v>
@@ -18776,7 +18776,7 @@
         <v>1417</v>
       </c>
       <c r="I368">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="J368">
         <v>77</v>
@@ -18820,7 +18820,7 @@
         <v>1417</v>
       </c>
       <c r="I369">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K369" t="s">
         <v>1424</v>
@@ -18858,7 +18858,7 @@
         <v>1417</v>
       </c>
       <c r="I370">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K370" t="s">
         <v>1424</v>
@@ -18896,7 +18896,7 @@
         <v>1417</v>
       </c>
       <c r="I371">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="J371">
         <v>16</v>
@@ -18984,7 +18984,7 @@
         <v>1417</v>
       </c>
       <c r="I373">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="K373" t="s">
         <v>1420</v>
@@ -19022,7 +19022,7 @@
         <v>1417</v>
       </c>
       <c r="I374">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="K374" t="s">
         <v>1420</v>
@@ -19060,7 +19060,7 @@
         <v>1417</v>
       </c>
       <c r="I375">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="J375">
         <v>94</v>
@@ -19101,7 +19101,7 @@
         <v>1417</v>
       </c>
       <c r="I376">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="K376" t="s">
         <v>1424</v>
@@ -19180,7 +19180,7 @@
         <v>1417</v>
       </c>
       <c r="I378">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="K378" t="s">
         <v>1424</v>
@@ -19218,7 +19218,7 @@
         <v>1417</v>
       </c>
       <c r="I379">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="J379">
         <v>20</v>
@@ -19262,7 +19262,7 @@
         <v>1417</v>
       </c>
       <c r="I380">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="J380">
         <v>94</v>
@@ -19306,7 +19306,7 @@
         <v>1417</v>
       </c>
       <c r="I381">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="K381" t="s">
         <v>1424</v>
@@ -19344,7 +19344,7 @@
         <v>1417</v>
       </c>
       <c r="I382">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="K382" t="s">
         <v>1424</v>
@@ -19382,7 +19382,7 @@
         <v>1417</v>
       </c>
       <c r="I383">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="J383">
         <v>71</v>
@@ -19426,7 +19426,7 @@
         <v>1417</v>
       </c>
       <c r="I384">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="K384" t="s">
         <v>1421</v>
@@ -19508,7 +19508,7 @@
         <v>1417</v>
       </c>
       <c r="I386">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="K386" t="s">
         <v>1424</v>
@@ -19546,7 +19546,7 @@
         <v>1417</v>
       </c>
       <c r="I387">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="K387" t="s">
         <v>1424</v>
@@ -19584,7 +19584,7 @@
         <v>1417</v>
       </c>
       <c r="I388">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="J388">
         <v>-85</v>
@@ -19628,7 +19628,7 @@
         <v>1417</v>
       </c>
       <c r="I389">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="K389" t="s">
         <v>1425</v>
@@ -20079,7 +20079,7 @@
         <v>1417</v>
       </c>
       <c r="I400">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="K400" t="s">
         <v>1424</v>
@@ -20155,7 +20155,7 @@
         <v>1417</v>
       </c>
       <c r="I402">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="K402" t="s">
         <v>1424</v>
@@ -20193,7 +20193,7 @@
         <v>1417</v>
       </c>
       <c r="I403">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="J403">
         <v>83</v>
@@ -20237,7 +20237,7 @@
         <v>1417</v>
       </c>
       <c r="I404">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="K404" t="s">
         <v>1424</v>
@@ -20307,7 +20307,7 @@
         <v>1417</v>
       </c>
       <c r="I406">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="Q406" t="b">
         <v>1</v>
@@ -20339,7 +20339,7 @@
         <v>1417</v>
       </c>
       <c r="I407">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="Q407" t="b">
         <v>1</v>
@@ -20371,7 +20371,7 @@
         <v>1417</v>
       </c>
       <c r="I408">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="Q408" t="b">
         <v>1</v>
@@ -20403,7 +20403,7 @@
         <v>1417</v>
       </c>
       <c r="I409">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="Q409" t="b">
         <v>1</v>
@@ -20435,7 +20435,7 @@
         <v>1417</v>
       </c>
       <c r="I410">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="Q410" t="b">
         <v>1</v>
@@ -20467,7 +20467,7 @@
         <v>1417</v>
       </c>
       <c r="I411">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="Q411" t="b">
         <v>1</v>
@@ -20499,7 +20499,7 @@
         <v>1417</v>
       </c>
       <c r="I412">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="Q412" t="b">
         <v>1</v>
@@ -20531,7 +20531,7 @@
         <v>1417</v>
       </c>
       <c r="I413">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="Q413" t="b">
         <v>1</v>
@@ -20621,7 +20621,7 @@
         <v>1417</v>
       </c>
       <c r="I416">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="Q416" t="b">
         <v>1</v>
@@ -20711,7 +20711,7 @@
         <v>1417</v>
       </c>
       <c r="I419">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="Q419" t="b">
         <v>1</v>
@@ -20743,7 +20743,7 @@
         <v>1417</v>
       </c>
       <c r="I420">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="Q420" t="b">
         <v>1</v>
@@ -20775,7 +20775,7 @@
         <v>1417</v>
       </c>
       <c r="I421">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="Q421" t="b">
         <v>1</v>
@@ -20807,7 +20807,7 @@
         <v>1417</v>
       </c>
       <c r="I422">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="Q422" t="b">
         <v>1</v>
@@ -20839,7 +20839,7 @@
         <v>1417</v>
       </c>
       <c r="I423">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="Q423" t="b">
         <v>1</v>
@@ -20871,7 +20871,7 @@
         <v>1417</v>
       </c>
       <c r="I424">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="Q424" t="b">
         <v>1</v>
@@ -20903,7 +20903,7 @@
         <v>1417</v>
       </c>
       <c r="I425">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="Q425" t="b">
         <v>1</v>
@@ -20935,7 +20935,7 @@
         <v>1417</v>
       </c>
       <c r="I426">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="Q426" t="b">
         <v>1</v>
@@ -20967,7 +20967,7 @@
         <v>1417</v>
       </c>
       <c r="I427">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="Q427" t="b">
         <v>1</v>
@@ -21057,7 +21057,7 @@
         <v>1417</v>
       </c>
       <c r="I430">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="Q430" t="b">
         <v>1</v>
@@ -21089,7 +21089,7 @@
         <v>1417</v>
       </c>
       <c r="I431">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="Q431" t="b">
         <v>1</v>
@@ -21121,7 +21121,7 @@
         <v>1417</v>
       </c>
       <c r="I432">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="Q432" t="b">
         <v>1</v>
@@ -21153,7 +21153,7 @@
         <v>1417</v>
       </c>
       <c r="I433">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="Q433" t="b">
         <v>1</v>
@@ -21185,7 +21185,7 @@
         <v>1417</v>
       </c>
       <c r="I434">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="Q434" t="b">
         <v>1</v>
@@ -21217,7 +21217,7 @@
         <v>1417</v>
       </c>
       <c r="I435">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="Q435" t="b">
         <v>1</v>
@@ -21249,7 +21249,7 @@
         <v>1417</v>
       </c>
       <c r="I436">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="Q436" t="b">
         <v>1</v>
@@ -21281,7 +21281,7 @@
         <v>1419</v>
       </c>
       <c r="I437">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="Q437" t="b">
         <v>1</v>
@@ -21313,7 +21313,7 @@
         <v>1419</v>
       </c>
       <c r="I438">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="Q438" t="b">
         <v>1</v>
@@ -21345,7 +21345,7 @@
         <v>1417</v>
       </c>
       <c r="I439">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="Q439" t="b">
         <v>1</v>
@@ -21377,7 +21377,7 @@
         <v>1417</v>
       </c>
       <c r="I440">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="Q440" t="b">
         <v>1</v>
@@ -21409,7 +21409,7 @@
         <v>1417</v>
       </c>
       <c r="I441">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="Q441" t="b">
         <v>1</v>
@@ -21470,7 +21470,7 @@
         <v>1417</v>
       </c>
       <c r="I443">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="Q443" t="b">
         <v>1</v>
@@ -21560,7 +21560,7 @@
         <v>1417</v>
       </c>
       <c r="I446">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="Q446" t="b">
         <v>1</v>
@@ -21592,7 +21592,7 @@
         <v>1417</v>
       </c>
       <c r="I447">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="Q447" t="b">
         <v>1</v>
@@ -21624,7 +21624,7 @@
         <v>1417</v>
       </c>
       <c r="I448">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="Q448" t="b">
         <v>1</v>
@@ -21656,7 +21656,7 @@
         <v>1417</v>
       </c>
       <c r="I449">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="Q449" t="b">
         <v>1</v>
@@ -21688,7 +21688,7 @@
         <v>1417</v>
       </c>
       <c r="I450">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="Q450" t="b">
         <v>1</v>
@@ -21720,7 +21720,7 @@
         <v>1417</v>
       </c>
       <c r="I451">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="Q451" t="b">
         <v>1</v>
@@ -21781,7 +21781,7 @@
         <v>1417</v>
       </c>
       <c r="I453">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="Q453" t="b">
         <v>1</v>
@@ -21813,7 +21813,7 @@
         <v>1417</v>
       </c>
       <c r="I454">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="Q454" t="b">
         <v>1</v>
@@ -21845,7 +21845,7 @@
         <v>1417</v>
       </c>
       <c r="I455">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="Q455" t="b">
         <v>1</v>
@@ -21906,7 +21906,7 @@
         <v>1417</v>
       </c>
       <c r="I457">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="Q457" t="b">
         <v>1</v>
@@ -21938,7 +21938,7 @@
         <v>1417</v>
       </c>
       <c r="I458">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q458" t="b">
         <v>1</v>
@@ -21970,7 +21970,7 @@
         <v>1417</v>
       </c>
       <c r="I459">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="Q459" t="b">
         <v>1</v>
@@ -22002,7 +22002,7 @@
         <v>1417</v>
       </c>
       <c r="I460">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="Q460" t="b">
         <v>1</v>
@@ -22034,7 +22034,7 @@
         <v>1417</v>
       </c>
       <c r="I461">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="Q461" t="b">
         <v>1</v>
@@ -22066,7 +22066,7 @@
         <v>1417</v>
       </c>
       <c r="I462">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="Q462" t="b">
         <v>1</v>
@@ -22098,7 +22098,7 @@
         <v>1417</v>
       </c>
       <c r="I463">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="Q463" t="b">
         <v>1</v>
@@ -22130,7 +22130,7 @@
         <v>1417</v>
       </c>
       <c r="I464">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="Q464" t="b">
         <v>1</v>
@@ -22162,7 +22162,7 @@
         <v>1417</v>
       </c>
       <c r="I465">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="Q465" t="b">
         <v>1</v>
@@ -22194,7 +22194,7 @@
         <v>1417</v>
       </c>
       <c r="I466">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="Q466" t="b">
         <v>1</v>
@@ -22226,7 +22226,7 @@
         <v>1417</v>
       </c>
       <c r="I467">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="Q467" t="b">
         <v>1</v>
@@ -22258,7 +22258,7 @@
         <v>1417</v>
       </c>
       <c r="I468">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="Q468" t="b">
         <v>1</v>
@@ -22290,7 +22290,7 @@
         <v>1417</v>
       </c>
       <c r="I469">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="Q469" t="b">
         <v>1</v>
@@ -22351,7 +22351,7 @@
         <v>1417</v>
       </c>
       <c r="I471">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="Q471" t="b">
         <v>1</v>
@@ -22383,7 +22383,7 @@
         <v>1417</v>
       </c>
       <c r="I472">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="Q472" t="b">
         <v>1</v>
@@ -22415,7 +22415,7 @@
         <v>1417</v>
       </c>
       <c r="I473">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="Q473" t="b">
         <v>1</v>
@@ -22447,7 +22447,7 @@
         <v>1417</v>
       </c>
       <c r="I474">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q474" t="b">
         <v>1</v>
@@ -22479,7 +22479,7 @@
         <v>1417</v>
       </c>
       <c r="I475">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q475" t="b">
         <v>1</v>
@@ -22511,7 +22511,7 @@
         <v>1417</v>
       </c>
       <c r="I476">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q476" t="b">
         <v>1</v>
@@ -22543,7 +22543,7 @@
         <v>1417</v>
       </c>
       <c r="I477">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q477" t="b">
         <v>1</v>
@@ -22575,7 +22575,7 @@
         <v>1417</v>
       </c>
       <c r="I478">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q478" t="b">
         <v>1</v>
@@ -22607,7 +22607,7 @@
         <v>1417</v>
       </c>
       <c r="I479">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q479" t="b">
         <v>1</v>
@@ -22639,7 +22639,7 @@
         <v>1417</v>
       </c>
       <c r="I480">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q480" t="b">
         <v>1</v>
@@ -22671,7 +22671,7 @@
         <v>1417</v>
       </c>
       <c r="I481">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q481" t="b">
         <v>1</v>
@@ -22703,7 +22703,7 @@
         <v>1417</v>
       </c>
       <c r="I482">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q482" t="b">
         <v>1</v>
@@ -22735,7 +22735,7 @@
         <v>1417</v>
       </c>
       <c r="I483">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q483" t="b">
         <v>1</v>
@@ -22767,7 +22767,7 @@
         <v>1417</v>
       </c>
       <c r="I484">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q484" t="b">
         <v>1</v>
@@ -22799,7 +22799,7 @@
         <v>1417</v>
       </c>
       <c r="I485">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q485" t="b">
         <v>1</v>
@@ -22831,7 +22831,7 @@
         <v>1417</v>
       </c>
       <c r="I486">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q486" t="b">
         <v>1</v>
@@ -22863,7 +22863,7 @@
         <v>1417</v>
       </c>
       <c r="I487">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q487" t="b">
         <v>1</v>
@@ -22895,7 +22895,7 @@
         <v>1417</v>
       </c>
       <c r="I488">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q488" t="b">
         <v>1</v>
@@ -22927,7 +22927,7 @@
         <v>1417</v>
       </c>
       <c r="I489">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q489" t="b">
         <v>1</v>
@@ -22959,7 +22959,7 @@
         <v>1417</v>
       </c>
       <c r="I490">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q490" t="b">
         <v>1</v>
@@ -22991,7 +22991,7 @@
         <v>1417</v>
       </c>
       <c r="I491">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q491" t="b">
         <v>1</v>
@@ -23023,7 +23023,7 @@
         <v>1419</v>
       </c>
       <c r="I492">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q492" t="b">
         <v>1</v>
@@ -23055,7 +23055,7 @@
         <v>1419</v>
       </c>
       <c r="I493">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q493" t="b">
         <v>1</v>
@@ -23087,7 +23087,7 @@
         <v>1419</v>
       </c>
       <c r="I494">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q494" t="b">
         <v>1</v>
@@ -23119,7 +23119,7 @@
         <v>1419</v>
       </c>
       <c r="I495">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q495" t="b">
         <v>1</v>
@@ -23151,7 +23151,7 @@
         <v>1419</v>
       </c>
       <c r="I496">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q496" t="b">
         <v>1</v>
@@ -23183,7 +23183,7 @@
         <v>1417</v>
       </c>
       <c r="I497">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q497" t="b">
         <v>1</v>
@@ -23215,7 +23215,7 @@
         <v>1417</v>
       </c>
       <c r="I498">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q498" t="b">
         <v>1</v>
@@ -23247,7 +23247,7 @@
         <v>1419</v>
       </c>
       <c r="I499">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q499" t="b">
         <v>1</v>
@@ -23279,7 +23279,7 @@
         <v>1417</v>
       </c>
       <c r="I500">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q500" t="b">
         <v>1</v>
@@ -23311,7 +23311,7 @@
         <v>1417</v>
       </c>
       <c r="I501">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q501" t="b">
         <v>1</v>
@@ -23343,7 +23343,7 @@
         <v>1417</v>
       </c>
       <c r="I502">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q502" t="b">
         <v>1</v>
@@ -23375,7 +23375,7 @@
         <v>1417</v>
       </c>
       <c r="I503">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q503" t="b">
         <v>1</v>
@@ -23407,7 +23407,7 @@
         <v>1417</v>
       </c>
       <c r="I504">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q504" t="b">
         <v>1</v>
@@ -23439,7 +23439,7 @@
         <v>1417</v>
       </c>
       <c r="I505">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q505" t="b">
         <v>1</v>
@@ -23471,7 +23471,7 @@
         <v>1417</v>
       </c>
       <c r="I506">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q506" t="b">
         <v>1</v>
@@ -23503,7 +23503,7 @@
         <v>1417</v>
       </c>
       <c r="I507">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="Q507" t="b">
         <v>1</v>
@@ -23564,7 +23564,7 @@
         <v>1417</v>
       </c>
       <c r="I509">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="Q509" t="b">
         <v>1</v>
@@ -23596,7 +23596,7 @@
         <v>1417</v>
       </c>
       <c r="I510">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="Q510" t="b">
         <v>1</v>
@@ -23628,7 +23628,7 @@
         <v>1417</v>
       </c>
       <c r="I511">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="Q511" t="b">
         <v>1</v>
@@ -23660,7 +23660,7 @@
         <v>1417</v>
       </c>
       <c r="I512">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="Q512" t="b">
         <v>1</v>
@@ -23692,7 +23692,7 @@
         <v>1417</v>
       </c>
       <c r="I513">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="Q513" t="b">
         <v>1</v>
@@ -23753,7 +23753,7 @@
         <v>1417</v>
       </c>
       <c r="I515">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="Q515" t="b">
         <v>1</v>
@@ -23785,7 +23785,7 @@
         <v>1417</v>
       </c>
       <c r="I516">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="Q516" t="b">
         <v>1</v>
@@ -23817,7 +23817,7 @@
         <v>1417</v>
       </c>
       <c r="I517">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="Q517" t="b">
         <v>1</v>
@@ -23849,7 +23849,7 @@
         <v>1417</v>
       </c>
       <c r="I518">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="Q518" t="b">
         <v>1</v>
@@ -23881,7 +23881,7 @@
         <v>1417</v>
       </c>
       <c r="I519">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="Q519" t="b">
         <v>1</v>
@@ -23913,7 +23913,7 @@
         <v>1417</v>
       </c>
       <c r="I520">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="Q520" t="b">
         <v>1</v>
@@ -23945,7 +23945,7 @@
         <v>1417</v>
       </c>
       <c r="I521">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="Q521" t="b">
         <v>1</v>
@@ -23977,7 +23977,7 @@
         <v>1417</v>
       </c>
       <c r="I522">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="Q522" t="b">
         <v>1</v>
@@ -24009,7 +24009,7 @@
         <v>1417</v>
       </c>
       <c r="I523">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="Q523" t="b">
         <v>1</v>
@@ -24041,7 +24041,7 @@
         <v>1417</v>
       </c>
       <c r="I524">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q524" t="b">
         <v>1</v>
@@ -24073,7 +24073,7 @@
         <v>1417</v>
       </c>
       <c r="I525">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q525" t="b">
         <v>1</v>
@@ -24105,7 +24105,7 @@
         <v>1417</v>
       </c>
       <c r="I526">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q526" t="b">
         <v>1</v>
@@ -24137,7 +24137,7 @@
         <v>1417</v>
       </c>
       <c r="I527">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q527" t="b">
         <v>1</v>
@@ -24169,7 +24169,7 @@
         <v>1417</v>
       </c>
       <c r="I528">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="Q528" t="b">
         <v>1</v>
@@ -24201,7 +24201,7 @@
         <v>1417</v>
       </c>
       <c r="I529">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Q529" t="b">
         <v>1</v>
@@ -24233,7 +24233,7 @@
         <v>1417</v>
       </c>
       <c r="I530">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Q530" t="b">
         <v>1</v>
@@ -24265,7 +24265,7 @@
         <v>1417</v>
       </c>
       <c r="I531">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Q531" t="b">
         <v>1</v>
@@ -24297,7 +24297,7 @@
         <v>1417</v>
       </c>
       <c r="I532">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Q532" t="b">
         <v>1</v>
@@ -24329,7 +24329,7 @@
         <v>1417</v>
       </c>
       <c r="I533">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Q533" t="b">
         <v>1</v>
@@ -24361,7 +24361,7 @@
         <v>1417</v>
       </c>
       <c r="I534">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Q534" t="b">
         <v>1</v>
@@ -24393,7 +24393,7 @@
         <v>1417</v>
       </c>
       <c r="I535">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Q535" t="b">
         <v>1</v>
@@ -24425,7 +24425,7 @@
         <v>1417</v>
       </c>
       <c r="I536">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Q536" t="b">
         <v>1</v>
@@ -24457,7 +24457,7 @@
         <v>1417</v>
       </c>
       <c r="I537">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Q537" t="b">
         <v>1</v>
@@ -24489,7 +24489,7 @@
         <v>1417</v>
       </c>
       <c r="I538">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Q538" t="b">
         <v>1</v>
@@ -24521,7 +24521,7 @@
         <v>1417</v>
       </c>
       <c r="I539">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Q539" t="b">
         <v>1</v>
@@ -24553,7 +24553,7 @@
         <v>1417</v>
       </c>
       <c r="I540">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Q540" t="b">
         <v>1</v>
@@ -24585,7 +24585,7 @@
         <v>1417</v>
       </c>
       <c r="I541">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Q541" t="b">
         <v>1</v>
@@ -24617,7 +24617,7 @@
         <v>1417</v>
       </c>
       <c r="I542">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Q542" t="b">
         <v>1</v>
@@ -24649,7 +24649,7 @@
         <v>1417</v>
       </c>
       <c r="I543">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Q543" t="b">
         <v>1</v>
@@ -24681,7 +24681,7 @@
         <v>1417</v>
       </c>
       <c r="I544">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Q544" t="b">
         <v>1</v>
@@ -24713,7 +24713,7 @@
         <v>1417</v>
       </c>
       <c r="I545">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Q545" t="b">
         <v>1</v>
@@ -24745,7 +24745,7 @@
         <v>1417</v>
       </c>
       <c r="I546">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q546" t="b">
         <v>1</v>
@@ -24777,7 +24777,7 @@
         <v>1417</v>
       </c>
       <c r="I547">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q547" t="b">
         <v>1</v>
@@ -24809,7 +24809,7 @@
         <v>1417</v>
       </c>
       <c r="I548">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q548" t="b">
         <v>1</v>
@@ -24841,7 +24841,7 @@
         <v>1417</v>
       </c>
       <c r="I549">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q549" t="b">
         <v>1</v>
@@ -24873,7 +24873,7 @@
         <v>1417</v>
       </c>
       <c r="I550">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q550" t="b">
         <v>1</v>
@@ -24905,7 +24905,7 @@
         <v>1417</v>
       </c>
       <c r="I551">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q551" t="b">
         <v>1</v>
@@ -24937,7 +24937,7 @@
         <v>1417</v>
       </c>
       <c r="I552">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q552" t="b">
         <v>1</v>
@@ -24969,7 +24969,7 @@
         <v>1417</v>
       </c>
       <c r="I553">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q553" t="b">
         <v>1</v>
@@ -25001,7 +25001,7 @@
         <v>1417</v>
       </c>
       <c r="I554">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q554" t="b">
         <v>1</v>
@@ -25033,7 +25033,7 @@
         <v>1417</v>
       </c>
       <c r="I555">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q555" t="b">
         <v>1</v>
@@ -25065,7 +25065,7 @@
         <v>1417</v>
       </c>
       <c r="I556">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q556" t="b">
         <v>1</v>
@@ -25097,7 +25097,7 @@
         <v>1417</v>
       </c>
       <c r="I557">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="Q557" t="b">
         <v>1</v>
@@ -25129,7 +25129,7 @@
         <v>1417</v>
       </c>
       <c r="I558">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="Q558" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: reparaveis (23/10/2026 12:44)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
@@ -5132,7 +5132,7 @@
         <v>1417</v>
       </c>
       <c r="I2">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="K2" t="s">
         <v>1420</v>
@@ -5170,7 +5170,7 @@
         <v>1417</v>
       </c>
       <c r="I3">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="K3" t="s">
         <v>1421</v>
@@ -5208,7 +5208,7 @@
         <v>1417</v>
       </c>
       <c r="I4">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="K4" t="s">
         <v>1421</v>
@@ -5246,7 +5246,7 @@
         <v>1417</v>
       </c>
       <c r="I5">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="J5">
         <v>279</v>
@@ -5290,7 +5290,7 @@
         <v>1417</v>
       </c>
       <c r="I6">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="J6">
         <v>153</v>
@@ -5334,7 +5334,7 @@
         <v>1417</v>
       </c>
       <c r="I7">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="J7">
         <v>112</v>
@@ -5410,7 +5410,7 @@
         <v>1417</v>
       </c>
       <c r="I9">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="J9">
         <v>362</v>
@@ -5457,7 +5457,7 @@
         <v>1417</v>
       </c>
       <c r="I10">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="J10">
         <v>378</v>
@@ -5504,7 +5504,7 @@
         <v>1417</v>
       </c>
       <c r="I11">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="J11">
         <v>112</v>
@@ -5551,7 +5551,7 @@
         <v>1417</v>
       </c>
       <c r="I12">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="J12">
         <v>124</v>
@@ -5624,7 +5624,7 @@
         <v>1417</v>
       </c>
       <c r="I14">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="J14">
         <v>64</v>
@@ -5703,7 +5703,7 @@
         <v>1417</v>
       </c>
       <c r="I16">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="K16" t="s">
         <v>1420</v>
@@ -5741,7 +5741,7 @@
         <v>1417</v>
       </c>
       <c r="I17">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="J17">
         <v>161</v>
@@ -5785,7 +5785,7 @@
         <v>1417</v>
       </c>
       <c r="I18">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="J18">
         <v>66</v>
@@ -5858,7 +5858,7 @@
         <v>1417</v>
       </c>
       <c r="I20">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="J20">
         <v>399</v>
@@ -5931,7 +5931,7 @@
         <v>1417</v>
       </c>
       <c r="I22">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="K22" t="s">
         <v>1424</v>
@@ -5969,7 +5969,7 @@
         <v>1417</v>
       </c>
       <c r="I23">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="J23">
         <v>229</v>
@@ -6074,7 +6074,7 @@
         <v>1417</v>
       </c>
       <c r="I26">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="J26">
         <v>155</v>
@@ -6121,7 +6121,7 @@
         <v>1417</v>
       </c>
       <c r="I27">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="K27" t="s">
         <v>1424</v>
@@ -6217,7 +6217,7 @@
         <v>1417</v>
       </c>
       <c r="I30">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="J30">
         <v>209</v>
@@ -6290,7 +6290,7 @@
         <v>1417</v>
       </c>
       <c r="I32">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="K32" t="s">
         <v>1420</v>
@@ -6499,7 +6499,7 @@
         <v>1417</v>
       </c>
       <c r="I39">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="K39" t="s">
         <v>1425</v>
@@ -6662,7 +6662,7 @@
         <v>1417</v>
       </c>
       <c r="I44">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="J44">
         <v>87</v>
@@ -6709,7 +6709,7 @@
         <v>1417</v>
       </c>
       <c r="I45">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="J45">
         <v>331</v>
@@ -6756,7 +6756,7 @@
         <v>1417</v>
       </c>
       <c r="I46">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="K46" t="s">
         <v>1424</v>
@@ -6797,7 +6797,7 @@
         <v>1417</v>
       </c>
       <c r="I47">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="J47">
         <v>344</v>
@@ -6844,7 +6844,7 @@
         <v>1417</v>
       </c>
       <c r="I48">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="K48" t="s">
         <v>1424</v>
@@ -6911,7 +6911,7 @@
         <v>1417</v>
       </c>
       <c r="I50">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="K50" t="s">
         <v>1424</v>
@@ -6978,7 +6978,7 @@
         <v>1417</v>
       </c>
       <c r="I52">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="K52" t="s">
         <v>1420</v>
@@ -7016,7 +7016,7 @@
         <v>1417</v>
       </c>
       <c r="I53">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="K53" t="s">
         <v>1421</v>
@@ -7054,7 +7054,7 @@
         <v>1417</v>
       </c>
       <c r="I54">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="K54" t="s">
         <v>1421</v>
@@ -7330,7 +7330,7 @@
         <v>1417</v>
       </c>
       <c r="I63">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="J63">
         <v>293</v>
@@ -7377,7 +7377,7 @@
         <v>1417</v>
       </c>
       <c r="I64">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="J64">
         <v>320</v>
@@ -7607,7 +7607,7 @@
         <v>1417</v>
       </c>
       <c r="I71">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="J71">
         <v>429</v>
@@ -7680,7 +7680,7 @@
         <v>1417</v>
       </c>
       <c r="I73">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="K73" t="s">
         <v>1420</v>
@@ -7788,7 +7788,7 @@
         <v>1417</v>
       </c>
       <c r="I76">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="K76" t="s">
         <v>1427</v>
@@ -7881,7 +7881,7 @@
         <v>1417</v>
       </c>
       <c r="I79">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="K79" t="s">
         <v>1427</v>
@@ -7986,7 +7986,7 @@
         <v>1417</v>
       </c>
       <c r="I82">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="K82" t="s">
         <v>1424</v>
@@ -8053,7 +8053,7 @@
         <v>1417</v>
       </c>
       <c r="I84">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="J84">
         <v>40</v>
@@ -8100,7 +8100,7 @@
         <v>1417</v>
       </c>
       <c r="I85">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="K85" t="s">
         <v>1421</v>
@@ -8138,7 +8138,7 @@
         <v>1417</v>
       </c>
       <c r="I86">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="K86" t="s">
         <v>1421</v>
@@ -8176,7 +8176,7 @@
         <v>1417</v>
       </c>
       <c r="I87">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="J87">
         <v>-16</v>
@@ -8299,7 +8299,7 @@
         <v>1417</v>
       </c>
       <c r="I90">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="K90" t="s">
         <v>1394</v>
@@ -8448,7 +8448,7 @@
         <v>1417</v>
       </c>
       <c r="I94">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="K94" t="s">
         <v>1424</v>
@@ -8527,7 +8527,7 @@
         <v>1417</v>
       </c>
       <c r="I96">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="J96">
         <v>17</v>
@@ -8574,7 +8574,7 @@
         <v>1417</v>
       </c>
       <c r="I97">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="J97">
         <v>20</v>
@@ -8621,7 +8621,7 @@
         <v>1417</v>
       </c>
       <c r="I98">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="K98" t="s">
         <v>1424</v>
@@ -8898,7 +8898,7 @@
         <v>1417</v>
       </c>
       <c r="I106">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="J106">
         <v>49</v>
@@ -8942,7 +8942,7 @@
         <v>1417</v>
       </c>
       <c r="I107">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="J107">
         <v>36</v>
@@ -8986,7 +8986,7 @@
         <v>1417</v>
       </c>
       <c r="I108">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="K108" t="s">
         <v>1421</v>
@@ -9024,7 +9024,7 @@
         <v>1417</v>
       </c>
       <c r="I109">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="K109" t="s">
         <v>1421</v>
@@ -9207,7 +9207,7 @@
         <v>1417</v>
       </c>
       <c r="I115">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="K115" t="s">
         <v>1421</v>
@@ -9245,7 +9245,7 @@
         <v>1417</v>
       </c>
       <c r="I116">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="K116" t="s">
         <v>1421</v>
@@ -9283,7 +9283,7 @@
         <v>1417</v>
       </c>
       <c r="I117">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="K117" t="s">
         <v>1421</v>
@@ -9321,7 +9321,7 @@
         <v>1417</v>
       </c>
       <c r="I118">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="K118" t="s">
         <v>1421</v>
@@ -9359,7 +9359,7 @@
         <v>1417</v>
       </c>
       <c r="I119">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="K119" t="s">
         <v>1421</v>
@@ -9397,7 +9397,7 @@
         <v>1417</v>
       </c>
       <c r="I120">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="K120" t="s">
         <v>1421</v>
@@ -9435,7 +9435,7 @@
         <v>1417</v>
       </c>
       <c r="I121">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="J121">
         <v>251</v>
@@ -9482,7 +9482,7 @@
         <v>1417</v>
       </c>
       <c r="I122">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="K122" t="s">
         <v>1421</v>
@@ -9549,7 +9549,7 @@
         <v>1417</v>
       </c>
       <c r="I124">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="K124" t="s">
         <v>1421</v>
@@ -9587,7 +9587,7 @@
         <v>1417</v>
       </c>
       <c r="I125">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="K125" t="s">
         <v>1427</v>
@@ -9683,7 +9683,7 @@
         <v>1417</v>
       </c>
       <c r="I128">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="K128" t="s">
         <v>1421</v>
@@ -9721,7 +9721,7 @@
         <v>1417</v>
       </c>
       <c r="I129">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="K129" t="s">
         <v>1420</v>
@@ -9759,7 +9759,7 @@
         <v>1417</v>
       </c>
       <c r="I130">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="J130">
         <v>47</v>
@@ -9835,7 +9835,7 @@
         <v>1417</v>
       </c>
       <c r="I132">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="J132">
         <v>145</v>
@@ -9911,7 +9911,7 @@
         <v>1417</v>
       </c>
       <c r="I134">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="K134" t="s">
         <v>1420</v>
@@ -10036,7 +10036,7 @@
         <v>1417</v>
       </c>
       <c r="I138">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="K138" t="s">
         <v>1421</v>
@@ -10420,7 +10420,7 @@
         <v>1417</v>
       </c>
       <c r="I150">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="J150">
         <v>201</v>
@@ -10607,7 +10607,7 @@
         <v>1417</v>
       </c>
       <c r="I155">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="K155" t="s">
         <v>1427</v>
@@ -10642,7 +10642,7 @@
         <v>1417</v>
       </c>
       <c r="I156">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="K156" t="s">
         <v>1421</v>
@@ -10680,7 +10680,7 @@
         <v>1417</v>
       </c>
       <c r="I157">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="J157">
         <v>371</v>
@@ -10724,7 +10724,7 @@
         <v>1417</v>
       </c>
       <c r="I158">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="J158">
         <v>52</v>
@@ -10768,7 +10768,7 @@
         <v>1417</v>
       </c>
       <c r="I159">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="K159" t="s">
         <v>1421</v>
@@ -10806,7 +10806,7 @@
         <v>1417</v>
       </c>
       <c r="I160">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="K160" t="s">
         <v>1421</v>
@@ -10844,7 +10844,7 @@
         <v>1417</v>
       </c>
       <c r="I161">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="J161">
         <v>55</v>
@@ -10979,7 +10979,7 @@
         <v>1417</v>
       </c>
       <c r="I164">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="O164" t="s">
         <v>1533</v>
@@ -11154,7 +11154,7 @@
         <v>1417</v>
       </c>
       <c r="I169">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="K169" t="s">
         <v>1394</v>
@@ -11364,7 +11364,7 @@
         <v>1417</v>
       </c>
       <c r="I175">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="J175">
         <v>205</v>
@@ -11411,7 +11411,7 @@
         <v>1417</v>
       </c>
       <c r="I176">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="K176" t="s">
         <v>1421</v>
@@ -11449,7 +11449,7 @@
         <v>1417</v>
       </c>
       <c r="I177">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="J177">
         <v>44</v>
@@ -11496,7 +11496,7 @@
         <v>1417</v>
       </c>
       <c r="I178">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="K178" t="s">
         <v>1420</v>
@@ -11563,7 +11563,7 @@
         <v>1417</v>
       </c>
       <c r="I180">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="K180" t="s">
         <v>1420</v>
@@ -11659,7 +11659,7 @@
         <v>1417</v>
       </c>
       <c r="I183">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="K183" t="s">
         <v>1421</v>
@@ -11697,7 +11697,7 @@
         <v>1417</v>
       </c>
       <c r="I184">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="K184" t="s">
         <v>1427</v>
@@ -11732,7 +11732,7 @@
         <v>1417</v>
       </c>
       <c r="I185">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="K185" t="s">
         <v>1421</v>
@@ -11770,7 +11770,7 @@
         <v>1417</v>
       </c>
       <c r="I186">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="K186" t="s">
         <v>1421</v>
@@ -11808,7 +11808,7 @@
         <v>1417</v>
       </c>
       <c r="I187">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="J187">
         <v>75</v>
@@ -11855,7 +11855,7 @@
         <v>1417</v>
       </c>
       <c r="I188">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="J188">
         <v>40</v>
@@ -11902,7 +11902,7 @@
         <v>1417</v>
       </c>
       <c r="I189">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="J189">
         <v>155</v>
@@ -11946,7 +11946,7 @@
         <v>1417</v>
       </c>
       <c r="I190">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="J190">
         <v>107</v>
@@ -11990,7 +11990,7 @@
         <v>1417</v>
       </c>
       <c r="I191">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="J191">
         <v>5</v>
@@ -12034,7 +12034,7 @@
         <v>1417</v>
       </c>
       <c r="I192">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="K192" t="s">
         <v>1421</v>
@@ -12072,7 +12072,7 @@
         <v>1417</v>
       </c>
       <c r="I193">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="K193" t="s">
         <v>1426</v>
@@ -12267,7 +12267,7 @@
         <v>1417</v>
       </c>
       <c r="I199">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="J199">
         <v>70</v>
@@ -12352,7 +12352,7 @@
         <v>1417</v>
       </c>
       <c r="I201">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="K201" t="s">
         <v>1421</v>
@@ -12390,7 +12390,7 @@
         <v>1417</v>
       </c>
       <c r="I202">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="K202" t="s">
         <v>1421</v>
@@ -12469,7 +12469,7 @@
         <v>1417</v>
       </c>
       <c r="I204">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="K204" t="s">
         <v>1420</v>
@@ -12507,7 +12507,7 @@
         <v>1417</v>
       </c>
       <c r="I205">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="K205" t="s">
         <v>1420</v>
@@ -12574,7 +12574,7 @@
         <v>1417</v>
       </c>
       <c r="I207">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="J207">
         <v>167</v>
@@ -12618,7 +12618,7 @@
         <v>1417</v>
       </c>
       <c r="I208">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="J208">
         <v>45</v>
@@ -12662,7 +12662,7 @@
         <v>1417</v>
       </c>
       <c r="I209">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="J209">
         <v>191</v>
@@ -12706,7 +12706,7 @@
         <v>1417</v>
       </c>
       <c r="I210">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="K210" t="s">
         <v>1424</v>
@@ -12802,7 +12802,7 @@
         <v>1417</v>
       </c>
       <c r="I213">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="K213" t="s">
         <v>1421</v>
@@ -12840,7 +12840,7 @@
         <v>1417</v>
       </c>
       <c r="I214">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="J214">
         <v>14</v>
@@ -12887,7 +12887,7 @@
         <v>1417</v>
       </c>
       <c r="I215">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="K215" t="s">
         <v>1421</v>
@@ -12954,7 +12954,7 @@
         <v>1417</v>
       </c>
       <c r="I217">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="J217">
         <v>42</v>
@@ -12998,7 +12998,7 @@
         <v>1417</v>
       </c>
       <c r="I218">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="J218">
         <v>166</v>
@@ -13086,7 +13086,7 @@
         <v>1417</v>
       </c>
       <c r="I220">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="J220">
         <v>154</v>
@@ -13472,7 +13472,7 @@
         <v>1417</v>
       </c>
       <c r="I230">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="J230">
         <v>197</v>
@@ -13516,7 +13516,7 @@
         <v>1417</v>
       </c>
       <c r="I231">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="J231">
         <v>35</v>
@@ -13618,7 +13618,7 @@
         <v>1417</v>
       </c>
       <c r="I234">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="J234">
         <v>35</v>
@@ -13665,7 +13665,7 @@
         <v>1417</v>
       </c>
       <c r="I235">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="J235">
         <v>35</v>
@@ -13712,7 +13712,7 @@
         <v>1417</v>
       </c>
       <c r="I236">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="J236">
         <v>86</v>
@@ -13829,7 +13829,7 @@
         <v>1417</v>
       </c>
       <c r="I239">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="K239" t="s">
         <v>1394</v>
@@ -13928,7 +13928,7 @@
         <v>1417</v>
       </c>
       <c r="I242">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="K242" t="s">
         <v>1420</v>
@@ -13995,7 +13995,7 @@
         <v>1417</v>
       </c>
       <c r="I244">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="J244">
         <v>15</v>
@@ -14036,7 +14036,7 @@
         <v>1417</v>
       </c>
       <c r="I245">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="J245">
         <v>15</v>
@@ -14179,7 +14179,7 @@
         <v>1417</v>
       </c>
       <c r="I249">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="K249" t="s">
         <v>1421</v>
@@ -14313,7 +14313,7 @@
         <v>1417</v>
       </c>
       <c r="I253">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="J253">
         <v>162</v>
@@ -14357,7 +14357,7 @@
         <v>1417</v>
       </c>
       <c r="I254">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="K254" t="s">
         <v>1424</v>
@@ -14436,7 +14436,7 @@
         <v>1417</v>
       </c>
       <c r="I256">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="J256">
         <v>23</v>
@@ -14620,7 +14620,7 @@
         <v>1417</v>
       </c>
       <c r="I261">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="J261">
         <v>162</v>
@@ -14778,7 +14778,7 @@
         <v>1417</v>
       </c>
       <c r="I265">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="J265">
         <v>162</v>
@@ -14863,7 +14863,7 @@
         <v>1417</v>
       </c>
       <c r="I267">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="K267" t="s">
         <v>1424</v>
@@ -14901,7 +14901,7 @@
         <v>1417</v>
       </c>
       <c r="I268">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="K268" t="s">
         <v>1421</v>
@@ -14936,7 +14936,7 @@
         <v>1417</v>
       </c>
       <c r="I269">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="K269" t="s">
         <v>1421</v>
@@ -14974,7 +14974,7 @@
         <v>1417</v>
       </c>
       <c r="I270">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="K270" t="s">
         <v>1424</v>
@@ -15012,7 +15012,7 @@
         <v>1417</v>
       </c>
       <c r="I271">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="K271" t="s">
         <v>1424</v>
@@ -15190,7 +15190,7 @@
         <v>1417</v>
       </c>
       <c r="I276">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="K276" t="s">
         <v>1425</v>
@@ -15228,7 +15228,7 @@
         <v>1417</v>
       </c>
       <c r="I277">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="K277" t="s">
         <v>1421</v>
@@ -15266,7 +15266,7 @@
         <v>1417</v>
       </c>
       <c r="I278">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="J278">
         <v>148</v>
@@ -15310,7 +15310,7 @@
         <v>1417</v>
       </c>
       <c r="I279">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="K279" t="s">
         <v>1423</v>
@@ -15351,7 +15351,7 @@
         <v>1417</v>
       </c>
       <c r="I280">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="K280" t="s">
         <v>1421</v>
@@ -15389,7 +15389,7 @@
         <v>1417</v>
       </c>
       <c r="I281">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="K281" t="s">
         <v>1421</v>
@@ -15430,7 +15430,7 @@
         <v>1417</v>
       </c>
       <c r="I282">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="K282" t="s">
         <v>1421</v>
@@ -15724,7 +15724,7 @@
         <v>1417</v>
       </c>
       <c r="I291">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="J291">
         <v>20</v>
@@ -15768,7 +15768,7 @@
         <v>1417</v>
       </c>
       <c r="I292">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="K292" t="s">
         <v>1424</v>
@@ -15806,7 +15806,7 @@
         <v>1417</v>
       </c>
       <c r="I293">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="K293" t="s">
         <v>1425</v>
@@ -15844,7 +15844,7 @@
         <v>1417</v>
       </c>
       <c r="I294">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="K294" t="s">
         <v>1430</v>
@@ -15981,7 +15981,7 @@
         <v>1417</v>
       </c>
       <c r="I298">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="J298">
         <v>58</v>
@@ -16145,7 +16145,7 @@
         <v>1417</v>
       </c>
       <c r="I302">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="K302" t="s">
         <v>1424</v>
@@ -16183,7 +16183,7 @@
         <v>1417</v>
       </c>
       <c r="I303">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="K303" t="s">
         <v>1421</v>
@@ -16221,7 +16221,7 @@
         <v>1417</v>
       </c>
       <c r="I304">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="K304" t="s">
         <v>1424</v>
@@ -16259,7 +16259,7 @@
         <v>1417</v>
       </c>
       <c r="I305">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="J305">
         <v>35</v>
@@ -16303,7 +16303,7 @@
         <v>1417</v>
       </c>
       <c r="I306">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="J306">
         <v>31</v>
@@ -16391,7 +16391,7 @@
         <v>1417</v>
       </c>
       <c r="I308">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="K308" t="s">
         <v>1420</v>
@@ -16508,7 +16508,7 @@
         <v>1417</v>
       </c>
       <c r="I311">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="K311" t="s">
         <v>1420</v>
@@ -16838,7 +16838,7 @@
         <v>1417</v>
       </c>
       <c r="I320">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="K320" t="s">
         <v>1425</v>
@@ -16876,7 +16876,7 @@
         <v>1417</v>
       </c>
       <c r="I321">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="K321" t="s">
         <v>1421</v>
@@ -16914,7 +16914,7 @@
         <v>1417</v>
       </c>
       <c r="I322">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="J322">
         <v>57</v>
@@ -17028,7 +17028,7 @@
         <v>1417</v>
       </c>
       <c r="I325">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="J325">
         <v>57</v>
@@ -17110,7 +17110,7 @@
         <v>1417</v>
       </c>
       <c r="I327">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="J327">
         <v>57</v>
@@ -17154,7 +17154,7 @@
         <v>1417</v>
       </c>
       <c r="I328">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="J328">
         <v>57</v>
@@ -17198,7 +17198,7 @@
         <v>1417</v>
       </c>
       <c r="I329">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="J329">
         <v>57</v>
@@ -17242,7 +17242,7 @@
         <v>1417</v>
       </c>
       <c r="I330">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="J330">
         <v>57</v>
@@ -17286,7 +17286,7 @@
         <v>1417</v>
       </c>
       <c r="I331">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="K331" t="s">
         <v>1420</v>
@@ -17324,7 +17324,7 @@
         <v>1417</v>
       </c>
       <c r="I332">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="K332" t="s">
         <v>1421</v>
@@ -17362,7 +17362,7 @@
         <v>1417</v>
       </c>
       <c r="I333">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="J333">
         <v>100</v>
@@ -17406,7 +17406,7 @@
         <v>1417</v>
       </c>
       <c r="I334">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="K334" t="s">
         <v>1421</v>
@@ -17631,7 +17631,7 @@
         <v>1417</v>
       </c>
       <c r="I340">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J340">
         <v>98</v>
@@ -17672,7 +17672,7 @@
         <v>1417</v>
       </c>
       <c r="I341">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J341">
         <v>90</v>
@@ -17713,7 +17713,7 @@
         <v>1417</v>
       </c>
       <c r="I342">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K342" t="s">
         <v>1420</v>
@@ -17827,7 +17827,7 @@
         <v>1417</v>
       </c>
       <c r="I345">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K345" t="s">
         <v>1420</v>
@@ -17947,7 +17947,7 @@
         <v>1417</v>
       </c>
       <c r="I348">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J348">
         <v>14</v>
@@ -17991,7 +17991,7 @@
         <v>1417</v>
       </c>
       <c r="I349">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K349" t="s">
         <v>1425</v>
@@ -18029,7 +18029,7 @@
         <v>1417</v>
       </c>
       <c r="I350">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J350">
         <v>46</v>
@@ -18067,7 +18067,7 @@
         <v>1417</v>
       </c>
       <c r="I351">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J351">
         <v>82</v>
@@ -18111,7 +18111,7 @@
         <v>1417</v>
       </c>
       <c r="I352">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J352">
         <v>78</v>
@@ -18155,7 +18155,7 @@
         <v>1417</v>
       </c>
       <c r="I353">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J353">
         <v>83</v>
@@ -18199,7 +18199,7 @@
         <v>1417</v>
       </c>
       <c r="I354">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K354" t="s">
         <v>1424</v>
@@ -18237,7 +18237,7 @@
         <v>1417</v>
       </c>
       <c r="I355">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J355">
         <v>8</v>
@@ -18319,7 +18319,7 @@
         <v>1417</v>
       </c>
       <c r="I357">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J357">
         <v>85</v>
@@ -18442,7 +18442,7 @@
         <v>1417</v>
       </c>
       <c r="I360">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J360">
         <v>83</v>
@@ -18489,7 +18489,7 @@
         <v>1417</v>
       </c>
       <c r="I361">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J361">
         <v>83</v>
@@ -18533,7 +18533,7 @@
         <v>1417</v>
       </c>
       <c r="I362">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K362" t="s">
         <v>1424</v>
@@ -18571,7 +18571,7 @@
         <v>1417</v>
       </c>
       <c r="I363">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K363" t="s">
         <v>1424</v>
@@ -18609,7 +18609,7 @@
         <v>1417</v>
       </c>
       <c r="I364">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J364">
         <v>83</v>
@@ -18653,7 +18653,7 @@
         <v>1417</v>
       </c>
       <c r="I365">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J365">
         <v>15</v>
@@ -18776,7 +18776,7 @@
         <v>1417</v>
       </c>
       <c r="I368">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="J368">
         <v>77</v>
@@ -18820,7 +18820,7 @@
         <v>1417</v>
       </c>
       <c r="I369">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="K369" t="s">
         <v>1424</v>
@@ -18858,7 +18858,7 @@
         <v>1417</v>
       </c>
       <c r="I370">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="K370" t="s">
         <v>1424</v>
@@ -18896,7 +18896,7 @@
         <v>1417</v>
       </c>
       <c r="I371">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="J371">
         <v>16</v>
@@ -18984,7 +18984,7 @@
         <v>1417</v>
       </c>
       <c r="I373">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="K373" t="s">
         <v>1420</v>
@@ -19022,7 +19022,7 @@
         <v>1417</v>
       </c>
       <c r="I374">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="K374" t="s">
         <v>1420</v>
@@ -19060,7 +19060,7 @@
         <v>1417</v>
       </c>
       <c r="I375">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J375">
         <v>94</v>
@@ -19101,7 +19101,7 @@
         <v>1417</v>
       </c>
       <c r="I376">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="K376" t="s">
         <v>1424</v>
@@ -19180,7 +19180,7 @@
         <v>1417</v>
       </c>
       <c r="I378">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="K378" t="s">
         <v>1424</v>
@@ -19218,7 +19218,7 @@
         <v>1417</v>
       </c>
       <c r="I379">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J379">
         <v>20</v>
@@ -19262,7 +19262,7 @@
         <v>1417</v>
       </c>
       <c r="I380">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J380">
         <v>94</v>
@@ -19306,7 +19306,7 @@
         <v>1417</v>
       </c>
       <c r="I381">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="K381" t="s">
         <v>1424</v>
@@ -19344,7 +19344,7 @@
         <v>1417</v>
       </c>
       <c r="I382">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="K382" t="s">
         <v>1424</v>
@@ -19382,7 +19382,7 @@
         <v>1417</v>
       </c>
       <c r="I383">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J383">
         <v>71</v>
@@ -19426,7 +19426,7 @@
         <v>1417</v>
       </c>
       <c r="I384">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="K384" t="s">
         <v>1421</v>
@@ -19508,7 +19508,7 @@
         <v>1417</v>
       </c>
       <c r="I386">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="K386" t="s">
         <v>1424</v>
@@ -19546,7 +19546,7 @@
         <v>1417</v>
       </c>
       <c r="I387">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="K387" t="s">
         <v>1424</v>
@@ -19584,7 +19584,7 @@
         <v>1417</v>
       </c>
       <c r="I388">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="J388">
         <v>-85</v>
@@ -19628,7 +19628,7 @@
         <v>1417</v>
       </c>
       <c r="I389">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="K389" t="s">
         <v>1425</v>
@@ -20079,7 +20079,7 @@
         <v>1417</v>
       </c>
       <c r="I400">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="K400" t="s">
         <v>1424</v>
@@ -20155,7 +20155,7 @@
         <v>1417</v>
       </c>
       <c r="I402">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="K402" t="s">
         <v>1424</v>
@@ -20193,7 +20193,7 @@
         <v>1417</v>
       </c>
       <c r="I403">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="J403">
         <v>83</v>
@@ -20237,7 +20237,7 @@
         <v>1417</v>
       </c>
       <c r="I404">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="K404" t="s">
         <v>1424</v>
@@ -20307,7 +20307,7 @@
         <v>1417</v>
       </c>
       <c r="I406">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="Q406" t="b">
         <v>1</v>
@@ -20339,7 +20339,7 @@
         <v>1417</v>
       </c>
       <c r="I407">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="Q407" t="b">
         <v>1</v>
@@ -20371,7 +20371,7 @@
         <v>1417</v>
       </c>
       <c r="I408">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="Q408" t="b">
         <v>1</v>
@@ -20403,7 +20403,7 @@
         <v>1417</v>
       </c>
       <c r="I409">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="Q409" t="b">
         <v>1</v>
@@ -20435,7 +20435,7 @@
         <v>1417</v>
       </c>
       <c r="I410">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="Q410" t="b">
         <v>1</v>
@@ -20467,7 +20467,7 @@
         <v>1417</v>
       </c>
       <c r="I411">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="Q411" t="b">
         <v>1</v>
@@ -20499,7 +20499,7 @@
         <v>1417</v>
       </c>
       <c r="I412">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="Q412" t="b">
         <v>1</v>
@@ -20531,7 +20531,7 @@
         <v>1417</v>
       </c>
       <c r="I413">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="Q413" t="b">
         <v>1</v>
@@ -20621,7 +20621,7 @@
         <v>1417</v>
       </c>
       <c r="I416">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="Q416" t="b">
         <v>1</v>
@@ -20711,7 +20711,7 @@
         <v>1417</v>
       </c>
       <c r="I419">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="Q419" t="b">
         <v>1</v>
@@ -20743,7 +20743,7 @@
         <v>1417</v>
       </c>
       <c r="I420">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="Q420" t="b">
         <v>1</v>
@@ -20775,7 +20775,7 @@
         <v>1417</v>
       </c>
       <c r="I421">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="Q421" t="b">
         <v>1</v>
@@ -20807,7 +20807,7 @@
         <v>1417</v>
       </c>
       <c r="I422">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="Q422" t="b">
         <v>1</v>
@@ -20839,7 +20839,7 @@
         <v>1417</v>
       </c>
       <c r="I423">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="Q423" t="b">
         <v>1</v>
@@ -20871,7 +20871,7 @@
         <v>1417</v>
       </c>
       <c r="I424">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="Q424" t="b">
         <v>1</v>
@@ -20903,7 +20903,7 @@
         <v>1417</v>
       </c>
       <c r="I425">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="Q425" t="b">
         <v>1</v>
@@ -20935,7 +20935,7 @@
         <v>1417</v>
       </c>
       <c r="I426">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="Q426" t="b">
         <v>1</v>
@@ -20967,7 +20967,7 @@
         <v>1417</v>
       </c>
       <c r="I427">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="Q427" t="b">
         <v>1</v>
@@ -21057,7 +21057,7 @@
         <v>1417</v>
       </c>
       <c r="I430">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="Q430" t="b">
         <v>1</v>
@@ -21089,7 +21089,7 @@
         <v>1417</v>
       </c>
       <c r="I431">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="Q431" t="b">
         <v>1</v>
@@ -21121,7 +21121,7 @@
         <v>1417</v>
       </c>
       <c r="I432">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="Q432" t="b">
         <v>1</v>
@@ -21153,7 +21153,7 @@
         <v>1417</v>
       </c>
       <c r="I433">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="Q433" t="b">
         <v>1</v>
@@ -21185,7 +21185,7 @@
         <v>1417</v>
       </c>
       <c r="I434">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="Q434" t="b">
         <v>1</v>
@@ -21217,7 +21217,7 @@
         <v>1417</v>
       </c>
       <c r="I435">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="Q435" t="b">
         <v>1</v>
@@ -21249,7 +21249,7 @@
         <v>1417</v>
       </c>
       <c r="I436">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="Q436" t="b">
         <v>1</v>
@@ -21281,7 +21281,7 @@
         <v>1419</v>
       </c>
       <c r="I437">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="Q437" t="b">
         <v>1</v>
@@ -21313,7 +21313,7 @@
         <v>1419</v>
       </c>
       <c r="I438">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="Q438" t="b">
         <v>1</v>
@@ -21345,7 +21345,7 @@
         <v>1417</v>
       </c>
       <c r="I439">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="Q439" t="b">
         <v>1</v>
@@ -21377,7 +21377,7 @@
         <v>1417</v>
       </c>
       <c r="I440">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="Q440" t="b">
         <v>1</v>
@@ -21409,7 +21409,7 @@
         <v>1417</v>
       </c>
       <c r="I441">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="Q441" t="b">
         <v>1</v>
@@ -21470,7 +21470,7 @@
         <v>1417</v>
       </c>
       <c r="I443">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="Q443" t="b">
         <v>1</v>
@@ -21560,7 +21560,7 @@
         <v>1417</v>
       </c>
       <c r="I446">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="Q446" t="b">
         <v>1</v>
@@ -21592,7 +21592,7 @@
         <v>1417</v>
       </c>
       <c r="I447">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="Q447" t="b">
         <v>1</v>
@@ -21624,7 +21624,7 @@
         <v>1417</v>
       </c>
       <c r="I448">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q448" t="b">
         <v>1</v>
@@ -21656,7 +21656,7 @@
         <v>1417</v>
       </c>
       <c r="I449">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q449" t="b">
         <v>1</v>
@@ -21688,7 +21688,7 @@
         <v>1417</v>
       </c>
       <c r="I450">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q450" t="b">
         <v>1</v>
@@ -21720,7 +21720,7 @@
         <v>1417</v>
       </c>
       <c r="I451">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="Q451" t="b">
         <v>1</v>
@@ -21781,7 +21781,7 @@
         <v>1417</v>
       </c>
       <c r="I453">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="Q453" t="b">
         <v>1</v>
@@ -21813,7 +21813,7 @@
         <v>1417</v>
       </c>
       <c r="I454">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="Q454" t="b">
         <v>1</v>
@@ -21845,7 +21845,7 @@
         <v>1417</v>
       </c>
       <c r="I455">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="Q455" t="b">
         <v>1</v>
@@ -21906,7 +21906,7 @@
         <v>1417</v>
       </c>
       <c r="I457">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="Q457" t="b">
         <v>1</v>
@@ -21938,7 +21938,7 @@
         <v>1417</v>
       </c>
       <c r="I458">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="Q458" t="b">
         <v>1</v>
@@ -21970,7 +21970,7 @@
         <v>1417</v>
       </c>
       <c r="I459">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q459" t="b">
         <v>1</v>
@@ -22002,7 +22002,7 @@
         <v>1417</v>
       </c>
       <c r="I460">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q460" t="b">
         <v>1</v>
@@ -22034,7 +22034,7 @@
         <v>1417</v>
       </c>
       <c r="I461">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q461" t="b">
         <v>1</v>
@@ -22066,7 +22066,7 @@
         <v>1417</v>
       </c>
       <c r="I462">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q462" t="b">
         <v>1</v>
@@ -22098,7 +22098,7 @@
         <v>1417</v>
       </c>
       <c r="I463">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q463" t="b">
         <v>1</v>
@@ -22130,7 +22130,7 @@
         <v>1417</v>
       </c>
       <c r="I464">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="Q464" t="b">
         <v>1</v>
@@ -22162,7 +22162,7 @@
         <v>1417</v>
       </c>
       <c r="I465">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="Q465" t="b">
         <v>1</v>
@@ -22194,7 +22194,7 @@
         <v>1417</v>
       </c>
       <c r="I466">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="Q466" t="b">
         <v>1</v>
@@ -22226,7 +22226,7 @@
         <v>1417</v>
       </c>
       <c r="I467">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="Q467" t="b">
         <v>1</v>
@@ -22258,7 +22258,7 @@
         <v>1417</v>
       </c>
       <c r="I468">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="Q468" t="b">
         <v>1</v>
@@ -22290,7 +22290,7 @@
         <v>1417</v>
       </c>
       <c r="I469">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="Q469" t="b">
         <v>1</v>
@@ -22351,7 +22351,7 @@
         <v>1417</v>
       </c>
       <c r="I471">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="Q471" t="b">
         <v>1</v>
@@ -22383,7 +22383,7 @@
         <v>1417</v>
       </c>
       <c r="I472">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="Q472" t="b">
         <v>1</v>
@@ -22415,7 +22415,7 @@
         <v>1417</v>
       </c>
       <c r="I473">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="Q473" t="b">
         <v>1</v>
@@ -22447,7 +22447,7 @@
         <v>1417</v>
       </c>
       <c r="I474">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="Q474" t="b">
         <v>1</v>
@@ -22479,7 +22479,7 @@
         <v>1417</v>
       </c>
       <c r="I475">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="Q475" t="b">
         <v>1</v>
@@ -22511,7 +22511,7 @@
         <v>1417</v>
       </c>
       <c r="I476">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="Q476" t="b">
         <v>1</v>
@@ -22543,7 +22543,7 @@
         <v>1417</v>
       </c>
       <c r="I477">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="Q477" t="b">
         <v>1</v>
@@ -22575,7 +22575,7 @@
         <v>1417</v>
       </c>
       <c r="I478">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="Q478" t="b">
         <v>1</v>
@@ -22607,7 +22607,7 @@
         <v>1417</v>
       </c>
       <c r="I479">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="Q479" t="b">
         <v>1</v>
@@ -22639,7 +22639,7 @@
         <v>1417</v>
       </c>
       <c r="I480">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="Q480" t="b">
         <v>1</v>
@@ -22671,7 +22671,7 @@
         <v>1417</v>
       </c>
       <c r="I481">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="Q481" t="b">
         <v>1</v>
@@ -22703,7 +22703,7 @@
         <v>1417</v>
       </c>
       <c r="I482">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="Q482" t="b">
         <v>1</v>
@@ -22735,7 +22735,7 @@
         <v>1417</v>
       </c>
       <c r="I483">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="Q483" t="b">
         <v>1</v>
@@ -22767,7 +22767,7 @@
         <v>1417</v>
       </c>
       <c r="I484">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="Q484" t="b">
         <v>1</v>
@@ -22799,7 +22799,7 @@
         <v>1417</v>
       </c>
       <c r="I485">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="Q485" t="b">
         <v>1</v>
@@ -22831,7 +22831,7 @@
         <v>1417</v>
       </c>
       <c r="I486">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="Q486" t="b">
         <v>1</v>
@@ -22863,7 +22863,7 @@
         <v>1417</v>
       </c>
       <c r="I487">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="Q487" t="b">
         <v>1</v>
@@ -22895,7 +22895,7 @@
         <v>1417</v>
       </c>
       <c r="I488">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="Q488" t="b">
         <v>1</v>
@@ -22927,7 +22927,7 @@
         <v>1417</v>
       </c>
       <c r="I489">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="Q489" t="b">
         <v>1</v>
@@ -22959,7 +22959,7 @@
         <v>1417</v>
       </c>
       <c r="I490">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="Q490" t="b">
         <v>1</v>
@@ -22991,7 +22991,7 @@
         <v>1417</v>
       </c>
       <c r="I491">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="Q491" t="b">
         <v>1</v>
@@ -23023,7 +23023,7 @@
         <v>1419</v>
       </c>
       <c r="I492">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="Q492" t="b">
         <v>1</v>
@@ -23055,7 +23055,7 @@
         <v>1419</v>
       </c>
       <c r="I493">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="Q493" t="b">
         <v>1</v>
@@ -23087,7 +23087,7 @@
         <v>1419</v>
       </c>
       <c r="I494">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="Q494" t="b">
         <v>1</v>
@@ -23119,7 +23119,7 @@
         <v>1419</v>
       </c>
       <c r="I495">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="Q495" t="b">
         <v>1</v>
@@ -23151,7 +23151,7 @@
         <v>1419</v>
       </c>
       <c r="I496">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="Q496" t="b">
         <v>1</v>
@@ -23183,7 +23183,7 @@
         <v>1417</v>
       </c>
       <c r="I497">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="Q497" t="b">
         <v>1</v>
@@ -23215,7 +23215,7 @@
         <v>1417</v>
       </c>
       <c r="I498">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="Q498" t="b">
         <v>1</v>
@@ -23247,7 +23247,7 @@
         <v>1419</v>
       </c>
       <c r="I499">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="Q499" t="b">
         <v>1</v>
@@ -23279,7 +23279,7 @@
         <v>1417</v>
       </c>
       <c r="I500">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="Q500" t="b">
         <v>1</v>
@@ -23311,7 +23311,7 @@
         <v>1417</v>
       </c>
       <c r="I501">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="Q501" t="b">
         <v>1</v>
@@ -23343,7 +23343,7 @@
         <v>1417</v>
       </c>
       <c r="I502">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="Q502" t="b">
         <v>1</v>
@@ -23375,7 +23375,7 @@
         <v>1417</v>
       </c>
       <c r="I503">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="Q503" t="b">
         <v>1</v>
@@ -23407,7 +23407,7 @@
         <v>1417</v>
       </c>
       <c r="I504">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="Q504" t="b">
         <v>1</v>
@@ -23439,7 +23439,7 @@
         <v>1417</v>
       </c>
       <c r="I505">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="Q505" t="b">
         <v>1</v>
@@ -23471,7 +23471,7 @@
         <v>1417</v>
       </c>
       <c r="I506">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="Q506" t="b">
         <v>1</v>
@@ -23503,7 +23503,7 @@
         <v>1417</v>
       </c>
       <c r="I507">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="Q507" t="b">
         <v>1</v>
@@ -23564,7 +23564,7 @@
         <v>1417</v>
       </c>
       <c r="I509">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="Q509" t="b">
         <v>1</v>
@@ -23596,7 +23596,7 @@
         <v>1417</v>
       </c>
       <c r="I510">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="Q510" t="b">
         <v>1</v>
@@ -23628,7 +23628,7 @@
         <v>1417</v>
       </c>
       <c r="I511">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Q511" t="b">
         <v>1</v>
@@ -23660,7 +23660,7 @@
         <v>1417</v>
       </c>
       <c r="I512">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Q512" t="b">
         <v>1</v>
@@ -23692,7 +23692,7 @@
         <v>1417</v>
       </c>
       <c r="I513">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="Q513" t="b">
         <v>1</v>
@@ -23753,7 +23753,7 @@
         <v>1417</v>
       </c>
       <c r="I515">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="Q515" t="b">
         <v>1</v>
@@ -23785,7 +23785,7 @@
         <v>1417</v>
       </c>
       <c r="I516">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="Q516" t="b">
         <v>1</v>
@@ -23817,7 +23817,7 @@
         <v>1417</v>
       </c>
       <c r="I517">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="Q517" t="b">
         <v>1</v>
@@ -23849,7 +23849,7 @@
         <v>1417</v>
       </c>
       <c r="I518">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="Q518" t="b">
         <v>1</v>
@@ -23881,7 +23881,7 @@
         <v>1417</v>
       </c>
       <c r="I519">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="Q519" t="b">
         <v>1</v>
@@ -23913,7 +23913,7 @@
         <v>1417</v>
       </c>
       <c r="I520">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="Q520" t="b">
         <v>1</v>
@@ -23945,7 +23945,7 @@
         <v>1417</v>
       </c>
       <c r="I521">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="Q521" t="b">
         <v>1</v>
@@ -23977,7 +23977,7 @@
         <v>1417</v>
       </c>
       <c r="I522">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="Q522" t="b">
         <v>1</v>
@@ -24009,7 +24009,7 @@
         <v>1417</v>
       </c>
       <c r="I523">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="Q523" t="b">
         <v>1</v>
@@ -24041,7 +24041,7 @@
         <v>1417</v>
       </c>
       <c r="I524">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Q524" t="b">
         <v>1</v>
@@ -24073,7 +24073,7 @@
         <v>1417</v>
       </c>
       <c r="I525">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Q525" t="b">
         <v>1</v>
@@ -24105,7 +24105,7 @@
         <v>1417</v>
       </c>
       <c r="I526">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Q526" t="b">
         <v>1</v>
@@ -24137,7 +24137,7 @@
         <v>1417</v>
       </c>
       <c r="I527">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Q527" t="b">
         <v>1</v>
@@ -24169,7 +24169,7 @@
         <v>1417</v>
       </c>
       <c r="I528">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="Q528" t="b">
         <v>1</v>
@@ -24201,7 +24201,7 @@
         <v>1417</v>
       </c>
       <c r="I529">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q529" t="b">
         <v>1</v>
@@ -24233,7 +24233,7 @@
         <v>1417</v>
       </c>
       <c r="I530">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q530" t="b">
         <v>1</v>
@@ -24265,7 +24265,7 @@
         <v>1417</v>
       </c>
       <c r="I531">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q531" t="b">
         <v>1</v>
@@ -24297,7 +24297,7 @@
         <v>1417</v>
       </c>
       <c r="I532">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q532" t="b">
         <v>1</v>
@@ -24329,7 +24329,7 @@
         <v>1417</v>
       </c>
       <c r="I533">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q533" t="b">
         <v>1</v>
@@ -24361,7 +24361,7 @@
         <v>1417</v>
       </c>
       <c r="I534">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q534" t="b">
         <v>1</v>
@@ -24393,7 +24393,7 @@
         <v>1417</v>
       </c>
       <c r="I535">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q535" t="b">
         <v>1</v>
@@ -24425,7 +24425,7 @@
         <v>1417</v>
       </c>
       <c r="I536">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q536" t="b">
         <v>1</v>
@@ -24457,7 +24457,7 @@
         <v>1417</v>
       </c>
       <c r="I537">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q537" t="b">
         <v>1</v>
@@ -24489,7 +24489,7 @@
         <v>1417</v>
       </c>
       <c r="I538">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q538" t="b">
         <v>1</v>
@@ -24521,7 +24521,7 @@
         <v>1417</v>
       </c>
       <c r="I539">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q539" t="b">
         <v>1</v>
@@ -24553,7 +24553,7 @@
         <v>1417</v>
       </c>
       <c r="I540">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q540" t="b">
         <v>1</v>
@@ -24585,7 +24585,7 @@
         <v>1417</v>
       </c>
       <c r="I541">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q541" t="b">
         <v>1</v>
@@ -24617,7 +24617,7 @@
         <v>1417</v>
       </c>
       <c r="I542">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q542" t="b">
         <v>1</v>
@@ -24649,7 +24649,7 @@
         <v>1417</v>
       </c>
       <c r="I543">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q543" t="b">
         <v>1</v>
@@ -24681,7 +24681,7 @@
         <v>1417</v>
       </c>
       <c r="I544">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q544" t="b">
         <v>1</v>
@@ -24713,7 +24713,7 @@
         <v>1417</v>
       </c>
       <c r="I545">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q545" t="b">
         <v>1</v>
@@ -24745,7 +24745,7 @@
         <v>1417</v>
       </c>
       <c r="I546">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Q546" t="b">
         <v>1</v>
@@ -24777,7 +24777,7 @@
         <v>1417</v>
       </c>
       <c r="I547">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Q547" t="b">
         <v>1</v>
@@ -24809,7 +24809,7 @@
         <v>1417</v>
       </c>
       <c r="I548">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Q548" t="b">
         <v>1</v>
@@ -24841,7 +24841,7 @@
         <v>1417</v>
       </c>
       <c r="I549">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Q549" t="b">
         <v>1</v>
@@ -24873,7 +24873,7 @@
         <v>1417</v>
       </c>
       <c r="I550">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Q550" t="b">
         <v>1</v>
@@ -24905,7 +24905,7 @@
         <v>1417</v>
       </c>
       <c r="I551">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Q551" t="b">
         <v>1</v>
@@ -24937,7 +24937,7 @@
         <v>1417</v>
       </c>
       <c r="I552">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Q552" t="b">
         <v>1</v>
@@ -24969,7 +24969,7 @@
         <v>1417</v>
       </c>
       <c r="I553">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Q553" t="b">
         <v>1</v>
@@ -25001,7 +25001,7 @@
         <v>1417</v>
       </c>
       <c r="I554">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Q554" t="b">
         <v>1</v>
@@ -25033,7 +25033,7 @@
         <v>1417</v>
       </c>
       <c r="I555">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Q555" t="b">
         <v>1</v>
@@ -25065,7 +25065,7 @@
         <v>1417</v>
       </c>
       <c r="I556">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Q556" t="b">
         <v>1</v>
@@ -25097,7 +25097,7 @@
         <v>1417</v>
       </c>
       <c r="I557">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="Q557" t="b">
         <v>1</v>
@@ -25129,7 +25129,7 @@
         <v>1417</v>
       </c>
       <c r="I558">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="Q558" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: reparaveis (27/10/2026 13:27)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
@@ -5132,7 +5132,7 @@
         <v>1417</v>
       </c>
       <c r="I2">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="K2" t="s">
         <v>1420</v>
@@ -5170,7 +5170,7 @@
         <v>1417</v>
       </c>
       <c r="I3">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="K3" t="s">
         <v>1421</v>
@@ -5208,7 +5208,7 @@
         <v>1417</v>
       </c>
       <c r="I4">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="K4" t="s">
         <v>1421</v>
@@ -5246,7 +5246,7 @@
         <v>1417</v>
       </c>
       <c r="I5">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="J5">
         <v>279</v>
@@ -5290,7 +5290,7 @@
         <v>1417</v>
       </c>
       <c r="I6">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="J6">
         <v>153</v>
@@ -5334,7 +5334,7 @@
         <v>1417</v>
       </c>
       <c r="I7">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="J7">
         <v>112</v>
@@ -5410,7 +5410,7 @@
         <v>1417</v>
       </c>
       <c r="I9">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="J9">
         <v>362</v>
@@ -5457,7 +5457,7 @@
         <v>1417</v>
       </c>
       <c r="I10">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="J10">
         <v>378</v>
@@ -5504,7 +5504,7 @@
         <v>1417</v>
       </c>
       <c r="I11">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="J11">
         <v>112</v>
@@ -5551,7 +5551,7 @@
         <v>1417</v>
       </c>
       <c r="I12">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="J12">
         <v>124</v>
@@ -5624,7 +5624,7 @@
         <v>1417</v>
       </c>
       <c r="I14">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="J14">
         <v>64</v>
@@ -5703,7 +5703,7 @@
         <v>1417</v>
       </c>
       <c r="I16">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="K16" t="s">
         <v>1420</v>
@@ -5741,7 +5741,7 @@
         <v>1417</v>
       </c>
       <c r="I17">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="J17">
         <v>161</v>
@@ -5785,7 +5785,7 @@
         <v>1417</v>
       </c>
       <c r="I18">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="J18">
         <v>66</v>
@@ -5858,7 +5858,7 @@
         <v>1417</v>
       </c>
       <c r="I20">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="J20">
         <v>399</v>
@@ -5931,7 +5931,7 @@
         <v>1417</v>
       </c>
       <c r="I22">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="K22" t="s">
         <v>1424</v>
@@ -5969,7 +5969,7 @@
         <v>1417</v>
       </c>
       <c r="I23">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="J23">
         <v>229</v>
@@ -6074,7 +6074,7 @@
         <v>1417</v>
       </c>
       <c r="I26">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="J26">
         <v>155</v>
@@ -6121,7 +6121,7 @@
         <v>1417</v>
       </c>
       <c r="I27">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="K27" t="s">
         <v>1424</v>
@@ -6217,7 +6217,7 @@
         <v>1417</v>
       </c>
       <c r="I30">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="J30">
         <v>209</v>
@@ -6290,7 +6290,7 @@
         <v>1417</v>
       </c>
       <c r="I32">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="K32" t="s">
         <v>1420</v>
@@ -6499,7 +6499,7 @@
         <v>1417</v>
       </c>
       <c r="I39">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="K39" t="s">
         <v>1425</v>
@@ -6662,7 +6662,7 @@
         <v>1417</v>
       </c>
       <c r="I44">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="J44">
         <v>87</v>
@@ -6709,7 +6709,7 @@
         <v>1417</v>
       </c>
       <c r="I45">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="J45">
         <v>331</v>
@@ -6756,7 +6756,7 @@
         <v>1417</v>
       </c>
       <c r="I46">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="K46" t="s">
         <v>1424</v>
@@ -6797,7 +6797,7 @@
         <v>1417</v>
       </c>
       <c r="I47">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="J47">
         <v>344</v>
@@ -6844,7 +6844,7 @@
         <v>1417</v>
       </c>
       <c r="I48">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="K48" t="s">
         <v>1424</v>
@@ -6911,7 +6911,7 @@
         <v>1417</v>
       </c>
       <c r="I50">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="K50" t="s">
         <v>1424</v>
@@ -6978,7 +6978,7 @@
         <v>1417</v>
       </c>
       <c r="I52">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="K52" t="s">
         <v>1420</v>
@@ -7016,7 +7016,7 @@
         <v>1417</v>
       </c>
       <c r="I53">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="K53" t="s">
         <v>1421</v>
@@ -7054,7 +7054,7 @@
         <v>1417</v>
       </c>
       <c r="I54">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="K54" t="s">
         <v>1421</v>
@@ -7330,7 +7330,7 @@
         <v>1417</v>
       </c>
       <c r="I63">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="J63">
         <v>293</v>
@@ -7377,7 +7377,7 @@
         <v>1417</v>
       </c>
       <c r="I64">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="J64">
         <v>320</v>
@@ -7607,7 +7607,7 @@
         <v>1417</v>
       </c>
       <c r="I71">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="J71">
         <v>429</v>
@@ -7680,7 +7680,7 @@
         <v>1417</v>
       </c>
       <c r="I73">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="K73" t="s">
         <v>1420</v>
@@ -7788,7 +7788,7 @@
         <v>1417</v>
       </c>
       <c r="I76">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="K76" t="s">
         <v>1427</v>
@@ -7881,7 +7881,7 @@
         <v>1417</v>
       </c>
       <c r="I79">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="K79" t="s">
         <v>1427</v>
@@ -7986,7 +7986,7 @@
         <v>1417</v>
       </c>
       <c r="I82">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="K82" t="s">
         <v>1424</v>
@@ -8053,7 +8053,7 @@
         <v>1417</v>
       </c>
       <c r="I84">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="J84">
         <v>40</v>
@@ -8100,7 +8100,7 @@
         <v>1417</v>
       </c>
       <c r="I85">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="K85" t="s">
         <v>1421</v>
@@ -8138,7 +8138,7 @@
         <v>1417</v>
       </c>
       <c r="I86">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="K86" t="s">
         <v>1421</v>
@@ -8176,7 +8176,7 @@
         <v>1417</v>
       </c>
       <c r="I87">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="J87">
         <v>-16</v>
@@ -8299,7 +8299,7 @@
         <v>1417</v>
       </c>
       <c r="I90">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="K90" t="s">
         <v>1394</v>
@@ -8448,7 +8448,7 @@
         <v>1417</v>
       </c>
       <c r="I94">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="K94" t="s">
         <v>1424</v>
@@ -8527,7 +8527,7 @@
         <v>1417</v>
       </c>
       <c r="I96">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="J96">
         <v>17</v>
@@ -8574,7 +8574,7 @@
         <v>1417</v>
       </c>
       <c r="I97">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="J97">
         <v>20</v>
@@ -8621,7 +8621,7 @@
         <v>1417</v>
       </c>
       <c r="I98">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="K98" t="s">
         <v>1424</v>
@@ -8898,7 +8898,7 @@
         <v>1417</v>
       </c>
       <c r="I106">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="J106">
         <v>49</v>
@@ -8942,7 +8942,7 @@
         <v>1417</v>
       </c>
       <c r="I107">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="J107">
         <v>36</v>
@@ -8986,7 +8986,7 @@
         <v>1417</v>
       </c>
       <c r="I108">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="K108" t="s">
         <v>1421</v>
@@ -9024,7 +9024,7 @@
         <v>1417</v>
       </c>
       <c r="I109">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="K109" t="s">
         <v>1421</v>
@@ -9207,7 +9207,7 @@
         <v>1417</v>
       </c>
       <c r="I115">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="K115" t="s">
         <v>1421</v>
@@ -9245,7 +9245,7 @@
         <v>1417</v>
       </c>
       <c r="I116">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="K116" t="s">
         <v>1421</v>
@@ -9283,7 +9283,7 @@
         <v>1417</v>
       </c>
       <c r="I117">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="K117" t="s">
         <v>1421</v>
@@ -9321,7 +9321,7 @@
         <v>1417</v>
       </c>
       <c r="I118">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="K118" t="s">
         <v>1421</v>
@@ -9359,7 +9359,7 @@
         <v>1417</v>
       </c>
       <c r="I119">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="K119" t="s">
         <v>1421</v>
@@ -9397,7 +9397,7 @@
         <v>1417</v>
       </c>
       <c r="I120">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="K120" t="s">
         <v>1421</v>
@@ -9435,7 +9435,7 @@
         <v>1417</v>
       </c>
       <c r="I121">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="J121">
         <v>251</v>
@@ -9482,7 +9482,7 @@
         <v>1417</v>
       </c>
       <c r="I122">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="K122" t="s">
         <v>1421</v>
@@ -9549,7 +9549,7 @@
         <v>1417</v>
       </c>
       <c r="I124">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="K124" t="s">
         <v>1421</v>
@@ -9587,7 +9587,7 @@
         <v>1417</v>
       </c>
       <c r="I125">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="K125" t="s">
         <v>1427</v>
@@ -9683,7 +9683,7 @@
         <v>1417</v>
       </c>
       <c r="I128">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="K128" t="s">
         <v>1421</v>
@@ -9721,7 +9721,7 @@
         <v>1417</v>
       </c>
       <c r="I129">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="K129" t="s">
         <v>1420</v>
@@ -9759,7 +9759,7 @@
         <v>1417</v>
       </c>
       <c r="I130">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="J130">
         <v>47</v>
@@ -9835,7 +9835,7 @@
         <v>1417</v>
       </c>
       <c r="I132">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="J132">
         <v>145</v>
@@ -9911,7 +9911,7 @@
         <v>1417</v>
       </c>
       <c r="I134">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="K134" t="s">
         <v>1420</v>
@@ -10036,7 +10036,7 @@
         <v>1417</v>
       </c>
       <c r="I138">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="K138" t="s">
         <v>1421</v>
@@ -10420,7 +10420,7 @@
         <v>1417</v>
       </c>
       <c r="I150">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="J150">
         <v>201</v>
@@ -10607,7 +10607,7 @@
         <v>1417</v>
       </c>
       <c r="I155">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="K155" t="s">
         <v>1427</v>
@@ -10642,7 +10642,7 @@
         <v>1417</v>
       </c>
       <c r="I156">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="K156" t="s">
         <v>1421</v>
@@ -10680,7 +10680,7 @@
         <v>1417</v>
       </c>
       <c r="I157">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="J157">
         <v>371</v>
@@ -10724,7 +10724,7 @@
         <v>1417</v>
       </c>
       <c r="I158">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="J158">
         <v>52</v>
@@ -10768,7 +10768,7 @@
         <v>1417</v>
       </c>
       <c r="I159">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="K159" t="s">
         <v>1421</v>
@@ -10806,7 +10806,7 @@
         <v>1417</v>
       </c>
       <c r="I160">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="K160" t="s">
         <v>1421</v>
@@ -10844,7 +10844,7 @@
         <v>1417</v>
       </c>
       <c r="I161">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="J161">
         <v>55</v>
@@ -10979,7 +10979,7 @@
         <v>1417</v>
       </c>
       <c r="I164">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="O164" t="s">
         <v>1533</v>
@@ -11154,7 +11154,7 @@
         <v>1417</v>
       </c>
       <c r="I169">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="K169" t="s">
         <v>1394</v>
@@ -11364,7 +11364,7 @@
         <v>1417</v>
       </c>
       <c r="I175">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="J175">
         <v>205</v>
@@ -11411,7 +11411,7 @@
         <v>1417</v>
       </c>
       <c r="I176">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="K176" t="s">
         <v>1421</v>
@@ -11449,7 +11449,7 @@
         <v>1417</v>
       </c>
       <c r="I177">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="J177">
         <v>44</v>
@@ -11496,7 +11496,7 @@
         <v>1417</v>
       </c>
       <c r="I178">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="K178" t="s">
         <v>1420</v>
@@ -11563,7 +11563,7 @@
         <v>1417</v>
       </c>
       <c r="I180">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="K180" t="s">
         <v>1420</v>
@@ -11659,7 +11659,7 @@
         <v>1417</v>
       </c>
       <c r="I183">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="K183" t="s">
         <v>1421</v>
@@ -11697,7 +11697,7 @@
         <v>1417</v>
       </c>
       <c r="I184">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="K184" t="s">
         <v>1427</v>
@@ -11732,7 +11732,7 @@
         <v>1417</v>
       </c>
       <c r="I185">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="K185" t="s">
         <v>1421</v>
@@ -11770,7 +11770,7 @@
         <v>1417</v>
       </c>
       <c r="I186">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="K186" t="s">
         <v>1421</v>
@@ -11808,7 +11808,7 @@
         <v>1417</v>
       </c>
       <c r="I187">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="J187">
         <v>75</v>
@@ -11855,7 +11855,7 @@
         <v>1417</v>
       </c>
       <c r="I188">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="J188">
         <v>40</v>
@@ -11902,7 +11902,7 @@
         <v>1417</v>
       </c>
       <c r="I189">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="J189">
         <v>155</v>
@@ -11946,7 +11946,7 @@
         <v>1417</v>
       </c>
       <c r="I190">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="J190">
         <v>107</v>
@@ -11990,7 +11990,7 @@
         <v>1417</v>
       </c>
       <c r="I191">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="J191">
         <v>5</v>
@@ -12034,7 +12034,7 @@
         <v>1417</v>
       </c>
       <c r="I192">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="K192" t="s">
         <v>1421</v>
@@ -12072,7 +12072,7 @@
         <v>1417</v>
       </c>
       <c r="I193">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="K193" t="s">
         <v>1426</v>
@@ -12267,7 +12267,7 @@
         <v>1417</v>
       </c>
       <c r="I199">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="J199">
         <v>70</v>
@@ -12352,7 +12352,7 @@
         <v>1417</v>
       </c>
       <c r="I201">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="K201" t="s">
         <v>1421</v>
@@ -12390,7 +12390,7 @@
         <v>1417</v>
       </c>
       <c r="I202">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="K202" t="s">
         <v>1421</v>
@@ -12469,7 +12469,7 @@
         <v>1417</v>
       </c>
       <c r="I204">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="K204" t="s">
         <v>1420</v>
@@ -12507,7 +12507,7 @@
         <v>1417</v>
       </c>
       <c r="I205">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="K205" t="s">
         <v>1420</v>
@@ -12574,7 +12574,7 @@
         <v>1417</v>
       </c>
       <c r="I207">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="J207">
         <v>167</v>
@@ -12618,7 +12618,7 @@
         <v>1417</v>
       </c>
       <c r="I208">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="J208">
         <v>45</v>
@@ -12662,7 +12662,7 @@
         <v>1417</v>
       </c>
       <c r="I209">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="J209">
         <v>191</v>
@@ -12706,7 +12706,7 @@
         <v>1417</v>
       </c>
       <c r="I210">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="K210" t="s">
         <v>1424</v>
@@ -12802,7 +12802,7 @@
         <v>1417</v>
       </c>
       <c r="I213">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="K213" t="s">
         <v>1421</v>
@@ -12840,7 +12840,7 @@
         <v>1417</v>
       </c>
       <c r="I214">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J214">
         <v>14</v>
@@ -12887,7 +12887,7 @@
         <v>1417</v>
       </c>
       <c r="I215">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="K215" t="s">
         <v>1421</v>
@@ -12954,7 +12954,7 @@
         <v>1417</v>
       </c>
       <c r="I217">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="J217">
         <v>42</v>
@@ -12998,7 +12998,7 @@
         <v>1417</v>
       </c>
       <c r="I218">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="J218">
         <v>166</v>
@@ -13086,7 +13086,7 @@
         <v>1417</v>
       </c>
       <c r="I220">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="J220">
         <v>154</v>
@@ -13472,7 +13472,7 @@
         <v>1417</v>
       </c>
       <c r="I230">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="J230">
         <v>197</v>
@@ -13516,7 +13516,7 @@
         <v>1417</v>
       </c>
       <c r="I231">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="J231">
         <v>35</v>
@@ -13618,7 +13618,7 @@
         <v>1417</v>
       </c>
       <c r="I234">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="J234">
         <v>35</v>
@@ -13665,7 +13665,7 @@
         <v>1417</v>
       </c>
       <c r="I235">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="J235">
         <v>35</v>
@@ -13712,7 +13712,7 @@
         <v>1417</v>
       </c>
       <c r="I236">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="J236">
         <v>86</v>
@@ -13829,7 +13829,7 @@
         <v>1417</v>
       </c>
       <c r="I239">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="K239" t="s">
         <v>1394</v>
@@ -13928,7 +13928,7 @@
         <v>1417</v>
       </c>
       <c r="I242">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="K242" t="s">
         <v>1420</v>
@@ -13995,7 +13995,7 @@
         <v>1417</v>
       </c>
       <c r="I244">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="J244">
         <v>15</v>
@@ -14036,7 +14036,7 @@
         <v>1417</v>
       </c>
       <c r="I245">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="J245">
         <v>15</v>
@@ -14179,7 +14179,7 @@
         <v>1417</v>
       </c>
       <c r="I249">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="K249" t="s">
         <v>1421</v>
@@ -14313,7 +14313,7 @@
         <v>1417</v>
       </c>
       <c r="I253">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="J253">
         <v>162</v>
@@ -14357,7 +14357,7 @@
         <v>1417</v>
       </c>
       <c r="I254">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="K254" t="s">
         <v>1424</v>
@@ -14436,7 +14436,7 @@
         <v>1417</v>
       </c>
       <c r="I256">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="J256">
         <v>23</v>
@@ -14620,7 +14620,7 @@
         <v>1417</v>
       </c>
       <c r="I261">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="J261">
         <v>162</v>
@@ -14778,7 +14778,7 @@
         <v>1417</v>
       </c>
       <c r="I265">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="J265">
         <v>162</v>
@@ -14863,7 +14863,7 @@
         <v>1417</v>
       </c>
       <c r="I267">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="K267" t="s">
         <v>1424</v>
@@ -14901,7 +14901,7 @@
         <v>1417</v>
       </c>
       <c r="I268">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="K268" t="s">
         <v>1421</v>
@@ -14936,7 +14936,7 @@
         <v>1417</v>
       </c>
       <c r="I269">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="K269" t="s">
         <v>1421</v>
@@ -14974,7 +14974,7 @@
         <v>1417</v>
       </c>
       <c r="I270">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="K270" t="s">
         <v>1424</v>
@@ -15012,7 +15012,7 @@
         <v>1417</v>
       </c>
       <c r="I271">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="K271" t="s">
         <v>1424</v>
@@ -15190,7 +15190,7 @@
         <v>1417</v>
       </c>
       <c r="I276">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="K276" t="s">
         <v>1425</v>
@@ -15228,7 +15228,7 @@
         <v>1417</v>
       </c>
       <c r="I277">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="K277" t="s">
         <v>1421</v>
@@ -15266,7 +15266,7 @@
         <v>1417</v>
       </c>
       <c r="I278">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="J278">
         <v>148</v>
@@ -15310,7 +15310,7 @@
         <v>1417</v>
       </c>
       <c r="I279">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="K279" t="s">
         <v>1423</v>
@@ -15351,7 +15351,7 @@
         <v>1417</v>
       </c>
       <c r="I280">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="K280" t="s">
         <v>1421</v>
@@ -15389,7 +15389,7 @@
         <v>1417</v>
       </c>
       <c r="I281">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="K281" t="s">
         <v>1421</v>
@@ -15430,7 +15430,7 @@
         <v>1417</v>
       </c>
       <c r="I282">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="K282" t="s">
         <v>1421</v>
@@ -15724,7 +15724,7 @@
         <v>1417</v>
       </c>
       <c r="I291">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="J291">
         <v>20</v>
@@ -15768,7 +15768,7 @@
         <v>1417</v>
       </c>
       <c r="I292">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="K292" t="s">
         <v>1424</v>
@@ -15806,7 +15806,7 @@
         <v>1417</v>
       </c>
       <c r="I293">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="K293" t="s">
         <v>1425</v>
@@ -15844,7 +15844,7 @@
         <v>1417</v>
       </c>
       <c r="I294">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="K294" t="s">
         <v>1430</v>
@@ -15981,7 +15981,7 @@
         <v>1417</v>
       </c>
       <c r="I298">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="J298">
         <v>58</v>
@@ -16145,7 +16145,7 @@
         <v>1417</v>
       </c>
       <c r="I302">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="K302" t="s">
         <v>1424</v>
@@ -16183,7 +16183,7 @@
         <v>1417</v>
       </c>
       <c r="I303">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="K303" t="s">
         <v>1421</v>
@@ -16221,7 +16221,7 @@
         <v>1417</v>
       </c>
       <c r="I304">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="K304" t="s">
         <v>1424</v>
@@ -16259,7 +16259,7 @@
         <v>1417</v>
       </c>
       <c r="I305">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="J305">
         <v>35</v>
@@ -16303,7 +16303,7 @@
         <v>1417</v>
       </c>
       <c r="I306">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="J306">
         <v>31</v>
@@ -16391,7 +16391,7 @@
         <v>1417</v>
       </c>
       <c r="I308">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="K308" t="s">
         <v>1420</v>
@@ -16508,7 +16508,7 @@
         <v>1417</v>
       </c>
       <c r="I311">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="K311" t="s">
         <v>1420</v>
@@ -16838,7 +16838,7 @@
         <v>1417</v>
       </c>
       <c r="I320">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="K320" t="s">
         <v>1425</v>
@@ -16876,7 +16876,7 @@
         <v>1417</v>
       </c>
       <c r="I321">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="K321" t="s">
         <v>1421</v>
@@ -16914,7 +16914,7 @@
         <v>1417</v>
       </c>
       <c r="I322">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="J322">
         <v>57</v>
@@ -17028,7 +17028,7 @@
         <v>1417</v>
       </c>
       <c r="I325">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="J325">
         <v>57</v>
@@ -17110,7 +17110,7 @@
         <v>1417</v>
       </c>
       <c r="I327">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="J327">
         <v>57</v>
@@ -17154,7 +17154,7 @@
         <v>1417</v>
       </c>
       <c r="I328">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="J328">
         <v>57</v>
@@ -17198,7 +17198,7 @@
         <v>1417</v>
       </c>
       <c r="I329">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="J329">
         <v>57</v>
@@ -17242,7 +17242,7 @@
         <v>1417</v>
       </c>
       <c r="I330">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="J330">
         <v>57</v>
@@ -17286,7 +17286,7 @@
         <v>1417</v>
       </c>
       <c r="I331">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="K331" t="s">
         <v>1420</v>
@@ -17324,7 +17324,7 @@
         <v>1417</v>
       </c>
       <c r="I332">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="K332" t="s">
         <v>1421</v>
@@ -17362,7 +17362,7 @@
         <v>1417</v>
       </c>
       <c r="I333">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="J333">
         <v>100</v>
@@ -17406,7 +17406,7 @@
         <v>1417</v>
       </c>
       <c r="I334">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="K334" t="s">
         <v>1421</v>
@@ -17631,7 +17631,7 @@
         <v>1417</v>
       </c>
       <c r="I340">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="J340">
         <v>98</v>
@@ -17672,7 +17672,7 @@
         <v>1417</v>
       </c>
       <c r="I341">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="J341">
         <v>90</v>
@@ -17713,7 +17713,7 @@
         <v>1417</v>
       </c>
       <c r="I342">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="K342" t="s">
         <v>1420</v>
@@ -17827,7 +17827,7 @@
         <v>1417</v>
       </c>
       <c r="I345">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="K345" t="s">
         <v>1420</v>
@@ -17947,7 +17947,7 @@
         <v>1417</v>
       </c>
       <c r="I348">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="J348">
         <v>14</v>
@@ -17991,7 +17991,7 @@
         <v>1417</v>
       </c>
       <c r="I349">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="K349" t="s">
         <v>1425</v>
@@ -18029,7 +18029,7 @@
         <v>1417</v>
       </c>
       <c r="I350">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="J350">
         <v>46</v>
@@ -18067,7 +18067,7 @@
         <v>1417</v>
       </c>
       <c r="I351">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="J351">
         <v>82</v>
@@ -18111,7 +18111,7 @@
         <v>1417</v>
       </c>
       <c r="I352">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="J352">
         <v>78</v>
@@ -18155,7 +18155,7 @@
         <v>1417</v>
       </c>
       <c r="I353">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="J353">
         <v>83</v>
@@ -18199,7 +18199,7 @@
         <v>1417</v>
       </c>
       <c r="I354">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="K354" t="s">
         <v>1424</v>
@@ -18237,7 +18237,7 @@
         <v>1417</v>
       </c>
       <c r="I355">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="J355">
         <v>8</v>
@@ -18319,7 +18319,7 @@
         <v>1417</v>
       </c>
       <c r="I357">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="J357">
         <v>85</v>
@@ -18442,7 +18442,7 @@
         <v>1417</v>
       </c>
       <c r="I360">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="J360">
         <v>83</v>
@@ -18489,7 +18489,7 @@
         <v>1417</v>
       </c>
       <c r="I361">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="J361">
         <v>83</v>
@@ -18533,7 +18533,7 @@
         <v>1417</v>
       </c>
       <c r="I362">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="K362" t="s">
         <v>1424</v>
@@ -18571,7 +18571,7 @@
         <v>1417</v>
       </c>
       <c r="I363">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="K363" t="s">
         <v>1424</v>
@@ -18609,7 +18609,7 @@
         <v>1417</v>
       </c>
       <c r="I364">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="J364">
         <v>83</v>
@@ -18653,7 +18653,7 @@
         <v>1417</v>
       </c>
       <c r="I365">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="J365">
         <v>15</v>
@@ -18776,7 +18776,7 @@
         <v>1417</v>
       </c>
       <c r="I368">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J368">
         <v>77</v>
@@ -18820,7 +18820,7 @@
         <v>1417</v>
       </c>
       <c r="I369">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="K369" t="s">
         <v>1424</v>
@@ -18858,7 +18858,7 @@
         <v>1417</v>
       </c>
       <c r="I370">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="K370" t="s">
         <v>1424</v>
@@ -18896,7 +18896,7 @@
         <v>1417</v>
       </c>
       <c r="I371">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J371">
         <v>16</v>
@@ -18984,7 +18984,7 @@
         <v>1417</v>
       </c>
       <c r="I373">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="K373" t="s">
         <v>1420</v>
@@ -19022,7 +19022,7 @@
         <v>1417</v>
       </c>
       <c r="I374">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="K374" t="s">
         <v>1420</v>
@@ -19060,7 +19060,7 @@
         <v>1417</v>
       </c>
       <c r="I375">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="J375">
         <v>94</v>
@@ -19101,7 +19101,7 @@
         <v>1417</v>
       </c>
       <c r="I376">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K376" t="s">
         <v>1424</v>
@@ -19180,7 +19180,7 @@
         <v>1417</v>
       </c>
       <c r="I378">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K378" t="s">
         <v>1424</v>
@@ -19218,7 +19218,7 @@
         <v>1417</v>
       </c>
       <c r="I379">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="J379">
         <v>20</v>
@@ -19262,7 +19262,7 @@
         <v>1417</v>
       </c>
       <c r="I380">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="J380">
         <v>94</v>
@@ -19306,7 +19306,7 @@
         <v>1417</v>
       </c>
       <c r="I381">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K381" t="s">
         <v>1424</v>
@@ -19344,7 +19344,7 @@
         <v>1417</v>
       </c>
       <c r="I382">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K382" t="s">
         <v>1424</v>
@@ -19382,7 +19382,7 @@
         <v>1417</v>
       </c>
       <c r="I383">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="J383">
         <v>71</v>
@@ -19426,7 +19426,7 @@
         <v>1417</v>
       </c>
       <c r="I384">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="K384" t="s">
         <v>1421</v>
@@ -19508,7 +19508,7 @@
         <v>1417</v>
       </c>
       <c r="I386">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="K386" t="s">
         <v>1424</v>
@@ -19546,7 +19546,7 @@
         <v>1417</v>
       </c>
       <c r="I387">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="K387" t="s">
         <v>1424</v>
@@ -19584,7 +19584,7 @@
         <v>1417</v>
       </c>
       <c r="I388">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="J388">
         <v>-85</v>
@@ -19628,7 +19628,7 @@
         <v>1417</v>
       </c>
       <c r="I389">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="K389" t="s">
         <v>1425</v>
@@ -20079,7 +20079,7 @@
         <v>1417</v>
       </c>
       <c r="I400">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="K400" t="s">
         <v>1424</v>
@@ -20155,7 +20155,7 @@
         <v>1417</v>
       </c>
       <c r="I402">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="K402" t="s">
         <v>1424</v>
@@ -20193,7 +20193,7 @@
         <v>1417</v>
       </c>
       <c r="I403">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="J403">
         <v>83</v>
@@ -20237,7 +20237,7 @@
         <v>1417</v>
       </c>
       <c r="I404">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="K404" t="s">
         <v>1424</v>
@@ -20307,7 +20307,7 @@
         <v>1417</v>
       </c>
       <c r="I406">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="Q406" t="b">
         <v>1</v>
@@ -20339,7 +20339,7 @@
         <v>1417</v>
       </c>
       <c r="I407">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="Q407" t="b">
         <v>1</v>
@@ -20371,7 +20371,7 @@
         <v>1417</v>
       </c>
       <c r="I408">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="Q408" t="b">
         <v>1</v>
@@ -20403,7 +20403,7 @@
         <v>1417</v>
       </c>
       <c r="I409">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="Q409" t="b">
         <v>1</v>
@@ -20435,7 +20435,7 @@
         <v>1417</v>
       </c>
       <c r="I410">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="Q410" t="b">
         <v>1</v>
@@ -20467,7 +20467,7 @@
         <v>1417</v>
       </c>
       <c r="I411">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="Q411" t="b">
         <v>1</v>
@@ -20499,7 +20499,7 @@
         <v>1417</v>
       </c>
       <c r="I412">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="Q412" t="b">
         <v>1</v>
@@ -20531,7 +20531,7 @@
         <v>1417</v>
       </c>
       <c r="I413">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="Q413" t="b">
         <v>1</v>
@@ -20621,7 +20621,7 @@
         <v>1417</v>
       </c>
       <c r="I416">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="Q416" t="b">
         <v>1</v>
@@ -20711,7 +20711,7 @@
         <v>1417</v>
       </c>
       <c r="I419">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="Q419" t="b">
         <v>1</v>
@@ -20743,7 +20743,7 @@
         <v>1417</v>
       </c>
       <c r="I420">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="Q420" t="b">
         <v>1</v>
@@ -20775,7 +20775,7 @@
         <v>1417</v>
       </c>
       <c r="I421">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="Q421" t="b">
         <v>1</v>
@@ -20807,7 +20807,7 @@
         <v>1417</v>
       </c>
       <c r="I422">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="Q422" t="b">
         <v>1</v>
@@ -20839,7 +20839,7 @@
         <v>1417</v>
       </c>
       <c r="I423">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="Q423" t="b">
         <v>1</v>
@@ -20871,7 +20871,7 @@
         <v>1417</v>
       </c>
       <c r="I424">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="Q424" t="b">
         <v>1</v>
@@ -20903,7 +20903,7 @@
         <v>1417</v>
       </c>
       <c r="I425">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="Q425" t="b">
         <v>1</v>
@@ -20935,7 +20935,7 @@
         <v>1417</v>
       </c>
       <c r="I426">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="Q426" t="b">
         <v>1</v>
@@ -20967,7 +20967,7 @@
         <v>1417</v>
       </c>
       <c r="I427">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="Q427" t="b">
         <v>1</v>
@@ -21057,7 +21057,7 @@
         <v>1417</v>
       </c>
       <c r="I430">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="Q430" t="b">
         <v>1</v>
@@ -21089,7 +21089,7 @@
         <v>1417</v>
       </c>
       <c r="I431">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="Q431" t="b">
         <v>1</v>
@@ -21121,7 +21121,7 @@
         <v>1417</v>
       </c>
       <c r="I432">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="Q432" t="b">
         <v>1</v>
@@ -21153,7 +21153,7 @@
         <v>1417</v>
       </c>
       <c r="I433">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="Q433" t="b">
         <v>1</v>
@@ -21185,7 +21185,7 @@
         <v>1417</v>
       </c>
       <c r="I434">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="Q434" t="b">
         <v>1</v>
@@ -21217,7 +21217,7 @@
         <v>1417</v>
       </c>
       <c r="I435">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="Q435" t="b">
         <v>1</v>
@@ -21249,7 +21249,7 @@
         <v>1417</v>
       </c>
       <c r="I436">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="Q436" t="b">
         <v>1</v>
@@ -21281,7 +21281,7 @@
         <v>1419</v>
       </c>
       <c r="I437">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="Q437" t="b">
         <v>1</v>
@@ -21313,7 +21313,7 @@
         <v>1419</v>
       </c>
       <c r="I438">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="Q438" t="b">
         <v>1</v>
@@ -21345,7 +21345,7 @@
         <v>1417</v>
       </c>
       <c r="I439">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="Q439" t="b">
         <v>1</v>
@@ -21377,7 +21377,7 @@
         <v>1417</v>
       </c>
       <c r="I440">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="Q440" t="b">
         <v>1</v>
@@ -21409,7 +21409,7 @@
         <v>1417</v>
       </c>
       <c r="I441">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="Q441" t="b">
         <v>1</v>
@@ -21470,7 +21470,7 @@
         <v>1417</v>
       </c>
       <c r="I443">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="Q443" t="b">
         <v>1</v>
@@ -21560,7 +21560,7 @@
         <v>1417</v>
       </c>
       <c r="I446">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="Q446" t="b">
         <v>1</v>
@@ -21592,7 +21592,7 @@
         <v>1417</v>
       </c>
       <c r="I447">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="Q447" t="b">
         <v>1</v>
@@ -21624,7 +21624,7 @@
         <v>1417</v>
       </c>
       <c r="I448">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="Q448" t="b">
         <v>1</v>
@@ -21656,7 +21656,7 @@
         <v>1417</v>
       </c>
       <c r="I449">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="Q449" t="b">
         <v>1</v>
@@ -21688,7 +21688,7 @@
         <v>1417</v>
       </c>
       <c r="I450">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="Q450" t="b">
         <v>1</v>
@@ -21720,7 +21720,7 @@
         <v>1417</v>
       </c>
       <c r="I451">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q451" t="b">
         <v>1</v>
@@ -21781,7 +21781,7 @@
         <v>1417</v>
       </c>
       <c r="I453">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q453" t="b">
         <v>1</v>
@@ -21813,7 +21813,7 @@
         <v>1417</v>
       </c>
       <c r="I454">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q454" t="b">
         <v>1</v>
@@ -21845,7 +21845,7 @@
         <v>1417</v>
       </c>
       <c r="I455">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q455" t="b">
         <v>1</v>
@@ -21906,7 +21906,7 @@
         <v>1417</v>
       </c>
       <c r="I457">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q457" t="b">
         <v>1</v>
@@ -21938,7 +21938,7 @@
         <v>1417</v>
       </c>
       <c r="I458">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="Q458" t="b">
         <v>1</v>
@@ -21970,7 +21970,7 @@
         <v>1417</v>
       </c>
       <c r="I459">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="Q459" t="b">
         <v>1</v>
@@ -22002,7 +22002,7 @@
         <v>1417</v>
       </c>
       <c r="I460">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="Q460" t="b">
         <v>1</v>
@@ -22034,7 +22034,7 @@
         <v>1417</v>
       </c>
       <c r="I461">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="Q461" t="b">
         <v>1</v>
@@ -22066,7 +22066,7 @@
         <v>1417</v>
       </c>
       <c r="I462">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="Q462" t="b">
         <v>1</v>
@@ -22098,7 +22098,7 @@
         <v>1417</v>
       </c>
       <c r="I463">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="Q463" t="b">
         <v>1</v>
@@ -22130,7 +22130,7 @@
         <v>1417</v>
       </c>
       <c r="I464">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q464" t="b">
         <v>1</v>
@@ -22162,7 +22162,7 @@
         <v>1417</v>
       </c>
       <c r="I465">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q465" t="b">
         <v>1</v>
@@ -22194,7 +22194,7 @@
         <v>1417</v>
       </c>
       <c r="I466">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q466" t="b">
         <v>1</v>
@@ -22226,7 +22226,7 @@
         <v>1417</v>
       </c>
       <c r="I467">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q467" t="b">
         <v>1</v>
@@ -22258,7 +22258,7 @@
         <v>1417</v>
       </c>
       <c r="I468">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q468" t="b">
         <v>1</v>
@@ -22290,7 +22290,7 @@
         <v>1417</v>
       </c>
       <c r="I469">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q469" t="b">
         <v>1</v>
@@ -22351,7 +22351,7 @@
         <v>1417</v>
       </c>
       <c r="I471">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q471" t="b">
         <v>1</v>
@@ -22383,7 +22383,7 @@
         <v>1417</v>
       </c>
       <c r="I472">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q472" t="b">
         <v>1</v>
@@ -22415,7 +22415,7 @@
         <v>1417</v>
       </c>
       <c r="I473">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q473" t="b">
         <v>1</v>
@@ -22447,7 +22447,7 @@
         <v>1417</v>
       </c>
       <c r="I474">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="Q474" t="b">
         <v>1</v>
@@ -22479,7 +22479,7 @@
         <v>1417</v>
       </c>
       <c r="I475">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="Q475" t="b">
         <v>1</v>
@@ -22511,7 +22511,7 @@
         <v>1417</v>
       </c>
       <c r="I476">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="Q476" t="b">
         <v>1</v>
@@ -22543,7 +22543,7 @@
         <v>1417</v>
       </c>
       <c r="I477">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="Q477" t="b">
         <v>1</v>
@@ -22575,7 +22575,7 @@
         <v>1417</v>
       </c>
       <c r="I478">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="Q478" t="b">
         <v>1</v>
@@ -22607,7 +22607,7 @@
         <v>1417</v>
       </c>
       <c r="I479">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="Q479" t="b">
         <v>1</v>
@@ -22639,7 +22639,7 @@
         <v>1417</v>
       </c>
       <c r="I480">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="Q480" t="b">
         <v>1</v>
@@ -22671,7 +22671,7 @@
         <v>1417</v>
       </c>
       <c r="I481">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="Q481" t="b">
         <v>1</v>
@@ -22703,7 +22703,7 @@
         <v>1417</v>
       </c>
       <c r="I482">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="Q482" t="b">
         <v>1</v>
@@ -22735,7 +22735,7 @@
         <v>1417</v>
       </c>
       <c r="I483">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="Q483" t="b">
         <v>1</v>
@@ -22767,7 +22767,7 @@
         <v>1417</v>
       </c>
       <c r="I484">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="Q484" t="b">
         <v>1</v>
@@ -22799,7 +22799,7 @@
         <v>1417</v>
       </c>
       <c r="I485">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="Q485" t="b">
         <v>1</v>
@@ -22831,7 +22831,7 @@
         <v>1417</v>
       </c>
       <c r="I486">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="Q486" t="b">
         <v>1</v>
@@ -22863,7 +22863,7 @@
         <v>1417</v>
       </c>
       <c r="I487">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="Q487" t="b">
         <v>1</v>
@@ -22895,7 +22895,7 @@
         <v>1417</v>
       </c>
       <c r="I488">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="Q488" t="b">
         <v>1</v>
@@ -22927,7 +22927,7 @@
         <v>1417</v>
       </c>
       <c r="I489">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="Q489" t="b">
         <v>1</v>
@@ -22959,7 +22959,7 @@
         <v>1417</v>
       </c>
       <c r="I490">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="Q490" t="b">
         <v>1</v>
@@ -22991,7 +22991,7 @@
         <v>1417</v>
       </c>
       <c r="I491">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="Q491" t="b">
         <v>1</v>
@@ -23023,7 +23023,7 @@
         <v>1419</v>
       </c>
       <c r="I492">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="Q492" t="b">
         <v>1</v>
@@ -23055,7 +23055,7 @@
         <v>1419</v>
       </c>
       <c r="I493">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="Q493" t="b">
         <v>1</v>
@@ -23087,7 +23087,7 @@
         <v>1419</v>
       </c>
       <c r="I494">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="Q494" t="b">
         <v>1</v>
@@ -23119,7 +23119,7 @@
         <v>1419</v>
       </c>
       <c r="I495">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="Q495" t="b">
         <v>1</v>
@@ -23151,7 +23151,7 @@
         <v>1419</v>
       </c>
       <c r="I496">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="Q496" t="b">
         <v>1</v>
@@ -23183,7 +23183,7 @@
         <v>1417</v>
       </c>
       <c r="I497">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="Q497" t="b">
         <v>1</v>
@@ -23215,7 +23215,7 @@
         <v>1417</v>
       </c>
       <c r="I498">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="Q498" t="b">
         <v>1</v>
@@ -23247,7 +23247,7 @@
         <v>1419</v>
       </c>
       <c r="I499">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="Q499" t="b">
         <v>1</v>
@@ -23279,7 +23279,7 @@
         <v>1417</v>
       </c>
       <c r="I500">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="Q500" t="b">
         <v>1</v>
@@ -23311,7 +23311,7 @@
         <v>1417</v>
       </c>
       <c r="I501">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="Q501" t="b">
         <v>1</v>
@@ -23343,7 +23343,7 @@
         <v>1417</v>
       </c>
       <c r="I502">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="Q502" t="b">
         <v>1</v>
@@ -23375,7 +23375,7 @@
         <v>1417</v>
       </c>
       <c r="I503">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="Q503" t="b">
         <v>1</v>
@@ -23407,7 +23407,7 @@
         <v>1417</v>
       </c>
       <c r="I504">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="Q504" t="b">
         <v>1</v>
@@ -23439,7 +23439,7 @@
         <v>1417</v>
       </c>
       <c r="I505">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="Q505" t="b">
         <v>1</v>
@@ -23471,7 +23471,7 @@
         <v>1417</v>
       </c>
       <c r="I506">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="Q506" t="b">
         <v>1</v>
@@ -23503,7 +23503,7 @@
         <v>1417</v>
       </c>
       <c r="I507">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q507" t="b">
         <v>1</v>
@@ -23564,7 +23564,7 @@
         <v>1417</v>
       </c>
       <c r="I509">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q509" t="b">
         <v>1</v>
@@ -23596,7 +23596,7 @@
         <v>1417</v>
       </c>
       <c r="I510">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q510" t="b">
         <v>1</v>
@@ -23628,7 +23628,7 @@
         <v>1417</v>
       </c>
       <c r="I511">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="Q511" t="b">
         <v>1</v>
@@ -23660,7 +23660,7 @@
         <v>1417</v>
       </c>
       <c r="I512">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="Q512" t="b">
         <v>1</v>
@@ -23692,7 +23692,7 @@
         <v>1417</v>
       </c>
       <c r="I513">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Q513" t="b">
         <v>1</v>
@@ -23753,7 +23753,7 @@
         <v>1417</v>
       </c>
       <c r="I515">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Q515" t="b">
         <v>1</v>
@@ -23785,7 +23785,7 @@
         <v>1417</v>
       </c>
       <c r="I516">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Q516" t="b">
         <v>1</v>
@@ -23817,7 +23817,7 @@
         <v>1417</v>
       </c>
       <c r="I517">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Q517" t="b">
         <v>1</v>
@@ -23849,7 +23849,7 @@
         <v>1417</v>
       </c>
       <c r="I518">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Q518" t="b">
         <v>1</v>
@@ -23881,7 +23881,7 @@
         <v>1417</v>
       </c>
       <c r="I519">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="Q519" t="b">
         <v>1</v>
@@ -23913,7 +23913,7 @@
         <v>1417</v>
       </c>
       <c r="I520">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="Q520" t="b">
         <v>1</v>
@@ -23945,7 +23945,7 @@
         <v>1417</v>
       </c>
       <c r="I521">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="Q521" t="b">
         <v>1</v>
@@ -23977,7 +23977,7 @@
         <v>1417</v>
       </c>
       <c r="I522">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="Q522" t="b">
         <v>1</v>
@@ -24009,7 +24009,7 @@
         <v>1417</v>
       </c>
       <c r="I523">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="Q523" t="b">
         <v>1</v>
@@ -24041,7 +24041,7 @@
         <v>1417</v>
       </c>
       <c r="I524">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q524" t="b">
         <v>1</v>
@@ -24073,7 +24073,7 @@
         <v>1417</v>
       </c>
       <c r="I525">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q525" t="b">
         <v>1</v>
@@ -24105,7 +24105,7 @@
         <v>1417</v>
       </c>
       <c r="I526">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q526" t="b">
         <v>1</v>
@@ -24137,7 +24137,7 @@
         <v>1417</v>
       </c>
       <c r="I527">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q527" t="b">
         <v>1</v>
@@ -24169,7 +24169,7 @@
         <v>1417</v>
       </c>
       <c r="I528">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Q528" t="b">
         <v>1</v>
@@ -24201,7 +24201,7 @@
         <v>1417</v>
       </c>
       <c r="I529">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="Q529" t="b">
         <v>1</v>
@@ -24233,7 +24233,7 @@
         <v>1417</v>
       </c>
       <c r="I530">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="Q530" t="b">
         <v>1</v>
@@ -24265,7 +24265,7 @@
         <v>1417</v>
       </c>
       <c r="I531">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="Q531" t="b">
         <v>1</v>
@@ -24297,7 +24297,7 @@
         <v>1417</v>
       </c>
       <c r="I532">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="Q532" t="b">
         <v>1</v>
@@ -24329,7 +24329,7 @@
         <v>1417</v>
       </c>
       <c r="I533">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="Q533" t="b">
         <v>1</v>
@@ -24361,7 +24361,7 @@
         <v>1417</v>
       </c>
       <c r="I534">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="Q534" t="b">
         <v>1</v>
@@ -24393,7 +24393,7 @@
         <v>1417</v>
       </c>
       <c r="I535">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="Q535" t="b">
         <v>1</v>
@@ -24425,7 +24425,7 @@
         <v>1417</v>
       </c>
       <c r="I536">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="Q536" t="b">
         <v>1</v>
@@ -24457,7 +24457,7 @@
         <v>1417</v>
       </c>
       <c r="I537">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="Q537" t="b">
         <v>1</v>
@@ -24489,7 +24489,7 @@
         <v>1417</v>
       </c>
       <c r="I538">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="Q538" t="b">
         <v>1</v>
@@ -24521,7 +24521,7 @@
         <v>1417</v>
       </c>
       <c r="I539">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="Q539" t="b">
         <v>1</v>
@@ -24553,7 +24553,7 @@
         <v>1417</v>
       </c>
       <c r="I540">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="Q540" t="b">
         <v>1</v>
@@ -24585,7 +24585,7 @@
         <v>1417</v>
       </c>
       <c r="I541">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="Q541" t="b">
         <v>1</v>
@@ -24617,7 +24617,7 @@
         <v>1417</v>
       </c>
       <c r="I542">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="Q542" t="b">
         <v>1</v>
@@ -24649,7 +24649,7 @@
         <v>1417</v>
       </c>
       <c r="I543">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="Q543" t="b">
         <v>1</v>
@@ -24681,7 +24681,7 @@
         <v>1417</v>
       </c>
       <c r="I544">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="Q544" t="b">
         <v>1</v>
@@ -24713,7 +24713,7 @@
         <v>1417</v>
       </c>
       <c r="I545">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="Q545" t="b">
         <v>1</v>
@@ -24745,7 +24745,7 @@
         <v>1417</v>
       </c>
       <c r="I546">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="Q546" t="b">
         <v>1</v>
@@ -24777,7 +24777,7 @@
         <v>1417</v>
       </c>
       <c r="I547">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="Q547" t="b">
         <v>1</v>
@@ -24809,7 +24809,7 @@
         <v>1417</v>
       </c>
       <c r="I548">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="Q548" t="b">
         <v>1</v>
@@ -24841,7 +24841,7 @@
         <v>1417</v>
       </c>
       <c r="I549">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="Q549" t="b">
         <v>1</v>
@@ -24873,7 +24873,7 @@
         <v>1417</v>
       </c>
       <c r="I550">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="Q550" t="b">
         <v>1</v>
@@ -24905,7 +24905,7 @@
         <v>1417</v>
       </c>
       <c r="I551">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="Q551" t="b">
         <v>1</v>
@@ -24937,7 +24937,7 @@
         <v>1417</v>
       </c>
       <c r="I552">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="Q552" t="b">
         <v>1</v>
@@ -24969,7 +24969,7 @@
         <v>1417</v>
       </c>
       <c r="I553">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="Q553" t="b">
         <v>1</v>
@@ -25001,7 +25001,7 @@
         <v>1417</v>
       </c>
       <c r="I554">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="Q554" t="b">
         <v>1</v>
@@ -25033,7 +25033,7 @@
         <v>1417</v>
       </c>
       <c r="I555">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="Q555" t="b">
         <v>1</v>
@@ -25065,7 +25065,7 @@
         <v>1417</v>
       </c>
       <c r="I556">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="Q556" t="b">
         <v>1</v>
@@ -25097,7 +25097,7 @@
         <v>1417</v>
       </c>
       <c r="I557">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q557" t="b">
         <v>1</v>
@@ -25129,7 +25129,7 @@
         <v>1417</v>
       </c>
       <c r="I558">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q558" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: reparaveis (28/10/2026 14:09)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
@@ -5132,7 +5132,7 @@
         <v>1417</v>
       </c>
       <c r="I2">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="K2" t="s">
         <v>1420</v>
@@ -5170,7 +5170,7 @@
         <v>1417</v>
       </c>
       <c r="I3">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="K3" t="s">
         <v>1421</v>
@@ -5208,7 +5208,7 @@
         <v>1417</v>
       </c>
       <c r="I4">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="K4" t="s">
         <v>1421</v>
@@ -5246,7 +5246,7 @@
         <v>1417</v>
       </c>
       <c r="I5">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="J5">
         <v>279</v>
@@ -5290,7 +5290,7 @@
         <v>1417</v>
       </c>
       <c r="I6">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="J6">
         <v>153</v>
@@ -5334,7 +5334,7 @@
         <v>1417</v>
       </c>
       <c r="I7">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="J7">
         <v>112</v>
@@ -5410,7 +5410,7 @@
         <v>1417</v>
       </c>
       <c r="I9">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="J9">
         <v>362</v>
@@ -5457,7 +5457,7 @@
         <v>1417</v>
       </c>
       <c r="I10">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="J10">
         <v>378</v>
@@ -5504,7 +5504,7 @@
         <v>1417</v>
       </c>
       <c r="I11">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="J11">
         <v>112</v>
@@ -5551,7 +5551,7 @@
         <v>1417</v>
       </c>
       <c r="I12">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="J12">
         <v>124</v>
@@ -5624,7 +5624,7 @@
         <v>1417</v>
       </c>
       <c r="I14">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="J14">
         <v>64</v>
@@ -5703,7 +5703,7 @@
         <v>1417</v>
       </c>
       <c r="I16">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="K16" t="s">
         <v>1420</v>
@@ -5741,7 +5741,7 @@
         <v>1417</v>
       </c>
       <c r="I17">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="J17">
         <v>161</v>
@@ -5785,7 +5785,7 @@
         <v>1417</v>
       </c>
       <c r="I18">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="J18">
         <v>66</v>
@@ -5858,7 +5858,7 @@
         <v>1417</v>
       </c>
       <c r="I20">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="J20">
         <v>399</v>
@@ -5931,7 +5931,7 @@
         <v>1417</v>
       </c>
       <c r="I22">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="K22" t="s">
         <v>1424</v>
@@ -5969,7 +5969,7 @@
         <v>1417</v>
       </c>
       <c r="I23">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="J23">
         <v>229</v>
@@ -6074,7 +6074,7 @@
         <v>1417</v>
       </c>
       <c r="I26">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="J26">
         <v>155</v>
@@ -6121,7 +6121,7 @@
         <v>1417</v>
       </c>
       <c r="I27">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="K27" t="s">
         <v>1424</v>
@@ -6217,7 +6217,7 @@
         <v>1417</v>
       </c>
       <c r="I30">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="J30">
         <v>209</v>
@@ -6290,7 +6290,7 @@
         <v>1417</v>
       </c>
       <c r="I32">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="K32" t="s">
         <v>1420</v>
@@ -6499,7 +6499,7 @@
         <v>1417</v>
       </c>
       <c r="I39">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="K39" t="s">
         <v>1425</v>
@@ -6662,7 +6662,7 @@
         <v>1417</v>
       </c>
       <c r="I44">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="J44">
         <v>87</v>
@@ -6709,7 +6709,7 @@
         <v>1417</v>
       </c>
       <c r="I45">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="J45">
         <v>331</v>
@@ -6756,7 +6756,7 @@
         <v>1417</v>
       </c>
       <c r="I46">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="K46" t="s">
         <v>1424</v>
@@ -6797,7 +6797,7 @@
         <v>1417</v>
       </c>
       <c r="I47">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="J47">
         <v>344</v>
@@ -6844,7 +6844,7 @@
         <v>1417</v>
       </c>
       <c r="I48">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="K48" t="s">
         <v>1424</v>
@@ -6911,7 +6911,7 @@
         <v>1417</v>
       </c>
       <c r="I50">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="K50" t="s">
         <v>1424</v>
@@ -6978,7 +6978,7 @@
         <v>1417</v>
       </c>
       <c r="I52">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="K52" t="s">
         <v>1420</v>
@@ -7016,7 +7016,7 @@
         <v>1417</v>
       </c>
       <c r="I53">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="K53" t="s">
         <v>1421</v>
@@ -7054,7 +7054,7 @@
         <v>1417</v>
       </c>
       <c r="I54">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="K54" t="s">
         <v>1421</v>
@@ -7330,7 +7330,7 @@
         <v>1417</v>
       </c>
       <c r="I63">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="J63">
         <v>293</v>
@@ -7377,7 +7377,7 @@
         <v>1417</v>
       </c>
       <c r="I64">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="J64">
         <v>320</v>
@@ -7607,7 +7607,7 @@
         <v>1417</v>
       </c>
       <c r="I71">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="J71">
         <v>429</v>
@@ -7680,7 +7680,7 @@
         <v>1417</v>
       </c>
       <c r="I73">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="K73" t="s">
         <v>1420</v>
@@ -7788,7 +7788,7 @@
         <v>1417</v>
       </c>
       <c r="I76">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="K76" t="s">
         <v>1427</v>
@@ -7881,7 +7881,7 @@
         <v>1417</v>
       </c>
       <c r="I79">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="K79" t="s">
         <v>1427</v>
@@ -7986,7 +7986,7 @@
         <v>1417</v>
       </c>
       <c r="I82">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="K82" t="s">
         <v>1424</v>
@@ -8053,7 +8053,7 @@
         <v>1417</v>
       </c>
       <c r="I84">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="J84">
         <v>40</v>
@@ -8100,7 +8100,7 @@
         <v>1417</v>
       </c>
       <c r="I85">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="K85" t="s">
         <v>1421</v>
@@ -8138,7 +8138,7 @@
         <v>1417</v>
       </c>
       <c r="I86">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="K86" t="s">
         <v>1421</v>
@@ -8176,7 +8176,7 @@
         <v>1417</v>
       </c>
       <c r="I87">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="J87">
         <v>-16</v>
@@ -8299,7 +8299,7 @@
         <v>1417</v>
       </c>
       <c r="I90">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="K90" t="s">
         <v>1394</v>
@@ -8448,7 +8448,7 @@
         <v>1417</v>
       </c>
       <c r="I94">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="K94" t="s">
         <v>1424</v>
@@ -8527,7 +8527,7 @@
         <v>1417</v>
       </c>
       <c r="I96">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="J96">
         <v>17</v>
@@ -8574,7 +8574,7 @@
         <v>1417</v>
       </c>
       <c r="I97">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="J97">
         <v>20</v>
@@ -8621,7 +8621,7 @@
         <v>1417</v>
       </c>
       <c r="I98">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="K98" t="s">
         <v>1424</v>
@@ -8898,7 +8898,7 @@
         <v>1417</v>
       </c>
       <c r="I106">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="J106">
         <v>49</v>
@@ -8942,7 +8942,7 @@
         <v>1417</v>
       </c>
       <c r="I107">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="J107">
         <v>36</v>
@@ -8986,7 +8986,7 @@
         <v>1417</v>
       </c>
       <c r="I108">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="K108" t="s">
         <v>1421</v>
@@ -9024,7 +9024,7 @@
         <v>1417</v>
       </c>
       <c r="I109">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="K109" t="s">
         <v>1421</v>
@@ -9207,7 +9207,7 @@
         <v>1417</v>
       </c>
       <c r="I115">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="K115" t="s">
         <v>1421</v>
@@ -9245,7 +9245,7 @@
         <v>1417</v>
       </c>
       <c r="I116">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="K116" t="s">
         <v>1421</v>
@@ -9283,7 +9283,7 @@
         <v>1417</v>
       </c>
       <c r="I117">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="K117" t="s">
         <v>1421</v>
@@ -9321,7 +9321,7 @@
         <v>1417</v>
       </c>
       <c r="I118">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="K118" t="s">
         <v>1421</v>
@@ -9359,7 +9359,7 @@
         <v>1417</v>
       </c>
       <c r="I119">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="K119" t="s">
         <v>1421</v>
@@ -9397,7 +9397,7 @@
         <v>1417</v>
       </c>
       <c r="I120">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="K120" t="s">
         <v>1421</v>
@@ -9435,7 +9435,7 @@
         <v>1417</v>
       </c>
       <c r="I121">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="J121">
         <v>251</v>
@@ -9482,7 +9482,7 @@
         <v>1417</v>
       </c>
       <c r="I122">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="K122" t="s">
         <v>1421</v>
@@ -9549,7 +9549,7 @@
         <v>1417</v>
       </c>
       <c r="I124">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="K124" t="s">
         <v>1421</v>
@@ -9587,7 +9587,7 @@
         <v>1417</v>
       </c>
       <c r="I125">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="K125" t="s">
         <v>1427</v>
@@ -9683,7 +9683,7 @@
         <v>1417</v>
       </c>
       <c r="I128">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="K128" t="s">
         <v>1421</v>
@@ -9721,7 +9721,7 @@
         <v>1417</v>
       </c>
       <c r="I129">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="K129" t="s">
         <v>1420</v>
@@ -9759,7 +9759,7 @@
         <v>1417</v>
       </c>
       <c r="I130">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="J130">
         <v>47</v>
@@ -9835,7 +9835,7 @@
         <v>1417</v>
       </c>
       <c r="I132">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="J132">
         <v>145</v>
@@ -9911,7 +9911,7 @@
         <v>1417</v>
       </c>
       <c r="I134">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="K134" t="s">
         <v>1420</v>
@@ -10036,7 +10036,7 @@
         <v>1417</v>
       </c>
       <c r="I138">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="K138" t="s">
         <v>1421</v>
@@ -10420,7 +10420,7 @@
         <v>1417</v>
       </c>
       <c r="I150">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="J150">
         <v>201</v>
@@ -10607,7 +10607,7 @@
         <v>1417</v>
       </c>
       <c r="I155">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="K155" t="s">
         <v>1427</v>
@@ -10642,7 +10642,7 @@
         <v>1417</v>
       </c>
       <c r="I156">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="K156" t="s">
         <v>1421</v>
@@ -10680,7 +10680,7 @@
         <v>1417</v>
       </c>
       <c r="I157">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="J157">
         <v>371</v>
@@ -10724,7 +10724,7 @@
         <v>1417</v>
       </c>
       <c r="I158">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="J158">
         <v>52</v>
@@ -10768,7 +10768,7 @@
         <v>1417</v>
       </c>
       <c r="I159">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="K159" t="s">
         <v>1421</v>
@@ -10806,7 +10806,7 @@
         <v>1417</v>
       </c>
       <c r="I160">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="K160" t="s">
         <v>1421</v>
@@ -10844,7 +10844,7 @@
         <v>1417</v>
       </c>
       <c r="I161">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="J161">
         <v>55</v>
@@ -10979,7 +10979,7 @@
         <v>1417</v>
       </c>
       <c r="I164">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="O164" t="s">
         <v>1533</v>
@@ -11154,7 +11154,7 @@
         <v>1417</v>
       </c>
       <c r="I169">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="K169" t="s">
         <v>1394</v>
@@ -11364,7 +11364,7 @@
         <v>1417</v>
       </c>
       <c r="I175">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="J175">
         <v>205</v>
@@ -11411,7 +11411,7 @@
         <v>1417</v>
       </c>
       <c r="I176">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="K176" t="s">
         <v>1421</v>
@@ -11449,7 +11449,7 @@
         <v>1417</v>
       </c>
       <c r="I177">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="J177">
         <v>44</v>
@@ -11496,7 +11496,7 @@
         <v>1417</v>
       </c>
       <c r="I178">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="K178" t="s">
         <v>1420</v>
@@ -11563,7 +11563,7 @@
         <v>1417</v>
       </c>
       <c r="I180">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="K180" t="s">
         <v>1420</v>
@@ -11659,7 +11659,7 @@
         <v>1417</v>
       </c>
       <c r="I183">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="K183" t="s">
         <v>1421</v>
@@ -11697,7 +11697,7 @@
         <v>1417</v>
       </c>
       <c r="I184">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="K184" t="s">
         <v>1427</v>
@@ -11732,7 +11732,7 @@
         <v>1417</v>
       </c>
       <c r="I185">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="K185" t="s">
         <v>1421</v>
@@ -11770,7 +11770,7 @@
         <v>1417</v>
       </c>
       <c r="I186">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="K186" t="s">
         <v>1421</v>
@@ -11808,7 +11808,7 @@
         <v>1417</v>
       </c>
       <c r="I187">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="J187">
         <v>75</v>
@@ -11855,7 +11855,7 @@
         <v>1417</v>
       </c>
       <c r="I188">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="J188">
         <v>40</v>
@@ -11902,7 +11902,7 @@
         <v>1417</v>
       </c>
       <c r="I189">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="J189">
         <v>155</v>
@@ -11946,7 +11946,7 @@
         <v>1417</v>
       </c>
       <c r="I190">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="J190">
         <v>107</v>
@@ -11990,7 +11990,7 @@
         <v>1417</v>
       </c>
       <c r="I191">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="J191">
         <v>5</v>
@@ -12034,7 +12034,7 @@
         <v>1417</v>
       </c>
       <c r="I192">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="K192" t="s">
         <v>1421</v>
@@ -12072,7 +12072,7 @@
         <v>1417</v>
       </c>
       <c r="I193">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="K193" t="s">
         <v>1426</v>
@@ -12267,7 +12267,7 @@
         <v>1417</v>
       </c>
       <c r="I199">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="J199">
         <v>70</v>
@@ -12352,7 +12352,7 @@
         <v>1417</v>
       </c>
       <c r="I201">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="K201" t="s">
         <v>1421</v>
@@ -12390,7 +12390,7 @@
         <v>1417</v>
       </c>
       <c r="I202">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="K202" t="s">
         <v>1421</v>
@@ -12469,7 +12469,7 @@
         <v>1417</v>
       </c>
       <c r="I204">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="K204" t="s">
         <v>1420</v>
@@ -12507,7 +12507,7 @@
         <v>1417</v>
       </c>
       <c r="I205">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="K205" t="s">
         <v>1420</v>
@@ -12574,7 +12574,7 @@
         <v>1417</v>
       </c>
       <c r="I207">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="J207">
         <v>167</v>
@@ -12618,7 +12618,7 @@
         <v>1417</v>
       </c>
       <c r="I208">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="J208">
         <v>45</v>
@@ -12662,7 +12662,7 @@
         <v>1417</v>
       </c>
       <c r="I209">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="J209">
         <v>191</v>
@@ -12706,7 +12706,7 @@
         <v>1417</v>
       </c>
       <c r="I210">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="K210" t="s">
         <v>1424</v>
@@ -12802,7 +12802,7 @@
         <v>1417</v>
       </c>
       <c r="I213">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="K213" t="s">
         <v>1421</v>
@@ -12840,7 +12840,7 @@
         <v>1417</v>
       </c>
       <c r="I214">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="J214">
         <v>14</v>
@@ -12887,7 +12887,7 @@
         <v>1417</v>
       </c>
       <c r="I215">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="K215" t="s">
         <v>1421</v>
@@ -12954,7 +12954,7 @@
         <v>1417</v>
       </c>
       <c r="I217">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="J217">
         <v>42</v>
@@ -12998,7 +12998,7 @@
         <v>1417</v>
       </c>
       <c r="I218">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="J218">
         <v>166</v>
@@ -13086,7 +13086,7 @@
         <v>1417</v>
       </c>
       <c r="I220">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="J220">
         <v>154</v>
@@ -13472,7 +13472,7 @@
         <v>1417</v>
       </c>
       <c r="I230">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="J230">
         <v>197</v>
@@ -13516,7 +13516,7 @@
         <v>1417</v>
       </c>
       <c r="I231">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="J231">
         <v>35</v>
@@ -13618,7 +13618,7 @@
         <v>1417</v>
       </c>
       <c r="I234">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="J234">
         <v>35</v>
@@ -13665,7 +13665,7 @@
         <v>1417</v>
       </c>
       <c r="I235">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="J235">
         <v>35</v>
@@ -13712,7 +13712,7 @@
         <v>1417</v>
       </c>
       <c r="I236">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="J236">
         <v>86</v>
@@ -13829,7 +13829,7 @@
         <v>1417</v>
       </c>
       <c r="I239">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="K239" t="s">
         <v>1394</v>
@@ -13928,7 +13928,7 @@
         <v>1417</v>
       </c>
       <c r="I242">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="K242" t="s">
         <v>1420</v>
@@ -13995,7 +13995,7 @@
         <v>1417</v>
       </c>
       <c r="I244">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="J244">
         <v>15</v>
@@ -14036,7 +14036,7 @@
         <v>1417</v>
       </c>
       <c r="I245">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="J245">
         <v>15</v>
@@ -14179,7 +14179,7 @@
         <v>1417</v>
       </c>
       <c r="I249">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="K249" t="s">
         <v>1421</v>
@@ -14313,7 +14313,7 @@
         <v>1417</v>
       </c>
       <c r="I253">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="J253">
         <v>162</v>
@@ -14357,7 +14357,7 @@
         <v>1417</v>
       </c>
       <c r="I254">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="K254" t="s">
         <v>1424</v>
@@ -14436,7 +14436,7 @@
         <v>1417</v>
       </c>
       <c r="I256">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="J256">
         <v>23</v>
@@ -14620,7 +14620,7 @@
         <v>1417</v>
       </c>
       <c r="I261">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="J261">
         <v>162</v>
@@ -14778,7 +14778,7 @@
         <v>1417</v>
       </c>
       <c r="I265">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="J265">
         <v>162</v>
@@ -14863,7 +14863,7 @@
         <v>1417</v>
       </c>
       <c r="I267">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="K267" t="s">
         <v>1424</v>
@@ -14901,7 +14901,7 @@
         <v>1417</v>
       </c>
       <c r="I268">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="K268" t="s">
         <v>1421</v>
@@ -14936,7 +14936,7 @@
         <v>1417</v>
       </c>
       <c r="I269">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="K269" t="s">
         <v>1421</v>
@@ -14974,7 +14974,7 @@
         <v>1417</v>
       </c>
       <c r="I270">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="K270" t="s">
         <v>1424</v>
@@ -15012,7 +15012,7 @@
         <v>1417</v>
       </c>
       <c r="I271">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="K271" t="s">
         <v>1424</v>
@@ -15190,7 +15190,7 @@
         <v>1417</v>
       </c>
       <c r="I276">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="K276" t="s">
         <v>1425</v>
@@ -15228,7 +15228,7 @@
         <v>1417</v>
       </c>
       <c r="I277">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="K277" t="s">
         <v>1421</v>
@@ -15266,7 +15266,7 @@
         <v>1417</v>
       </c>
       <c r="I278">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="J278">
         <v>148</v>
@@ -15310,7 +15310,7 @@
         <v>1417</v>
       </c>
       <c r="I279">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="K279" t="s">
         <v>1423</v>
@@ -15351,7 +15351,7 @@
         <v>1417</v>
       </c>
       <c r="I280">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="K280" t="s">
         <v>1421</v>
@@ -15389,7 +15389,7 @@
         <v>1417</v>
       </c>
       <c r="I281">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="K281" t="s">
         <v>1421</v>
@@ -15430,7 +15430,7 @@
         <v>1417</v>
       </c>
       <c r="I282">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="K282" t="s">
         <v>1421</v>
@@ -15724,7 +15724,7 @@
         <v>1417</v>
       </c>
       <c r="I291">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="J291">
         <v>20</v>
@@ -15768,7 +15768,7 @@
         <v>1417</v>
       </c>
       <c r="I292">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="K292" t="s">
         <v>1424</v>
@@ -15806,7 +15806,7 @@
         <v>1417</v>
       </c>
       <c r="I293">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="K293" t="s">
         <v>1425</v>
@@ -15844,7 +15844,7 @@
         <v>1417</v>
       </c>
       <c r="I294">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="K294" t="s">
         <v>1430</v>
@@ -15981,7 +15981,7 @@
         <v>1417</v>
       </c>
       <c r="I298">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="J298">
         <v>58</v>
@@ -16145,7 +16145,7 @@
         <v>1417</v>
       </c>
       <c r="I302">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="K302" t="s">
         <v>1424</v>
@@ -16183,7 +16183,7 @@
         <v>1417</v>
       </c>
       <c r="I303">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="K303" t="s">
         <v>1421</v>
@@ -16221,7 +16221,7 @@
         <v>1417</v>
       </c>
       <c r="I304">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="K304" t="s">
         <v>1424</v>
@@ -16259,7 +16259,7 @@
         <v>1417</v>
       </c>
       <c r="I305">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="J305">
         <v>35</v>
@@ -16303,7 +16303,7 @@
         <v>1417</v>
       </c>
       <c r="I306">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="J306">
         <v>31</v>
@@ -16391,7 +16391,7 @@
         <v>1417</v>
       </c>
       <c r="I308">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="K308" t="s">
         <v>1420</v>
@@ -16508,7 +16508,7 @@
         <v>1417</v>
       </c>
       <c r="I311">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="K311" t="s">
         <v>1420</v>
@@ -16838,7 +16838,7 @@
         <v>1417</v>
       </c>
       <c r="I320">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="K320" t="s">
         <v>1425</v>
@@ -16876,7 +16876,7 @@
         <v>1417</v>
       </c>
       <c r="I321">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="K321" t="s">
         <v>1421</v>
@@ -16914,7 +16914,7 @@
         <v>1417</v>
       </c>
       <c r="I322">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="J322">
         <v>57</v>
@@ -17028,7 +17028,7 @@
         <v>1417</v>
       </c>
       <c r="I325">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="J325">
         <v>57</v>
@@ -17110,7 +17110,7 @@
         <v>1417</v>
       </c>
       <c r="I327">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="J327">
         <v>57</v>
@@ -17154,7 +17154,7 @@
         <v>1417</v>
       </c>
       <c r="I328">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="J328">
         <v>57</v>
@@ -17198,7 +17198,7 @@
         <v>1417</v>
       </c>
       <c r="I329">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="J329">
         <v>57</v>
@@ -17242,7 +17242,7 @@
         <v>1417</v>
       </c>
       <c r="I330">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="J330">
         <v>57</v>
@@ -17286,7 +17286,7 @@
         <v>1417</v>
       </c>
       <c r="I331">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="K331" t="s">
         <v>1420</v>
@@ -17324,7 +17324,7 @@
         <v>1417</v>
       </c>
       <c r="I332">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="K332" t="s">
         <v>1421</v>
@@ -17362,7 +17362,7 @@
         <v>1417</v>
       </c>
       <c r="I333">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="J333">
         <v>100</v>
@@ -17406,7 +17406,7 @@
         <v>1417</v>
       </c>
       <c r="I334">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="K334" t="s">
         <v>1421</v>
@@ -17631,7 +17631,7 @@
         <v>1417</v>
       </c>
       <c r="I340">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="J340">
         <v>98</v>
@@ -17672,7 +17672,7 @@
         <v>1417</v>
       </c>
       <c r="I341">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="J341">
         <v>90</v>
@@ -17713,7 +17713,7 @@
         <v>1417</v>
       </c>
       <c r="I342">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="K342" t="s">
         <v>1420</v>
@@ -17827,7 +17827,7 @@
         <v>1417</v>
       </c>
       <c r="I345">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="K345" t="s">
         <v>1420</v>
@@ -17947,7 +17947,7 @@
         <v>1417</v>
       </c>
       <c r="I348">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="J348">
         <v>14</v>
@@ -17991,7 +17991,7 @@
         <v>1417</v>
       </c>
       <c r="I349">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="K349" t="s">
         <v>1425</v>
@@ -18029,7 +18029,7 @@
         <v>1417</v>
       </c>
       <c r="I350">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="J350">
         <v>46</v>
@@ -18067,7 +18067,7 @@
         <v>1417</v>
       </c>
       <c r="I351">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="J351">
         <v>82</v>
@@ -18111,7 +18111,7 @@
         <v>1417</v>
       </c>
       <c r="I352">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="J352">
         <v>78</v>
@@ -18155,7 +18155,7 @@
         <v>1417</v>
       </c>
       <c r="I353">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="J353">
         <v>83</v>
@@ -18199,7 +18199,7 @@
         <v>1417</v>
       </c>
       <c r="I354">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="K354" t="s">
         <v>1424</v>
@@ -18237,7 +18237,7 @@
         <v>1417</v>
       </c>
       <c r="I355">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="J355">
         <v>8</v>
@@ -18319,7 +18319,7 @@
         <v>1417</v>
       </c>
       <c r="I357">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="J357">
         <v>85</v>
@@ -18442,7 +18442,7 @@
         <v>1417</v>
       </c>
       <c r="I360">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="J360">
         <v>83</v>
@@ -18489,7 +18489,7 @@
         <v>1417</v>
       </c>
       <c r="I361">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="J361">
         <v>83</v>
@@ -18533,7 +18533,7 @@
         <v>1417</v>
       </c>
       <c r="I362">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="K362" t="s">
         <v>1424</v>
@@ -18571,7 +18571,7 @@
         <v>1417</v>
       </c>
       <c r="I363">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="K363" t="s">
         <v>1424</v>
@@ -18609,7 +18609,7 @@
         <v>1417</v>
       </c>
       <c r="I364">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="J364">
         <v>83</v>
@@ -18653,7 +18653,7 @@
         <v>1417</v>
       </c>
       <c r="I365">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="J365">
         <v>15</v>
@@ -18776,7 +18776,7 @@
         <v>1417</v>
       </c>
       <c r="I368">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="J368">
         <v>77</v>
@@ -18820,7 +18820,7 @@
         <v>1417</v>
       </c>
       <c r="I369">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="K369" t="s">
         <v>1424</v>
@@ -18858,7 +18858,7 @@
         <v>1417</v>
       </c>
       <c r="I370">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="K370" t="s">
         <v>1424</v>
@@ -18896,7 +18896,7 @@
         <v>1417</v>
       </c>
       <c r="I371">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="J371">
         <v>16</v>
@@ -18984,7 +18984,7 @@
         <v>1417</v>
       </c>
       <c r="I373">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="K373" t="s">
         <v>1420</v>
@@ -19022,7 +19022,7 @@
         <v>1417</v>
       </c>
       <c r="I374">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="K374" t="s">
         <v>1420</v>
@@ -19060,7 +19060,7 @@
         <v>1417</v>
       </c>
       <c r="I375">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="J375">
         <v>94</v>
@@ -19101,7 +19101,7 @@
         <v>1417</v>
       </c>
       <c r="I376">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="K376" t="s">
         <v>1424</v>
@@ -19180,7 +19180,7 @@
         <v>1417</v>
       </c>
       <c r="I378">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="K378" t="s">
         <v>1424</v>
@@ -19218,7 +19218,7 @@
         <v>1417</v>
       </c>
       <c r="I379">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="J379">
         <v>20</v>
@@ -19262,7 +19262,7 @@
         <v>1417</v>
       </c>
       <c r="I380">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="J380">
         <v>94</v>
@@ -19306,7 +19306,7 @@
         <v>1417</v>
       </c>
       <c r="I381">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="K381" t="s">
         <v>1424</v>
@@ -19344,7 +19344,7 @@
         <v>1417</v>
       </c>
       <c r="I382">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="K382" t="s">
         <v>1424</v>
@@ -19382,7 +19382,7 @@
         <v>1417</v>
       </c>
       <c r="I383">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="J383">
         <v>71</v>
@@ -19426,7 +19426,7 @@
         <v>1417</v>
       </c>
       <c r="I384">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="K384" t="s">
         <v>1421</v>
@@ -19508,7 +19508,7 @@
         <v>1417</v>
       </c>
       <c r="I386">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="K386" t="s">
         <v>1424</v>
@@ -19546,7 +19546,7 @@
         <v>1417</v>
       </c>
       <c r="I387">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="K387" t="s">
         <v>1424</v>
@@ -19584,7 +19584,7 @@
         <v>1417</v>
       </c>
       <c r="I388">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="J388">
         <v>-85</v>
@@ -19628,7 +19628,7 @@
         <v>1417</v>
       </c>
       <c r="I389">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="K389" t="s">
         <v>1425</v>
@@ -20079,7 +20079,7 @@
         <v>1417</v>
       </c>
       <c r="I400">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="K400" t="s">
         <v>1424</v>
@@ -20155,7 +20155,7 @@
         <v>1417</v>
       </c>
       <c r="I402">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="K402" t="s">
         <v>1424</v>
@@ -20193,7 +20193,7 @@
         <v>1417</v>
       </c>
       <c r="I403">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="J403">
         <v>83</v>
@@ -20237,7 +20237,7 @@
         <v>1417</v>
       </c>
       <c r="I404">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="K404" t="s">
         <v>1424</v>
@@ -20307,7 +20307,7 @@
         <v>1417</v>
       </c>
       <c r="I406">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="Q406" t="b">
         <v>1</v>
@@ -20339,7 +20339,7 @@
         <v>1417</v>
       </c>
       <c r="I407">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="Q407" t="b">
         <v>1</v>
@@ -20371,7 +20371,7 @@
         <v>1417</v>
       </c>
       <c r="I408">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="Q408" t="b">
         <v>1</v>
@@ -20403,7 +20403,7 @@
         <v>1417</v>
       </c>
       <c r="I409">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="Q409" t="b">
         <v>1</v>
@@ -20435,7 +20435,7 @@
         <v>1417</v>
       </c>
       <c r="I410">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="Q410" t="b">
         <v>1</v>
@@ -20467,7 +20467,7 @@
         <v>1417</v>
       </c>
       <c r="I411">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="Q411" t="b">
         <v>1</v>
@@ -20499,7 +20499,7 @@
         <v>1417</v>
       </c>
       <c r="I412">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="Q412" t="b">
         <v>1</v>
@@ -20531,7 +20531,7 @@
         <v>1417</v>
       </c>
       <c r="I413">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="Q413" t="b">
         <v>1</v>
@@ -20621,7 +20621,7 @@
         <v>1417</v>
       </c>
       <c r="I416">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="Q416" t="b">
         <v>1</v>
@@ -20711,7 +20711,7 @@
         <v>1417</v>
       </c>
       <c r="I419">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="Q419" t="b">
         <v>1</v>
@@ -20743,7 +20743,7 @@
         <v>1417</v>
       </c>
       <c r="I420">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="Q420" t="b">
         <v>1</v>
@@ -20775,7 +20775,7 @@
         <v>1417</v>
       </c>
       <c r="I421">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="Q421" t="b">
         <v>1</v>
@@ -20807,7 +20807,7 @@
         <v>1417</v>
       </c>
       <c r="I422">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="Q422" t="b">
         <v>1</v>
@@ -20839,7 +20839,7 @@
         <v>1417</v>
       </c>
       <c r="I423">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="Q423" t="b">
         <v>1</v>
@@ -20871,7 +20871,7 @@
         <v>1417</v>
       </c>
       <c r="I424">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="Q424" t="b">
         <v>1</v>
@@ -20903,7 +20903,7 @@
         <v>1417</v>
       </c>
       <c r="I425">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="Q425" t="b">
         <v>1</v>
@@ -20935,7 +20935,7 @@
         <v>1417</v>
       </c>
       <c r="I426">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="Q426" t="b">
         <v>1</v>
@@ -20967,7 +20967,7 @@
         <v>1417</v>
       </c>
       <c r="I427">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="Q427" t="b">
         <v>1</v>
@@ -21057,7 +21057,7 @@
         <v>1417</v>
       </c>
       <c r="I430">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="Q430" t="b">
         <v>1</v>
@@ -21089,7 +21089,7 @@
         <v>1417</v>
       </c>
       <c r="I431">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="Q431" t="b">
         <v>1</v>
@@ -21121,7 +21121,7 @@
         <v>1417</v>
       </c>
       <c r="I432">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="Q432" t="b">
         <v>1</v>
@@ -21153,7 +21153,7 @@
         <v>1417</v>
       </c>
       <c r="I433">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="Q433" t="b">
         <v>1</v>
@@ -21185,7 +21185,7 @@
         <v>1417</v>
       </c>
       <c r="I434">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="Q434" t="b">
         <v>1</v>
@@ -21217,7 +21217,7 @@
         <v>1417</v>
       </c>
       <c r="I435">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="Q435" t="b">
         <v>1</v>
@@ -21249,7 +21249,7 @@
         <v>1417</v>
       </c>
       <c r="I436">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="Q436" t="b">
         <v>1</v>
@@ -21281,7 +21281,7 @@
         <v>1419</v>
       </c>
       <c r="I437">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="Q437" t="b">
         <v>1</v>
@@ -21313,7 +21313,7 @@
         <v>1419</v>
       </c>
       <c r="I438">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="Q438" t="b">
         <v>1</v>
@@ -21345,7 +21345,7 @@
         <v>1417</v>
       </c>
       <c r="I439">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="Q439" t="b">
         <v>1</v>
@@ -21377,7 +21377,7 @@
         <v>1417</v>
       </c>
       <c r="I440">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="Q440" t="b">
         <v>1</v>
@@ -21409,7 +21409,7 @@
         <v>1417</v>
       </c>
       <c r="I441">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="Q441" t="b">
         <v>1</v>
@@ -21470,7 +21470,7 @@
         <v>1417</v>
       </c>
       <c r="I443">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="Q443" t="b">
         <v>1</v>
@@ -21560,7 +21560,7 @@
         <v>1417</v>
       </c>
       <c r="I446">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="Q446" t="b">
         <v>1</v>
@@ -21592,7 +21592,7 @@
         <v>1417</v>
       </c>
       <c r="I447">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="Q447" t="b">
         <v>1</v>
@@ -21624,7 +21624,7 @@
         <v>1417</v>
       </c>
       <c r="I448">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="Q448" t="b">
         <v>1</v>
@@ -21656,7 +21656,7 @@
         <v>1417</v>
       </c>
       <c r="I449">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="Q449" t="b">
         <v>1</v>
@@ -21688,7 +21688,7 @@
         <v>1417</v>
       </c>
       <c r="I450">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="Q450" t="b">
         <v>1</v>
@@ -21720,7 +21720,7 @@
         <v>1417</v>
       </c>
       <c r="I451">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q451" t="b">
         <v>1</v>
@@ -21781,7 +21781,7 @@
         <v>1417</v>
       </c>
       <c r="I453">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q453" t="b">
         <v>1</v>
@@ -21813,7 +21813,7 @@
         <v>1417</v>
       </c>
       <c r="I454">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q454" t="b">
         <v>1</v>
@@ -21845,7 +21845,7 @@
         <v>1417</v>
       </c>
       <c r="I455">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q455" t="b">
         <v>1</v>
@@ -21906,7 +21906,7 @@
         <v>1417</v>
       </c>
       <c r="I457">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q457" t="b">
         <v>1</v>
@@ -21938,7 +21938,7 @@
         <v>1417</v>
       </c>
       <c r="I458">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q458" t="b">
         <v>1</v>
@@ -21970,7 +21970,7 @@
         <v>1417</v>
       </c>
       <c r="I459">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="Q459" t="b">
         <v>1</v>
@@ -22002,7 +22002,7 @@
         <v>1417</v>
       </c>
       <c r="I460">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="Q460" t="b">
         <v>1</v>
@@ -22034,7 +22034,7 @@
         <v>1417</v>
       </c>
       <c r="I461">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="Q461" t="b">
         <v>1</v>
@@ -22066,7 +22066,7 @@
         <v>1417</v>
       </c>
       <c r="I462">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="Q462" t="b">
         <v>1</v>
@@ -22098,7 +22098,7 @@
         <v>1417</v>
       </c>
       <c r="I463">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="Q463" t="b">
         <v>1</v>
@@ -22130,7 +22130,7 @@
         <v>1417</v>
       </c>
       <c r="I464">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q464" t="b">
         <v>1</v>
@@ -22162,7 +22162,7 @@
         <v>1417</v>
       </c>
       <c r="I465">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q465" t="b">
         <v>1</v>
@@ -22194,7 +22194,7 @@
         <v>1417</v>
       </c>
       <c r="I466">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q466" t="b">
         <v>1</v>
@@ -22226,7 +22226,7 @@
         <v>1417</v>
       </c>
       <c r="I467">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q467" t="b">
         <v>1</v>
@@ -22258,7 +22258,7 @@
         <v>1417</v>
       </c>
       <c r="I468">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q468" t="b">
         <v>1</v>
@@ -22290,7 +22290,7 @@
         <v>1417</v>
       </c>
       <c r="I469">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q469" t="b">
         <v>1</v>
@@ -22351,7 +22351,7 @@
         <v>1417</v>
       </c>
       <c r="I471">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q471" t="b">
         <v>1</v>
@@ -22383,7 +22383,7 @@
         <v>1417</v>
       </c>
       <c r="I472">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q472" t="b">
         <v>1</v>
@@ -22415,7 +22415,7 @@
         <v>1417</v>
       </c>
       <c r="I473">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q473" t="b">
         <v>1</v>
@@ -22447,7 +22447,7 @@
         <v>1417</v>
       </c>
       <c r="I474">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q474" t="b">
         <v>1</v>
@@ -22479,7 +22479,7 @@
         <v>1417</v>
       </c>
       <c r="I475">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q475" t="b">
         <v>1</v>
@@ -22511,7 +22511,7 @@
         <v>1417</v>
       </c>
       <c r="I476">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q476" t="b">
         <v>1</v>
@@ -22543,7 +22543,7 @@
         <v>1417</v>
       </c>
       <c r="I477">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q477" t="b">
         <v>1</v>
@@ -22575,7 +22575,7 @@
         <v>1417</v>
       </c>
       <c r="I478">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q478" t="b">
         <v>1</v>
@@ -22607,7 +22607,7 @@
         <v>1417</v>
       </c>
       <c r="I479">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q479" t="b">
         <v>1</v>
@@ -22639,7 +22639,7 @@
         <v>1417</v>
       </c>
       <c r="I480">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q480" t="b">
         <v>1</v>
@@ -22671,7 +22671,7 @@
         <v>1417</v>
       </c>
       <c r="I481">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q481" t="b">
         <v>1</v>
@@ -22703,7 +22703,7 @@
         <v>1417</v>
       </c>
       <c r="I482">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q482" t="b">
         <v>1</v>
@@ -22735,7 +22735,7 @@
         <v>1417</v>
       </c>
       <c r="I483">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q483" t="b">
         <v>1</v>
@@ -22767,7 +22767,7 @@
         <v>1417</v>
       </c>
       <c r="I484">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q484" t="b">
         <v>1</v>
@@ -22799,7 +22799,7 @@
         <v>1417</v>
       </c>
       <c r="I485">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q485" t="b">
         <v>1</v>
@@ -22831,7 +22831,7 @@
         <v>1417</v>
       </c>
       <c r="I486">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q486" t="b">
         <v>1</v>
@@ -22863,7 +22863,7 @@
         <v>1417</v>
       </c>
       <c r="I487">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q487" t="b">
         <v>1</v>
@@ -22895,7 +22895,7 @@
         <v>1417</v>
       </c>
       <c r="I488">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q488" t="b">
         <v>1</v>
@@ -22927,7 +22927,7 @@
         <v>1417</v>
       </c>
       <c r="I489">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q489" t="b">
         <v>1</v>
@@ -22959,7 +22959,7 @@
         <v>1417</v>
       </c>
       <c r="I490">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q490" t="b">
         <v>1</v>
@@ -22991,7 +22991,7 @@
         <v>1417</v>
       </c>
       <c r="I491">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q491" t="b">
         <v>1</v>
@@ -23023,7 +23023,7 @@
         <v>1419</v>
       </c>
       <c r="I492">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q492" t="b">
         <v>1</v>
@@ -23055,7 +23055,7 @@
         <v>1419</v>
       </c>
       <c r="I493">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q493" t="b">
         <v>1</v>
@@ -23087,7 +23087,7 @@
         <v>1419</v>
       </c>
       <c r="I494">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q494" t="b">
         <v>1</v>
@@ -23119,7 +23119,7 @@
         <v>1419</v>
       </c>
       <c r="I495">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q495" t="b">
         <v>1</v>
@@ -23151,7 +23151,7 @@
         <v>1419</v>
       </c>
       <c r="I496">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q496" t="b">
         <v>1</v>
@@ -23183,7 +23183,7 @@
         <v>1417</v>
       </c>
       <c r="I497">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q497" t="b">
         <v>1</v>
@@ -23215,7 +23215,7 @@
         <v>1417</v>
       </c>
       <c r="I498">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q498" t="b">
         <v>1</v>
@@ -23247,7 +23247,7 @@
         <v>1419</v>
       </c>
       <c r="I499">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q499" t="b">
         <v>1</v>
@@ -23279,7 +23279,7 @@
         <v>1417</v>
       </c>
       <c r="I500">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q500" t="b">
         <v>1</v>
@@ -23311,7 +23311,7 @@
         <v>1417</v>
       </c>
       <c r="I501">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q501" t="b">
         <v>1</v>
@@ -23343,7 +23343,7 @@
         <v>1417</v>
       </c>
       <c r="I502">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q502" t="b">
         <v>1</v>
@@ -23375,7 +23375,7 @@
         <v>1417</v>
       </c>
       <c r="I503">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q503" t="b">
         <v>1</v>
@@ -23407,7 +23407,7 @@
         <v>1417</v>
       </c>
       <c r="I504">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="Q504" t="b">
         <v>1</v>
@@ -23439,7 +23439,7 @@
         <v>1417</v>
       </c>
       <c r="I505">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="Q505" t="b">
         <v>1</v>
@@ -23471,7 +23471,7 @@
         <v>1417</v>
       </c>
       <c r="I506">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="Q506" t="b">
         <v>1</v>
@@ -23503,7 +23503,7 @@
         <v>1417</v>
       </c>
       <c r="I507">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="Q507" t="b">
         <v>1</v>
@@ -23564,7 +23564,7 @@
         <v>1417</v>
       </c>
       <c r="I509">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="Q509" t="b">
         <v>1</v>
@@ -23596,7 +23596,7 @@
         <v>1417</v>
       </c>
       <c r="I510">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="Q510" t="b">
         <v>1</v>
@@ -23628,7 +23628,7 @@
         <v>1417</v>
       </c>
       <c r="I511">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="Q511" t="b">
         <v>1</v>
@@ -23660,7 +23660,7 @@
         <v>1417</v>
       </c>
       <c r="I512">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="Q512" t="b">
         <v>1</v>
@@ -23692,7 +23692,7 @@
         <v>1417</v>
       </c>
       <c r="I513">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="Q513" t="b">
         <v>1</v>
@@ -23753,7 +23753,7 @@
         <v>1417</v>
       </c>
       <c r="I515">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="Q515" t="b">
         <v>1</v>
@@ -23785,7 +23785,7 @@
         <v>1417</v>
       </c>
       <c r="I516">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="Q516" t="b">
         <v>1</v>
@@ -23817,7 +23817,7 @@
         <v>1417</v>
       </c>
       <c r="I517">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="Q517" t="b">
         <v>1</v>
@@ -23849,7 +23849,7 @@
         <v>1417</v>
       </c>
       <c r="I518">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="Q518" t="b">
         <v>1</v>
@@ -23881,7 +23881,7 @@
         <v>1417</v>
       </c>
       <c r="I519">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="Q519" t="b">
         <v>1</v>
@@ -23913,7 +23913,7 @@
         <v>1417</v>
       </c>
       <c r="I520">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="Q520" t="b">
         <v>1</v>
@@ -23945,7 +23945,7 @@
         <v>1417</v>
       </c>
       <c r="I521">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="Q521" t="b">
         <v>1</v>
@@ -23977,7 +23977,7 @@
         <v>1417</v>
       </c>
       <c r="I522">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="Q522" t="b">
         <v>1</v>
@@ -24009,7 +24009,7 @@
         <v>1417</v>
       </c>
       <c r="I523">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="Q523" t="b">
         <v>1</v>
@@ -24041,7 +24041,7 @@
         <v>1417</v>
       </c>
       <c r="I524">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q524" t="b">
         <v>1</v>
@@ -24073,7 +24073,7 @@
         <v>1417</v>
       </c>
       <c r="I525">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q525" t="b">
         <v>1</v>
@@ -24105,7 +24105,7 @@
         <v>1417</v>
       </c>
       <c r="I526">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q526" t="b">
         <v>1</v>
@@ -24137,7 +24137,7 @@
         <v>1417</v>
       </c>
       <c r="I527">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q527" t="b">
         <v>1</v>
@@ -24169,7 +24169,7 @@
         <v>1417</v>
       </c>
       <c r="I528">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="Q528" t="b">
         <v>1</v>
@@ -24201,7 +24201,7 @@
         <v>1417</v>
       </c>
       <c r="I529">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="Q529" t="b">
         <v>1</v>
@@ -24233,7 +24233,7 @@
         <v>1417</v>
       </c>
       <c r="I530">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="Q530" t="b">
         <v>1</v>
@@ -24265,7 +24265,7 @@
         <v>1417</v>
       </c>
       <c r="I531">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="Q531" t="b">
         <v>1</v>
@@ -24297,7 +24297,7 @@
         <v>1417</v>
       </c>
       <c r="I532">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="Q532" t="b">
         <v>1</v>
@@ -24329,7 +24329,7 @@
         <v>1417</v>
       </c>
       <c r="I533">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="Q533" t="b">
         <v>1</v>
@@ -24361,7 +24361,7 @@
         <v>1417</v>
       </c>
       <c r="I534">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="Q534" t="b">
         <v>1</v>
@@ -24393,7 +24393,7 @@
         <v>1417</v>
       </c>
       <c r="I535">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="Q535" t="b">
         <v>1</v>
@@ -24425,7 +24425,7 @@
         <v>1417</v>
       </c>
       <c r="I536">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="Q536" t="b">
         <v>1</v>
@@ -24457,7 +24457,7 @@
         <v>1417</v>
       </c>
       <c r="I537">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="Q537" t="b">
         <v>1</v>
@@ -24489,7 +24489,7 @@
         <v>1417</v>
       </c>
       <c r="I538">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="Q538" t="b">
         <v>1</v>
@@ -24521,7 +24521,7 @@
         <v>1417</v>
       </c>
       <c r="I539">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="Q539" t="b">
         <v>1</v>
@@ -24553,7 +24553,7 @@
         <v>1417</v>
       </c>
       <c r="I540">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="Q540" t="b">
         <v>1</v>
@@ -24585,7 +24585,7 @@
         <v>1417</v>
       </c>
       <c r="I541">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="Q541" t="b">
         <v>1</v>
@@ -24617,7 +24617,7 @@
         <v>1417</v>
       </c>
       <c r="I542">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="Q542" t="b">
         <v>1</v>
@@ -24649,7 +24649,7 @@
         <v>1417</v>
       </c>
       <c r="I543">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="Q543" t="b">
         <v>1</v>
@@ -24681,7 +24681,7 @@
         <v>1417</v>
       </c>
       <c r="I544">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="Q544" t="b">
         <v>1</v>
@@ -24713,7 +24713,7 @@
         <v>1417</v>
       </c>
       <c r="I545">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="Q545" t="b">
         <v>1</v>
@@ -24745,7 +24745,7 @@
         <v>1417</v>
       </c>
       <c r="I546">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Q546" t="b">
         <v>1</v>
@@ -24777,7 +24777,7 @@
         <v>1417</v>
       </c>
       <c r="I547">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Q547" t="b">
         <v>1</v>
@@ -24809,7 +24809,7 @@
         <v>1417</v>
       </c>
       <c r="I548">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Q548" t="b">
         <v>1</v>
@@ -24841,7 +24841,7 @@
         <v>1417</v>
       </c>
       <c r="I549">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Q549" t="b">
         <v>1</v>
@@ -24873,7 +24873,7 @@
         <v>1417</v>
       </c>
       <c r="I550">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Q550" t="b">
         <v>1</v>
@@ -24905,7 +24905,7 @@
         <v>1417</v>
       </c>
       <c r="I551">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Q551" t="b">
         <v>1</v>
@@ -24937,7 +24937,7 @@
         <v>1417</v>
       </c>
       <c r="I552">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Q552" t="b">
         <v>1</v>
@@ -24969,7 +24969,7 @@
         <v>1417</v>
       </c>
       <c r="I553">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Q553" t="b">
         <v>1</v>
@@ -25001,7 +25001,7 @@
         <v>1417</v>
       </c>
       <c r="I554">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Q554" t="b">
         <v>1</v>
@@ -25033,7 +25033,7 @@
         <v>1417</v>
       </c>
       <c r="I555">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Q555" t="b">
         <v>1</v>
@@ -25065,7 +25065,7 @@
         <v>1417</v>
       </c>
       <c r="I556">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Q556" t="b">
         <v>1</v>
@@ -25097,7 +25097,7 @@
         <v>1417</v>
       </c>
       <c r="I557">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q557" t="b">
         <v>1</v>
@@ -25129,7 +25129,7 @@
         <v>1417</v>
       </c>
       <c r="I558">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q558" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: reparaveis (29/10/2026 14:25)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
@@ -5132,7 +5132,7 @@
         <v>1417</v>
       </c>
       <c r="I2">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="K2" t="s">
         <v>1420</v>
@@ -5170,7 +5170,7 @@
         <v>1417</v>
       </c>
       <c r="I3">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="K3" t="s">
         <v>1421</v>
@@ -5208,7 +5208,7 @@
         <v>1417</v>
       </c>
       <c r="I4">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="K4" t="s">
         <v>1421</v>
@@ -5246,7 +5246,7 @@
         <v>1417</v>
       </c>
       <c r="I5">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="J5">
         <v>279</v>
@@ -5290,7 +5290,7 @@
         <v>1417</v>
       </c>
       <c r="I6">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="J6">
         <v>153</v>
@@ -5334,7 +5334,7 @@
         <v>1417</v>
       </c>
       <c r="I7">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="J7">
         <v>112</v>
@@ -5410,7 +5410,7 @@
         <v>1417</v>
       </c>
       <c r="I9">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="J9">
         <v>362</v>
@@ -5457,7 +5457,7 @@
         <v>1417</v>
       </c>
       <c r="I10">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="J10">
         <v>378</v>
@@ -5504,7 +5504,7 @@
         <v>1417</v>
       </c>
       <c r="I11">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="J11">
         <v>112</v>
@@ -5551,7 +5551,7 @@
         <v>1417</v>
       </c>
       <c r="I12">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="J12">
         <v>124</v>
@@ -5624,7 +5624,7 @@
         <v>1417</v>
       </c>
       <c r="I14">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="J14">
         <v>64</v>
@@ -5703,7 +5703,7 @@
         <v>1417</v>
       </c>
       <c r="I16">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="K16" t="s">
         <v>1420</v>
@@ -5741,7 +5741,7 @@
         <v>1417</v>
       </c>
       <c r="I17">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="J17">
         <v>161</v>
@@ -5785,7 +5785,7 @@
         <v>1417</v>
       </c>
       <c r="I18">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="J18">
         <v>66</v>
@@ -5858,7 +5858,7 @@
         <v>1417</v>
       </c>
       <c r="I20">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="J20">
         <v>399</v>
@@ -5931,7 +5931,7 @@
         <v>1417</v>
       </c>
       <c r="I22">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="K22" t="s">
         <v>1424</v>
@@ -5969,7 +5969,7 @@
         <v>1417</v>
       </c>
       <c r="I23">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="J23">
         <v>229</v>
@@ -6074,7 +6074,7 @@
         <v>1417</v>
       </c>
       <c r="I26">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="J26">
         <v>155</v>
@@ -6121,7 +6121,7 @@
         <v>1417</v>
       </c>
       <c r="I27">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="K27" t="s">
         <v>1424</v>
@@ -6217,7 +6217,7 @@
         <v>1417</v>
       </c>
       <c r="I30">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="J30">
         <v>209</v>
@@ -6290,7 +6290,7 @@
         <v>1417</v>
       </c>
       <c r="I32">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="K32" t="s">
         <v>1420</v>
@@ -6499,7 +6499,7 @@
         <v>1417</v>
       </c>
       <c r="I39">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="K39" t="s">
         <v>1425</v>
@@ -6662,7 +6662,7 @@
         <v>1417</v>
       </c>
       <c r="I44">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="J44">
         <v>87</v>
@@ -6709,7 +6709,7 @@
         <v>1417</v>
       </c>
       <c r="I45">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="J45">
         <v>331</v>
@@ -6756,7 +6756,7 @@
         <v>1417</v>
       </c>
       <c r="I46">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="K46" t="s">
         <v>1424</v>
@@ -6797,7 +6797,7 @@
         <v>1417</v>
       </c>
       <c r="I47">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="J47">
         <v>344</v>
@@ -6844,7 +6844,7 @@
         <v>1417</v>
       </c>
       <c r="I48">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="K48" t="s">
         <v>1424</v>
@@ -6911,7 +6911,7 @@
         <v>1417</v>
       </c>
       <c r="I50">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="K50" t="s">
         <v>1424</v>
@@ -6978,7 +6978,7 @@
         <v>1417</v>
       </c>
       <c r="I52">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="K52" t="s">
         <v>1420</v>
@@ -7016,7 +7016,7 @@
         <v>1417</v>
       </c>
       <c r="I53">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="K53" t="s">
         <v>1421</v>
@@ -7054,7 +7054,7 @@
         <v>1417</v>
       </c>
       <c r="I54">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="K54" t="s">
         <v>1421</v>
@@ -7330,7 +7330,7 @@
         <v>1417</v>
       </c>
       <c r="I63">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="J63">
         <v>293</v>
@@ -7377,7 +7377,7 @@
         <v>1417</v>
       </c>
       <c r="I64">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="J64">
         <v>320</v>
@@ -7607,7 +7607,7 @@
         <v>1417</v>
       </c>
       <c r="I71">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="J71">
         <v>429</v>
@@ -7680,7 +7680,7 @@
         <v>1417</v>
       </c>
       <c r="I73">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="K73" t="s">
         <v>1420</v>
@@ -7788,7 +7788,7 @@
         <v>1417</v>
       </c>
       <c r="I76">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="K76" t="s">
         <v>1427</v>
@@ -7881,7 +7881,7 @@
         <v>1417</v>
       </c>
       <c r="I79">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="K79" t="s">
         <v>1427</v>
@@ -7986,7 +7986,7 @@
         <v>1417</v>
       </c>
       <c r="I82">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="K82" t="s">
         <v>1424</v>
@@ -8053,7 +8053,7 @@
         <v>1417</v>
       </c>
       <c r="I84">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="J84">
         <v>40</v>
@@ -8100,7 +8100,7 @@
         <v>1417</v>
       </c>
       <c r="I85">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="K85" t="s">
         <v>1421</v>
@@ -8138,7 +8138,7 @@
         <v>1417</v>
       </c>
       <c r="I86">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="K86" t="s">
         <v>1421</v>
@@ -8176,7 +8176,7 @@
         <v>1417</v>
       </c>
       <c r="I87">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="J87">
         <v>-16</v>
@@ -8299,7 +8299,7 @@
         <v>1417</v>
       </c>
       <c r="I90">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="K90" t="s">
         <v>1394</v>
@@ -8448,7 +8448,7 @@
         <v>1417</v>
       </c>
       <c r="I94">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="K94" t="s">
         <v>1424</v>
@@ -8527,7 +8527,7 @@
         <v>1417</v>
       </c>
       <c r="I96">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="J96">
         <v>17</v>
@@ -8574,7 +8574,7 @@
         <v>1417</v>
       </c>
       <c r="I97">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="J97">
         <v>20</v>
@@ -8621,7 +8621,7 @@
         <v>1417</v>
       </c>
       <c r="I98">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="K98" t="s">
         <v>1424</v>
@@ -8898,7 +8898,7 @@
         <v>1417</v>
       </c>
       <c r="I106">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="J106">
         <v>49</v>
@@ -8942,7 +8942,7 @@
         <v>1417</v>
       </c>
       <c r="I107">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="J107">
         <v>36</v>
@@ -8986,7 +8986,7 @@
         <v>1417</v>
       </c>
       <c r="I108">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="K108" t="s">
         <v>1421</v>
@@ -9024,7 +9024,7 @@
         <v>1417</v>
       </c>
       <c r="I109">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="K109" t="s">
         <v>1421</v>
@@ -9207,7 +9207,7 @@
         <v>1417</v>
       </c>
       <c r="I115">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="K115" t="s">
         <v>1421</v>
@@ -9245,7 +9245,7 @@
         <v>1417</v>
       </c>
       <c r="I116">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="K116" t="s">
         <v>1421</v>
@@ -9283,7 +9283,7 @@
         <v>1417</v>
       </c>
       <c r="I117">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="K117" t="s">
         <v>1421</v>
@@ -9321,7 +9321,7 @@
         <v>1417</v>
       </c>
       <c r="I118">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="K118" t="s">
         <v>1421</v>
@@ -9359,7 +9359,7 @@
         <v>1417</v>
       </c>
       <c r="I119">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="K119" t="s">
         <v>1421</v>
@@ -9397,7 +9397,7 @@
         <v>1417</v>
       </c>
       <c r="I120">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="K120" t="s">
         <v>1421</v>
@@ -9435,7 +9435,7 @@
         <v>1417</v>
       </c>
       <c r="I121">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="J121">
         <v>251</v>
@@ -9482,7 +9482,7 @@
         <v>1417</v>
       </c>
       <c r="I122">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="K122" t="s">
         <v>1421</v>
@@ -9549,7 +9549,7 @@
         <v>1417</v>
       </c>
       <c r="I124">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="K124" t="s">
         <v>1421</v>
@@ -9587,7 +9587,7 @@
         <v>1417</v>
       </c>
       <c r="I125">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="K125" t="s">
         <v>1427</v>
@@ -9683,7 +9683,7 @@
         <v>1417</v>
       </c>
       <c r="I128">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="K128" t="s">
         <v>1421</v>
@@ -9721,7 +9721,7 @@
         <v>1417</v>
       </c>
       <c r="I129">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="K129" t="s">
         <v>1420</v>
@@ -9759,7 +9759,7 @@
         <v>1417</v>
       </c>
       <c r="I130">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="J130">
         <v>47</v>
@@ -9835,7 +9835,7 @@
         <v>1417</v>
       </c>
       <c r="I132">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="J132">
         <v>145</v>
@@ -9911,7 +9911,7 @@
         <v>1417</v>
       </c>
       <c r="I134">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="K134" t="s">
         <v>1420</v>
@@ -10036,7 +10036,7 @@
         <v>1417</v>
       </c>
       <c r="I138">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="K138" t="s">
         <v>1421</v>
@@ -10420,7 +10420,7 @@
         <v>1417</v>
       </c>
       <c r="I150">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="J150">
         <v>201</v>
@@ -10607,7 +10607,7 @@
         <v>1417</v>
       </c>
       <c r="I155">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="K155" t="s">
         <v>1427</v>
@@ -10642,7 +10642,7 @@
         <v>1417</v>
       </c>
       <c r="I156">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="K156" t="s">
         <v>1421</v>
@@ -10680,7 +10680,7 @@
         <v>1417</v>
       </c>
       <c r="I157">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="J157">
         <v>371</v>
@@ -10724,7 +10724,7 @@
         <v>1417</v>
       </c>
       <c r="I158">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="J158">
         <v>52</v>
@@ -10768,7 +10768,7 @@
         <v>1417</v>
       </c>
       <c r="I159">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="K159" t="s">
         <v>1421</v>
@@ -10806,7 +10806,7 @@
         <v>1417</v>
       </c>
       <c r="I160">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="K160" t="s">
         <v>1421</v>
@@ -10844,7 +10844,7 @@
         <v>1417</v>
       </c>
       <c r="I161">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="J161">
         <v>55</v>
@@ -10979,7 +10979,7 @@
         <v>1417</v>
       </c>
       <c r="I164">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="O164" t="s">
         <v>1533</v>
@@ -11154,7 +11154,7 @@
         <v>1417</v>
       </c>
       <c r="I169">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="K169" t="s">
         <v>1394</v>
@@ -11364,7 +11364,7 @@
         <v>1417</v>
       </c>
       <c r="I175">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="J175">
         <v>205</v>
@@ -11411,7 +11411,7 @@
         <v>1417</v>
       </c>
       <c r="I176">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="K176" t="s">
         <v>1421</v>
@@ -11449,7 +11449,7 @@
         <v>1417</v>
       </c>
       <c r="I177">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="J177">
         <v>44</v>
@@ -11496,7 +11496,7 @@
         <v>1417</v>
       </c>
       <c r="I178">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="K178" t="s">
         <v>1420</v>
@@ -11563,7 +11563,7 @@
         <v>1417</v>
       </c>
       <c r="I180">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="K180" t="s">
         <v>1420</v>
@@ -11659,7 +11659,7 @@
         <v>1417</v>
       </c>
       <c r="I183">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="K183" t="s">
         <v>1421</v>
@@ -11697,7 +11697,7 @@
         <v>1417</v>
       </c>
       <c r="I184">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="K184" t="s">
         <v>1427</v>
@@ -11732,7 +11732,7 @@
         <v>1417</v>
       </c>
       <c r="I185">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="K185" t="s">
         <v>1421</v>
@@ -11770,7 +11770,7 @@
         <v>1417</v>
       </c>
       <c r="I186">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="K186" t="s">
         <v>1421</v>
@@ -11808,7 +11808,7 @@
         <v>1417</v>
       </c>
       <c r="I187">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="J187">
         <v>75</v>
@@ -11855,7 +11855,7 @@
         <v>1417</v>
       </c>
       <c r="I188">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="J188">
         <v>40</v>
@@ -11902,7 +11902,7 @@
         <v>1417</v>
       </c>
       <c r="I189">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="J189">
         <v>155</v>
@@ -11946,7 +11946,7 @@
         <v>1417</v>
       </c>
       <c r="I190">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="J190">
         <v>107</v>
@@ -11990,7 +11990,7 @@
         <v>1417</v>
       </c>
       <c r="I191">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="J191">
         <v>5</v>
@@ -12034,7 +12034,7 @@
         <v>1417</v>
       </c>
       <c r="I192">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="K192" t="s">
         <v>1421</v>
@@ -12072,7 +12072,7 @@
         <v>1417</v>
       </c>
       <c r="I193">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="K193" t="s">
         <v>1426</v>
@@ -12267,7 +12267,7 @@
         <v>1417</v>
       </c>
       <c r="I199">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="J199">
         <v>70</v>
@@ -12352,7 +12352,7 @@
         <v>1417</v>
       </c>
       <c r="I201">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="K201" t="s">
         <v>1421</v>
@@ -12390,7 +12390,7 @@
         <v>1417</v>
       </c>
       <c r="I202">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="K202" t="s">
         <v>1421</v>
@@ -12469,7 +12469,7 @@
         <v>1417</v>
       </c>
       <c r="I204">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="K204" t="s">
         <v>1420</v>
@@ -12507,7 +12507,7 @@
         <v>1417</v>
       </c>
       <c r="I205">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="K205" t="s">
         <v>1420</v>
@@ -12574,7 +12574,7 @@
         <v>1417</v>
       </c>
       <c r="I207">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="J207">
         <v>167</v>
@@ -12618,7 +12618,7 @@
         <v>1417</v>
       </c>
       <c r="I208">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="J208">
         <v>45</v>
@@ -12662,7 +12662,7 @@
         <v>1417</v>
       </c>
       <c r="I209">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="J209">
         <v>191</v>
@@ -12706,7 +12706,7 @@
         <v>1417</v>
       </c>
       <c r="I210">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="K210" t="s">
         <v>1424</v>
@@ -12802,7 +12802,7 @@
         <v>1417</v>
       </c>
       <c r="I213">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="K213" t="s">
         <v>1421</v>
@@ -12840,7 +12840,7 @@
         <v>1417</v>
       </c>
       <c r="I214">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="J214">
         <v>14</v>
@@ -12887,7 +12887,7 @@
         <v>1417</v>
       </c>
       <c r="I215">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="K215" t="s">
         <v>1421</v>
@@ -12954,7 +12954,7 @@
         <v>1417</v>
       </c>
       <c r="I217">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="J217">
         <v>42</v>
@@ -12998,7 +12998,7 @@
         <v>1417</v>
       </c>
       <c r="I218">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="J218">
         <v>166</v>
@@ -13086,7 +13086,7 @@
         <v>1417</v>
       </c>
       <c r="I220">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="J220">
         <v>154</v>
@@ -13472,7 +13472,7 @@
         <v>1417</v>
       </c>
       <c r="I230">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="J230">
         <v>197</v>
@@ -13516,7 +13516,7 @@
         <v>1417</v>
       </c>
       <c r="I231">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="J231">
         <v>35</v>
@@ -13618,7 +13618,7 @@
         <v>1417</v>
       </c>
       <c r="I234">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="J234">
         <v>35</v>
@@ -13665,7 +13665,7 @@
         <v>1417</v>
       </c>
       <c r="I235">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="J235">
         <v>35</v>
@@ -13712,7 +13712,7 @@
         <v>1417</v>
       </c>
       <c r="I236">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="J236">
         <v>86</v>
@@ -13829,7 +13829,7 @@
         <v>1417</v>
       </c>
       <c r="I239">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="K239" t="s">
         <v>1394</v>
@@ -13928,7 +13928,7 @@
         <v>1417</v>
       </c>
       <c r="I242">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="K242" t="s">
         <v>1420</v>
@@ -13995,7 +13995,7 @@
         <v>1417</v>
       </c>
       <c r="I244">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="J244">
         <v>15</v>
@@ -14036,7 +14036,7 @@
         <v>1417</v>
       </c>
       <c r="I245">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="J245">
         <v>15</v>
@@ -14179,7 +14179,7 @@
         <v>1417</v>
       </c>
       <c r="I249">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="K249" t="s">
         <v>1421</v>
@@ -14313,7 +14313,7 @@
         <v>1417</v>
       </c>
       <c r="I253">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="J253">
         <v>162</v>
@@ -14357,7 +14357,7 @@
         <v>1417</v>
       </c>
       <c r="I254">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="K254" t="s">
         <v>1424</v>
@@ -14436,7 +14436,7 @@
         <v>1417</v>
       </c>
       <c r="I256">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="J256">
         <v>23</v>
@@ -14620,7 +14620,7 @@
         <v>1417</v>
       </c>
       <c r="I261">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="J261">
         <v>162</v>
@@ -14778,7 +14778,7 @@
         <v>1417</v>
       </c>
       <c r="I265">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="J265">
         <v>162</v>
@@ -14863,7 +14863,7 @@
         <v>1417</v>
       </c>
       <c r="I267">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="K267" t="s">
         <v>1424</v>
@@ -14901,7 +14901,7 @@
         <v>1417</v>
       </c>
       <c r="I268">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="K268" t="s">
         <v>1421</v>
@@ -14936,7 +14936,7 @@
         <v>1417</v>
       </c>
       <c r="I269">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="K269" t="s">
         <v>1421</v>
@@ -14974,7 +14974,7 @@
         <v>1417</v>
       </c>
       <c r="I270">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="K270" t="s">
         <v>1424</v>
@@ -15012,7 +15012,7 @@
         <v>1417</v>
       </c>
       <c r="I271">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="K271" t="s">
         <v>1424</v>
@@ -15190,7 +15190,7 @@
         <v>1417</v>
       </c>
       <c r="I276">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="K276" t="s">
         <v>1425</v>
@@ -15228,7 +15228,7 @@
         <v>1417</v>
       </c>
       <c r="I277">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="K277" t="s">
         <v>1421</v>
@@ -15266,7 +15266,7 @@
         <v>1417</v>
       </c>
       <c r="I278">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="J278">
         <v>148</v>
@@ -15310,7 +15310,7 @@
         <v>1417</v>
       </c>
       <c r="I279">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="K279" t="s">
         <v>1423</v>
@@ -15351,7 +15351,7 @@
         <v>1417</v>
       </c>
       <c r="I280">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="K280" t="s">
         <v>1421</v>
@@ -15389,7 +15389,7 @@
         <v>1417</v>
       </c>
       <c r="I281">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="K281" t="s">
         <v>1421</v>
@@ -15430,7 +15430,7 @@
         <v>1417</v>
       </c>
       <c r="I282">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="K282" t="s">
         <v>1421</v>
@@ -15724,7 +15724,7 @@
         <v>1417</v>
       </c>
       <c r="I291">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="J291">
         <v>20</v>
@@ -15768,7 +15768,7 @@
         <v>1417</v>
       </c>
       <c r="I292">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="K292" t="s">
         <v>1424</v>
@@ -15806,7 +15806,7 @@
         <v>1417</v>
       </c>
       <c r="I293">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="K293" t="s">
         <v>1425</v>
@@ -15844,7 +15844,7 @@
         <v>1417</v>
       </c>
       <c r="I294">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="K294" t="s">
         <v>1430</v>
@@ -15981,7 +15981,7 @@
         <v>1417</v>
       </c>
       <c r="I298">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="J298">
         <v>58</v>
@@ -16145,7 +16145,7 @@
         <v>1417</v>
       </c>
       <c r="I302">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="K302" t="s">
         <v>1424</v>
@@ -16183,7 +16183,7 @@
         <v>1417</v>
       </c>
       <c r="I303">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="K303" t="s">
         <v>1421</v>
@@ -16221,7 +16221,7 @@
         <v>1417</v>
       </c>
       <c r="I304">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="K304" t="s">
         <v>1424</v>
@@ -16259,7 +16259,7 @@
         <v>1417</v>
       </c>
       <c r="I305">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="J305">
         <v>35</v>
@@ -16303,7 +16303,7 @@
         <v>1417</v>
       </c>
       <c r="I306">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="J306">
         <v>31</v>
@@ -16391,7 +16391,7 @@
         <v>1417</v>
       </c>
       <c r="I308">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="K308" t="s">
         <v>1420</v>
@@ -16508,7 +16508,7 @@
         <v>1417</v>
       </c>
       <c r="I311">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="K311" t="s">
         <v>1420</v>
@@ -16838,7 +16838,7 @@
         <v>1417</v>
       </c>
       <c r="I320">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="K320" t="s">
         <v>1425</v>
@@ -16876,7 +16876,7 @@
         <v>1417</v>
       </c>
       <c r="I321">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="K321" t="s">
         <v>1421</v>
@@ -16914,7 +16914,7 @@
         <v>1417</v>
       </c>
       <c r="I322">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="J322">
         <v>57</v>
@@ -17028,7 +17028,7 @@
         <v>1417</v>
       </c>
       <c r="I325">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="J325">
         <v>57</v>
@@ -17110,7 +17110,7 @@
         <v>1417</v>
       </c>
       <c r="I327">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="J327">
         <v>57</v>
@@ -17154,7 +17154,7 @@
         <v>1417</v>
       </c>
       <c r="I328">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="J328">
         <v>57</v>
@@ -17198,7 +17198,7 @@
         <v>1417</v>
       </c>
       <c r="I329">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="J329">
         <v>57</v>
@@ -17242,7 +17242,7 @@
         <v>1417</v>
       </c>
       <c r="I330">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="J330">
         <v>57</v>
@@ -17286,7 +17286,7 @@
         <v>1417</v>
       </c>
       <c r="I331">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="K331" t="s">
         <v>1420</v>
@@ -17324,7 +17324,7 @@
         <v>1417</v>
       </c>
       <c r="I332">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="K332" t="s">
         <v>1421</v>
@@ -17362,7 +17362,7 @@
         <v>1417</v>
       </c>
       <c r="I333">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="J333">
         <v>100</v>
@@ -17406,7 +17406,7 @@
         <v>1417</v>
       </c>
       <c r="I334">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="K334" t="s">
         <v>1421</v>
@@ -17631,7 +17631,7 @@
         <v>1417</v>
       </c>
       <c r="I340">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="J340">
         <v>98</v>
@@ -17672,7 +17672,7 @@
         <v>1417</v>
       </c>
       <c r="I341">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="J341">
         <v>90</v>
@@ -17713,7 +17713,7 @@
         <v>1417</v>
       </c>
       <c r="I342">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="K342" t="s">
         <v>1420</v>
@@ -17827,7 +17827,7 @@
         <v>1417</v>
       </c>
       <c r="I345">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="K345" t="s">
         <v>1420</v>
@@ -17947,7 +17947,7 @@
         <v>1417</v>
       </c>
       <c r="I348">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="J348">
         <v>14</v>
@@ -17991,7 +17991,7 @@
         <v>1417</v>
       </c>
       <c r="I349">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="K349" t="s">
         <v>1425</v>
@@ -18029,7 +18029,7 @@
         <v>1417</v>
       </c>
       <c r="I350">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="J350">
         <v>46</v>
@@ -18067,7 +18067,7 @@
         <v>1417</v>
       </c>
       <c r="I351">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="J351">
         <v>82</v>
@@ -18111,7 +18111,7 @@
         <v>1417</v>
       </c>
       <c r="I352">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="J352">
         <v>78</v>
@@ -18155,7 +18155,7 @@
         <v>1417</v>
       </c>
       <c r="I353">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="J353">
         <v>83</v>
@@ -18199,7 +18199,7 @@
         <v>1417</v>
       </c>
       <c r="I354">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="K354" t="s">
         <v>1424</v>
@@ -18237,7 +18237,7 @@
         <v>1417</v>
       </c>
       <c r="I355">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="J355">
         <v>8</v>
@@ -18319,7 +18319,7 @@
         <v>1417</v>
       </c>
       <c r="I357">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="J357">
         <v>85</v>
@@ -18442,7 +18442,7 @@
         <v>1417</v>
       </c>
       <c r="I360">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="J360">
         <v>83</v>
@@ -18489,7 +18489,7 @@
         <v>1417</v>
       </c>
       <c r="I361">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="J361">
         <v>83</v>
@@ -18533,7 +18533,7 @@
         <v>1417</v>
       </c>
       <c r="I362">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="K362" t="s">
         <v>1424</v>
@@ -18571,7 +18571,7 @@
         <v>1417</v>
       </c>
       <c r="I363">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="K363" t="s">
         <v>1424</v>
@@ -18609,7 +18609,7 @@
         <v>1417</v>
       </c>
       <c r="I364">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="J364">
         <v>83</v>
@@ -18653,7 +18653,7 @@
         <v>1417</v>
       </c>
       <c r="I365">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="J365">
         <v>15</v>
@@ -18776,7 +18776,7 @@
         <v>1417</v>
       </c>
       <c r="I368">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J368">
         <v>77</v>
@@ -18820,7 +18820,7 @@
         <v>1417</v>
       </c>
       <c r="I369">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K369" t="s">
         <v>1424</v>
@@ -18858,7 +18858,7 @@
         <v>1417</v>
       </c>
       <c r="I370">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K370" t="s">
         <v>1424</v>
@@ -18896,7 +18896,7 @@
         <v>1417</v>
       </c>
       <c r="I371">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J371">
         <v>16</v>
@@ -18984,7 +18984,7 @@
         <v>1417</v>
       </c>
       <c r="I373">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="K373" t="s">
         <v>1420</v>
@@ -19022,7 +19022,7 @@
         <v>1417</v>
       </c>
       <c r="I374">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="K374" t="s">
         <v>1420</v>
@@ -19060,7 +19060,7 @@
         <v>1417</v>
       </c>
       <c r="I375">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="J375">
         <v>94</v>
@@ -19101,7 +19101,7 @@
         <v>1417</v>
       </c>
       <c r="I376">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="K376" t="s">
         <v>1424</v>
@@ -19180,7 +19180,7 @@
         <v>1417</v>
       </c>
       <c r="I378">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="K378" t="s">
         <v>1424</v>
@@ -19218,7 +19218,7 @@
         <v>1417</v>
       </c>
       <c r="I379">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="J379">
         <v>20</v>
@@ -19262,7 +19262,7 @@
         <v>1417</v>
       </c>
       <c r="I380">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="J380">
         <v>94</v>
@@ -19306,7 +19306,7 @@
         <v>1417</v>
       </c>
       <c r="I381">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="K381" t="s">
         <v>1424</v>
@@ -19344,7 +19344,7 @@
         <v>1417</v>
       </c>
       <c r="I382">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="K382" t="s">
         <v>1424</v>
@@ -19382,7 +19382,7 @@
         <v>1417</v>
       </c>
       <c r="I383">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="J383">
         <v>71</v>
@@ -19426,7 +19426,7 @@
         <v>1417</v>
       </c>
       <c r="I384">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="K384" t="s">
         <v>1421</v>
@@ -19508,7 +19508,7 @@
         <v>1417</v>
       </c>
       <c r="I386">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="K386" t="s">
         <v>1424</v>
@@ -19546,7 +19546,7 @@
         <v>1417</v>
       </c>
       <c r="I387">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="K387" t="s">
         <v>1424</v>
@@ -19584,7 +19584,7 @@
         <v>1417</v>
       </c>
       <c r="I388">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J388">
         <v>-85</v>
@@ -19628,7 +19628,7 @@
         <v>1417</v>
       </c>
       <c r="I389">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="K389" t="s">
         <v>1425</v>
@@ -20079,7 +20079,7 @@
         <v>1417</v>
       </c>
       <c r="I400">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="K400" t="s">
         <v>1424</v>
@@ -20155,7 +20155,7 @@
         <v>1417</v>
       </c>
       <c r="I402">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="K402" t="s">
         <v>1424</v>
@@ -20193,7 +20193,7 @@
         <v>1417</v>
       </c>
       <c r="I403">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J403">
         <v>83</v>
@@ -20237,7 +20237,7 @@
         <v>1417</v>
       </c>
       <c r="I404">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="K404" t="s">
         <v>1424</v>
@@ -20307,7 +20307,7 @@
         <v>1417</v>
       </c>
       <c r="I406">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="Q406" t="b">
         <v>1</v>
@@ -20339,7 +20339,7 @@
         <v>1417</v>
       </c>
       <c r="I407">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="Q407" t="b">
         <v>1</v>
@@ -20371,7 +20371,7 @@
         <v>1417</v>
       </c>
       <c r="I408">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="Q408" t="b">
         <v>1</v>
@@ -20403,7 +20403,7 @@
         <v>1417</v>
       </c>
       <c r="I409">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="Q409" t="b">
         <v>1</v>
@@ -20435,7 +20435,7 @@
         <v>1417</v>
       </c>
       <c r="I410">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="Q410" t="b">
         <v>1</v>
@@ -20467,7 +20467,7 @@
         <v>1417</v>
       </c>
       <c r="I411">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="Q411" t="b">
         <v>1</v>
@@ -20499,7 +20499,7 @@
         <v>1417</v>
       </c>
       <c r="I412">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="Q412" t="b">
         <v>1</v>
@@ -20531,7 +20531,7 @@
         <v>1417</v>
       </c>
       <c r="I413">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="Q413" t="b">
         <v>1</v>
@@ -20621,7 +20621,7 @@
         <v>1417</v>
       </c>
       <c r="I416">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="Q416" t="b">
         <v>1</v>
@@ -20711,7 +20711,7 @@
         <v>1417</v>
       </c>
       <c r="I419">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="Q419" t="b">
         <v>1</v>
@@ -20743,7 +20743,7 @@
         <v>1417</v>
       </c>
       <c r="I420">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="Q420" t="b">
         <v>1</v>
@@ -20775,7 +20775,7 @@
         <v>1417</v>
       </c>
       <c r="I421">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="Q421" t="b">
         <v>1</v>
@@ -20807,7 +20807,7 @@
         <v>1417</v>
       </c>
       <c r="I422">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="Q422" t="b">
         <v>1</v>
@@ -20839,7 +20839,7 @@
         <v>1417</v>
       </c>
       <c r="I423">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="Q423" t="b">
         <v>1</v>
@@ -20871,7 +20871,7 @@
         <v>1417</v>
       </c>
       <c r="I424">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="Q424" t="b">
         <v>1</v>
@@ -20903,7 +20903,7 @@
         <v>1417</v>
       </c>
       <c r="I425">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="Q425" t="b">
         <v>1</v>
@@ -20935,7 +20935,7 @@
         <v>1417</v>
       </c>
       <c r="I426">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="Q426" t="b">
         <v>1</v>
@@ -20967,7 +20967,7 @@
         <v>1417</v>
       </c>
       <c r="I427">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="Q427" t="b">
         <v>1</v>
@@ -21057,7 +21057,7 @@
         <v>1417</v>
       </c>
       <c r="I430">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="Q430" t="b">
         <v>1</v>
@@ -21089,7 +21089,7 @@
         <v>1417</v>
       </c>
       <c r="I431">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="Q431" t="b">
         <v>1</v>
@@ -21121,7 +21121,7 @@
         <v>1417</v>
       </c>
       <c r="I432">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="Q432" t="b">
         <v>1</v>
@@ -21153,7 +21153,7 @@
         <v>1417</v>
       </c>
       <c r="I433">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="Q433" t="b">
         <v>1</v>
@@ -21185,7 +21185,7 @@
         <v>1417</v>
       </c>
       <c r="I434">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="Q434" t="b">
         <v>1</v>
@@ -21217,7 +21217,7 @@
         <v>1417</v>
       </c>
       <c r="I435">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="Q435" t="b">
         <v>1</v>
@@ -21249,7 +21249,7 @@
         <v>1417</v>
       </c>
       <c r="I436">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="Q436" t="b">
         <v>1</v>
@@ -21281,7 +21281,7 @@
         <v>1419</v>
       </c>
       <c r="I437">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="Q437" t="b">
         <v>1</v>
@@ -21313,7 +21313,7 @@
         <v>1419</v>
       </c>
       <c r="I438">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="Q438" t="b">
         <v>1</v>
@@ -21345,7 +21345,7 @@
         <v>1417</v>
       </c>
       <c r="I439">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="Q439" t="b">
         <v>1</v>
@@ -21377,7 +21377,7 @@
         <v>1417</v>
       </c>
       <c r="I440">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="Q440" t="b">
         <v>1</v>
@@ -21409,7 +21409,7 @@
         <v>1417</v>
       </c>
       <c r="I441">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="Q441" t="b">
         <v>1</v>
@@ -21470,7 +21470,7 @@
         <v>1417</v>
       </c>
       <c r="I443">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="Q443" t="b">
         <v>1</v>
@@ -21560,7 +21560,7 @@
         <v>1417</v>
       </c>
       <c r="I446">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="Q446" t="b">
         <v>1</v>
@@ -21592,7 +21592,7 @@
         <v>1417</v>
       </c>
       <c r="I447">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="Q447" t="b">
         <v>1</v>
@@ -21624,7 +21624,7 @@
         <v>1417</v>
       </c>
       <c r="I448">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="Q448" t="b">
         <v>1</v>
@@ -21656,7 +21656,7 @@
         <v>1417</v>
       </c>
       <c r="I449">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="Q449" t="b">
         <v>1</v>
@@ -21688,7 +21688,7 @@
         <v>1417</v>
       </c>
       <c r="I450">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="Q450" t="b">
         <v>1</v>
@@ -21720,7 +21720,7 @@
         <v>1417</v>
       </c>
       <c r="I451">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="Q451" t="b">
         <v>1</v>
@@ -21781,7 +21781,7 @@
         <v>1417</v>
       </c>
       <c r="I453">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="Q453" t="b">
         <v>1</v>
@@ -21813,7 +21813,7 @@
         <v>1417</v>
       </c>
       <c r="I454">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="Q454" t="b">
         <v>1</v>
@@ -21845,7 +21845,7 @@
         <v>1417</v>
       </c>
       <c r="I455">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="Q455" t="b">
         <v>1</v>
@@ -21906,7 +21906,7 @@
         <v>1417</v>
       </c>
       <c r="I457">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="Q457" t="b">
         <v>1</v>
@@ -21938,7 +21938,7 @@
         <v>1417</v>
       </c>
       <c r="I458">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q458" t="b">
         <v>1</v>
@@ -21970,7 +21970,7 @@
         <v>1417</v>
       </c>
       <c r="I459">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="Q459" t="b">
         <v>1</v>
@@ -22002,7 +22002,7 @@
         <v>1417</v>
       </c>
       <c r="I460">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="Q460" t="b">
         <v>1</v>
@@ -22034,7 +22034,7 @@
         <v>1417</v>
       </c>
       <c r="I461">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="Q461" t="b">
         <v>1</v>
@@ -22066,7 +22066,7 @@
         <v>1417</v>
       </c>
       <c r="I462">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="Q462" t="b">
         <v>1</v>
@@ -22098,7 +22098,7 @@
         <v>1417</v>
       </c>
       <c r="I463">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="Q463" t="b">
         <v>1</v>
@@ -22130,7 +22130,7 @@
         <v>1417</v>
       </c>
       <c r="I464">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="Q464" t="b">
         <v>1</v>
@@ -22162,7 +22162,7 @@
         <v>1417</v>
       </c>
       <c r="I465">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="Q465" t="b">
         <v>1</v>
@@ -22194,7 +22194,7 @@
         <v>1417</v>
       </c>
       <c r="I466">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="Q466" t="b">
         <v>1</v>
@@ -22226,7 +22226,7 @@
         <v>1417</v>
       </c>
       <c r="I467">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="Q467" t="b">
         <v>1</v>
@@ -22258,7 +22258,7 @@
         <v>1417</v>
       </c>
       <c r="I468">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="Q468" t="b">
         <v>1</v>
@@ -22290,7 +22290,7 @@
         <v>1417</v>
       </c>
       <c r="I469">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="Q469" t="b">
         <v>1</v>
@@ -22351,7 +22351,7 @@
         <v>1417</v>
       </c>
       <c r="I471">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="Q471" t="b">
         <v>1</v>
@@ -22383,7 +22383,7 @@
         <v>1417</v>
       </c>
       <c r="I472">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="Q472" t="b">
         <v>1</v>
@@ -22415,7 +22415,7 @@
         <v>1417</v>
       </c>
       <c r="I473">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="Q473" t="b">
         <v>1</v>
@@ -22447,7 +22447,7 @@
         <v>1417</v>
       </c>
       <c r="I474">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q474" t="b">
         <v>1</v>
@@ -22479,7 +22479,7 @@
         <v>1417</v>
       </c>
       <c r="I475">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q475" t="b">
         <v>1</v>
@@ -22511,7 +22511,7 @@
         <v>1417</v>
       </c>
       <c r="I476">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q476" t="b">
         <v>1</v>
@@ -22543,7 +22543,7 @@
         <v>1417</v>
       </c>
       <c r="I477">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q477" t="b">
         <v>1</v>
@@ -22575,7 +22575,7 @@
         <v>1417</v>
       </c>
       <c r="I478">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q478" t="b">
         <v>1</v>
@@ -22607,7 +22607,7 @@
         <v>1417</v>
       </c>
       <c r="I479">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q479" t="b">
         <v>1</v>
@@ -22639,7 +22639,7 @@
         <v>1417</v>
       </c>
       <c r="I480">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q480" t="b">
         <v>1</v>
@@ -22671,7 +22671,7 @@
         <v>1417</v>
       </c>
       <c r="I481">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q481" t="b">
         <v>1</v>
@@ -22703,7 +22703,7 @@
         <v>1417</v>
       </c>
       <c r="I482">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q482" t="b">
         <v>1</v>
@@ -22735,7 +22735,7 @@
         <v>1417</v>
       </c>
       <c r="I483">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q483" t="b">
         <v>1</v>
@@ -22767,7 +22767,7 @@
         <v>1417</v>
       </c>
       <c r="I484">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q484" t="b">
         <v>1</v>
@@ -22799,7 +22799,7 @@
         <v>1417</v>
       </c>
       <c r="I485">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q485" t="b">
         <v>1</v>
@@ -22831,7 +22831,7 @@
         <v>1417</v>
       </c>
       <c r="I486">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q486" t="b">
         <v>1</v>
@@ -22863,7 +22863,7 @@
         <v>1417</v>
       </c>
       <c r="I487">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q487" t="b">
         <v>1</v>
@@ -22895,7 +22895,7 @@
         <v>1417</v>
       </c>
       <c r="I488">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q488" t="b">
         <v>1</v>
@@ -22927,7 +22927,7 @@
         <v>1417</v>
       </c>
       <c r="I489">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q489" t="b">
         <v>1</v>
@@ -22959,7 +22959,7 @@
         <v>1417</v>
       </c>
       <c r="I490">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q490" t="b">
         <v>1</v>
@@ -22991,7 +22991,7 @@
         <v>1417</v>
       </c>
       <c r="I491">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q491" t="b">
         <v>1</v>
@@ -23023,7 +23023,7 @@
         <v>1419</v>
       </c>
       <c r="I492">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q492" t="b">
         <v>1</v>
@@ -23055,7 +23055,7 @@
         <v>1419</v>
       </c>
       <c r="I493">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q493" t="b">
         <v>1</v>
@@ -23087,7 +23087,7 @@
         <v>1419</v>
       </c>
       <c r="I494">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q494" t="b">
         <v>1</v>
@@ -23119,7 +23119,7 @@
         <v>1419</v>
       </c>
       <c r="I495">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q495" t="b">
         <v>1</v>
@@ -23151,7 +23151,7 @@
         <v>1419</v>
       </c>
       <c r="I496">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q496" t="b">
         <v>1</v>
@@ -23183,7 +23183,7 @@
         <v>1417</v>
       </c>
       <c r="I497">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q497" t="b">
         <v>1</v>
@@ -23215,7 +23215,7 @@
         <v>1417</v>
       </c>
       <c r="I498">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q498" t="b">
         <v>1</v>
@@ -23247,7 +23247,7 @@
         <v>1419</v>
       </c>
       <c r="I499">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q499" t="b">
         <v>1</v>
@@ -23279,7 +23279,7 @@
         <v>1417</v>
       </c>
       <c r="I500">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q500" t="b">
         <v>1</v>
@@ -23311,7 +23311,7 @@
         <v>1417</v>
       </c>
       <c r="I501">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q501" t="b">
         <v>1</v>
@@ -23343,7 +23343,7 @@
         <v>1417</v>
       </c>
       <c r="I502">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q502" t="b">
         <v>1</v>
@@ -23375,7 +23375,7 @@
         <v>1417</v>
       </c>
       <c r="I503">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q503" t="b">
         <v>1</v>
@@ -23407,7 +23407,7 @@
         <v>1417</v>
       </c>
       <c r="I504">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q504" t="b">
         <v>1</v>
@@ -23439,7 +23439,7 @@
         <v>1417</v>
       </c>
       <c r="I505">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q505" t="b">
         <v>1</v>
@@ -23471,7 +23471,7 @@
         <v>1417</v>
       </c>
       <c r="I506">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q506" t="b">
         <v>1</v>
@@ -23503,7 +23503,7 @@
         <v>1417</v>
       </c>
       <c r="I507">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="Q507" t="b">
         <v>1</v>
@@ -23564,7 +23564,7 @@
         <v>1417</v>
       </c>
       <c r="I509">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="Q509" t="b">
         <v>1</v>
@@ -23596,7 +23596,7 @@
         <v>1417</v>
       </c>
       <c r="I510">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="Q510" t="b">
         <v>1</v>
@@ -23628,7 +23628,7 @@
         <v>1417</v>
       </c>
       <c r="I511">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q511" t="b">
         <v>1</v>
@@ -23660,7 +23660,7 @@
         <v>1417</v>
       </c>
       <c r="I512">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q512" t="b">
         <v>1</v>
@@ -23692,7 +23692,7 @@
         <v>1417</v>
       </c>
       <c r="I513">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="Q513" t="b">
         <v>1</v>
@@ -23753,7 +23753,7 @@
         <v>1417</v>
       </c>
       <c r="I515">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="Q515" t="b">
         <v>1</v>
@@ -23785,7 +23785,7 @@
         <v>1417</v>
       </c>
       <c r="I516">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="Q516" t="b">
         <v>1</v>
@@ -23817,7 +23817,7 @@
         <v>1417</v>
       </c>
       <c r="I517">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="Q517" t="b">
         <v>1</v>
@@ -23849,7 +23849,7 @@
         <v>1417</v>
       </c>
       <c r="I518">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="Q518" t="b">
         <v>1</v>
@@ -23881,7 +23881,7 @@
         <v>1417</v>
       </c>
       <c r="I519">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Q519" t="b">
         <v>1</v>
@@ -23913,7 +23913,7 @@
         <v>1417</v>
       </c>
       <c r="I520">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Q520" t="b">
         <v>1</v>
@@ -23945,7 +23945,7 @@
         <v>1417</v>
       </c>
       <c r="I521">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Q521" t="b">
         <v>1</v>
@@ -23977,7 +23977,7 @@
         <v>1417</v>
       </c>
       <c r="I522">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Q522" t="b">
         <v>1</v>
@@ -24009,7 +24009,7 @@
         <v>1417</v>
       </c>
       <c r="I523">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Q523" t="b">
         <v>1</v>
@@ -24041,7 +24041,7 @@
         <v>1417</v>
       </c>
       <c r="I524">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q524" t="b">
         <v>1</v>
@@ -24073,7 +24073,7 @@
         <v>1417</v>
       </c>
       <c r="I525">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q525" t="b">
         <v>1</v>
@@ -24105,7 +24105,7 @@
         <v>1417</v>
       </c>
       <c r="I526">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q526" t="b">
         <v>1</v>
@@ -24137,7 +24137,7 @@
         <v>1417</v>
       </c>
       <c r="I527">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q527" t="b">
         <v>1</v>
@@ -24169,7 +24169,7 @@
         <v>1417</v>
       </c>
       <c r="I528">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="Q528" t="b">
         <v>1</v>
@@ -24201,7 +24201,7 @@
         <v>1417</v>
       </c>
       <c r="I529">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q529" t="b">
         <v>1</v>
@@ -24233,7 +24233,7 @@
         <v>1417</v>
       </c>
       <c r="I530">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q530" t="b">
         <v>1</v>
@@ -24265,7 +24265,7 @@
         <v>1417</v>
       </c>
       <c r="I531">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q531" t="b">
         <v>1</v>
@@ -24297,7 +24297,7 @@
         <v>1417</v>
       </c>
       <c r="I532">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q532" t="b">
         <v>1</v>
@@ -24329,7 +24329,7 @@
         <v>1417</v>
       </c>
       <c r="I533">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q533" t="b">
         <v>1</v>
@@ -24361,7 +24361,7 @@
         <v>1417</v>
       </c>
       <c r="I534">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q534" t="b">
         <v>1</v>
@@ -24393,7 +24393,7 @@
         <v>1417</v>
       </c>
       <c r="I535">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q535" t="b">
         <v>1</v>
@@ -24425,7 +24425,7 @@
         <v>1417</v>
       </c>
       <c r="I536">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q536" t="b">
         <v>1</v>
@@ -24457,7 +24457,7 @@
         <v>1417</v>
       </c>
       <c r="I537">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q537" t="b">
         <v>1</v>
@@ -24489,7 +24489,7 @@
         <v>1417</v>
       </c>
       <c r="I538">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q538" t="b">
         <v>1</v>
@@ -24521,7 +24521,7 @@
         <v>1417</v>
       </c>
       <c r="I539">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q539" t="b">
         <v>1</v>
@@ -24553,7 +24553,7 @@
         <v>1417</v>
       </c>
       <c r="I540">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q540" t="b">
         <v>1</v>
@@ -24585,7 +24585,7 @@
         <v>1417</v>
       </c>
       <c r="I541">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q541" t="b">
         <v>1</v>
@@ -24617,7 +24617,7 @@
         <v>1417</v>
       </c>
       <c r="I542">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q542" t="b">
         <v>1</v>
@@ -24649,7 +24649,7 @@
         <v>1417</v>
       </c>
       <c r="I543">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q543" t="b">
         <v>1</v>
@@ -24681,7 +24681,7 @@
         <v>1417</v>
       </c>
       <c r="I544">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q544" t="b">
         <v>1</v>
@@ -24713,7 +24713,7 @@
         <v>1417</v>
       </c>
       <c r="I545">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q545" t="b">
         <v>1</v>
@@ -24745,7 +24745,7 @@
         <v>1417</v>
       </c>
       <c r="I546">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q546" t="b">
         <v>1</v>
@@ -24777,7 +24777,7 @@
         <v>1417</v>
       </c>
       <c r="I547">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q547" t="b">
         <v>1</v>
@@ -24809,7 +24809,7 @@
         <v>1417</v>
       </c>
       <c r="I548">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q548" t="b">
         <v>1</v>
@@ -24841,7 +24841,7 @@
         <v>1417</v>
       </c>
       <c r="I549">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q549" t="b">
         <v>1</v>
@@ -24873,7 +24873,7 @@
         <v>1417</v>
       </c>
       <c r="I550">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q550" t="b">
         <v>1</v>
@@ -24905,7 +24905,7 @@
         <v>1417</v>
       </c>
       <c r="I551">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q551" t="b">
         <v>1</v>
@@ -24937,7 +24937,7 @@
         <v>1417</v>
       </c>
       <c r="I552">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q552" t="b">
         <v>1</v>
@@ -24969,7 +24969,7 @@
         <v>1417</v>
       </c>
       <c r="I553">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q553" t="b">
         <v>1</v>
@@ -25001,7 +25001,7 @@
         <v>1417</v>
       </c>
       <c r="I554">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q554" t="b">
         <v>1</v>
@@ -25033,7 +25033,7 @@
         <v>1417</v>
       </c>
       <c r="I555">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q555" t="b">
         <v>1</v>
@@ -25065,7 +25065,7 @@
         <v>1417</v>
       </c>
       <c r="I556">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q556" t="b">
         <v>1</v>
@@ -25097,7 +25097,7 @@
         <v>1417</v>
       </c>
       <c r="I557">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q557" t="b">
         <v>1</v>
@@ -25129,7 +25129,7 @@
         <v>1417</v>
       </c>
       <c r="I558">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q558" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: reparaveis (30/10/2026 14:01)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reparaveis_tratada.xlsx
@@ -5132,7 +5132,7 @@
         <v>1417</v>
       </c>
       <c r="I2">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="K2" t="s">
         <v>1420</v>
@@ -5170,7 +5170,7 @@
         <v>1417</v>
       </c>
       <c r="I3">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="K3" t="s">
         <v>1421</v>
@@ -5208,7 +5208,7 @@
         <v>1417</v>
       </c>
       <c r="I4">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="K4" t="s">
         <v>1421</v>
@@ -5246,7 +5246,7 @@
         <v>1417</v>
       </c>
       <c r="I5">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="J5">
         <v>279</v>
@@ -5290,7 +5290,7 @@
         <v>1417</v>
       </c>
       <c r="I6">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="J6">
         <v>153</v>
@@ -5334,7 +5334,7 @@
         <v>1417</v>
       </c>
       <c r="I7">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="J7">
         <v>112</v>
@@ -5410,7 +5410,7 @@
         <v>1417</v>
       </c>
       <c r="I9">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="J9">
         <v>362</v>
@@ -5457,7 +5457,7 @@
         <v>1417</v>
       </c>
       <c r="I10">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="J10">
         <v>378</v>
@@ -5504,7 +5504,7 @@
         <v>1417</v>
       </c>
       <c r="I11">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="J11">
         <v>112</v>
@@ -5551,7 +5551,7 @@
         <v>1417</v>
       </c>
       <c r="I12">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="J12">
         <v>124</v>
@@ -5624,7 +5624,7 @@
         <v>1417</v>
       </c>
       <c r="I14">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="J14">
         <v>64</v>
@@ -5703,7 +5703,7 @@
         <v>1417</v>
       </c>
       <c r="I16">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="K16" t="s">
         <v>1420</v>
@@ -5741,7 +5741,7 @@
         <v>1417</v>
       </c>
       <c r="I17">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="J17">
         <v>161</v>
@@ -5785,7 +5785,7 @@
         <v>1417</v>
       </c>
       <c r="I18">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="J18">
         <v>66</v>
@@ -5858,7 +5858,7 @@
         <v>1417</v>
       </c>
       <c r="I20">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="J20">
         <v>399</v>
@@ -5931,7 +5931,7 @@
         <v>1417</v>
       </c>
       <c r="I22">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="K22" t="s">
         <v>1424</v>
@@ -5969,7 +5969,7 @@
         <v>1417</v>
       </c>
       <c r="I23">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="J23">
         <v>229</v>
@@ -6074,7 +6074,7 @@
         <v>1417</v>
       </c>
       <c r="I26">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="J26">
         <v>155</v>
@@ -6121,7 +6121,7 @@
         <v>1417</v>
       </c>
       <c r="I27">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="K27" t="s">
         <v>1424</v>
@@ -6217,7 +6217,7 @@
         <v>1417</v>
       </c>
       <c r="I30">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="J30">
         <v>209</v>
@@ -6290,7 +6290,7 @@
         <v>1417</v>
       </c>
       <c r="I32">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="K32" t="s">
         <v>1420</v>
@@ -6499,7 +6499,7 @@
         <v>1417</v>
       </c>
       <c r="I39">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="K39" t="s">
         <v>1425</v>
@@ -6662,7 +6662,7 @@
         <v>1417</v>
       </c>
       <c r="I44">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="J44">
         <v>87</v>
@@ -6709,7 +6709,7 @@
         <v>1417</v>
       </c>
       <c r="I45">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="J45">
         <v>331</v>
@@ -6756,7 +6756,7 @@
         <v>1417</v>
       </c>
       <c r="I46">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="K46" t="s">
         <v>1424</v>
@@ -6797,7 +6797,7 @@
         <v>1417</v>
       </c>
       <c r="I47">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="J47">
         <v>344</v>
@@ -6844,7 +6844,7 @@
         <v>1417</v>
       </c>
       <c r="I48">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="K48" t="s">
         <v>1424</v>
@@ -6911,7 +6911,7 @@
         <v>1417</v>
       </c>
       <c r="I50">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="K50" t="s">
         <v>1424</v>
@@ -6978,7 +6978,7 @@
         <v>1417</v>
       </c>
       <c r="I52">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="K52" t="s">
         <v>1420</v>
@@ -7016,7 +7016,7 @@
         <v>1417</v>
       </c>
       <c r="I53">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="K53" t="s">
         <v>1421</v>
@@ -7054,7 +7054,7 @@
         <v>1417</v>
       </c>
       <c r="I54">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="K54" t="s">
         <v>1421</v>
@@ -7330,7 +7330,7 @@
         <v>1417</v>
       </c>
       <c r="I63">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="J63">
         <v>293</v>
@@ -7377,7 +7377,7 @@
         <v>1417</v>
       </c>
       <c r="I64">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="J64">
         <v>320</v>
@@ -7607,7 +7607,7 @@
         <v>1417</v>
       </c>
       <c r="I71">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="J71">
         <v>429</v>
@@ -7680,7 +7680,7 @@
         <v>1417</v>
       </c>
       <c r="I73">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="K73" t="s">
         <v>1420</v>
@@ -7788,7 +7788,7 @@
         <v>1417</v>
       </c>
       <c r="I76">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="K76" t="s">
         <v>1427</v>
@@ -7881,7 +7881,7 @@
         <v>1417</v>
       </c>
       <c r="I79">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="K79" t="s">
         <v>1427</v>
@@ -7986,7 +7986,7 @@
         <v>1417</v>
       </c>
       <c r="I82">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="K82" t="s">
         <v>1424</v>
@@ -8053,7 +8053,7 @@
         <v>1417</v>
       </c>
       <c r="I84">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="J84">
         <v>40</v>
@@ -8100,7 +8100,7 @@
         <v>1417</v>
       </c>
       <c r="I85">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="K85" t="s">
         <v>1421</v>
@@ -8138,7 +8138,7 @@
         <v>1417</v>
       </c>
       <c r="I86">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="K86" t="s">
         <v>1421</v>
@@ -8176,7 +8176,7 @@
         <v>1417</v>
       </c>
       <c r="I87">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="J87">
         <v>-16</v>
@@ -8299,7 +8299,7 @@
         <v>1417</v>
       </c>
       <c r="I90">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="K90" t="s">
         <v>1394</v>
@@ -8448,7 +8448,7 @@
         <v>1417</v>
       </c>
       <c r="I94">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="K94" t="s">
         <v>1424</v>
@@ -8527,7 +8527,7 @@
         <v>1417</v>
       </c>
       <c r="I96">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="J96">
         <v>17</v>
@@ -8574,7 +8574,7 @@
         <v>1417</v>
       </c>
       <c r="I97">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="J97">
         <v>20</v>
@@ -8621,7 +8621,7 @@
         <v>1417</v>
       </c>
       <c r="I98">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="K98" t="s">
         <v>1424</v>
@@ -8898,7 +8898,7 @@
         <v>1417</v>
       </c>
       <c r="I106">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="J106">
         <v>49</v>
@@ -8942,7 +8942,7 @@
         <v>1417</v>
       </c>
       <c r="I107">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="J107">
         <v>36</v>
@@ -8986,7 +8986,7 @@
         <v>1417</v>
       </c>
       <c r="I108">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="K108" t="s">
         <v>1421</v>
@@ -9024,7 +9024,7 @@
         <v>1417</v>
       </c>
       <c r="I109">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="K109" t="s">
         <v>1421</v>
@@ -9207,7 +9207,7 @@
         <v>1417</v>
       </c>
       <c r="I115">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="K115" t="s">
         <v>1421</v>
@@ -9245,7 +9245,7 @@
         <v>1417</v>
       </c>
       <c r="I116">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="K116" t="s">
         <v>1421</v>
@@ -9283,7 +9283,7 @@
         <v>1417</v>
       </c>
       <c r="I117">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="K117" t="s">
         <v>1421</v>
@@ -9321,7 +9321,7 @@
         <v>1417</v>
       </c>
       <c r="I118">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="K118" t="s">
         <v>1421</v>
@@ -9359,7 +9359,7 @@
         <v>1417</v>
       </c>
       <c r="I119">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="K119" t="s">
         <v>1421</v>
@@ -9397,7 +9397,7 @@
         <v>1417</v>
       </c>
       <c r="I120">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="K120" t="s">
         <v>1421</v>
@@ -9435,7 +9435,7 @@
         <v>1417</v>
       </c>
       <c r="I121">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="J121">
         <v>251</v>
@@ -9482,7 +9482,7 @@
         <v>1417</v>
       </c>
       <c r="I122">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="K122" t="s">
         <v>1421</v>
@@ -9549,7 +9549,7 @@
         <v>1417</v>
       </c>
       <c r="I124">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="K124" t="s">
         <v>1421</v>
@@ -9587,7 +9587,7 @@
         <v>1417</v>
       </c>
       <c r="I125">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="K125" t="s">
         <v>1427</v>
@@ -9683,7 +9683,7 @@
         <v>1417</v>
       </c>
       <c r="I128">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="K128" t="s">
         <v>1421</v>
@@ -9721,7 +9721,7 @@
         <v>1417</v>
       </c>
       <c r="I129">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="K129" t="s">
         <v>1420</v>
@@ -9759,7 +9759,7 @@
         <v>1417</v>
       </c>
       <c r="I130">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="J130">
         <v>47</v>
@@ -9835,7 +9835,7 @@
         <v>1417</v>
       </c>
       <c r="I132">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="J132">
         <v>145</v>
@@ -9911,7 +9911,7 @@
         <v>1417</v>
       </c>
       <c r="I134">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="K134" t="s">
         <v>1420</v>
@@ -10036,7 +10036,7 @@
         <v>1417</v>
       </c>
       <c r="I138">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="K138" t="s">
         <v>1421</v>
@@ -10420,7 +10420,7 @@
         <v>1417</v>
       </c>
       <c r="I150">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="J150">
         <v>201</v>
@@ -10607,7 +10607,7 @@
         <v>1417</v>
       </c>
       <c r="I155">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="K155" t="s">
         <v>1427</v>
@@ -10642,7 +10642,7 @@
         <v>1417</v>
       </c>
       <c r="I156">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="K156" t="s">
         <v>1421</v>
@@ -10680,7 +10680,7 @@
         <v>1417</v>
       </c>
       <c r="I157">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="J157">
         <v>371</v>
@@ -10724,7 +10724,7 @@
         <v>1417</v>
       </c>
       <c r="I158">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="J158">
         <v>52</v>
@@ -10768,7 +10768,7 @@
         <v>1417</v>
       </c>
       <c r="I159">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="K159" t="s">
         <v>1421</v>
@@ -10806,7 +10806,7 @@
         <v>1417</v>
       </c>
       <c r="I160">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="K160" t="s">
         <v>1421</v>
@@ -10844,7 +10844,7 @@
         <v>1417</v>
       </c>
       <c r="I161">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="J161">
         <v>55</v>
@@ -10979,7 +10979,7 @@
         <v>1417</v>
       </c>
       <c r="I164">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="O164" t="s">
         <v>1533</v>
@@ -11154,7 +11154,7 @@
         <v>1417</v>
       </c>
       <c r="I169">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="K169" t="s">
         <v>1394</v>
@@ -11364,7 +11364,7 @@
         <v>1417</v>
       </c>
       <c r="I175">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="J175">
         <v>205</v>
@@ -11411,7 +11411,7 @@
         <v>1417</v>
       </c>
       <c r="I176">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="K176" t="s">
         <v>1421</v>
@@ -11449,7 +11449,7 @@
         <v>1417</v>
       </c>
       <c r="I177">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="J177">
         <v>44</v>
@@ -11496,7 +11496,7 @@
         <v>1417</v>
       </c>
       <c r="I178">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="K178" t="s">
         <v>1420</v>
@@ -11563,7 +11563,7 @@
         <v>1417</v>
       </c>
       <c r="I180">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="K180" t="s">
         <v>1420</v>
@@ -11659,7 +11659,7 @@
         <v>1417</v>
       </c>
       <c r="I183">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="K183" t="s">
         <v>1421</v>
@@ -11697,7 +11697,7 @@
         <v>1417</v>
       </c>
       <c r="I184">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="K184" t="s">
         <v>1427</v>
@@ -11732,7 +11732,7 @@
         <v>1417</v>
       </c>
       <c r="I185">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="K185" t="s">
         <v>1421</v>
@@ -11770,7 +11770,7 @@
         <v>1417</v>
       </c>
       <c r="I186">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="K186" t="s">
         <v>1421</v>
@@ -11808,7 +11808,7 @@
         <v>1417</v>
       </c>
       <c r="I187">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J187">
         <v>75</v>
@@ -11855,7 +11855,7 @@
         <v>1417</v>
       </c>
       <c r="I188">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="J188">
         <v>40</v>
@@ -11902,7 +11902,7 @@
         <v>1417</v>
       </c>
       <c r="I189">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="J189">
         <v>155</v>
@@ -11946,7 +11946,7 @@
         <v>1417</v>
       </c>
       <c r="I190">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="J190">
         <v>107</v>
@@ -11990,7 +11990,7 @@
         <v>1417</v>
       </c>
       <c r="I191">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="J191">
         <v>5</v>
@@ -12034,7 +12034,7 @@
         <v>1417</v>
       </c>
       <c r="I192">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="K192" t="s">
         <v>1421</v>
@@ -12072,7 +12072,7 @@
         <v>1417</v>
       </c>
       <c r="I193">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="K193" t="s">
         <v>1426</v>
@@ -12267,7 +12267,7 @@
         <v>1417</v>
       </c>
       <c r="I199">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="J199">
         <v>70</v>
@@ -12352,7 +12352,7 @@
         <v>1417</v>
       </c>
       <c r="I201">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="K201" t="s">
         <v>1421</v>
@@ -12390,7 +12390,7 @@
         <v>1417</v>
       </c>
       <c r="I202">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="K202" t="s">
         <v>1421</v>
@@ -12469,7 +12469,7 @@
         <v>1417</v>
       </c>
       <c r="I204">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="K204" t="s">
         <v>1420</v>
@@ -12507,7 +12507,7 @@
         <v>1417</v>
       </c>
       <c r="I205">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="K205" t="s">
         <v>1420</v>
@@ -12574,7 +12574,7 @@
         <v>1417</v>
       </c>
       <c r="I207">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="J207">
         <v>167</v>
@@ -12618,7 +12618,7 @@
         <v>1417</v>
       </c>
       <c r="I208">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="J208">
         <v>45</v>
@@ -12662,7 +12662,7 @@
         <v>1417</v>
       </c>
       <c r="I209">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="J209">
         <v>191</v>
@@ -12706,7 +12706,7 @@
         <v>1417</v>
       </c>
       <c r="I210">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="K210" t="s">
         <v>1424</v>
@@ -12802,7 +12802,7 @@
         <v>1417</v>
       </c>
       <c r="I213">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="K213" t="s">
         <v>1421</v>
@@ -12840,7 +12840,7 @@
         <v>1417</v>
       </c>
       <c r="I214">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="J214">
         <v>14</v>
@@ -12887,7 +12887,7 @@
         <v>1417</v>
       </c>
       <c r="I215">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="K215" t="s">
         <v>1421</v>
@@ -12954,7 +12954,7 @@
         <v>1417</v>
       </c>
       <c r="I217">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J217">
         <v>42</v>
@@ -12998,7 +12998,7 @@
         <v>1417</v>
       </c>
       <c r="I218">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J218">
         <v>166</v>
@@ -13086,7 +13086,7 @@
         <v>1417</v>
       </c>
       <c r="I220">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J220">
         <v>154</v>
@@ -13472,7 +13472,7 @@
         <v>1417</v>
       </c>
       <c r="I230">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="J230">
         <v>197</v>
@@ -13516,7 +13516,7 @@
         <v>1417</v>
       </c>
       <c r="I231">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="J231">
         <v>35</v>
@@ -13618,7 +13618,7 @@
         <v>1417</v>
       </c>
       <c r="I234">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="J234">
         <v>35</v>
@@ -13665,7 +13665,7 @@
         <v>1417</v>
       </c>
       <c r="I235">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="J235">
         <v>35</v>
@@ -13712,7 +13712,7 @@
         <v>1417</v>
       </c>
       <c r="I236">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="J236">
         <v>86</v>
@@ -13829,7 +13829,7 @@
         <v>1417</v>
       </c>
       <c r="I239">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="K239" t="s">
         <v>1394</v>
@@ -13928,7 +13928,7 @@
         <v>1417</v>
       </c>
       <c r="I242">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="K242" t="s">
         <v>1420</v>
@@ -13995,7 +13995,7 @@
         <v>1417</v>
       </c>
       <c r="I244">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="J244">
         <v>15</v>
@@ -14036,7 +14036,7 @@
         <v>1417</v>
       </c>
       <c r="I245">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="J245">
         <v>15</v>
@@ -14179,7 +14179,7 @@
         <v>1417</v>
       </c>
       <c r="I249">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="K249" t="s">
         <v>1421</v>
@@ -14313,7 +14313,7 @@
         <v>1417</v>
       </c>
       <c r="I253">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="J253">
         <v>162</v>
@@ -14357,7 +14357,7 @@
         <v>1417</v>
       </c>
       <c r="I254">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="K254" t="s">
         <v>1424</v>
@@ -14436,7 +14436,7 @@
         <v>1417</v>
       </c>
       <c r="I256">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="J256">
         <v>23</v>
@@ -14620,7 +14620,7 @@
         <v>1417</v>
       </c>
       <c r="I261">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="J261">
         <v>162</v>
@@ -14778,7 +14778,7 @@
         <v>1417</v>
       </c>
       <c r="I265">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="J265">
         <v>162</v>
@@ -14863,7 +14863,7 @@
         <v>1417</v>
       </c>
       <c r="I267">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="K267" t="s">
         <v>1424</v>
@@ -14901,7 +14901,7 @@
         <v>1417</v>
       </c>
       <c r="I268">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="K268" t="s">
         <v>1421</v>
@@ -14936,7 +14936,7 @@
         <v>1417</v>
       </c>
       <c r="I269">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="K269" t="s">
         <v>1421</v>
@@ -14974,7 +14974,7 @@
         <v>1417</v>
       </c>
       <c r="I270">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="K270" t="s">
         <v>1424</v>
@@ -15012,7 +15012,7 @@
         <v>1417</v>
       </c>
       <c r="I271">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="K271" t="s">
         <v>1424</v>
@@ -15190,7 +15190,7 @@
         <v>1417</v>
       </c>
       <c r="I276">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="K276" t="s">
         <v>1425</v>
@@ -15228,7 +15228,7 @@
         <v>1417</v>
       </c>
       <c r="I277">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="K277" t="s">
         <v>1421</v>
@@ -15266,7 +15266,7 @@
         <v>1417</v>
       </c>
       <c r="I278">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="J278">
         <v>148</v>
@@ -15310,7 +15310,7 @@
         <v>1417</v>
       </c>
       <c r="I279">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="K279" t="s">
         <v>1423</v>
@@ -15351,7 +15351,7 @@
         <v>1417</v>
       </c>
       <c r="I280">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="K280" t="s">
         <v>1421</v>
@@ -15389,7 +15389,7 @@
         <v>1417</v>
       </c>
       <c r="I281">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="K281" t="s">
         <v>1421</v>
@@ -15430,7 +15430,7 @@
         <v>1417</v>
       </c>
       <c r="I282">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="K282" t="s">
         <v>1421</v>
@@ -15724,7 +15724,7 @@
         <v>1417</v>
       </c>
       <c r="I291">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="J291">
         <v>20</v>
@@ -15768,7 +15768,7 @@
         <v>1417</v>
       </c>
       <c r="I292">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="K292" t="s">
         <v>1424</v>
@@ -15806,7 +15806,7 @@
         <v>1417</v>
       </c>
       <c r="I293">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="K293" t="s">
         <v>1425</v>
@@ -15844,7 +15844,7 @@
         <v>1417</v>
       </c>
       <c r="I294">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="K294" t="s">
         <v>1430</v>
@@ -15981,7 +15981,7 @@
         <v>1417</v>
       </c>
       <c r="I298">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="J298">
         <v>58</v>
@@ -16145,7 +16145,7 @@
         <v>1417</v>
       </c>
       <c r="I302">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="K302" t="s">
         <v>1424</v>
@@ -16183,7 +16183,7 @@
         <v>1417</v>
       </c>
       <c r="I303">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="K303" t="s">
         <v>1421</v>
@@ -16221,7 +16221,7 @@
         <v>1417</v>
       </c>
       <c r="I304">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="K304" t="s">
         <v>1424</v>
@@ -16259,7 +16259,7 @@
         <v>1417</v>
       </c>
       <c r="I305">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="J305">
         <v>35</v>
@@ -16303,7 +16303,7 @@
         <v>1417</v>
       </c>
       <c r="I306">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="J306">
         <v>31</v>
@@ -16391,7 +16391,7 @@
         <v>1417</v>
       </c>
       <c r="I308">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="K308" t="s">
         <v>1420</v>
@@ -16508,7 +16508,7 @@
         <v>1417</v>
       </c>
       <c r="I311">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="K311" t="s">
         <v>1420</v>
@@ -16838,7 +16838,7 @@
         <v>1417</v>
       </c>
       <c r="I320">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="K320" t="s">
         <v>1425</v>
@@ -16876,7 +16876,7 @@
         <v>1417</v>
       </c>
       <c r="I321">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="K321" t="s">
         <v>1421</v>
@@ -16914,7 +16914,7 @@
         <v>1417</v>
       </c>
       <c r="I322">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="J322">
         <v>57</v>
@@ -17028,7 +17028,7 @@
         <v>1417</v>
       </c>
       <c r="I325">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="J325">
         <v>57</v>
@@ -17110,7 +17110,7 @@
         <v>1417</v>
       </c>
       <c r="I327">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="J327">
         <v>57</v>
@@ -17154,7 +17154,7 @@
         <v>1417</v>
       </c>
       <c r="I328">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="J328">
         <v>57</v>
@@ -17198,7 +17198,7 @@
         <v>1417</v>
       </c>
       <c r="I329">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="J329">
         <v>57</v>
@@ -17242,7 +17242,7 @@
         <v>1417</v>
       </c>
       <c r="I330">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="J330">
         <v>57</v>
@@ -17286,7 +17286,7 @@
         <v>1417</v>
       </c>
       <c r="I331">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="K331" t="s">
         <v>1420</v>
@@ -17324,7 +17324,7 @@
         <v>1417</v>
       </c>
       <c r="I332">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="K332" t="s">
         <v>1421</v>
@@ -17362,7 +17362,7 @@
         <v>1417</v>
       </c>
       <c r="I333">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="J333">
         <v>100</v>
@@ -17406,7 +17406,7 @@
         <v>1417</v>
       </c>
       <c r="I334">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="K334" t="s">
         <v>1421</v>
@@ -17631,7 +17631,7 @@
         <v>1417</v>
       </c>
       <c r="I340">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="J340">
         <v>98</v>
@@ -17672,7 +17672,7 @@
         <v>1417</v>
       </c>
       <c r="I341">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="J341">
         <v>90</v>
@@ -17713,7 +17713,7 @@
         <v>1417</v>
       </c>
       <c r="I342">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="K342" t="s">
         <v>1420</v>
@@ -17827,7 +17827,7 @@
         <v>1417</v>
       </c>
       <c r="I345">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="K345" t="s">
         <v>1420</v>
@@ -17947,7 +17947,7 @@
         <v>1417</v>
       </c>
       <c r="I348">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="J348">
         <v>14</v>
@@ -17991,7 +17991,7 @@
         <v>1417</v>
       </c>
       <c r="I349">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="K349" t="s">
         <v>1425</v>
@@ -18029,7 +18029,7 @@
         <v>1417</v>
       </c>
       <c r="I350">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="J350">
         <v>46</v>
@@ -18067,7 +18067,7 @@
         <v>1417</v>
       </c>
       <c r="I351">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="J351">
         <v>82</v>
@@ -18111,7 +18111,7 @@
         <v>1417</v>
       </c>
       <c r="I352">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="J352">
         <v>78</v>
@@ -18155,7 +18155,7 @@
         <v>1417</v>
       </c>
       <c r="I353">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="J353">
         <v>83</v>
@@ -18199,7 +18199,7 @@
         <v>1417</v>
       </c>
       <c r="I354">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="K354" t="s">
         <v>1424</v>
@@ -18237,7 +18237,7 @@
         <v>1417</v>
       </c>
       <c r="I355">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="J355">
         <v>8</v>
@@ -18319,7 +18319,7 @@
         <v>1417</v>
       </c>
       <c r="I357">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="J357">
         <v>85</v>
@@ -18442,7 +18442,7 @@
         <v>1417</v>
       </c>
       <c r="I360">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="J360">
         <v>83</v>
@@ -18489,7 +18489,7 @@
         <v>1417</v>
       </c>
       <c r="I361">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="J361">
         <v>83</v>
@@ -18533,7 +18533,7 @@
         <v>1417</v>
       </c>
       <c r="I362">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="K362" t="s">
         <v>1424</v>
@@ -18571,7 +18571,7 @@
         <v>1417</v>
       </c>
       <c r="I363">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="K363" t="s">
         <v>1424</v>
@@ -18609,7 +18609,7 @@
         <v>1417</v>
       </c>
       <c r="I364">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="J364">
         <v>83</v>
@@ -18653,7 +18653,7 @@
         <v>1417</v>
       </c>
       <c r="I365">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="J365">
         <v>15</v>
@@ -18776,7 +18776,7 @@
         <v>1417</v>
       </c>
       <c r="I368">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="J368">
         <v>77</v>
@@ -18820,7 +18820,7 @@
         <v>1417</v>
       </c>
       <c r="I369">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="K369" t="s">
         <v>1424</v>
@@ -18858,7 +18858,7 @@
         <v>1417</v>
       </c>
       <c r="I370">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="K370" t="s">
         <v>1424</v>
@@ -18896,7 +18896,7 @@
         <v>1417</v>
       </c>
       <c r="I371">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="J371">
         <v>16</v>
@@ -18984,7 +18984,7 @@
         <v>1417</v>
       </c>
       <c r="I373">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K373" t="s">
         <v>1420</v>
@@ -19022,7 +19022,7 @@
         <v>1417</v>
       </c>
       <c r="I374">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K374" t="s">
         <v>1420</v>
@@ -19060,7 +19060,7 @@
         <v>1417</v>
       </c>
       <c r="I375">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="J375">
         <v>94</v>
@@ -19101,7 +19101,7 @@
         <v>1417</v>
       </c>
       <c r="I376">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="K376" t="s">
         <v>1424</v>
@@ -19180,7 +19180,7 @@
         <v>1417</v>
       </c>
       <c r="I378">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="K378" t="s">
         <v>1424</v>
@@ -19218,7 +19218,7 @@
         <v>1417</v>
       </c>
       <c r="I379">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="J379">
         <v>20</v>
@@ -19262,7 +19262,7 @@
         <v>1417</v>
       </c>
       <c r="I380">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="J380">
         <v>94</v>
@@ -19306,7 +19306,7 @@
         <v>1417</v>
       </c>
       <c r="I381">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="K381" t="s">
         <v>1424</v>
@@ -19344,7 +19344,7 @@
         <v>1417</v>
       </c>
       <c r="I382">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="K382" t="s">
         <v>1424</v>
@@ -19382,7 +19382,7 @@
         <v>1417</v>
       </c>
       <c r="I383">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="J383">
         <v>71</v>
@@ -19426,7 +19426,7 @@
         <v>1417</v>
       </c>
       <c r="I384">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="K384" t="s">
         <v>1421</v>
@@ -19508,7 +19508,7 @@
         <v>1417</v>
       </c>
       <c r="I386">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="K386" t="s">
         <v>1424</v>
@@ -19546,7 +19546,7 @@
         <v>1417</v>
       </c>
       <c r="I387">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="K387" t="s">
         <v>1424</v>
@@ -19584,7 +19584,7 @@
         <v>1417</v>
       </c>
       <c r="I388">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J388">
         <v>-85</v>
@@ -19628,7 +19628,7 @@
         <v>1417</v>
       </c>
       <c r="I389">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="K389" t="s">
         <v>1425</v>
@@ -20079,7 +20079,7 @@
         <v>1417</v>
       </c>
       <c r="I400">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="K400" t="s">
         <v>1424</v>
@@ -20155,7 +20155,7 @@
         <v>1417</v>
       </c>
       <c r="I402">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="K402" t="s">
         <v>1424</v>
@@ -20193,7 +20193,7 @@
         <v>1417</v>
       </c>
       <c r="I403">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J403">
         <v>83</v>
@@ -20237,7 +20237,7 @@
         <v>1417</v>
       </c>
       <c r="I404">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="K404" t="s">
         <v>1424</v>
@@ -20307,7 +20307,7 @@
         <v>1417</v>
       </c>
       <c r="I406">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="Q406" t="b">
         <v>1</v>
@@ -20339,7 +20339,7 @@
         <v>1417</v>
       </c>
       <c r="I407">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="Q407" t="b">
         <v>1</v>
@@ -20371,7 +20371,7 @@
         <v>1417</v>
       </c>
       <c r="I408">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="Q408" t="b">
         <v>1</v>
@@ -20403,7 +20403,7 @@
         <v>1417</v>
       </c>
       <c r="I409">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="Q409" t="b">
         <v>1</v>
@@ -20435,7 +20435,7 @@
         <v>1417</v>
       </c>
       <c r="I410">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="Q410" t="b">
         <v>1</v>
@@ -20467,7 +20467,7 @@
         <v>1417</v>
       </c>
       <c r="I411">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="Q411" t="b">
         <v>1</v>
@@ -20499,7 +20499,7 @@
         <v>1417</v>
       </c>
       <c r="I412">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="Q412" t="b">
         <v>1</v>
@@ -20531,7 +20531,7 @@
         <v>1417</v>
       </c>
       <c r="I413">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="Q413" t="b">
         <v>1</v>
@@ -20621,7 +20621,7 @@
         <v>1417</v>
       </c>
       <c r="I416">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="Q416" t="b">
         <v>1</v>
@@ -20711,7 +20711,7 @@
         <v>1417</v>
       </c>
       <c r="I419">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="Q419" t="b">
         <v>1</v>
@@ -20743,7 +20743,7 @@
         <v>1417</v>
       </c>
       <c r="I420">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="Q420" t="b">
         <v>1</v>
@@ -20775,7 +20775,7 @@
         <v>1417</v>
       </c>
       <c r="I421">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="Q421" t="b">
         <v>1</v>
@@ -20807,7 +20807,7 @@
         <v>1417</v>
       </c>
       <c r="I422">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="Q422" t="b">
         <v>1</v>
@@ -20839,7 +20839,7 @@
         <v>1417</v>
       </c>
       <c r="I423">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="Q423" t="b">
         <v>1</v>
@@ -20871,7 +20871,7 @@
         <v>1417</v>
       </c>
       <c r="I424">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="Q424" t="b">
         <v>1</v>
@@ -20903,7 +20903,7 @@
         <v>1417</v>
       </c>
       <c r="I425">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="Q425" t="b">
         <v>1</v>
@@ -20935,7 +20935,7 @@
         <v>1417</v>
       </c>
       <c r="I426">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="Q426" t="b">
         <v>1</v>
@@ -20967,7 +20967,7 @@
         <v>1417</v>
       </c>
       <c r="I427">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="Q427" t="b">
         <v>1</v>
@@ -21057,7 +21057,7 @@
         <v>1417</v>
       </c>
       <c r="I430">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="Q430" t="b">
         <v>1</v>
@@ -21089,7 +21089,7 @@
         <v>1417</v>
       </c>
       <c r="I431">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="Q431" t="b">
         <v>1</v>
@@ -21121,7 +21121,7 @@
         <v>1417</v>
       </c>
       <c r="I432">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="Q432" t="b">
         <v>1</v>
@@ -21153,7 +21153,7 @@
         <v>1417</v>
       </c>
       <c r="I433">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="Q433" t="b">
         <v>1</v>
@@ -21185,7 +21185,7 @@
         <v>1417</v>
       </c>
       <c r="I434">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="Q434" t="b">
         <v>1</v>
@@ -21217,7 +21217,7 @@
         <v>1417</v>
       </c>
       <c r="I435">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="Q435" t="b">
         <v>1</v>
@@ -21249,7 +21249,7 @@
         <v>1417</v>
       </c>
       <c r="I436">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="Q436" t="b">
         <v>1</v>
@@ -21281,7 +21281,7 @@
         <v>1419</v>
       </c>
       <c r="I437">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="Q437" t="b">
         <v>1</v>
@@ -21313,7 +21313,7 @@
         <v>1419</v>
       </c>
       <c r="I438">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="Q438" t="b">
         <v>1</v>
@@ -21345,7 +21345,7 @@
         <v>1417</v>
       </c>
       <c r="I439">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="Q439" t="b">
         <v>1</v>
@@ -21377,7 +21377,7 @@
         <v>1417</v>
       </c>
       <c r="I440">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="Q440" t="b">
         <v>1</v>
@@ -21409,7 +21409,7 @@
         <v>1417</v>
       </c>
       <c r="I441">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="Q441" t="b">
         <v>1</v>
@@ -21470,7 +21470,7 @@
         <v>1417</v>
       </c>
       <c r="I443">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="Q443" t="b">
         <v>1</v>
@@ -21560,7 +21560,7 @@
         <v>1417</v>
       </c>
       <c r="I446">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="Q446" t="b">
         <v>1</v>
@@ -21592,7 +21592,7 @@
         <v>1417</v>
       </c>
       <c r="I447">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="Q447" t="b">
         <v>1</v>
@@ -21624,7 +21624,7 @@
         <v>1417</v>
       </c>
       <c r="I448">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="Q448" t="b">
         <v>1</v>
@@ -21656,7 +21656,7 @@
         <v>1417</v>
       </c>
       <c r="I449">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="Q449" t="b">
         <v>1</v>
@@ -21688,7 +21688,7 @@
         <v>1417</v>
       </c>
       <c r="I450">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="Q450" t="b">
         <v>1</v>
@@ -21720,7 +21720,7 @@
         <v>1417</v>
       </c>
       <c r="I451">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="Q451" t="b">
         <v>1</v>
@@ -21781,7 +21781,7 @@
         <v>1417</v>
       </c>
       <c r="I453">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="Q453" t="b">
         <v>1</v>
@@ -21813,7 +21813,7 @@
         <v>1417</v>
       </c>
       <c r="I454">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="Q454" t="b">
         <v>1</v>
@@ -21845,7 +21845,7 @@
         <v>1417</v>
       </c>
       <c r="I455">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="Q455" t="b">
         <v>1</v>
@@ -21906,7 +21906,7 @@
         <v>1417</v>
       </c>
       <c r="I457">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="Q457" t="b">
         <v>1</v>
@@ -21938,7 +21938,7 @@
         <v>1417</v>
       </c>
       <c r="I458">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="Q458" t="b">
         <v>1</v>
@@ -21970,7 +21970,7 @@
         <v>1417</v>
       </c>
       <c r="I459">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q459" t="b">
         <v>1</v>
@@ -22002,7 +22002,7 @@
         <v>1417</v>
       </c>
       <c r="I460">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q460" t="b">
         <v>1</v>
@@ -22034,7 +22034,7 @@
         <v>1417</v>
       </c>
       <c r="I461">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q461" t="b">
         <v>1</v>
@@ -22066,7 +22066,7 @@
         <v>1417</v>
       </c>
       <c r="I462">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q462" t="b">
         <v>1</v>
@@ -22098,7 +22098,7 @@
         <v>1417</v>
       </c>
       <c r="I463">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="Q463" t="b">
         <v>1</v>
@@ -22130,7 +22130,7 @@
         <v>1417</v>
       </c>
       <c r="I464">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="Q464" t="b">
         <v>1</v>
@@ -22162,7 +22162,7 @@
         <v>1417</v>
       </c>
       <c r="I465">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="Q465" t="b">
         <v>1</v>
@@ -22194,7 +22194,7 @@
         <v>1417</v>
       </c>
       <c r="I466">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="Q466" t="b">
         <v>1</v>
@@ -22226,7 +22226,7 @@
         <v>1417</v>
       </c>
       <c r="I467">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="Q467" t="b">
         <v>1</v>
@@ -22258,7 +22258,7 @@
         <v>1417</v>
       </c>
       <c r="I468">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="Q468" t="b">
         <v>1</v>
@@ -22290,7 +22290,7 @@
         <v>1417</v>
       </c>
       <c r="I469">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="Q469" t="b">
         <v>1</v>
@@ -22351,7 +22351,7 @@
         <v>1417</v>
       </c>
       <c r="I471">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="Q471" t="b">
         <v>1</v>
@@ -22383,7 +22383,7 @@
         <v>1417</v>
       </c>
       <c r="I472">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="Q472" t="b">
         <v>1</v>
@@ -22415,7 +22415,7 @@
         <v>1417</v>
       </c>
       <c r="I473">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="Q473" t="b">
         <v>1</v>
@@ -22447,7 +22447,7 @@
         <v>1417</v>
       </c>
       <c r="I474">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="Q474" t="b">
         <v>1</v>
@@ -22479,7 +22479,7 @@
         <v>1417</v>
       </c>
       <c r="I475">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="Q475" t="b">
         <v>1</v>
@@ -22511,7 +22511,7 @@
         <v>1417</v>
       </c>
       <c r="I476">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="Q476" t="b">
         <v>1</v>
@@ -22543,7 +22543,7 @@
         <v>1417</v>
       </c>
       <c r="I477">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="Q477" t="b">
         <v>1</v>
@@ -22575,7 +22575,7 @@
         <v>1417</v>
       </c>
       <c r="I478">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="Q478" t="b">
         <v>1</v>
@@ -22607,7 +22607,7 @@
         <v>1417</v>
       </c>
       <c r="I479">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="Q479" t="b">
         <v>1</v>
@@ -22639,7 +22639,7 @@
         <v>1417</v>
       </c>
       <c r="I480">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="Q480" t="b">
         <v>1</v>
@@ -22671,7 +22671,7 @@
         <v>1417</v>
       </c>
       <c r="I481">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="Q481" t="b">
         <v>1</v>
@@ -22703,7 +22703,7 @@
         <v>1417</v>
       </c>
       <c r="I482">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="Q482" t="b">
         <v>1</v>
@@ -22735,7 +22735,7 @@
         <v>1417</v>
       </c>
       <c r="I483">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="Q483" t="b">
         <v>1</v>
@@ -22767,7 +22767,7 @@
         <v>1417</v>
       </c>
       <c r="I484">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="Q484" t="b">
         <v>1</v>
@@ -22799,7 +22799,7 @@
         <v>1417</v>
       </c>
       <c r="I485">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="Q485" t="b">
         <v>1</v>
@@ -22831,7 +22831,7 @@
         <v>1417</v>
       </c>
       <c r="I486">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="Q486" t="b">
         <v>1</v>
@@ -22863,7 +22863,7 @@
         <v>1417</v>
       </c>
       <c r="I487">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="Q487" t="b">
         <v>1</v>
@@ -22895,7 +22895,7 @@
         <v>1417</v>
       </c>
       <c r="I488">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="Q488" t="b">
         <v>1</v>
@@ -22927,7 +22927,7 @@
         <v>1417</v>
       </c>
       <c r="I489">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="Q489" t="b">
         <v>1</v>
@@ -22959,7 +22959,7 @@
         <v>1417</v>
       </c>
       <c r="I490">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="Q490" t="b">
         <v>1</v>
@@ -22991,7 +22991,7 @@
         <v>1417</v>
       </c>
       <c r="I491">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="Q491" t="b">
         <v>1</v>
@@ -23023,7 +23023,7 @@
         <v>1419</v>
       </c>
       <c r="I492">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="Q492" t="b">
         <v>1</v>
@@ -23055,7 +23055,7 @@
         <v>1419</v>
       </c>
       <c r="I493">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="Q493" t="b">
         <v>1</v>
@@ -23087,7 +23087,7 @@
         <v>1419</v>
       </c>
       <c r="I494">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="Q494" t="b">
         <v>1</v>
@@ -23119,7 +23119,7 @@
         <v>1419</v>
       </c>
       <c r="I495">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="Q495" t="b">
         <v>1</v>
@@ -23151,7 +23151,7 @@
         <v>1419</v>
       </c>
       <c r="I496">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="Q496" t="b">
         <v>1</v>
@@ -23183,7 +23183,7 @@
         <v>1417</v>
       </c>
       <c r="I497">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="Q497" t="b">
         <v>1</v>
@@ -23215,7 +23215,7 @@
         <v>1417</v>
       </c>
       <c r="I498">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="Q498" t="b">
         <v>1</v>
@@ -23247,7 +23247,7 @@
         <v>1419</v>
       </c>
       <c r="I499">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="Q499" t="b">
         <v>1</v>
@@ -23279,7 +23279,7 @@
         <v>1417</v>
       </c>
       <c r="I500">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="Q500" t="b">
         <v>1</v>
@@ -23311,7 +23311,7 @@
         <v>1417</v>
       </c>
       <c r="I501">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="Q501" t="b">
         <v>1</v>
@@ -23343,7 +23343,7 @@
         <v>1417</v>
       </c>
       <c r="I502">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="Q502" t="b">
         <v>1</v>
@@ -23375,7 +23375,7 @@
         <v>1417</v>
       </c>
       <c r="I503">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="Q503" t="b">
         <v>1</v>
@@ -23407,7 +23407,7 @@
         <v>1417</v>
       </c>
       <c r="I504">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q504" t="b">
         <v>1</v>
@@ -23439,7 +23439,7 @@
         <v>1417</v>
       </c>
       <c r="I505">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q505" t="b">
         <v>1</v>
@@ -23471,7 +23471,7 @@
         <v>1417</v>
       </c>
       <c r="I506">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q506" t="b">
         <v>1</v>
@@ -23503,7 +23503,7 @@
         <v>1417</v>
       </c>
       <c r="I507">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="Q507" t="b">
         <v>1</v>
@@ -23564,7 +23564,7 @@
         <v>1417</v>
       </c>
       <c r="I509">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="Q509" t="b">
         <v>1</v>
@@ -23596,7 +23596,7 @@
         <v>1417</v>
       </c>
       <c r="I510">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="Q510" t="b">
         <v>1</v>
@@ -23628,7 +23628,7 @@
         <v>1417</v>
       </c>
       <c r="I511">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q511" t="b">
         <v>1</v>
@@ -23660,7 +23660,7 @@
         <v>1417</v>
       </c>
       <c r="I512">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q512" t="b">
         <v>1</v>
@@ -23692,7 +23692,7 @@
         <v>1417</v>
       </c>
       <c r="I513">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="Q513" t="b">
         <v>1</v>
@@ -23753,7 +23753,7 @@
         <v>1417</v>
       </c>
       <c r="I515">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="Q515" t="b">
         <v>1</v>
@@ -23785,7 +23785,7 @@
         <v>1417</v>
       </c>
       <c r="I516">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q516" t="b">
         <v>1</v>
@@ -23817,7 +23817,7 @@
         <v>1417</v>
       </c>
       <c r="I517">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q517" t="b">
         <v>1</v>
@@ -23849,7 +23849,7 @@
         <v>1417</v>
       </c>
       <c r="I518">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q518" t="b">
         <v>1</v>
@@ -23881,7 +23881,7 @@
         <v>1417</v>
       </c>
       <c r="I519">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="Q519" t="b">
         <v>1</v>
@@ -23913,7 +23913,7 @@
         <v>1417</v>
       </c>
       <c r="I520">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="Q520" t="b">
         <v>1</v>
@@ -23945,7 +23945,7 @@
         <v>1417</v>
       </c>
       <c r="I521">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="Q521" t="b">
         <v>1</v>
@@ -23977,7 +23977,7 @@
         <v>1417</v>
       </c>
       <c r="I522">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="Q522" t="b">
         <v>1</v>
@@ -24009,7 +24009,7 @@
         <v>1417</v>
       </c>
       <c r="I523">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="Q523" t="b">
         <v>1</v>
@@ -24041,7 +24041,7 @@
         <v>1417</v>
       </c>
       <c r="I524">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="Q524" t="b">
         <v>1</v>
@@ -24073,7 +24073,7 @@
         <v>1417</v>
       </c>
       <c r="I525">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="Q525" t="b">
         <v>1</v>
@@ -24105,7 +24105,7 @@
         <v>1417</v>
       </c>
       <c r="I526">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="Q526" t="b">
         <v>1</v>
@@ -24137,7 +24137,7 @@
         <v>1417</v>
       </c>
       <c r="I527">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="Q527" t="b">
         <v>1</v>
@@ -24169,7 +24169,7 @@
         <v>1417</v>
       </c>
       <c r="I528">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="Q528" t="b">
         <v>1</v>
@@ -24201,7 +24201,7 @@
         <v>1417</v>
       </c>
       <c r="I529">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q529" t="b">
         <v>1</v>
@@ -24233,7 +24233,7 @@
         <v>1417</v>
       </c>
       <c r="I530">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q530" t="b">
         <v>1</v>
@@ -24265,7 +24265,7 @@
         <v>1417</v>
       </c>
       <c r="I531">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q531" t="b">
         <v>1</v>
@@ -24297,7 +24297,7 @@
         <v>1417</v>
       </c>
       <c r="I532">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q532" t="b">
         <v>1</v>
@@ -24329,7 +24329,7 @@
         <v>1417</v>
       </c>
       <c r="I533">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q533" t="b">
         <v>1</v>
@@ -24361,7 +24361,7 @@
         <v>1417</v>
       </c>
       <c r="I534">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q534" t="b">
         <v>1</v>
@@ -24393,7 +24393,7 @@
         <v>1417</v>
       </c>
       <c r="I535">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q535" t="b">
         <v>1</v>
@@ -24425,7 +24425,7 @@
         <v>1417</v>
       </c>
       <c r="I536">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q536" t="b">
         <v>1</v>
@@ -24457,7 +24457,7 @@
         <v>1417</v>
       </c>
       <c r="I537">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q537" t="b">
         <v>1</v>
@@ -24489,7 +24489,7 @@
         <v>1417</v>
       </c>
       <c r="I538">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q538" t="b">
         <v>1</v>
@@ -24521,7 +24521,7 @@
         <v>1417</v>
       </c>
       <c r="I539">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q539" t="b">
         <v>1</v>
@@ -24553,7 +24553,7 @@
         <v>1417</v>
       </c>
       <c r="I540">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q540" t="b">
         <v>1</v>
@@ -24585,7 +24585,7 @@
         <v>1417</v>
       </c>
       <c r="I541">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q541" t="b">
         <v>1</v>
@@ -24617,7 +24617,7 @@
         <v>1417</v>
       </c>
       <c r="I542">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q542" t="b">
         <v>1</v>
@@ -24649,7 +24649,7 @@
         <v>1417</v>
       </c>
       <c r="I543">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q543" t="b">
         <v>1</v>
@@ -24681,7 +24681,7 @@
         <v>1417</v>
       </c>
       <c r="I544">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q544" t="b">
         <v>1</v>
@@ -24713,7 +24713,7 @@
         <v>1417</v>
       </c>
       <c r="I545">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q545" t="b">
         <v>1</v>
@@ -24745,7 +24745,7 @@
         <v>1417</v>
       </c>
       <c r="I546">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q546" t="b">
         <v>1</v>
@@ -24777,7 +24777,7 @@
         <v>1417</v>
       </c>
       <c r="I547">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q547" t="b">
         <v>1</v>
@@ -24809,7 +24809,7 @@
         <v>1417</v>
       </c>
       <c r="I548">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q548" t="b">
         <v>1</v>
@@ -24841,7 +24841,7 @@
         <v>1417</v>
       </c>
       <c r="I549">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q549" t="b">
         <v>1</v>
@@ -24873,7 +24873,7 @@
         <v>1417</v>
       </c>
       <c r="I550">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q550" t="b">
         <v>1</v>
@@ -24905,7 +24905,7 @@
         <v>1417</v>
       </c>
       <c r="I551">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q551" t="b">
         <v>1</v>
@@ -24937,7 +24937,7 @@
         <v>1417</v>
       </c>
       <c r="I552">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q552" t="b">
         <v>1</v>
@@ -24969,7 +24969,7 @@
         <v>1417</v>
       </c>
       <c r="I553">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q553" t="b">
         <v>1</v>
@@ -25001,7 +25001,7 @@
         <v>1417</v>
       </c>
       <c r="I554">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q554" t="b">
         <v>1</v>
@@ -25033,7 +25033,7 @@
         <v>1417</v>
       </c>
       <c r="I555">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q555" t="b">
         <v>1</v>
@@ -25065,7 +25065,7 @@
         <v>1417</v>
       </c>
       <c r="I556">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q556" t="b">
         <v>1</v>
@@ -25097,7 +25097,7 @@
         <v>1417</v>
       </c>
       <c r="I557">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Q557" t="b">
         <v>1</v>
@@ -25129,7 +25129,7 @@
         <v>1417</v>
       </c>
       <c r="I558">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Q558" t="b">
         <v>1</v>

</xml_diff>